<commit_message>
Add Section A: market size, firm concentration metrics and growth drivers
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01Tu61bPEQej1E6sErbEFanY
</commit_message>
<xml_diff>
--- a/research/swedish_legal_market.xlsx
+++ b/research/swedish_legal_market.xlsx
@@ -7,11 +7,14 @@
     <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" tabRatio="600" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
   </bookViews>
   <sheets>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="B. Practice rankings" sheetId="1" state="visible" r:id="rId1"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="B. Rankings raw" sheetId="2" state="visible" r:id="rId2"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="A. Market size" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="A. Firms" sheetId="2" state="visible" r:id="rId2"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="A. Growth drivers" sheetId="3" state="visible" r:id="rId3"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="B. Practice rankings" sheetId="4" state="visible" r:id="rId4"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="B. Rankings raw" sheetId="5" state="visible" r:id="rId5"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'B. Rankings raw'!$A$1:$E$661</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="4" hidden="1">'B. Rankings raw'!$A$1:$E$661</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -19,8 +22,10 @@
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <numFmts count="0"/>
-  <fonts count="7">
+  <numFmts count="1">
+    <numFmt numFmtId="164" formatCode="0.0"/>
+  </numFmts>
+  <fonts count="8">
     <font>
       <name val="Calibri"/>
       <family val="2"/>
@@ -47,6 +52,10 @@
     <font>
       <i val="1"/>
       <sz val="9"/>
+    </font>
+    <font>
+      <b val="1"/>
+      <sz val="11"/>
     </font>
   </fonts>
   <fills count="10">
@@ -277,7 +286,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="47">
+  <cellXfs count="63">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
@@ -393,6 +402,44 @@
     </xf>
     <xf numFmtId="0" fontId="6" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="5" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="7" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="2" fillId="2" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="3" fontId="2" fillId="2" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="3" fontId="0" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="2" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="top"/>
+    </xf>
+    <xf numFmtId="3" fontId="0" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="top"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="5" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="top"/>
+    </xf>
+    <xf numFmtId="164" fontId="0" fillId="0" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="0" fillId="5" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="3" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="9" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="top"/>
+    </xf>
+    <xf numFmtId="3" fontId="0" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="top"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="5" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="top"/>
+    </xf>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0" hidden="0"/>
@@ -758,6 +805,2312 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
+  <dimension ref="A1:E24"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="58" customWidth="1" min="1" max="1"/>
+    <col width="40" customWidth="1" min="2" max="2"/>
+    <col width="20" customWidth="1" min="3" max="3"/>
+    <col width="24" customWidth="1" min="4" max="4"/>
+    <col width="20" customWidth="1" min="5" max="5"/>
+  </cols>
+  <sheetData>
+    <row r="1">
+      <c r="A1" s="1" t="inlineStr">
+        <is>
+          <t>Section A. Swedish (corporate) legal market: size</t>
+        </is>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" s="47" t="inlineStr">
+        <is>
+          <t>A1. Headline estimates</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" s="48" t="inlineStr">
+        <is>
+          <t>Scope</t>
+        </is>
+      </c>
+      <c r="B4" s="48" t="inlineStr">
+        <is>
+          <t>Figure</t>
+        </is>
+      </c>
+      <c r="C4" s="48" t="inlineStr">
+        <is>
+          <t>Year</t>
+        </is>
+      </c>
+      <c r="D4" s="48" t="inlineStr">
+        <is>
+          <t>Source</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" s="49" t="inlineStr">
+        <is>
+          <t>Business law: fee income, 56 largest firms (Affärsvärlden panel)</t>
+        </is>
+      </c>
+      <c r="B5" s="49" t="inlineStr">
+        <is>
+          <t>~SEK 16bn (+5.3%)</t>
+        </is>
+      </c>
+      <c r="C5" s="49" t="inlineStr">
+        <is>
+          <t>2025</t>
+        </is>
+      </c>
+      <c r="D5" s="49" t="inlineStr">
+        <is>
+          <t>https://www.affarsvarlden.se/artikel/affarsjuridiken-vaxer-igen-men-jattarna-tappar-mark</t>
+        </is>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" s="49" t="inlineStr">
+        <is>
+          <t>Same panel, prior year (revised Oct-25, split FYs)</t>
+        </is>
+      </c>
+      <c r="B6" s="49" t="inlineStr">
+        <is>
+          <t>SEK 15.4bn (+8.6%); SEK 4.13m fee per lawyer</t>
+        </is>
+      </c>
+      <c r="C6" s="49" t="inlineStr">
+        <is>
+          <t>2024</t>
+        </is>
+      </c>
+      <c r="D6" s="49" t="inlineStr">
+        <is>
+          <t>https://www.realtid.se/affarer/154-miljarder-sa-klarade-affarsjuristerna-tullchocken/</t>
+        </is>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" s="49" t="inlineStr">
+        <is>
+          <t>Business law market, total (industry estimate, method not given)</t>
+        </is>
+      </c>
+      <c r="B7" s="49" t="inlineStr">
+        <is>
+          <t>&gt;SEK 25bn p.a.</t>
+        </is>
+      </c>
+      <c r="C7" s="49" t="inlineStr">
+        <is>
+          <t>n/a</t>
+        </is>
+      </c>
+      <c r="D7" s="49" t="inlineStr">
+        <is>
+          <t>https://www.affarsvarlden.se/debatt/okad-konkurrens-starker-svensk-affarsjuridik</t>
+        </is>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" s="49" t="inlineStr">
+        <is>
+          <t>All legal services (MarketLine)</t>
+        </is>
+      </c>
+      <c r="B8" s="49" t="inlineStr">
+        <is>
+          <t>USD 3.1bn (CAGR 5.9% 2019-24)</t>
+        </is>
+      </c>
+      <c r="C8" s="49" t="inlineStr">
+        <is>
+          <t>2024</t>
+        </is>
+      </c>
+      <c r="D8" s="49" t="inlineStr">
+        <is>
+          <t>https://store.marketline.com/report/legal-services-in-sweden/</t>
+        </is>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" s="49" t="inlineStr">
+        <is>
+          <t>All legal activities (IBISWorld)</t>
+        </is>
+      </c>
+      <c r="B9" s="49" t="inlineStr">
+        <is>
+          <t>EUR 3.5bn (CAGR -0.5% 2020-25)</t>
+        </is>
+      </c>
+      <c r="C9" s="49" t="inlineStr">
+        <is>
+          <t>2026e</t>
+        </is>
+      </c>
+      <c r="D9" s="49" t="inlineStr">
+        <is>
+          <t>https://www.ibisworld.com/sweden/industry/legal-activities/200283/</t>
+        </is>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" s="49" t="inlineStr">
+        <is>
+          <t>All law firms (advokatbyråer), estimate from SCB</t>
+        </is>
+      </c>
+      <c r="B10" s="49" t="inlineStr">
+        <is>
+          <t>~SEK 29bn</t>
+        </is>
+      </c>
+      <c r="C10" s="49" t="inlineStr">
+        <is>
+          <t>2024e</t>
+        </is>
+      </c>
+      <c r="D10" s="49" t="inlineStr">
+        <is>
+          <t>74.5% share of SNI 69.1 in 2021 applied to 2024 (SCB, below)</t>
+        </is>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" s="47" t="inlineStr">
+        <is>
+          <t>A2. Official statistics: SCB Företagens ekonomi, net turnover (SEK m)</t>
+        </is>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" s="48" t="inlineStr">
+        <is>
+          <t>Year</t>
+        </is>
+      </c>
+      <c r="B13" s="50" t="inlineStr">
+        <is>
+          <t>69.1 Legal activities (total)</t>
+        </is>
+      </c>
+      <c r="C13" s="50" t="inlineStr">
+        <is>
+          <t>69.101 Advokatbyråer</t>
+        </is>
+      </c>
+      <c r="D13" s="50" t="inlineStr">
+        <is>
+          <t>69.102 Other legal offices</t>
+        </is>
+      </c>
+      <c r="E13" s="50" t="inlineStr">
+        <is>
+          <t>69.103 Patent agents</t>
+        </is>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" s="49" t="n">
+        <v>2010</v>
+      </c>
+      <c r="B14" s="51" t="n">
+        <v>18738</v>
+      </c>
+      <c r="C14" s="51" t="n">
+        <v>13904</v>
+      </c>
+      <c r="D14" s="51" t="n">
+        <v>1956</v>
+      </c>
+      <c r="E14" s="51" t="n">
+        <v>2879</v>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" s="49" t="n">
+        <v>2015</v>
+      </c>
+      <c r="B15" s="51" t="n">
+        <v>23986</v>
+      </c>
+      <c r="C15" s="51" t="n">
+        <v>17936</v>
+      </c>
+      <c r="D15" s="51" t="n">
+        <v>2750</v>
+      </c>
+      <c r="E15" s="51" t="n">
+        <v>3300</v>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" s="49" t="n">
+        <v>2019</v>
+      </c>
+      <c r="B16" s="51" t="n">
+        <v>31237</v>
+      </c>
+      <c r="C16" s="51" t="n">
+        <v>22277</v>
+      </c>
+      <c r="D16" s="51" t="n">
+        <v>4194</v>
+      </c>
+      <c r="E16" s="51" t="n">
+        <v>4765</v>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" s="49" t="n">
+        <v>2020</v>
+      </c>
+      <c r="B17" s="51" t="n">
+        <v>32628</v>
+      </c>
+      <c r="C17" s="51" t="n">
+        <v>23298</v>
+      </c>
+      <c r="D17" s="51" t="n">
+        <v>4371</v>
+      </c>
+      <c r="E17" s="51" t="n">
+        <v>4958</v>
+      </c>
+    </row>
+    <row r="18">
+      <c r="A18" s="49" t="n">
+        <v>2021</v>
+      </c>
+      <c r="B18" s="51" t="n">
+        <v>34693</v>
+      </c>
+      <c r="C18" s="51" t="n">
+        <v>25864</v>
+      </c>
+      <c r="D18" s="51" t="n">
+        <v>4558</v>
+      </c>
+      <c r="E18" s="51" t="n">
+        <v>4270</v>
+      </c>
+    </row>
+    <row r="19">
+      <c r="A19" s="49" t="inlineStr">
+        <is>
+          <t>2022*</t>
+        </is>
+      </c>
+      <c r="B19" s="51" t="n">
+        <v>33276</v>
+      </c>
+      <c r="C19" s="51" t="inlineStr">
+        <is>
+          <t>n/p</t>
+        </is>
+      </c>
+      <c r="D19" s="51" t="inlineStr">
+        <is>
+          <t>n/p</t>
+        </is>
+      </c>
+      <c r="E19" s="51" t="inlineStr">
+        <is>
+          <t>n/p</t>
+        </is>
+      </c>
+    </row>
+    <row r="20">
+      <c r="A20" s="49" t="inlineStr">
+        <is>
+          <t>2023*</t>
+        </is>
+      </c>
+      <c r="B20" s="51" t="n">
+        <v>36525</v>
+      </c>
+      <c r="C20" s="51" t="inlineStr">
+        <is>
+          <t>n/p</t>
+        </is>
+      </c>
+      <c r="D20" s="51" t="inlineStr">
+        <is>
+          <t>n/p</t>
+        </is>
+      </c>
+      <c r="E20" s="51" t="inlineStr">
+        <is>
+          <t>n/p</t>
+        </is>
+      </c>
+    </row>
+    <row r="21">
+      <c r="A21" s="49" t="inlineStr">
+        <is>
+          <t>2024*</t>
+        </is>
+      </c>
+      <c r="B21" s="51" t="n">
+        <v>38921</v>
+      </c>
+      <c r="C21" s="51" t="inlineStr">
+        <is>
+          <t>n/p</t>
+        </is>
+      </c>
+      <c r="D21" s="51" t="inlineStr">
+        <is>
+          <t>n/p</t>
+        </is>
+      </c>
+      <c r="E21" s="51" t="inlineStr">
+        <is>
+          <t>n/p</t>
+        </is>
+      </c>
+    </row>
+    <row r="22">
+      <c r="A22" s="45" t="inlineStr">
+        <is>
+          <t>* New SCB series from 2022 (NV0109P): 2022 onward is not directly comparable to 2021; sub-industry splits not published (n/p).</t>
+        </is>
+      </c>
+    </row>
+    <row r="23">
+      <c r="A23" s="45" t="inlineStr">
+        <is>
+          <t>69.1 in 2024: 6,965 companies, 13,446 employees; production value SEK 39.1bn, value added SEK 25.3bn, EBITDA margin 28.2%.</t>
+        </is>
+      </c>
+    </row>
+    <row r="24">
+      <c r="A24" s="45" t="inlineStr">
+        <is>
+          <t>69.101 turnover CAGR 2010-21: ~5.8%. Source: https://api.scb.se/OV0104/v1/doris/sv/ssd/NV/NV0109/ (BasfaktaFEngs07, NSEBasfaktaFEngs07, NSEBasfaktaVEngs07N).</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:N39"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="4" customWidth="1" min="1" max="1"/>
+    <col width="26" customWidth="1" min="2" max="2"/>
+    <col width="13" customWidth="1" min="3" max="3"/>
+    <col width="11" customWidth="1" min="4" max="4"/>
+    <col width="30" customWidth="1" min="5" max="5"/>
+    <col width="9" customWidth="1" min="6" max="6"/>
+    <col width="30" customWidth="1" min="7" max="7"/>
+    <col width="9" customWidth="1" min="8" max="8"/>
+    <col width="11" customWidth="1" min="9" max="9"/>
+    <col width="24" customWidth="1" min="10" max="10"/>
+    <col width="10" customWidth="1" min="11" max="11"/>
+    <col width="10" customWidth="1" min="12" max="12"/>
+    <col width="10" customWidth="1" min="13" max="13"/>
+    <col width="40" customWidth="1" min="14" max="14"/>
+  </cols>
+  <sheetData>
+    <row r="1">
+      <c r="A1" s="1" t="inlineStr">
+        <is>
+          <t>A3. Concentration: largest Swedish business law firms ranked by latest revenue</t>
+        </is>
+      </c>
+    </row>
+    <row r="2" ht="55" customHeight="1">
+      <c r="A2" s="2" t="inlineStr">
+        <is>
+          <t>Revenue = latest available year per firm (SEK m). Affärsvärlden figures are fee income; company accounts (AB) are net sales of the main legal entity and are not strictly comparable. Partners and lawyers mostly firm-supplied to Chambers (2026). Employees = headcount, used as a proxy for FTEs (no FTE data is published); AB headcounts usually exclude partners who bill via own companies. Ratios are calculated only where both inputs exist. Grey = not found.</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" s="52" t="inlineStr">
+        <is>
+          <t>#</t>
+        </is>
+      </c>
+      <c r="B4" s="52" t="inlineStr">
+        <is>
+          <t>Firm</t>
+        </is>
+      </c>
+      <c r="C4" s="52" t="inlineStr">
+        <is>
+          <t>FY</t>
+        </is>
+      </c>
+      <c r="D4" s="52" t="inlineStr">
+        <is>
+          <t>Revenue SEK m</t>
+        </is>
+      </c>
+      <c r="E4" s="52" t="inlineStr">
+        <is>
+          <t>Revenue basis</t>
+        </is>
+      </c>
+      <c r="F4" s="52" t="inlineStr">
+        <is>
+          <t>Partners</t>
+        </is>
+      </c>
+      <c r="G4" s="52" t="inlineStr">
+        <is>
+          <t>Partner source</t>
+        </is>
+      </c>
+      <c r="H4" s="52" t="inlineStr">
+        <is>
+          <t>Lawyers</t>
+        </is>
+      </c>
+      <c r="I4" s="52" t="inlineStr">
+        <is>
+          <t>Employees (FTE proxy)</t>
+        </is>
+      </c>
+      <c r="J4" s="52" t="inlineStr">
+        <is>
+          <t>Employee source</t>
+        </is>
+      </c>
+      <c r="K4" s="52" t="inlineStr">
+        <is>
+          <t>Rev / partner SEK m</t>
+        </is>
+      </c>
+      <c r="L4" s="52" t="inlineStr">
+        <is>
+          <t>Rev / employee SEK m</t>
+        </is>
+      </c>
+      <c r="M4" s="52" t="inlineStr">
+        <is>
+          <t>Rev / lawyer SEK m</t>
+        </is>
+      </c>
+      <c r="N4" s="52" t="inlineStr">
+        <is>
+          <t>Notes</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" s="60" t="n">
+        <v>1</v>
+      </c>
+      <c r="B5" s="60" t="inlineStr">
+        <is>
+          <t>Vinge</t>
+        </is>
+      </c>
+      <c r="C5" s="60" t="inlineStr">
+        <is>
+          <t>2025</t>
+        </is>
+      </c>
+      <c r="D5" s="61" t="n">
+        <v>2036</v>
+      </c>
+      <c r="E5" s="49" t="inlineStr">
+        <is>
+          <t>Group, annual reports (DJ via Realtid)</t>
+        </is>
+      </c>
+      <c r="F5" s="60" t="n">
+        <v>63</v>
+      </c>
+      <c r="G5" s="49" t="inlineStr">
+        <is>
+          <t>Dividend recipients: Stockholm 49 + Malmö 14; excl. Göteborg (understated)</t>
+        </is>
+      </c>
+      <c r="H5" s="62" t="n"/>
+      <c r="I5" s="60" t="n">
+        <v>550</v>
+      </c>
+      <c r="J5" s="49" t="inlineStr">
+        <is>
+          <t>Website, 2026 (~550)</t>
+        </is>
+      </c>
+      <c r="K5" s="56">
+        <f>D5/F5</f>
+        <v/>
+      </c>
+      <c r="L5" s="56">
+        <f>D5/I5</f>
+        <v/>
+      </c>
+      <c r="M5" s="57" t="n"/>
+      <c r="N5" s="49" t="inlineStr">
+        <is>
+          <t>-2% y/y; 2024 was a record (2,083-2,085)</t>
+        </is>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" s="60" t="n">
+        <v>2</v>
+      </c>
+      <c r="B6" s="60" t="inlineStr">
+        <is>
+          <t>Mannheimer Swartling</t>
+        </is>
+      </c>
+      <c r="C6" s="60" t="inlineStr">
+        <is>
+          <t>2025</t>
+        </is>
+      </c>
+      <c r="D6" s="61" t="n">
+        <v>2002</v>
+      </c>
+      <c r="E6" s="49" t="inlineStr">
+        <is>
+          <t>Group, annual report (DJ via Realtid)</t>
+        </is>
+      </c>
+      <c r="F6" s="60" t="n">
+        <v>92</v>
+      </c>
+      <c r="G6" s="49" t="inlineStr">
+        <is>
+          <t>DJ (dividend split), 2025</t>
+        </is>
+      </c>
+      <c r="H6" s="60" t="n">
+        <v>430</v>
+      </c>
+      <c r="I6" s="60" t="n">
+        <v>650</v>
+      </c>
+      <c r="J6" s="49" t="inlineStr">
+        <is>
+          <t>Chambers 2026 / AB 649</t>
+        </is>
+      </c>
+      <c r="K6" s="56">
+        <f>D6/F6</f>
+        <v/>
+      </c>
+      <c r="L6" s="56">
+        <f>D6/I6</f>
+        <v/>
+      </c>
+      <c r="M6" s="56">
+        <f>D6/H6</f>
+        <v/>
+      </c>
+      <c r="N6" s="49" t="inlineStr">
+        <is>
+          <t>+4%; EBIT SEK 796m; dividend SEK 617m</t>
+        </is>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" s="60" t="n">
+        <v>3</v>
+      </c>
+      <c r="B7" s="60" t="inlineStr">
+        <is>
+          <t>Roschier (Sweden)</t>
+        </is>
+      </c>
+      <c r="C7" s="60" t="inlineStr">
+        <is>
+          <t>FY Jun24-May25</t>
+        </is>
+      </c>
+      <c r="D7" s="61" t="n">
+        <v>1254</v>
+      </c>
+      <c r="E7" s="49" t="inlineStr">
+        <is>
+          <t>Affärsvärlden Oct-25</t>
+        </is>
+      </c>
+      <c r="F7" s="62" t="n"/>
+      <c r="G7" s="49" t="inlineStr">
+        <is>
+          <t>Group 52 incl. Finland (not used)</t>
+        </is>
+      </c>
+      <c r="H7" s="62" t="n"/>
+      <c r="I7" s="60" t="n">
+        <v>226</v>
+      </c>
+      <c r="J7" s="49" t="inlineStr">
+        <is>
+          <t>Company accounts (AB)</t>
+        </is>
+      </c>
+      <c r="K7" s="57" t="n"/>
+      <c r="L7" s="56">
+        <f>D7/I7</f>
+        <v/>
+      </c>
+      <c r="M7" s="57" t="n"/>
+      <c r="N7" s="49" t="inlineStr">
+        <is>
+          <t>FY25/26 net sales 1,304 (220 staff)</t>
+        </is>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" s="60" t="n">
+        <v>4</v>
+      </c>
+      <c r="B8" s="60" t="inlineStr">
+        <is>
+          <t>White &amp; Case (Stockholm)</t>
+        </is>
+      </c>
+      <c r="C8" s="60" t="inlineStr">
+        <is>
+          <t>2025</t>
+        </is>
+      </c>
+      <c r="D8" s="61" t="n">
+        <v>1108</v>
+      </c>
+      <c r="E8" s="49" t="inlineStr">
+        <is>
+          <t>Company accounts, net sales (AB)</t>
+        </is>
+      </c>
+      <c r="F8" s="60" t="n">
+        <v>16</v>
+      </c>
+      <c r="G8" s="49" t="inlineStr">
+        <is>
+          <t>Implied (est.): DJ "&gt;SEK 69m per partner"</t>
+        </is>
+      </c>
+      <c r="H8" s="60" t="n">
+        <v>70</v>
+      </c>
+      <c r="I8" s="60" t="n">
+        <v>120</v>
+      </c>
+      <c r="J8" s="49" t="inlineStr">
+        <is>
+          <t>Company accounts (AB)</t>
+        </is>
+      </c>
+      <c r="K8" s="56">
+        <f>D8/F8</f>
+        <v/>
+      </c>
+      <c r="L8" s="56">
+        <f>D8/I8</f>
+        <v/>
+      </c>
+      <c r="M8" s="56">
+        <f>D8/H8</f>
+        <v/>
+      </c>
+      <c r="N8" s="49" t="inlineStr">
+        <is>
+          <t>2024: 859; +29%. AB net sales may include intra-group billing; per-head ratios look high, treat with caution</t>
+        </is>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" s="60" t="n">
+        <v>5</v>
+      </c>
+      <c r="B9" s="60" t="inlineStr">
+        <is>
+          <t>Setterwalls</t>
+        </is>
+      </c>
+      <c r="C9" s="60" t="inlineStr">
+        <is>
+          <t>2025</t>
+        </is>
+      </c>
+      <c r="D9" s="61" t="n">
+        <v>1000</v>
+      </c>
+      <c r="E9" s="49" t="inlineStr">
+        <is>
+          <t>Affärsvärlden ("&gt;1bn"); parent AB 1,056</t>
+        </is>
+      </c>
+      <c r="F9" s="60" t="n">
+        <v>37</v>
+      </c>
+      <c r="G9" s="49" t="inlineStr">
+        <is>
+          <t>Chambers 2026 (firm-supplied; looks low)</t>
+        </is>
+      </c>
+      <c r="H9" s="62" t="n"/>
+      <c r="I9" s="60" t="n">
+        <v>306</v>
+      </c>
+      <c r="J9" s="49" t="inlineStr">
+        <is>
+          <t>Sum of 3 entities (AB)</t>
+        </is>
+      </c>
+      <c r="K9" s="56">
+        <f>D9/F9</f>
+        <v/>
+      </c>
+      <c r="L9" s="56">
+        <f>D9/I9</f>
+        <v/>
+      </c>
+      <c r="M9" s="57" t="n"/>
+      <c r="N9" s="49" t="inlineStr">
+        <is>
+          <t>Malmö office (SEK 305m) left Sep-26 for AGRD</t>
+        </is>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" s="60" t="n">
+        <v>6</v>
+      </c>
+      <c r="B10" s="60" t="inlineStr">
+        <is>
+          <t>Lindahl</t>
+        </is>
+      </c>
+      <c r="C10" s="60" t="inlineStr">
+        <is>
+          <t>2024</t>
+        </is>
+      </c>
+      <c r="D10" s="61" t="n">
+        <v>737</v>
+      </c>
+      <c r="E10" s="49" t="inlineStr">
+        <is>
+          <t>Affärsvärlden Apr-25</t>
+        </is>
+      </c>
+      <c r="F10" s="62" t="n"/>
+      <c r="G10" s="49" t="inlineStr"/>
+      <c r="H10" s="60" t="n">
+        <v>153</v>
+      </c>
+      <c r="I10" s="60" t="n">
+        <v>300</v>
+      </c>
+      <c r="J10" s="49" t="inlineStr">
+        <is>
+          <t>Chambers 2026</t>
+        </is>
+      </c>
+      <c r="K10" s="57" t="n"/>
+      <c r="L10" s="56">
+        <f>D10/I10</f>
+        <v/>
+      </c>
+      <c r="M10" s="56">
+        <f>D10/H10</f>
+        <v/>
+      </c>
+      <c r="N10" s="49" t="inlineStr">
+        <is>
+          <t>2025 entity sum ~635 (est., not comparable)</t>
+        </is>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" s="60" t="n">
+        <v>7</v>
+      </c>
+      <c r="B11" s="60" t="inlineStr">
+        <is>
+          <t>Gernandt &amp; Danielsson</t>
+        </is>
+      </c>
+      <c r="C11" s="60" t="inlineStr">
+        <is>
+          <t>FY24/25</t>
+        </is>
+      </c>
+      <c r="D11" s="61" t="n">
+        <v>676</v>
+      </c>
+      <c r="E11" s="49" t="inlineStr">
+        <is>
+          <t>Affärsvärlden Oct-25</t>
+        </is>
+      </c>
+      <c r="F11" s="60" t="n">
+        <v>21</v>
+      </c>
+      <c r="G11" s="49" t="inlineStr">
+        <is>
+          <t>Chambers 2026</t>
+        </is>
+      </c>
+      <c r="H11" s="60" t="n">
+        <v>80</v>
+      </c>
+      <c r="I11" s="60" t="n">
+        <v>150</v>
+      </c>
+      <c r="J11" s="49" t="inlineStr">
+        <is>
+          <t>Firm website</t>
+        </is>
+      </c>
+      <c r="K11" s="56">
+        <f>D11/F11</f>
+        <v/>
+      </c>
+      <c r="L11" s="56">
+        <f>D11/I11</f>
+        <v/>
+      </c>
+      <c r="M11" s="56">
+        <f>D11/H11</f>
+        <v/>
+      </c>
+      <c r="N11" s="49" t="inlineStr">
+        <is>
+          <t>+12% (FY23/24: 601)</t>
+        </is>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" s="60" t="n">
+        <v>8</v>
+      </c>
+      <c r="B12" s="60" t="inlineStr">
+        <is>
+          <t>DLA Piper (Sweden)</t>
+        </is>
+      </c>
+      <c r="C12" s="60" t="inlineStr">
+        <is>
+          <t>FY24/25</t>
+        </is>
+      </c>
+      <c r="D12" s="61" t="n">
+        <v>602</v>
+      </c>
+      <c r="E12" s="49" t="inlineStr">
+        <is>
+          <t>Affärsvärlden Oct-25</t>
+        </is>
+      </c>
+      <c r="F12" s="62" t="n"/>
+      <c r="G12" s="49" t="inlineStr"/>
+      <c r="H12" s="62" t="n"/>
+      <c r="I12" s="62" t="n"/>
+      <c r="J12" s="49" t="inlineStr"/>
+      <c r="K12" s="57" t="n"/>
+      <c r="L12" s="57" t="n"/>
+      <c r="M12" s="57" t="n"/>
+      <c r="N12" s="49" t="inlineStr">
+        <is>
+          <t>-9%</t>
+        </is>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" s="60" t="n">
+        <v>9</v>
+      </c>
+      <c r="B13" s="60" t="inlineStr">
+        <is>
+          <t>CMS Wistrand</t>
+        </is>
+      </c>
+      <c r="C13" s="60" t="inlineStr">
+        <is>
+          <t>2024</t>
+        </is>
+      </c>
+      <c r="D13" s="61" t="n">
+        <v>558</v>
+      </c>
+      <c r="E13" s="49" t="inlineStr">
+        <is>
+          <t>Affärsvärlden Apr-25</t>
+        </is>
+      </c>
+      <c r="F13" s="62" t="n"/>
+      <c r="G13" s="49" t="inlineStr"/>
+      <c r="H13" s="62" t="n"/>
+      <c r="I13" s="62" t="n"/>
+      <c r="J13" s="49" t="inlineStr"/>
+      <c r="K13" s="57" t="n"/>
+      <c r="L13" s="57" t="n"/>
+      <c r="M13" s="57" t="n"/>
+      <c r="N13" s="49" t="inlineStr"/>
+    </row>
+    <row r="14">
+      <c r="A14" s="60" t="n">
+        <v>10</v>
+      </c>
+      <c r="B14" s="60" t="inlineStr">
+        <is>
+          <t>Schjødt (Sweden)</t>
+        </is>
+      </c>
+      <c r="C14" s="60" t="inlineStr">
+        <is>
+          <t>2025</t>
+        </is>
+      </c>
+      <c r="D14" s="61" t="n">
+        <v>534</v>
+      </c>
+      <c r="E14" s="49" t="inlineStr">
+        <is>
+          <t>Est.: "&gt;SEK 0.5bn", +25% on 427</t>
+        </is>
+      </c>
+      <c r="F14" s="62" t="n"/>
+      <c r="G14" s="49" t="inlineStr"/>
+      <c r="H14" s="62" t="n"/>
+      <c r="I14" s="62" t="n"/>
+      <c r="J14" s="49" t="inlineStr"/>
+      <c r="K14" s="57" t="n"/>
+      <c r="L14" s="57" t="n"/>
+      <c r="M14" s="57" t="n"/>
+      <c r="N14" s="49" t="inlineStr">
+        <is>
+          <t>Branch, no Swedish accounts; 8 Sthlm partners left for BAHR (2026)</t>
+        </is>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" s="60" t="n">
+        <v>11</v>
+      </c>
+      <c r="B15" s="60" t="inlineStr">
+        <is>
+          <t>Delphi</t>
+        </is>
+      </c>
+      <c r="C15" s="60" t="inlineStr">
+        <is>
+          <t>2024</t>
+        </is>
+      </c>
+      <c r="D15" s="61" t="n">
+        <v>516</v>
+      </c>
+      <c r="E15" s="49" t="inlineStr">
+        <is>
+          <t>Affärsvärlden Apr-25</t>
+        </is>
+      </c>
+      <c r="F15" s="60" t="n">
+        <v>49</v>
+      </c>
+      <c r="G15" s="49" t="inlineStr">
+        <is>
+          <t>Chambers 2026</t>
+        </is>
+      </c>
+      <c r="H15" s="60" t="n">
+        <v>150</v>
+      </c>
+      <c r="I15" s="60" t="n">
+        <v>220</v>
+      </c>
+      <c r="J15" s="49" t="inlineStr">
+        <is>
+          <t>Firm website</t>
+        </is>
+      </c>
+      <c r="K15" s="56">
+        <f>D15/F15</f>
+        <v/>
+      </c>
+      <c r="L15" s="56">
+        <f>D15/I15</f>
+        <v/>
+      </c>
+      <c r="M15" s="56">
+        <f>D15/H15</f>
+        <v/>
+      </c>
+      <c r="N15" s="49" t="inlineStr">
+        <is>
+          <t>+2%</t>
+        </is>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" s="60" t="n">
+        <v>12</v>
+      </c>
+      <c r="B16" s="60" t="inlineStr">
+        <is>
+          <t>Cirio</t>
+        </is>
+      </c>
+      <c r="C16" s="60" t="inlineStr">
+        <is>
+          <t>2025</t>
+        </is>
+      </c>
+      <c r="D16" s="61" t="n">
+        <v>431</v>
+      </c>
+      <c r="E16" s="49" t="inlineStr">
+        <is>
+          <t>Company accounts, net sales (AB)</t>
+        </is>
+      </c>
+      <c r="F16" s="62" t="n"/>
+      <c r="G16" s="49" t="inlineStr"/>
+      <c r="H16" s="62" t="n"/>
+      <c r="I16" s="60" t="n">
+        <v>127</v>
+      </c>
+      <c r="J16" s="49" t="inlineStr">
+        <is>
+          <t>Company accounts (AB)</t>
+        </is>
+      </c>
+      <c r="K16" s="57" t="n"/>
+      <c r="L16" s="56">
+        <f>D16/I16</f>
+        <v/>
+      </c>
+      <c r="M16" s="57" t="n"/>
+      <c r="N16" s="49" t="inlineStr">
+        <is>
+          <t>+15% (Afv); 2024 Afv 363</t>
+        </is>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" s="60" t="n">
+        <v>13</v>
+      </c>
+      <c r="B17" s="60" t="inlineStr">
+        <is>
+          <t>MAQS</t>
+        </is>
+      </c>
+      <c r="C17" s="60" t="inlineStr">
+        <is>
+          <t>2024</t>
+        </is>
+      </c>
+      <c r="D17" s="61" t="n">
+        <v>417</v>
+      </c>
+      <c r="E17" s="49" t="inlineStr">
+        <is>
+          <t>Affärsvärlden Apr-25</t>
+        </is>
+      </c>
+      <c r="F17" s="62" t="n"/>
+      <c r="G17" s="49" t="inlineStr"/>
+      <c r="H17" s="60" t="n">
+        <v>127</v>
+      </c>
+      <c r="I17" s="60" t="n">
+        <v>180</v>
+      </c>
+      <c r="J17" s="49" t="inlineStr">
+        <is>
+          <t>Chambers 2026</t>
+        </is>
+      </c>
+      <c r="K17" s="57" t="n"/>
+      <c r="L17" s="56">
+        <f>D17/I17</f>
+        <v/>
+      </c>
+      <c r="M17" s="56">
+        <f>D17/H17</f>
+        <v/>
+      </c>
+      <c r="N17" s="49" t="inlineStr">
+        <is>
+          <t>+21%</t>
+        </is>
+      </c>
+    </row>
+    <row r="18">
+      <c r="A18" s="60" t="n">
+        <v>14</v>
+      </c>
+      <c r="B18" s="60" t="inlineStr">
+        <is>
+          <t>Baker McKenzie (Stockholm)</t>
+        </is>
+      </c>
+      <c r="C18" s="60" t="inlineStr">
+        <is>
+          <t>FY23/24</t>
+        </is>
+      </c>
+      <c r="D18" s="61" t="n">
+        <v>334</v>
+      </c>
+      <c r="E18" s="49" t="inlineStr">
+        <is>
+          <t>Affärsvärlden Apr-25</t>
+        </is>
+      </c>
+      <c r="F18" s="62" t="n"/>
+      <c r="G18" s="49" t="inlineStr"/>
+      <c r="H18" s="62" t="n"/>
+      <c r="I18" s="62" t="n"/>
+      <c r="J18" s="49" t="inlineStr"/>
+      <c r="K18" s="57" t="n"/>
+      <c r="L18" s="57" t="n"/>
+      <c r="M18" s="57" t="n"/>
+      <c r="N18" s="49" t="inlineStr">
+        <is>
+          <t>KB, no public accounts</t>
+        </is>
+      </c>
+    </row>
+    <row r="19">
+      <c r="A19" s="60" t="n">
+        <v>15</v>
+      </c>
+      <c r="B19" s="60" t="inlineStr">
+        <is>
+          <t>Snellman (Sweden)</t>
+        </is>
+      </c>
+      <c r="C19" s="60" t="inlineStr">
+        <is>
+          <t>2025</t>
+        </is>
+      </c>
+      <c r="D19" s="61" t="n">
+        <v>279</v>
+      </c>
+      <c r="E19" s="49" t="inlineStr">
+        <is>
+          <t>Company accounts, net sales (AB)</t>
+        </is>
+      </c>
+      <c r="F19" s="62" t="n"/>
+      <c r="G19" s="49" t="inlineStr"/>
+      <c r="H19" s="62" t="n"/>
+      <c r="I19" s="60" t="n">
+        <v>107</v>
+      </c>
+      <c r="J19" s="49" t="inlineStr">
+        <is>
+          <t>Company accounts (AB)</t>
+        </is>
+      </c>
+      <c r="K19" s="57" t="n"/>
+      <c r="L19" s="56">
+        <f>D19/I19</f>
+        <v/>
+      </c>
+      <c r="M19" s="57" t="n"/>
+      <c r="N19" s="49" t="inlineStr">
+        <is>
+          <t>2024 Afv 295</t>
+        </is>
+      </c>
+    </row>
+    <row r="20">
+      <c r="A20" s="60" t="n">
+        <v>16</v>
+      </c>
+      <c r="B20" s="60" t="inlineStr">
+        <is>
+          <t>Foyen</t>
+        </is>
+      </c>
+      <c r="C20" s="60" t="inlineStr">
+        <is>
+          <t>2024</t>
+        </is>
+      </c>
+      <c r="D20" s="61" t="n">
+        <v>277</v>
+      </c>
+      <c r="E20" s="49" t="inlineStr">
+        <is>
+          <t>Affärsvärlden Apr-25</t>
+        </is>
+      </c>
+      <c r="F20" s="62" t="n"/>
+      <c r="G20" s="49" t="inlineStr"/>
+      <c r="H20" s="62" t="n"/>
+      <c r="I20" s="60" t="n">
+        <v>106</v>
+      </c>
+      <c r="J20" s="49" t="inlineStr">
+        <is>
+          <t>Company accounts (AB)</t>
+        </is>
+      </c>
+      <c r="K20" s="57" t="n"/>
+      <c r="L20" s="56">
+        <f>D20/I20</f>
+        <v/>
+      </c>
+      <c r="M20" s="57" t="n"/>
+      <c r="N20" s="49" t="inlineStr"/>
+    </row>
+    <row r="21">
+      <c r="A21" s="60" t="n">
+        <v>17</v>
+      </c>
+      <c r="B21" s="60" t="inlineStr">
+        <is>
+          <t>Glimstedt</t>
+        </is>
+      </c>
+      <c r="C21" s="60" t="inlineStr">
+        <is>
+          <t>2024</t>
+        </is>
+      </c>
+      <c r="D21" s="61" t="n">
+        <v>196</v>
+      </c>
+      <c r="E21" s="49" t="inlineStr">
+        <is>
+          <t>Affärsvärlden Apr-25</t>
+        </is>
+      </c>
+      <c r="F21" s="62" t="n"/>
+      <c r="G21" s="49" t="inlineStr"/>
+      <c r="H21" s="62" t="n"/>
+      <c r="I21" s="62" t="n"/>
+      <c r="J21" s="49" t="inlineStr"/>
+      <c r="K21" s="57" t="n"/>
+      <c r="L21" s="57" t="n"/>
+      <c r="M21" s="57" t="n"/>
+      <c r="N21" s="49" t="inlineStr">
+        <is>
+          <t>~200 staff on website includes Baltics (not used)</t>
+        </is>
+      </c>
+    </row>
+    <row r="22">
+      <c r="A22" s="60" t="n">
+        <v>18</v>
+      </c>
+      <c r="B22" s="60" t="inlineStr">
+        <is>
+          <t>Eversheds Sutherland</t>
+        </is>
+      </c>
+      <c r="C22" s="60" t="inlineStr">
+        <is>
+          <t>2025</t>
+        </is>
+      </c>
+      <c r="D22" s="61" t="n">
+        <v>166</v>
+      </c>
+      <c r="E22" s="49" t="inlineStr">
+        <is>
+          <t>Company accounts, net sales (AB)</t>
+        </is>
+      </c>
+      <c r="F22" s="62" t="n"/>
+      <c r="G22" s="49" t="inlineStr"/>
+      <c r="H22" s="62" t="n"/>
+      <c r="I22" s="60" t="n">
+        <v>59</v>
+      </c>
+      <c r="J22" s="49" t="inlineStr">
+        <is>
+          <t>Company accounts (AB)</t>
+        </is>
+      </c>
+      <c r="K22" s="57" t="n"/>
+      <c r="L22" s="56">
+        <f>D22/I22</f>
+        <v/>
+      </c>
+      <c r="M22" s="57" t="n"/>
+      <c r="N22" s="49" t="inlineStr">
+        <is>
+          <t>2024 Afv 140</t>
+        </is>
+      </c>
+    </row>
+    <row r="23">
+      <c r="A23" s="60" t="n">
+        <v>19</v>
+      </c>
+      <c r="B23" s="60" t="inlineStr">
+        <is>
+          <t>Fylgia</t>
+        </is>
+      </c>
+      <c r="C23" s="60" t="inlineStr">
+        <is>
+          <t>2024</t>
+        </is>
+      </c>
+      <c r="D23" s="61" t="n">
+        <v>131</v>
+      </c>
+      <c r="E23" s="49" t="inlineStr">
+        <is>
+          <t>Affärsvärlden Apr-25</t>
+        </is>
+      </c>
+      <c r="F23" s="62" t="n"/>
+      <c r="G23" s="49" t="inlineStr"/>
+      <c r="H23" s="62" t="n"/>
+      <c r="I23" s="62" t="n"/>
+      <c r="J23" s="49" t="inlineStr"/>
+      <c r="K23" s="57" t="n"/>
+      <c r="L23" s="57" t="n"/>
+      <c r="M23" s="57" t="n"/>
+      <c r="N23" s="49" t="inlineStr">
+        <is>
+          <t>Record 2025 (firm)</t>
+        </is>
+      </c>
+    </row>
+    <row r="24">
+      <c r="A24" s="60" t="n">
+        <v>20</v>
+      </c>
+      <c r="B24" s="60" t="inlineStr">
+        <is>
+          <t>Westerberg &amp; Partners</t>
+        </is>
+      </c>
+      <c r="C24" s="60" t="inlineStr">
+        <is>
+          <t>2025</t>
+        </is>
+      </c>
+      <c r="D24" s="61" t="n">
+        <v>107</v>
+      </c>
+      <c r="E24" s="49" t="inlineStr">
+        <is>
+          <t>Company accounts, net sales (AB)</t>
+        </is>
+      </c>
+      <c r="F24" s="60" t="n">
+        <v>12</v>
+      </c>
+      <c r="G24" s="49" t="inlineStr">
+        <is>
+          <t>Chambers 2026</t>
+        </is>
+      </c>
+      <c r="H24" s="62" t="n"/>
+      <c r="I24" s="60" t="n">
+        <v>35</v>
+      </c>
+      <c r="J24" s="49" t="inlineStr">
+        <is>
+          <t>Company accounts (AB)</t>
+        </is>
+      </c>
+      <c r="K24" s="56">
+        <f>D24/F24</f>
+        <v/>
+      </c>
+      <c r="L24" s="56">
+        <f>D24/I24</f>
+        <v/>
+      </c>
+      <c r="M24" s="57" t="n"/>
+      <c r="N24" s="49" t="inlineStr"/>
+    </row>
+    <row r="25">
+      <c r="A25" s="60" t="n">
+        <v>21</v>
+      </c>
+      <c r="B25" s="60" t="inlineStr">
+        <is>
+          <t>Moll Wendén</t>
+        </is>
+      </c>
+      <c r="C25" s="60" t="inlineStr">
+        <is>
+          <t>2025</t>
+        </is>
+      </c>
+      <c r="D25" s="61" t="n">
+        <v>101</v>
+      </c>
+      <c r="E25" s="49" t="inlineStr">
+        <is>
+          <t>Company accounts, net sales (AB)</t>
+        </is>
+      </c>
+      <c r="F25" s="62" t="n"/>
+      <c r="G25" s="49" t="inlineStr"/>
+      <c r="H25" s="62" t="n"/>
+      <c r="I25" s="60" t="n">
+        <v>44</v>
+      </c>
+      <c r="J25" s="49" t="inlineStr">
+        <is>
+          <t>Company accounts (AB)</t>
+        </is>
+      </c>
+      <c r="K25" s="57" t="n"/>
+      <c r="L25" s="56">
+        <f>D25/I25</f>
+        <v/>
+      </c>
+      <c r="M25" s="57" t="n"/>
+      <c r="N25" s="49" t="inlineStr"/>
+    </row>
+    <row r="26">
+      <c r="A26" s="60" t="n">
+        <v>22</v>
+      </c>
+      <c r="B26" s="60" t="inlineStr">
+        <is>
+          <t>Born</t>
+        </is>
+      </c>
+      <c r="C26" s="60" t="inlineStr">
+        <is>
+          <t>2024</t>
+        </is>
+      </c>
+      <c r="D26" s="61" t="n">
+        <v>86</v>
+      </c>
+      <c r="E26" s="49" t="inlineStr">
+        <is>
+          <t>Affärsvärlden Apr-25</t>
+        </is>
+      </c>
+      <c r="F26" s="62" t="n"/>
+      <c r="G26" s="49" t="inlineStr"/>
+      <c r="H26" s="62" t="n"/>
+      <c r="I26" s="62" t="n"/>
+      <c r="J26" s="49" t="inlineStr"/>
+      <c r="K26" s="57" t="n"/>
+      <c r="L26" s="57" t="n"/>
+      <c r="M26" s="57" t="n"/>
+      <c r="N26" s="49" t="inlineStr">
+        <is>
+          <t>Part of AGRD since 2025</t>
+        </is>
+      </c>
+    </row>
+    <row r="27">
+      <c r="A27" s="60" t="n">
+        <v>23</v>
+      </c>
+      <c r="B27" s="60" t="inlineStr">
+        <is>
+          <t>Harvest</t>
+        </is>
+      </c>
+      <c r="C27" s="60" t="inlineStr">
+        <is>
+          <t>2025</t>
+        </is>
+      </c>
+      <c r="D27" s="61" t="n">
+        <v>82</v>
+      </c>
+      <c r="E27" s="49" t="inlineStr">
+        <is>
+          <t>Company accounts, net sales (AB)</t>
+        </is>
+      </c>
+      <c r="F27" s="62" t="n"/>
+      <c r="G27" s="49" t="inlineStr"/>
+      <c r="H27" s="62" t="n"/>
+      <c r="I27" s="60" t="n">
+        <v>27</v>
+      </c>
+      <c r="J27" s="49" t="inlineStr">
+        <is>
+          <t>Company accounts (AB)</t>
+        </is>
+      </c>
+      <c r="K27" s="57" t="n"/>
+      <c r="L27" s="56">
+        <f>D27/I27</f>
+        <v/>
+      </c>
+      <c r="M27" s="57" t="n"/>
+      <c r="N27" s="49" t="inlineStr"/>
+    </row>
+    <row r="28">
+      <c r="A28" s="60" t="n">
+        <v>24</v>
+      </c>
+      <c r="B28" s="60" t="inlineStr">
+        <is>
+          <t>Synch</t>
+        </is>
+      </c>
+      <c r="C28" s="60" t="inlineStr">
+        <is>
+          <t>2025</t>
+        </is>
+      </c>
+      <c r="D28" s="61" t="n">
+        <v>81</v>
+      </c>
+      <c r="E28" s="49" t="inlineStr">
+        <is>
+          <t>Company accounts, net sales (AB)</t>
+        </is>
+      </c>
+      <c r="F28" s="62" t="n"/>
+      <c r="G28" s="49" t="inlineStr"/>
+      <c r="H28" s="62" t="n"/>
+      <c r="I28" s="60" t="n">
+        <v>38</v>
+      </c>
+      <c r="J28" s="49" t="inlineStr">
+        <is>
+          <t>Company accounts (AB)</t>
+        </is>
+      </c>
+      <c r="K28" s="57" t="n"/>
+      <c r="L28" s="56">
+        <f>D28/I28</f>
+        <v/>
+      </c>
+      <c r="M28" s="57" t="n"/>
+      <c r="N28" s="49" t="inlineStr">
+        <is>
+          <t>Part of AGRD since 2025</t>
+        </is>
+      </c>
+    </row>
+    <row r="29">
+      <c r="A29" s="60" t="n">
+        <v>25</v>
+      </c>
+      <c r="B29" s="60" t="inlineStr">
+        <is>
+          <t>Kastell</t>
+        </is>
+      </c>
+      <c r="C29" s="60" t="inlineStr">
+        <is>
+          <t>2025</t>
+        </is>
+      </c>
+      <c r="D29" s="61" t="n">
+        <v>80</v>
+      </c>
+      <c r="E29" s="49" t="inlineStr">
+        <is>
+          <t>Company accounts, net sales (AB)</t>
+        </is>
+      </c>
+      <c r="F29" s="60" t="n">
+        <v>9</v>
+      </c>
+      <c r="G29" s="49" t="inlineStr">
+        <is>
+          <t>Chambers 2026</t>
+        </is>
+      </c>
+      <c r="H29" s="60" t="n">
+        <v>19</v>
+      </c>
+      <c r="I29" s="60" t="n">
+        <v>21</v>
+      </c>
+      <c r="J29" s="49" t="inlineStr">
+        <is>
+          <t>Company accounts (AB)</t>
+        </is>
+      </c>
+      <c r="K29" s="56">
+        <f>D29/F29</f>
+        <v/>
+      </c>
+      <c r="L29" s="56">
+        <f>D29/I29</f>
+        <v/>
+      </c>
+      <c r="M29" s="56">
+        <f>D29/H29</f>
+        <v/>
+      </c>
+      <c r="N29" s="49" t="inlineStr"/>
+    </row>
+    <row r="30">
+      <c r="B30" s="46" t="inlineStr">
+        <is>
+          <t>Total shown</t>
+        </is>
+      </c>
+      <c r="D30" s="58">
+        <f>SUM(D5:D29)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="31">
+      <c r="B31" t="inlineStr">
+        <is>
+          <t>Top 5 share of ~SEK 16bn panel (indicative, mixed years/bases)</t>
+        </is>
+      </c>
+      <c r="D31" s="59">
+        <f>SUM(D5:D9)/16000</f>
+        <v/>
+      </c>
+    </row>
+    <row r="32">
+      <c r="B32" t="inlineStr">
+        <is>
+          <t>Top 10 share of ~SEK 16bn panel (indicative)</t>
+        </is>
+      </c>
+      <c r="D32" s="59">
+        <f>SUM(D5:D14)/16000</f>
+        <v/>
+      </c>
+    </row>
+    <row r="34">
+      <c r="A34" s="45" t="inlineStr">
+        <is>
+          <t>Caveats: Vinge partner count covers only the Stockholm and Malmö dividend-receiving partners (no Göteborg), so Vinge rev/partner is overstated. White &amp; Case partners are implied from Dagens Juridik "&gt;SEK 69m per partner" (paywalled).</t>
+        </is>
+      </c>
+    </row>
+    <row r="35">
+      <c r="A35" s="45" t="inlineStr">
+        <is>
+          <t>Setterwalls partner count (37) is as supplied to Chambers and looks low against the firm size. Roschier group partner count (52) includes Finland and is not used. Magnusson: no Swedish revenue or headcount found.</t>
+        </is>
+      </c>
+    </row>
+    <row r="36">
+      <c r="A36" s="45" t="inlineStr">
+        <is>
+          <t>Sources: Affärsvärlden 12-Apr-25 https://www.affarsvarlden.se/artikel/vinge-gar-om-msa-sa-gar-det-for-affarsjuristerna ; 3-Oct-25 https://www.affarsvarlden.se/artikel/affarsjuristerna-gar-starkt-finns-fler-bolag-i-ipo-pipelinen ;</t>
+        </is>
+      </c>
+    </row>
+    <row r="37">
+      <c r="A37" s="45" t="inlineStr">
+        <is>
+          <t>Realtid 7-Aug-26 https://www.realtid.se/juridik/vinge-tappar-mark-mannheimer-swartling-drar-ifran/ ; Realtid 26-Apr-26 https://www.realtid.se/juridik/affarsjuridiken-vaxer-men-sprickorna-syns/ ; Realtid 27-Nov-25 https://www.realtid.se/juridik/white-case-dubblade-omsattningen-var-styrka/ ;</t>
+        </is>
+      </c>
+    </row>
+    <row r="38">
+      <c r="A38" s="45" t="inlineStr">
+        <is>
+          <t>Realtid 1-Sep-26 https://www.realtid.se/juridik/setterwalls-malmokontor-gar-till-riskkapitalagda-agrd/ ; Affärsvärlden 5-Oct-26 (Schjødt) https://www.affarsvarlden.se/artikel/schjdt-vaxer-snabbast--men-konkurrensen-hardnar ;</t>
+        </is>
+      </c>
+    </row>
+    <row r="39">
+      <c r="A39" s="45" t="inlineStr">
+        <is>
+          <t>company accounts via https://www.allabolag.se/{org.nr} ; Chambers Europe 2026 firm profiles (firm-supplied "top figures"); firm websites.</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+  <mergeCells count="1">
+    <mergeCell ref="A2:N2"/>
+  </mergeCells>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:F23"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="24" customWidth="1" min="1" max="1"/>
+    <col width="22" customWidth="1" min="2" max="2"/>
+    <col width="16" customWidth="1" min="3" max="3"/>
+    <col width="14" customWidth="1" min="4" max="4"/>
+    <col width="80" customWidth="1" min="5" max="5"/>
+    <col width="60" customWidth="1" min="6" max="6"/>
+  </cols>
+  <sheetData>
+    <row r="1">
+      <c r="A1" s="1" t="inlineStr">
+        <is>
+          <t>A4. Fastest growers and growth drivers</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" s="45" t="inlineStr">
+        <is>
+          <t>Driver tags: Lateral hire / M&amp;A / New office / Organic. Only drivers found in a cited source are listed.</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" s="48" t="inlineStr">
+        <is>
+          <t>Firm</t>
+        </is>
+      </c>
+      <c r="B4" s="48" t="inlineStr">
+        <is>
+          <t>Growth</t>
+        </is>
+      </c>
+      <c r="C4" s="48" t="inlineStr">
+        <is>
+          <t>Period</t>
+        </is>
+      </c>
+      <c r="D4" s="48" t="inlineStr">
+        <is>
+          <t>Driver</t>
+        </is>
+      </c>
+      <c r="E4" s="48" t="inlineStr">
+        <is>
+          <t>Detail</t>
+        </is>
+      </c>
+      <c r="F4" s="48" t="inlineStr">
+        <is>
+          <t>Source</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" s="49" t="inlineStr">
+        <is>
+          <t>Carthiel</t>
+        </is>
+      </c>
+      <c r="B5" s="49" t="inlineStr">
+        <is>
+          <t>+155%</t>
+        </is>
+      </c>
+      <c r="C5" s="49" t="inlineStr">
+        <is>
+          <t>2024</t>
+        </is>
+      </c>
+      <c r="D5" s="49" t="inlineStr">
+        <is>
+          <t>M&amp;A</t>
+        </is>
+      </c>
+      <c r="E5" s="49" t="inlineStr">
+        <is>
+          <t>Merged with Grey Advokatbyrå (operating from Feb-2024), adding a disputes team. Small base (~10 people).</t>
+        </is>
+      </c>
+      <c r="F5" s="49" t="inlineStr">
+        <is>
+          <t>https://www.carthiel.se/post/advokatfirman-carthiel-g%C3%A5r-ihop-med-grey-advokatbyr%C3%A5</t>
+        </is>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" s="49" t="inlineStr">
+        <is>
+          <t>White &amp; Case (Stockholm)</t>
+        </is>
+      </c>
+      <c r="B6" s="49" t="inlineStr">
+        <is>
+          <t>+29% (AB net sales 859 to 1,108)</t>
+        </is>
+      </c>
+      <c r="C6" s="49" t="inlineStr">
+        <is>
+          <t>2025</t>
+        </is>
+      </c>
+      <c r="D6" s="49" t="inlineStr">
+        <is>
+          <t>Organic</t>
+        </is>
+      </c>
+      <c r="E6" s="49" t="inlineStr">
+        <is>
+          <t>Fastest grower in 2023 (+24%) on PE deals and selective hiring; "doubled revenue" coverage Nov-25. Lost Magnus Wennerhorn to Linklaters (Sep-24).</t>
+        </is>
+      </c>
+      <c r="F6" s="49" t="inlineStr">
+        <is>
+          <t>https://www.realtid.se/juridik/white-case-dubblade-omsattningen-var-styrka/</t>
+        </is>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" s="49" t="inlineStr">
+        <is>
+          <t>Schjødt (Sweden)</t>
+        </is>
+      </c>
+      <c r="B7" s="49" t="inlineStr">
+        <is>
+          <t>+24% / ~+25%</t>
+        </is>
+      </c>
+      <c r="C7" s="49" t="inlineStr">
+        <is>
+          <t>2024 / 2025</t>
+        </is>
+      </c>
+      <c r="D7" s="49" t="inlineStr">
+        <is>
+          <t>Lateral hire</t>
+        </is>
+      </c>
+      <c r="E7" s="49" t="inlineStr">
+        <is>
+          <t>Tom Wehtje (M&amp;A) joined 2024 from Mannheimer Swartling after 15 years as partner; Karl Klackenberg (M&amp;A/PE) reportedly from Vinge May-24 (unconfirmed).</t>
+        </is>
+      </c>
+      <c r="F7" s="49" t="inlineStr">
+        <is>
+          <t>https://www.legal500.com/firms/10502-advokatfirmaet-schjodt-as/c-sweden/lawyers/2101480-tom-wehtje</t>
+        </is>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" s="49" t="inlineStr"/>
+      <c r="B8" s="49" t="inlineStr"/>
+      <c r="C8" s="49" t="inlineStr"/>
+      <c r="D8" s="49" t="inlineStr">
+        <is>
+          <t>Organic</t>
+        </is>
+      </c>
+      <c r="E8" s="49" t="inlineStr">
+        <is>
+          <t>Demand for pan-Scandinavian cross-border offering, FDI and regulatory work.</t>
+        </is>
+      </c>
+      <c r="F8" s="49" t="inlineStr">
+        <is>
+          <t>https://www.affarsvarlden.se/artikel/vinge-gar-om-msa-sa-gar-det-for-affarsjuristerna</t>
+        </is>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" s="49" t="inlineStr"/>
+      <c r="B9" s="49" t="inlineStr"/>
+      <c r="C9" s="49" t="inlineStr"/>
+      <c r="D9" s="49" t="inlineStr">
+        <is>
+          <t>M&amp;A (historic)</t>
+        </is>
+      </c>
+      <c r="E9" s="49" t="inlineStr">
+        <is>
+          <t>Entered Sweden via merger with Hamilton (2019/20). Risk: 54 people (23 partners, group-wide) left for BAHR, which opened Stockholm Jan-26.</t>
+        </is>
+      </c>
+      <c r="F9" s="49" t="inlineStr">
+        <is>
+          <t>https://www.realtid.se/juridik/oppnar-stockholmskontor-efter-massvarvning-fran-rivalen/</t>
+        </is>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" s="49" t="inlineStr">
+        <is>
+          <t>Roschier (Sweden)</t>
+        </is>
+      </c>
+      <c r="B10" s="49" t="inlineStr">
+        <is>
+          <t>+23% / +22%</t>
+        </is>
+      </c>
+      <c r="C10" s="49" t="inlineStr">
+        <is>
+          <t>FY23/24 / FY24/25</t>
+        </is>
+      </c>
+      <c r="D10" s="49" t="inlineStr">
+        <is>
+          <t>Organic</t>
+        </is>
+      </c>
+      <c r="E10" s="49" t="inlineStr">
+        <is>
+          <t>Swedish transaction market pick-up, larger mandates, high disputes demand, closer Finland-Sweden integration; Northvolt Expansion Ett restructuring. Stockholm now larger than Helsinki.</t>
+        </is>
+      </c>
+      <c r="F10" s="49" t="inlineStr">
+        <is>
+          <t>https://www.realtid.se/affarer/154-miljarder-sa-klarade-affarsjuristerna-tullchocken/</t>
+        </is>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" s="49" t="inlineStr">
+        <is>
+          <t>MAQS</t>
+        </is>
+      </c>
+      <c r="B11" s="49" t="inlineStr">
+        <is>
+          <t>+21%</t>
+        </is>
+      </c>
+      <c r="C11" s="49" t="inlineStr">
+        <is>
+          <t>2024</t>
+        </is>
+      </c>
+      <c r="D11" s="49" t="inlineStr">
+        <is>
+          <t>Organic</t>
+        </is>
+      </c>
+      <c r="E11" s="49" t="inlineStr">
+        <is>
+          <t>Strong demand in M&amp;A, capital markets and disputes (CEO Katrin Troedsson).</t>
+        </is>
+      </c>
+      <c r="F11" s="49" t="inlineStr">
+        <is>
+          <t>https://www.affarsvarlden.se/artikel/vinge-gar-om-msa-sa-gar-det-for-affarsjuristerna</t>
+        </is>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" s="49" t="inlineStr"/>
+      <c r="B12" s="49" t="inlineStr"/>
+      <c r="C12" s="49" t="inlineStr"/>
+      <c r="D12" s="49" t="inlineStr">
+        <is>
+          <t>Lateral hire</t>
+        </is>
+      </c>
+      <c r="E12" s="49" t="inlineStr">
+        <is>
+          <t>Strategic sustainability hires, e.g. Anna Domander (ex head of legal, Systembolaget); date not given.</t>
+        </is>
+      </c>
+      <c r="F12" s="49" t="inlineStr">
+        <is>
+          <t>https://www.affarsvarlden.se/artikel/vinge-gar-om-msa-sa-gar-det-for-affarsjuristerna</t>
+        </is>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" s="49" t="inlineStr">
+        <is>
+          <t>Vinge</t>
+        </is>
+      </c>
+      <c r="B13" s="49" t="inlineStr">
+        <is>
+          <t>+19%</t>
+        </is>
+      </c>
+      <c r="C13" s="49" t="inlineStr">
+        <is>
+          <t>2024</t>
+        </is>
+      </c>
+      <c r="D13" s="49" t="inlineStr">
+        <is>
+          <t>Organic</t>
+        </is>
+      </c>
+      <c r="E13" s="49" t="inlineStr">
+        <is>
+          <t>Broad client activity and full-service model; accounted for ~25% of total market growth. Then -2% in 2025 ("2024 exceptional").</t>
+        </is>
+      </c>
+      <c r="F13" s="49" t="inlineStr">
+        <is>
+          <t>https://www.affarsvarlden.se/artikel/vinge-gar-om-msa-sa-gar-det-for-affarsjuristerna</t>
+        </is>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" s="49" t="inlineStr">
+        <is>
+          <t>Gernandt &amp; Danielsson</t>
+        </is>
+      </c>
+      <c r="B14" s="49" t="inlineStr">
+        <is>
+          <t>+19% / +12%</t>
+        </is>
+      </c>
+      <c r="C14" s="49" t="inlineStr">
+        <is>
+          <t>FY23/24 / FY24/25</t>
+        </is>
+      </c>
+      <c r="D14" s="49" t="inlineStr">
+        <is>
+          <t>Lateral hire</t>
+        </is>
+      </c>
+      <c r="E14" s="49" t="inlineStr">
+        <is>
+          <t>Linklaters Stockholm real estate team: partners Magnus Lidman and Anna Eriksson + 5 associates (dated Jun-24 by Global Legal Post/Legal 500; Afv says early 2025).</t>
+        </is>
+      </c>
+      <c r="F14" s="49" t="inlineStr">
+        <is>
+          <t>https://www.affarsvarlden.se/artikel/affarsjuristerna-gar-starkt-finns-fler-bolag-i-ipo-pipelinen</t>
+        </is>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" s="49" t="inlineStr"/>
+      <c r="B15" s="49" t="inlineStr"/>
+      <c r="C15" s="49" t="inlineStr"/>
+      <c r="D15" s="49" t="inlineStr">
+        <is>
+          <t>Organic</t>
+        </is>
+      </c>
+      <c r="E15" s="49" t="inlineStr">
+        <is>
+          <t>Strong bond and M&amp;A teams.</t>
+        </is>
+      </c>
+      <c r="F15" s="49" t="inlineStr">
+        <is>
+          <t>https://www.affarsvarlden.se/artikel/affarsjuristerna-gar-starkt-finns-fler-bolag-i-ipo-pipelinen</t>
+        </is>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" s="49" t="inlineStr">
+        <is>
+          <t>Cirio</t>
+        </is>
+      </c>
+      <c r="B16" s="49" t="inlineStr">
+        <is>
+          <t>~+15%</t>
+        </is>
+      </c>
+      <c r="C16" s="49" t="inlineStr">
+        <is>
+          <t>2025</t>
+        </is>
+      </c>
+      <c r="D16" s="49" t="inlineStr">
+        <is>
+          <t>Lateral hire</t>
+        </is>
+      </c>
+      <c r="E16" s="49" t="inlineStr">
+        <is>
+          <t>12-person real estate and construction team from AG Advokat from Jan-25, incl. partners Johan Lindberg, Johan Rosén, Måns Derk; new construction disputes offering.</t>
+        </is>
+      </c>
+      <c r="F16" s="49" t="inlineStr">
+        <is>
+          <t>https://www.realtid.se/juridik/cirio-expanderar-inom-fastighets-och-entreprenadjuridik/</t>
+        </is>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" s="49" t="inlineStr"/>
+      <c r="B17" s="49" t="inlineStr"/>
+      <c r="C17" s="49" t="inlineStr"/>
+      <c r="D17" s="49" t="inlineStr">
+        <is>
+          <t>Organic</t>
+        </is>
+      </c>
+      <c r="E17" s="49" t="inlineStr">
+        <is>
+          <t>Investment in real estate transactions and insolvency.</t>
+        </is>
+      </c>
+      <c r="F17" s="49" t="inlineStr">
+        <is>
+          <t>https://www.realtid.se/juridik/affarsjuridiken-vaxer-men-sprickorna-syns/</t>
+        </is>
+      </c>
+    </row>
+    <row r="18">
+      <c r="A18" s="49" t="inlineStr">
+        <is>
+          <t>Setterwalls</t>
+        </is>
+      </c>
+      <c r="B18" s="49" t="inlineStr">
+        <is>
+          <t>+2% / ~+9% (passed SEK 1bn)</t>
+        </is>
+      </c>
+      <c r="C18" s="49" t="inlineStr">
+        <is>
+          <t>2024 / 2025</t>
+        </is>
+      </c>
+      <c r="D18" s="49" t="inlineStr">
+        <is>
+          <t>Organic</t>
+        </is>
+      </c>
+      <c r="E18" s="49" t="inlineStr">
+        <is>
+          <t>Large complex mandates: public M&amp;A and PE take-privates (MedHelp, Integrum, Norva24), bank finance, disputes; lawyers +10% to 235 in 2024. Malmö office left for AGRD in Sep-26.</t>
+        </is>
+      </c>
+      <c r="F18" s="49" t="inlineStr">
+        <is>
+          <t>https://www.realtid.se/affarer/154-miljarder-sa-klarade-affarsjuristerna-tullchocken/</t>
+        </is>
+      </c>
+    </row>
+    <row r="19">
+      <c r="A19" s="49" t="inlineStr">
+        <is>
+          <t>Fylgia</t>
+        </is>
+      </c>
+      <c r="B19" s="49" t="inlineStr">
+        <is>
+          <t>n/a (record 2025)</t>
+        </is>
+      </c>
+      <c r="C19" s="49" t="inlineStr">
+        <is>
+          <t>2025</t>
+        </is>
+      </c>
+      <c r="D19" s="49" t="inlineStr">
+        <is>
+          <t>Organic</t>
+        </is>
+      </c>
+      <c r="E19" s="49" t="inlineStr">
+        <is>
+          <t>Transactions, construction/real estate, public procurement, restructuring/insolvency; four new partners appointed.</t>
+        </is>
+      </c>
+      <c r="F19" s="49" t="inlineStr">
+        <is>
+          <t>https://www.fylgia.se/en/news/following-a-record-breaking-year-fylgia-appoints-four-new-partners</t>
+        </is>
+      </c>
+    </row>
+    <row r="20">
+      <c r="A20" s="49" t="inlineStr">
+        <is>
+          <t>AGRD Partners (Axcel)</t>
+        </is>
+      </c>
+      <c r="B20" s="49" t="inlineStr">
+        <is>
+          <t>n/a (~SEK 660m combined)</t>
+        </is>
+      </c>
+      <c r="C20" s="49" t="inlineStr">
+        <is>
+          <t>2025</t>
+        </is>
+      </c>
+      <c r="D20" s="49" t="inlineStr">
+        <is>
+          <t>M&amp;A</t>
+        </is>
+      </c>
+      <c r="E20" s="49" t="inlineStr">
+        <is>
+          <t>PE-backed roll-up of six firms in Aug-25: Allié, Born, Morris Law, Next, Synch, TM &amp; Partners (~130 lawyers gave up advokat title). Added Setterwalls Malmö (Ascente Law) Sep-26.</t>
+        </is>
+      </c>
+      <c r="F20" s="49" t="inlineStr">
+        <is>
+          <t>https://www.realtid.se/juridik/setterwalls-malmokontor-gar-till-riskkapitalagda-agrd/</t>
+        </is>
+      </c>
+    </row>
+    <row r="21">
+      <c r="A21" s="49" t="inlineStr">
+        <is>
+          <t>DLA Piper (Sweden)</t>
+        </is>
+      </c>
+      <c r="B21" s="49" t="inlineStr">
+        <is>
+          <t>-9%</t>
+        </is>
+      </c>
+      <c r="C21" s="49" t="inlineStr">
+        <is>
+          <t>FY24/25</t>
+        </is>
+      </c>
+      <c r="D21" s="49" t="inlineStr">
+        <is>
+          <t>Decline</t>
+        </is>
+      </c>
+      <c r="E21" s="49" t="inlineStr">
+        <is>
+          <t>Consolidation year: generational shift and hesitant deal market; restructuring group busy (Northvolt, Oscar Properties, SAS).</t>
+        </is>
+      </c>
+      <c r="F21" s="49" t="inlineStr">
+        <is>
+          <t>https://www.affarsvarlden.se/artikel/affarsjuristerna-gar-starkt-finns-fler-bolag-i-ipo-pipelinen</t>
+        </is>
+      </c>
+    </row>
+    <row r="23">
+      <c r="A23" s="45" t="inlineStr">
+        <is>
+          <t>Market context: 2025 growth came from international transactions, disputes and regulatory work; IPOs were the weakest segment. Firms expect +6.8% in 2026 (Affärsvärlden/Realtid).</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
   <dimension ref="A1:BB66"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
@@ -857,157 +3210,128 @@
           <t>Corporate / M&amp;A</t>
         </is>
       </c>
-      <c r="F4" s="3" t="n"/>
       <c r="G4" s="3" t="inlineStr">
         <is>
           <t>Private equity</t>
         </is>
       </c>
-      <c r="H4" s="3" t="n"/>
       <c r="I4" s="3" t="inlineStr">
         <is>
           <t>PE fund formation</t>
         </is>
       </c>
-      <c r="J4" s="3" t="n"/>
       <c r="K4" s="3" t="inlineStr">
         <is>
           <t>Banking &amp; finance</t>
         </is>
       </c>
-      <c r="L4" s="3" t="n"/>
       <c r="M4" s="3" t="inlineStr">
         <is>
           <t>Capital markets: equity</t>
         </is>
       </c>
-      <c r="N4" s="3" t="n"/>
       <c r="O4" s="3" t="inlineStr">
         <is>
           <t>Capital markets: debt</t>
         </is>
       </c>
-      <c r="P4" s="3" t="n"/>
       <c r="Q4" s="3" t="inlineStr">
         <is>
           <t>Dispute resolution</t>
         </is>
       </c>
-      <c r="R4" s="3" t="n"/>
       <c r="S4" s="3" t="inlineStr">
         <is>
           <t>Restructuring / insolvency</t>
         </is>
       </c>
-      <c r="T4" s="3" t="n"/>
       <c r="U4" s="3" t="inlineStr">
         <is>
           <t>Insolvency trustees</t>
         </is>
       </c>
-      <c r="V4" s="3" t="n"/>
       <c r="W4" s="3" t="inlineStr">
         <is>
           <t>Competition / EU</t>
         </is>
       </c>
-      <c r="X4" s="3" t="n"/>
       <c r="Y4" s="3" t="inlineStr">
         <is>
           <t>Employment</t>
         </is>
       </c>
-      <c r="Z4" s="3" t="n"/>
       <c r="AA4" s="3" t="inlineStr">
         <is>
           <t>Tax</t>
         </is>
       </c>
-      <c r="AB4" s="3" t="n"/>
       <c r="AC4" s="3" t="inlineStr">
         <is>
           <t>Real estate</t>
         </is>
       </c>
-      <c r="AD4" s="3" t="n"/>
       <c r="AE4" s="3" t="inlineStr">
         <is>
           <t>Construction</t>
         </is>
       </c>
-      <c r="AF4" s="3" t="n"/>
       <c r="AG4" s="3" t="inlineStr">
         <is>
           <t>IP</t>
         </is>
       </c>
-      <c r="AH4" s="3" t="n"/>
       <c r="AI4" s="3" t="inlineStr">
         <is>
           <t>IT / TMT</t>
         </is>
       </c>
-      <c r="AJ4" s="3" t="n"/>
       <c r="AK4" s="3" t="inlineStr">
         <is>
           <t>Data protection</t>
         </is>
       </c>
-      <c r="AL4" s="3" t="n"/>
       <c r="AM4" s="3" t="inlineStr">
         <is>
           <t>Fintech</t>
         </is>
       </c>
-      <c r="AN4" s="3" t="n"/>
       <c r="AO4" s="3" t="inlineStr">
         <is>
           <t>Energy</t>
         </is>
       </c>
-      <c r="AP4" s="3" t="n"/>
       <c r="AQ4" s="3" t="inlineStr">
         <is>
           <t>Environment</t>
         </is>
       </c>
-      <c r="AR4" s="3" t="n"/>
       <c r="AS4" s="3" t="inlineStr">
         <is>
           <t>Insurance</t>
         </is>
       </c>
-      <c r="AT4" s="3" t="n"/>
       <c r="AU4" s="3" t="inlineStr">
         <is>
           <t>Public procurement</t>
         </is>
       </c>
-      <c r="AV4" s="3" t="n"/>
       <c r="AW4" s="3" t="inlineStr">
         <is>
           <t>Healthcare / life sciences</t>
         </is>
       </c>
-      <c r="AX4" s="3" t="n"/>
       <c r="AY4" s="3" t="inlineStr">
         <is>
           <t>Shipping</t>
         </is>
       </c>
-      <c r="AZ4" s="3" t="n"/>
       <c r="BA4" s="3" t="inlineStr">
         <is>
           <t>Corporate investigations</t>
         </is>
       </c>
-      <c r="BB4" s="3" t="n"/>
     </row>
     <row r="5">
-      <c r="A5" s="4" t="n"/>
-      <c r="B5" s="4" t="n"/>
-      <c r="C5" s="4" t="n"/>
-      <c r="D5" s="4" t="n"/>
       <c r="E5" s="4" t="inlineStr">
         <is>
           <t>CH</t>
@@ -7694,7 +10018,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
     <outlinePr summaryBelow="1" summaryRight="1"/>

</xml_diff>

<commit_message>
Add leverage ratio (partners / lawyers) to firms sheet
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01Tu61bPEQej1E6sErbEFanY
</commit_message>
<xml_diff>
--- a/research/swedish_legal_market.xlsx
+++ b/research/swedish_legal_market.xlsx
@@ -286,7 +286,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="63">
+  <cellXfs count="67">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
@@ -440,6 +440,16 @@
     <xf numFmtId="0" fontId="0" fillId="5" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="top"/>
     </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="top"/>
+    </xf>
+    <xf numFmtId="3" fontId="0" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="top"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="5" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="top"/>
+    </xf>
+    <xf numFmtId="9" fontId="0" fillId="0" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0" hidden="0"/>
@@ -1209,7 +1219,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:N39"/>
+  <dimension ref="A1:O40"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="4" customWidth="1" min="1" max="1"/>
@@ -1225,7 +1235,8 @@
     <col width="10" customWidth="1" min="11" max="11"/>
     <col width="10" customWidth="1" min="12" max="12"/>
     <col width="10" customWidth="1" min="13" max="13"/>
-    <col width="40" customWidth="1" min="14" max="14"/>
+    <col width="11" customWidth="1" min="14" max="14"/>
+    <col width="40" customWidth="1" min="15" max="15"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -1310,25 +1321,30 @@
       </c>
       <c r="N4" s="52" t="inlineStr">
         <is>
+          <t>Leverage (partners / lawyers)</t>
+        </is>
+      </c>
+      <c r="O4" s="52" t="inlineStr">
+        <is>
           <t>Notes</t>
         </is>
       </c>
     </row>
     <row r="5">
-      <c r="A5" s="60" t="n">
+      <c r="A5" s="63" t="n">
         <v>1</v>
       </c>
-      <c r="B5" s="60" t="inlineStr">
+      <c r="B5" s="63" t="inlineStr">
         <is>
           <t>Vinge</t>
         </is>
       </c>
-      <c r="C5" s="60" t="inlineStr">
+      <c r="C5" s="63" t="inlineStr">
         <is>
           <t>2025</t>
         </is>
       </c>
-      <c r="D5" s="61" t="n">
+      <c r="D5" s="64" t="n">
         <v>2036</v>
       </c>
       <c r="E5" s="49" t="inlineStr">
@@ -1336,7 +1352,7 @@
           <t>Group, annual reports (DJ via Realtid)</t>
         </is>
       </c>
-      <c r="F5" s="60" t="n">
+      <c r="F5" s="63" t="n">
         <v>63</v>
       </c>
       <c r="G5" s="49" t="inlineStr">
@@ -1344,8 +1360,8 @@
           <t>Dividend recipients: Stockholm 49 + Malmö 14; excl. Göteborg (understated)</t>
         </is>
       </c>
-      <c r="H5" s="62" t="n"/>
-      <c r="I5" s="60" t="n">
+      <c r="H5" s="65" t="n"/>
+      <c r="I5" s="63" t="n">
         <v>550</v>
       </c>
       <c r="J5" s="49" t="inlineStr">
@@ -1362,27 +1378,28 @@
         <v/>
       </c>
       <c r="M5" s="57" t="n"/>
-      <c r="N5" s="49" t="inlineStr">
+      <c r="N5" s="57" t="n"/>
+      <c r="O5" s="49" t="inlineStr">
         <is>
           <t>-2% y/y; 2024 was a record (2,083-2,085)</t>
         </is>
       </c>
     </row>
     <row r="6">
-      <c r="A6" s="60" t="n">
+      <c r="A6" s="63" t="n">
         <v>2</v>
       </c>
-      <c r="B6" s="60" t="inlineStr">
+      <c r="B6" s="63" t="inlineStr">
         <is>
           <t>Mannheimer Swartling</t>
         </is>
       </c>
-      <c r="C6" s="60" t="inlineStr">
+      <c r="C6" s="63" t="inlineStr">
         <is>
           <t>2025</t>
         </is>
       </c>
-      <c r="D6" s="61" t="n">
+      <c r="D6" s="64" t="n">
         <v>2002</v>
       </c>
       <c r="E6" s="49" t="inlineStr">
@@ -1390,7 +1407,7 @@
           <t>Group, annual report (DJ via Realtid)</t>
         </is>
       </c>
-      <c r="F6" s="60" t="n">
+      <c r="F6" s="63" t="n">
         <v>92</v>
       </c>
       <c r="G6" s="49" t="inlineStr">
@@ -1398,10 +1415,10 @@
           <t>DJ (dividend split), 2025</t>
         </is>
       </c>
-      <c r="H6" s="60" t="n">
+      <c r="H6" s="63" t="n">
         <v>430</v>
       </c>
-      <c r="I6" s="60" t="n">
+      <c r="I6" s="63" t="n">
         <v>650</v>
       </c>
       <c r="J6" s="49" t="inlineStr">
@@ -1421,27 +1438,31 @@
         <f>D6/H6</f>
         <v/>
       </c>
-      <c r="N6" s="49" t="inlineStr">
+      <c r="N6" s="66">
+        <f>F6/H6</f>
+        <v/>
+      </c>
+      <c r="O6" s="49" t="inlineStr">
         <is>
           <t>+4%; EBIT SEK 796m; dividend SEK 617m</t>
         </is>
       </c>
     </row>
     <row r="7">
-      <c r="A7" s="60" t="n">
+      <c r="A7" s="63" t="n">
         <v>3</v>
       </c>
-      <c r="B7" s="60" t="inlineStr">
+      <c r="B7" s="63" t="inlineStr">
         <is>
           <t>Roschier (Sweden)</t>
         </is>
       </c>
-      <c r="C7" s="60" t="inlineStr">
+      <c r="C7" s="63" t="inlineStr">
         <is>
           <t>FY Jun24-May25</t>
         </is>
       </c>
-      <c r="D7" s="61" t="n">
+      <c r="D7" s="64" t="n">
         <v>1254</v>
       </c>
       <c r="E7" s="49" t="inlineStr">
@@ -1449,14 +1470,14 @@
           <t>Affärsvärlden Oct-25</t>
         </is>
       </c>
-      <c r="F7" s="62" t="n"/>
+      <c r="F7" s="65" t="n"/>
       <c r="G7" s="49" t="inlineStr">
         <is>
           <t>Group 52 incl. Finland (not used)</t>
         </is>
       </c>
-      <c r="H7" s="62" t="n"/>
-      <c r="I7" s="60" t="n">
+      <c r="H7" s="65" t="n"/>
+      <c r="I7" s="63" t="n">
         <v>226</v>
       </c>
       <c r="J7" s="49" t="inlineStr">
@@ -1470,27 +1491,28 @@
         <v/>
       </c>
       <c r="M7" s="57" t="n"/>
-      <c r="N7" s="49" t="inlineStr">
+      <c r="N7" s="57" t="n"/>
+      <c r="O7" s="49" t="inlineStr">
         <is>
           <t>FY25/26 net sales 1,304 (220 staff)</t>
         </is>
       </c>
     </row>
     <row r="8">
-      <c r="A8" s="60" t="n">
+      <c r="A8" s="63" t="n">
         <v>4</v>
       </c>
-      <c r="B8" s="60" t="inlineStr">
+      <c r="B8" s="63" t="inlineStr">
         <is>
           <t>White &amp; Case (Stockholm)</t>
         </is>
       </c>
-      <c r="C8" s="60" t="inlineStr">
+      <c r="C8" s="63" t="inlineStr">
         <is>
           <t>2025</t>
         </is>
       </c>
-      <c r="D8" s="61" t="n">
+      <c r="D8" s="64" t="n">
         <v>1108</v>
       </c>
       <c r="E8" s="49" t="inlineStr">
@@ -1498,7 +1520,7 @@
           <t>Company accounts, net sales (AB)</t>
         </is>
       </c>
-      <c r="F8" s="60" t="n">
+      <c r="F8" s="63" t="n">
         <v>16</v>
       </c>
       <c r="G8" s="49" t="inlineStr">
@@ -1506,10 +1528,10 @@
           <t>Implied (est.): DJ "&gt;SEK 69m per partner"</t>
         </is>
       </c>
-      <c r="H8" s="60" t="n">
+      <c r="H8" s="63" t="n">
         <v>70</v>
       </c>
-      <c r="I8" s="60" t="n">
+      <c r="I8" s="63" t="n">
         <v>120</v>
       </c>
       <c r="J8" s="49" t="inlineStr">
@@ -1529,27 +1551,31 @@
         <f>D8/H8</f>
         <v/>
       </c>
-      <c r="N8" s="49" t="inlineStr">
+      <c r="N8" s="66">
+        <f>F8/H8</f>
+        <v/>
+      </c>
+      <c r="O8" s="49" t="inlineStr">
         <is>
           <t>2024: 859; +29%. AB net sales may include intra-group billing; per-head ratios look high, treat with caution</t>
         </is>
       </c>
     </row>
     <row r="9">
-      <c r="A9" s="60" t="n">
+      <c r="A9" s="63" t="n">
         <v>5</v>
       </c>
-      <c r="B9" s="60" t="inlineStr">
+      <c r="B9" s="63" t="inlineStr">
         <is>
           <t>Setterwalls</t>
         </is>
       </c>
-      <c r="C9" s="60" t="inlineStr">
+      <c r="C9" s="63" t="inlineStr">
         <is>
           <t>2025</t>
         </is>
       </c>
-      <c r="D9" s="61" t="n">
+      <c r="D9" s="64" t="n">
         <v>1000</v>
       </c>
       <c r="E9" s="49" t="inlineStr">
@@ -1557,7 +1583,7 @@
           <t>Affärsvärlden ("&gt;1bn"); parent AB 1,056</t>
         </is>
       </c>
-      <c r="F9" s="60" t="n">
+      <c r="F9" s="63" t="n">
         <v>37</v>
       </c>
       <c r="G9" s="49" t="inlineStr">
@@ -1565,8 +1591,8 @@
           <t>Chambers 2026 (firm-supplied; looks low)</t>
         </is>
       </c>
-      <c r="H9" s="62" t="n"/>
-      <c r="I9" s="60" t="n">
+      <c r="H9" s="65" t="n"/>
+      <c r="I9" s="63" t="n">
         <v>306</v>
       </c>
       <c r="J9" s="49" t="inlineStr">
@@ -1583,27 +1609,28 @@
         <v/>
       </c>
       <c r="M9" s="57" t="n"/>
-      <c r="N9" s="49" t="inlineStr">
+      <c r="N9" s="57" t="n"/>
+      <c r="O9" s="49" t="inlineStr">
         <is>
           <t>Malmö office (SEK 305m) left Sep-26 for AGRD</t>
         </is>
       </c>
     </row>
     <row r="10">
-      <c r="A10" s="60" t="n">
+      <c r="A10" s="63" t="n">
         <v>6</v>
       </c>
-      <c r="B10" s="60" t="inlineStr">
+      <c r="B10" s="63" t="inlineStr">
         <is>
           <t>Lindahl</t>
         </is>
       </c>
-      <c r="C10" s="60" t="inlineStr">
+      <c r="C10" s="63" t="inlineStr">
         <is>
           <t>2024</t>
         </is>
       </c>
-      <c r="D10" s="61" t="n">
+      <c r="D10" s="64" t="n">
         <v>737</v>
       </c>
       <c r="E10" s="49" t="inlineStr">
@@ -1611,12 +1638,12 @@
           <t>Affärsvärlden Apr-25</t>
         </is>
       </c>
-      <c r="F10" s="62" t="n"/>
+      <c r="F10" s="65" t="n"/>
       <c r="G10" s="49" t="inlineStr"/>
-      <c r="H10" s="60" t="n">
+      <c r="H10" s="63" t="n">
         <v>153</v>
       </c>
-      <c r="I10" s="60" t="n">
+      <c r="I10" s="63" t="n">
         <v>300</v>
       </c>
       <c r="J10" s="49" t="inlineStr">
@@ -1633,27 +1660,28 @@
         <f>D10/H10</f>
         <v/>
       </c>
-      <c r="N10" s="49" t="inlineStr">
+      <c r="N10" s="57" t="n"/>
+      <c r="O10" s="49" t="inlineStr">
         <is>
           <t>2025 entity sum ~635 (est., not comparable)</t>
         </is>
       </c>
     </row>
     <row r="11">
-      <c r="A11" s="60" t="n">
+      <c r="A11" s="63" t="n">
         <v>7</v>
       </c>
-      <c r="B11" s="60" t="inlineStr">
+      <c r="B11" s="63" t="inlineStr">
         <is>
           <t>Gernandt &amp; Danielsson</t>
         </is>
       </c>
-      <c r="C11" s="60" t="inlineStr">
+      <c r="C11" s="63" t="inlineStr">
         <is>
           <t>FY24/25</t>
         </is>
       </c>
-      <c r="D11" s="61" t="n">
+      <c r="D11" s="64" t="n">
         <v>676</v>
       </c>
       <c r="E11" s="49" t="inlineStr">
@@ -1661,7 +1689,7 @@
           <t>Affärsvärlden Oct-25</t>
         </is>
       </c>
-      <c r="F11" s="60" t="n">
+      <c r="F11" s="63" t="n">
         <v>21</v>
       </c>
       <c r="G11" s="49" t="inlineStr">
@@ -1669,10 +1697,10 @@
           <t>Chambers 2026</t>
         </is>
       </c>
-      <c r="H11" s="60" t="n">
+      <c r="H11" s="63" t="n">
         <v>80</v>
       </c>
-      <c r="I11" s="60" t="n">
+      <c r="I11" s="63" t="n">
         <v>150</v>
       </c>
       <c r="J11" s="49" t="inlineStr">
@@ -1692,27 +1720,31 @@
         <f>D11/H11</f>
         <v/>
       </c>
-      <c r="N11" s="49" t="inlineStr">
+      <c r="N11" s="66">
+        <f>F11/H11</f>
+        <v/>
+      </c>
+      <c r="O11" s="49" t="inlineStr">
         <is>
           <t>+12% (FY23/24: 601)</t>
         </is>
       </c>
     </row>
     <row r="12">
-      <c r="A12" s="60" t="n">
+      <c r="A12" s="63" t="n">
         <v>8</v>
       </c>
-      <c r="B12" s="60" t="inlineStr">
+      <c r="B12" s="63" t="inlineStr">
         <is>
           <t>DLA Piper (Sweden)</t>
         </is>
       </c>
-      <c r="C12" s="60" t="inlineStr">
+      <c r="C12" s="63" t="inlineStr">
         <is>
           <t>FY24/25</t>
         </is>
       </c>
-      <c r="D12" s="61" t="n">
+      <c r="D12" s="64" t="n">
         <v>602</v>
       </c>
       <c r="E12" s="49" t="inlineStr">
@@ -1720,35 +1752,36 @@
           <t>Affärsvärlden Oct-25</t>
         </is>
       </c>
-      <c r="F12" s="62" t="n"/>
+      <c r="F12" s="65" t="n"/>
       <c r="G12" s="49" t="inlineStr"/>
-      <c r="H12" s="62" t="n"/>
-      <c r="I12" s="62" t="n"/>
+      <c r="H12" s="65" t="n"/>
+      <c r="I12" s="65" t="n"/>
       <c r="J12" s="49" t="inlineStr"/>
       <c r="K12" s="57" t="n"/>
       <c r="L12" s="57" t="n"/>
       <c r="M12" s="57" t="n"/>
-      <c r="N12" s="49" t="inlineStr">
+      <c r="N12" s="57" t="n"/>
+      <c r="O12" s="49" t="inlineStr">
         <is>
           <t>-9%</t>
         </is>
       </c>
     </row>
     <row r="13">
-      <c r="A13" s="60" t="n">
+      <c r="A13" s="63" t="n">
         <v>9</v>
       </c>
-      <c r="B13" s="60" t="inlineStr">
+      <c r="B13" s="63" t="inlineStr">
         <is>
           <t>CMS Wistrand</t>
         </is>
       </c>
-      <c r="C13" s="60" t="inlineStr">
+      <c r="C13" s="63" t="inlineStr">
         <is>
           <t>2024</t>
         </is>
       </c>
-      <c r="D13" s="61" t="n">
+      <c r="D13" s="64" t="n">
         <v>558</v>
       </c>
       <c r="E13" s="49" t="inlineStr">
@@ -1756,31 +1789,32 @@
           <t>Affärsvärlden Apr-25</t>
         </is>
       </c>
-      <c r="F13" s="62" t="n"/>
+      <c r="F13" s="65" t="n"/>
       <c r="G13" s="49" t="inlineStr"/>
-      <c r="H13" s="62" t="n"/>
-      <c r="I13" s="62" t="n"/>
+      <c r="H13" s="65" t="n"/>
+      <c r="I13" s="65" t="n"/>
       <c r="J13" s="49" t="inlineStr"/>
       <c r="K13" s="57" t="n"/>
       <c r="L13" s="57" t="n"/>
       <c r="M13" s="57" t="n"/>
-      <c r="N13" s="49" t="inlineStr"/>
+      <c r="N13" s="57" t="n"/>
+      <c r="O13" s="49" t="inlineStr"/>
     </row>
     <row r="14">
-      <c r="A14" s="60" t="n">
+      <c r="A14" s="63" t="n">
         <v>10</v>
       </c>
-      <c r="B14" s="60" t="inlineStr">
+      <c r="B14" s="63" t="inlineStr">
         <is>
           <t>Schjødt (Sweden)</t>
         </is>
       </c>
-      <c r="C14" s="60" t="inlineStr">
+      <c r="C14" s="63" t="inlineStr">
         <is>
           <t>2025</t>
         </is>
       </c>
-      <c r="D14" s="61" t="n">
+      <c r="D14" s="64" t="n">
         <v>534</v>
       </c>
       <c r="E14" s="49" t="inlineStr">
@@ -1788,35 +1822,36 @@
           <t>Est.: "&gt;SEK 0.5bn", +25% on 427</t>
         </is>
       </c>
-      <c r="F14" s="62" t="n"/>
+      <c r="F14" s="65" t="n"/>
       <c r="G14" s="49" t="inlineStr"/>
-      <c r="H14" s="62" t="n"/>
-      <c r="I14" s="62" t="n"/>
+      <c r="H14" s="65" t="n"/>
+      <c r="I14" s="65" t="n"/>
       <c r="J14" s="49" t="inlineStr"/>
       <c r="K14" s="57" t="n"/>
       <c r="L14" s="57" t="n"/>
       <c r="M14" s="57" t="n"/>
-      <c r="N14" s="49" t="inlineStr">
+      <c r="N14" s="57" t="n"/>
+      <c r="O14" s="49" t="inlineStr">
         <is>
           <t>Branch, no Swedish accounts; 8 Sthlm partners left for BAHR (2026)</t>
         </is>
       </c>
     </row>
     <row r="15">
-      <c r="A15" s="60" t="n">
+      <c r="A15" s="63" t="n">
         <v>11</v>
       </c>
-      <c r="B15" s="60" t="inlineStr">
+      <c r="B15" s="63" t="inlineStr">
         <is>
           <t>Delphi</t>
         </is>
       </c>
-      <c r="C15" s="60" t="inlineStr">
+      <c r="C15" s="63" t="inlineStr">
         <is>
           <t>2024</t>
         </is>
       </c>
-      <c r="D15" s="61" t="n">
+      <c r="D15" s="64" t="n">
         <v>516</v>
       </c>
       <c r="E15" s="49" t="inlineStr">
@@ -1824,7 +1859,7 @@
           <t>Affärsvärlden Apr-25</t>
         </is>
       </c>
-      <c r="F15" s="60" t="n">
+      <c r="F15" s="63" t="n">
         <v>49</v>
       </c>
       <c r="G15" s="49" t="inlineStr">
@@ -1832,10 +1867,10 @@
           <t>Chambers 2026</t>
         </is>
       </c>
-      <c r="H15" s="60" t="n">
+      <c r="H15" s="63" t="n">
         <v>150</v>
       </c>
-      <c r="I15" s="60" t="n">
+      <c r="I15" s="63" t="n">
         <v>220</v>
       </c>
       <c r="J15" s="49" t="inlineStr">
@@ -1855,27 +1890,31 @@
         <f>D15/H15</f>
         <v/>
       </c>
-      <c r="N15" s="49" t="inlineStr">
+      <c r="N15" s="66">
+        <f>F15/H15</f>
+        <v/>
+      </c>
+      <c r="O15" s="49" t="inlineStr">
         <is>
           <t>+2%</t>
         </is>
       </c>
     </row>
     <row r="16">
-      <c r="A16" s="60" t="n">
+      <c r="A16" s="63" t="n">
         <v>12</v>
       </c>
-      <c r="B16" s="60" t="inlineStr">
+      <c r="B16" s="63" t="inlineStr">
         <is>
           <t>Cirio</t>
         </is>
       </c>
-      <c r="C16" s="60" t="inlineStr">
+      <c r="C16" s="63" t="inlineStr">
         <is>
           <t>2025</t>
         </is>
       </c>
-      <c r="D16" s="61" t="n">
+      <c r="D16" s="64" t="n">
         <v>431</v>
       </c>
       <c r="E16" s="49" t="inlineStr">
@@ -1883,10 +1922,10 @@
           <t>Company accounts, net sales (AB)</t>
         </is>
       </c>
-      <c r="F16" s="62" t="n"/>
+      <c r="F16" s="65" t="n"/>
       <c r="G16" s="49" t="inlineStr"/>
-      <c r="H16" s="62" t="n"/>
-      <c r="I16" s="60" t="n">
+      <c r="H16" s="65" t="n"/>
+      <c r="I16" s="63" t="n">
         <v>127</v>
       </c>
       <c r="J16" s="49" t="inlineStr">
@@ -1900,27 +1939,28 @@
         <v/>
       </c>
       <c r="M16" s="57" t="n"/>
-      <c r="N16" s="49" t="inlineStr">
+      <c r="N16" s="57" t="n"/>
+      <c r="O16" s="49" t="inlineStr">
         <is>
           <t>+15% (Afv); 2024 Afv 363</t>
         </is>
       </c>
     </row>
     <row r="17">
-      <c r="A17" s="60" t="n">
+      <c r="A17" s="63" t="n">
         <v>13</v>
       </c>
-      <c r="B17" s="60" t="inlineStr">
+      <c r="B17" s="63" t="inlineStr">
         <is>
           <t>MAQS</t>
         </is>
       </c>
-      <c r="C17" s="60" t="inlineStr">
+      <c r="C17" s="63" t="inlineStr">
         <is>
           <t>2024</t>
         </is>
       </c>
-      <c r="D17" s="61" t="n">
+      <c r="D17" s="64" t="n">
         <v>417</v>
       </c>
       <c r="E17" s="49" t="inlineStr">
@@ -1928,12 +1968,12 @@
           <t>Affärsvärlden Apr-25</t>
         </is>
       </c>
-      <c r="F17" s="62" t="n"/>
+      <c r="F17" s="65" t="n"/>
       <c r="G17" s="49" t="inlineStr"/>
-      <c r="H17" s="60" t="n">
+      <c r="H17" s="63" t="n">
         <v>127</v>
       </c>
-      <c r="I17" s="60" t="n">
+      <c r="I17" s="63" t="n">
         <v>180</v>
       </c>
       <c r="J17" s="49" t="inlineStr">
@@ -1950,27 +1990,28 @@
         <f>D17/H17</f>
         <v/>
       </c>
-      <c r="N17" s="49" t="inlineStr">
+      <c r="N17" s="57" t="n"/>
+      <c r="O17" s="49" t="inlineStr">
         <is>
           <t>+21%</t>
         </is>
       </c>
     </row>
     <row r="18">
-      <c r="A18" s="60" t="n">
+      <c r="A18" s="63" t="n">
         <v>14</v>
       </c>
-      <c r="B18" s="60" t="inlineStr">
+      <c r="B18" s="63" t="inlineStr">
         <is>
           <t>Baker McKenzie (Stockholm)</t>
         </is>
       </c>
-      <c r="C18" s="60" t="inlineStr">
+      <c r="C18" s="63" t="inlineStr">
         <is>
           <t>FY23/24</t>
         </is>
       </c>
-      <c r="D18" s="61" t="n">
+      <c r="D18" s="64" t="n">
         <v>334</v>
       </c>
       <c r="E18" s="49" t="inlineStr">
@@ -1978,35 +2019,36 @@
           <t>Affärsvärlden Apr-25</t>
         </is>
       </c>
-      <c r="F18" s="62" t="n"/>
+      <c r="F18" s="65" t="n"/>
       <c r="G18" s="49" t="inlineStr"/>
-      <c r="H18" s="62" t="n"/>
-      <c r="I18" s="62" t="n"/>
+      <c r="H18" s="65" t="n"/>
+      <c r="I18" s="65" t="n"/>
       <c r="J18" s="49" t="inlineStr"/>
       <c r="K18" s="57" t="n"/>
       <c r="L18" s="57" t="n"/>
       <c r="M18" s="57" t="n"/>
-      <c r="N18" s="49" t="inlineStr">
+      <c r="N18" s="57" t="n"/>
+      <c r="O18" s="49" t="inlineStr">
         <is>
           <t>KB, no public accounts</t>
         </is>
       </c>
     </row>
     <row r="19">
-      <c r="A19" s="60" t="n">
+      <c r="A19" s="63" t="n">
         <v>15</v>
       </c>
-      <c r="B19" s="60" t="inlineStr">
+      <c r="B19" s="63" t="inlineStr">
         <is>
           <t>Snellman (Sweden)</t>
         </is>
       </c>
-      <c r="C19" s="60" t="inlineStr">
+      <c r="C19" s="63" t="inlineStr">
         <is>
           <t>2025</t>
         </is>
       </c>
-      <c r="D19" s="61" t="n">
+      <c r="D19" s="64" t="n">
         <v>279</v>
       </c>
       <c r="E19" s="49" t="inlineStr">
@@ -2014,10 +2056,10 @@
           <t>Company accounts, net sales (AB)</t>
         </is>
       </c>
-      <c r="F19" s="62" t="n"/>
+      <c r="F19" s="65" t="n"/>
       <c r="G19" s="49" t="inlineStr"/>
-      <c r="H19" s="62" t="n"/>
-      <c r="I19" s="60" t="n">
+      <c r="H19" s="65" t="n"/>
+      <c r="I19" s="63" t="n">
         <v>107</v>
       </c>
       <c r="J19" s="49" t="inlineStr">
@@ -2031,27 +2073,28 @@
         <v/>
       </c>
       <c r="M19" s="57" t="n"/>
-      <c r="N19" s="49" t="inlineStr">
+      <c r="N19" s="57" t="n"/>
+      <c r="O19" s="49" t="inlineStr">
         <is>
           <t>2024 Afv 295</t>
         </is>
       </c>
     </row>
     <row r="20">
-      <c r="A20" s="60" t="n">
+      <c r="A20" s="63" t="n">
         <v>16</v>
       </c>
-      <c r="B20" s="60" t="inlineStr">
+      <c r="B20" s="63" t="inlineStr">
         <is>
           <t>Foyen</t>
         </is>
       </c>
-      <c r="C20" s="60" t="inlineStr">
+      <c r="C20" s="63" t="inlineStr">
         <is>
           <t>2024</t>
         </is>
       </c>
-      <c r="D20" s="61" t="n">
+      <c r="D20" s="64" t="n">
         <v>277</v>
       </c>
       <c r="E20" s="49" t="inlineStr">
@@ -2059,10 +2102,10 @@
           <t>Affärsvärlden Apr-25</t>
         </is>
       </c>
-      <c r="F20" s="62" t="n"/>
+      <c r="F20" s="65" t="n"/>
       <c r="G20" s="49" t="inlineStr"/>
-      <c r="H20" s="62" t="n"/>
-      <c r="I20" s="60" t="n">
+      <c r="H20" s="65" t="n"/>
+      <c r="I20" s="63" t="n">
         <v>106</v>
       </c>
       <c r="J20" s="49" t="inlineStr">
@@ -2076,23 +2119,24 @@
         <v/>
       </c>
       <c r="M20" s="57" t="n"/>
-      <c r="N20" s="49" t="inlineStr"/>
+      <c r="N20" s="57" t="n"/>
+      <c r="O20" s="49" t="inlineStr"/>
     </row>
     <row r="21">
-      <c r="A21" s="60" t="n">
+      <c r="A21" s="63" t="n">
         <v>17</v>
       </c>
-      <c r="B21" s="60" t="inlineStr">
+      <c r="B21" s="63" t="inlineStr">
         <is>
           <t>Glimstedt</t>
         </is>
       </c>
-      <c r="C21" s="60" t="inlineStr">
+      <c r="C21" s="63" t="inlineStr">
         <is>
           <t>2024</t>
         </is>
       </c>
-      <c r="D21" s="61" t="n">
+      <c r="D21" s="64" t="n">
         <v>196</v>
       </c>
       <c r="E21" s="49" t="inlineStr">
@@ -2100,35 +2144,36 @@
           <t>Affärsvärlden Apr-25</t>
         </is>
       </c>
-      <c r="F21" s="62" t="n"/>
+      <c r="F21" s="65" t="n"/>
       <c r="G21" s="49" t="inlineStr"/>
-      <c r="H21" s="62" t="n"/>
-      <c r="I21" s="62" t="n"/>
+      <c r="H21" s="65" t="n"/>
+      <c r="I21" s="65" t="n"/>
       <c r="J21" s="49" t="inlineStr"/>
       <c r="K21" s="57" t="n"/>
       <c r="L21" s="57" t="n"/>
       <c r="M21" s="57" t="n"/>
-      <c r="N21" s="49" t="inlineStr">
+      <c r="N21" s="57" t="n"/>
+      <c r="O21" s="49" t="inlineStr">
         <is>
           <t>~200 staff on website includes Baltics (not used)</t>
         </is>
       </c>
     </row>
     <row r="22">
-      <c r="A22" s="60" t="n">
+      <c r="A22" s="63" t="n">
         <v>18</v>
       </c>
-      <c r="B22" s="60" t="inlineStr">
+      <c r="B22" s="63" t="inlineStr">
         <is>
           <t>Eversheds Sutherland</t>
         </is>
       </c>
-      <c r="C22" s="60" t="inlineStr">
+      <c r="C22" s="63" t="inlineStr">
         <is>
           <t>2025</t>
         </is>
       </c>
-      <c r="D22" s="61" t="n">
+      <c r="D22" s="64" t="n">
         <v>166</v>
       </c>
       <c r="E22" s="49" t="inlineStr">
@@ -2136,10 +2181,10 @@
           <t>Company accounts, net sales (AB)</t>
         </is>
       </c>
-      <c r="F22" s="62" t="n"/>
+      <c r="F22" s="65" t="n"/>
       <c r="G22" s="49" t="inlineStr"/>
-      <c r="H22" s="62" t="n"/>
-      <c r="I22" s="60" t="n">
+      <c r="H22" s="65" t="n"/>
+      <c r="I22" s="63" t="n">
         <v>59</v>
       </c>
       <c r="J22" s="49" t="inlineStr">
@@ -2153,27 +2198,28 @@
         <v/>
       </c>
       <c r="M22" s="57" t="n"/>
-      <c r="N22" s="49" t="inlineStr">
+      <c r="N22" s="57" t="n"/>
+      <c r="O22" s="49" t="inlineStr">
         <is>
           <t>2024 Afv 140</t>
         </is>
       </c>
     </row>
     <row r="23">
-      <c r="A23" s="60" t="n">
+      <c r="A23" s="63" t="n">
         <v>19</v>
       </c>
-      <c r="B23" s="60" t="inlineStr">
+      <c r="B23" s="63" t="inlineStr">
         <is>
           <t>Fylgia</t>
         </is>
       </c>
-      <c r="C23" s="60" t="inlineStr">
+      <c r="C23" s="63" t="inlineStr">
         <is>
           <t>2024</t>
         </is>
       </c>
-      <c r="D23" s="61" t="n">
+      <c r="D23" s="64" t="n">
         <v>131</v>
       </c>
       <c r="E23" s="49" t="inlineStr">
@@ -2181,35 +2227,36 @@
           <t>Affärsvärlden Apr-25</t>
         </is>
       </c>
-      <c r="F23" s="62" t="n"/>
+      <c r="F23" s="65" t="n"/>
       <c r="G23" s="49" t="inlineStr"/>
-      <c r="H23" s="62" t="n"/>
-      <c r="I23" s="62" t="n"/>
+      <c r="H23" s="65" t="n"/>
+      <c r="I23" s="65" t="n"/>
       <c r="J23" s="49" t="inlineStr"/>
       <c r="K23" s="57" t="n"/>
       <c r="L23" s="57" t="n"/>
       <c r="M23" s="57" t="n"/>
-      <c r="N23" s="49" t="inlineStr">
+      <c r="N23" s="57" t="n"/>
+      <c r="O23" s="49" t="inlineStr">
         <is>
           <t>Record 2025 (firm)</t>
         </is>
       </c>
     </row>
     <row r="24">
-      <c r="A24" s="60" t="n">
+      <c r="A24" s="63" t="n">
         <v>20</v>
       </c>
-      <c r="B24" s="60" t="inlineStr">
+      <c r="B24" s="63" t="inlineStr">
         <is>
           <t>Westerberg &amp; Partners</t>
         </is>
       </c>
-      <c r="C24" s="60" t="inlineStr">
+      <c r="C24" s="63" t="inlineStr">
         <is>
           <t>2025</t>
         </is>
       </c>
-      <c r="D24" s="61" t="n">
+      <c r="D24" s="64" t="n">
         <v>107</v>
       </c>
       <c r="E24" s="49" t="inlineStr">
@@ -2217,7 +2264,7 @@
           <t>Company accounts, net sales (AB)</t>
         </is>
       </c>
-      <c r="F24" s="60" t="n">
+      <c r="F24" s="63" t="n">
         <v>12</v>
       </c>
       <c r="G24" s="49" t="inlineStr">
@@ -2225,8 +2272,8 @@
           <t>Chambers 2026</t>
         </is>
       </c>
-      <c r="H24" s="62" t="n"/>
-      <c r="I24" s="60" t="n">
+      <c r="H24" s="65" t="n"/>
+      <c r="I24" s="63" t="n">
         <v>35</v>
       </c>
       <c r="J24" s="49" t="inlineStr">
@@ -2243,23 +2290,24 @@
         <v/>
       </c>
       <c r="M24" s="57" t="n"/>
-      <c r="N24" s="49" t="inlineStr"/>
+      <c r="N24" s="57" t="n"/>
+      <c r="O24" s="49" t="inlineStr"/>
     </row>
     <row r="25">
-      <c r="A25" s="60" t="n">
+      <c r="A25" s="63" t="n">
         <v>21</v>
       </c>
-      <c r="B25" s="60" t="inlineStr">
+      <c r="B25" s="63" t="inlineStr">
         <is>
           <t>Moll Wendén</t>
         </is>
       </c>
-      <c r="C25" s="60" t="inlineStr">
+      <c r="C25" s="63" t="inlineStr">
         <is>
           <t>2025</t>
         </is>
       </c>
-      <c r="D25" s="61" t="n">
+      <c r="D25" s="64" t="n">
         <v>101</v>
       </c>
       <c r="E25" s="49" t="inlineStr">
@@ -2267,10 +2315,10 @@
           <t>Company accounts, net sales (AB)</t>
         </is>
       </c>
-      <c r="F25" s="62" t="n"/>
+      <c r="F25" s="65" t="n"/>
       <c r="G25" s="49" t="inlineStr"/>
-      <c r="H25" s="62" t="n"/>
-      <c r="I25" s="60" t="n">
+      <c r="H25" s="65" t="n"/>
+      <c r="I25" s="63" t="n">
         <v>44</v>
       </c>
       <c r="J25" s="49" t="inlineStr">
@@ -2284,23 +2332,24 @@
         <v/>
       </c>
       <c r="M25" s="57" t="n"/>
-      <c r="N25" s="49" t="inlineStr"/>
+      <c r="N25" s="57" t="n"/>
+      <c r="O25" s="49" t="inlineStr"/>
     </row>
     <row r="26">
-      <c r="A26" s="60" t="n">
+      <c r="A26" s="63" t="n">
         <v>22</v>
       </c>
-      <c r="B26" s="60" t="inlineStr">
+      <c r="B26" s="63" t="inlineStr">
         <is>
           <t>Born</t>
         </is>
       </c>
-      <c r="C26" s="60" t="inlineStr">
+      <c r="C26" s="63" t="inlineStr">
         <is>
           <t>2024</t>
         </is>
       </c>
-      <c r="D26" s="61" t="n">
+      <c r="D26" s="64" t="n">
         <v>86</v>
       </c>
       <c r="E26" s="49" t="inlineStr">
@@ -2308,35 +2357,36 @@
           <t>Affärsvärlden Apr-25</t>
         </is>
       </c>
-      <c r="F26" s="62" t="n"/>
+      <c r="F26" s="65" t="n"/>
       <c r="G26" s="49" t="inlineStr"/>
-      <c r="H26" s="62" t="n"/>
-      <c r="I26" s="62" t="n"/>
+      <c r="H26" s="65" t="n"/>
+      <c r="I26" s="65" t="n"/>
       <c r="J26" s="49" t="inlineStr"/>
       <c r="K26" s="57" t="n"/>
       <c r="L26" s="57" t="n"/>
       <c r="M26" s="57" t="n"/>
-      <c r="N26" s="49" t="inlineStr">
+      <c r="N26" s="57" t="n"/>
+      <c r="O26" s="49" t="inlineStr">
         <is>
           <t>Part of AGRD since 2025</t>
         </is>
       </c>
     </row>
     <row r="27">
-      <c r="A27" s="60" t="n">
+      <c r="A27" s="63" t="n">
         <v>23</v>
       </c>
-      <c r="B27" s="60" t="inlineStr">
+      <c r="B27" s="63" t="inlineStr">
         <is>
           <t>Harvest</t>
         </is>
       </c>
-      <c r="C27" s="60" t="inlineStr">
+      <c r="C27" s="63" t="inlineStr">
         <is>
           <t>2025</t>
         </is>
       </c>
-      <c r="D27" s="61" t="n">
+      <c r="D27" s="64" t="n">
         <v>82</v>
       </c>
       <c r="E27" s="49" t="inlineStr">
@@ -2344,10 +2394,10 @@
           <t>Company accounts, net sales (AB)</t>
         </is>
       </c>
-      <c r="F27" s="62" t="n"/>
+      <c r="F27" s="65" t="n"/>
       <c r="G27" s="49" t="inlineStr"/>
-      <c r="H27" s="62" t="n"/>
-      <c r="I27" s="60" t="n">
+      <c r="H27" s="65" t="n"/>
+      <c r="I27" s="63" t="n">
         <v>27</v>
       </c>
       <c r="J27" s="49" t="inlineStr">
@@ -2361,23 +2411,24 @@
         <v/>
       </c>
       <c r="M27" s="57" t="n"/>
-      <c r="N27" s="49" t="inlineStr"/>
+      <c r="N27" s="57" t="n"/>
+      <c r="O27" s="49" t="inlineStr"/>
     </row>
     <row r="28">
-      <c r="A28" s="60" t="n">
+      <c r="A28" s="63" t="n">
         <v>24</v>
       </c>
-      <c r="B28" s="60" t="inlineStr">
+      <c r="B28" s="63" t="inlineStr">
         <is>
           <t>Synch</t>
         </is>
       </c>
-      <c r="C28" s="60" t="inlineStr">
+      <c r="C28" s="63" t="inlineStr">
         <is>
           <t>2025</t>
         </is>
       </c>
-      <c r="D28" s="61" t="n">
+      <c r="D28" s="64" t="n">
         <v>81</v>
       </c>
       <c r="E28" s="49" t="inlineStr">
@@ -2385,10 +2436,10 @@
           <t>Company accounts, net sales (AB)</t>
         </is>
       </c>
-      <c r="F28" s="62" t="n"/>
+      <c r="F28" s="65" t="n"/>
       <c r="G28" s="49" t="inlineStr"/>
-      <c r="H28" s="62" t="n"/>
-      <c r="I28" s="60" t="n">
+      <c r="H28" s="65" t="n"/>
+      <c r="I28" s="63" t="n">
         <v>38</v>
       </c>
       <c r="J28" s="49" t="inlineStr">
@@ -2402,27 +2453,28 @@
         <v/>
       </c>
       <c r="M28" s="57" t="n"/>
-      <c r="N28" s="49" t="inlineStr">
+      <c r="N28" s="57" t="n"/>
+      <c r="O28" s="49" t="inlineStr">
         <is>
           <t>Part of AGRD since 2025</t>
         </is>
       </c>
     </row>
     <row r="29">
-      <c r="A29" s="60" t="n">
+      <c r="A29" s="63" t="n">
         <v>25</v>
       </c>
-      <c r="B29" s="60" t="inlineStr">
+      <c r="B29" s="63" t="inlineStr">
         <is>
           <t>Kastell</t>
         </is>
       </c>
-      <c r="C29" s="60" t="inlineStr">
+      <c r="C29" s="63" t="inlineStr">
         <is>
           <t>2025</t>
         </is>
       </c>
-      <c r="D29" s="61" t="n">
+      <c r="D29" s="64" t="n">
         <v>80</v>
       </c>
       <c r="E29" s="49" t="inlineStr">
@@ -2430,7 +2482,7 @@
           <t>Company accounts, net sales (AB)</t>
         </is>
       </c>
-      <c r="F29" s="60" t="n">
+      <c r="F29" s="63" t="n">
         <v>9</v>
       </c>
       <c r="G29" s="49" t="inlineStr">
@@ -2438,10 +2490,10 @@
           <t>Chambers 2026</t>
         </is>
       </c>
-      <c r="H29" s="60" t="n">
+      <c r="H29" s="63" t="n">
         <v>19</v>
       </c>
-      <c r="I29" s="60" t="n">
+      <c r="I29" s="63" t="n">
         <v>21</v>
       </c>
       <c r="J29" s="49" t="inlineStr">
@@ -2461,7 +2513,11 @@
         <f>D29/H29</f>
         <v/>
       </c>
-      <c r="N29" s="49" t="inlineStr"/>
+      <c r="N29" s="66">
+        <f>F29/H29</f>
+        <v/>
+      </c>
+      <c r="O29" s="49" t="inlineStr"/>
     </row>
     <row r="30">
       <c r="B30" s="46" t="inlineStr">
@@ -2506,41 +2562,48 @@
     <row r="35">
       <c r="A35" s="45" t="inlineStr">
         <is>
-          <t>Setterwalls partner count (37) is as supplied to Chambers and looks low against the firm size. Roschier group partner count (52) includes Finland and is not used. Magnusson: no Swedish revenue or headcount found.</t>
+          <t>Leverage = partners / lawyers (lawyer counts as supplied to Chambers include partners); shown only where both counts exist. White &amp; Case uses the implied partner count.</t>
         </is>
       </c>
     </row>
     <row r="36">
       <c r="A36" s="45" t="inlineStr">
         <is>
-          <t>Sources: Affärsvärlden 12-Apr-25 https://www.affarsvarlden.se/artikel/vinge-gar-om-msa-sa-gar-det-for-affarsjuristerna ; 3-Oct-25 https://www.affarsvarlden.se/artikel/affarsjuristerna-gar-starkt-finns-fler-bolag-i-ipo-pipelinen ;</t>
+          <t>Setterwalls partner count (37) is as supplied to Chambers and looks low against the firm size. Roschier group partner count (52) includes Finland and is not used. Magnusson: no Swedish revenue or headcount found.</t>
         </is>
       </c>
     </row>
     <row r="37">
       <c r="A37" s="45" t="inlineStr">
         <is>
-          <t>Realtid 7-Aug-26 https://www.realtid.se/juridik/vinge-tappar-mark-mannheimer-swartling-drar-ifran/ ; Realtid 26-Apr-26 https://www.realtid.se/juridik/affarsjuridiken-vaxer-men-sprickorna-syns/ ; Realtid 27-Nov-25 https://www.realtid.se/juridik/white-case-dubblade-omsattningen-var-styrka/ ;</t>
+          <t>Sources: Affärsvärlden 12-Apr-25 https://www.affarsvarlden.se/artikel/vinge-gar-om-msa-sa-gar-det-for-affarsjuristerna ; 3-Oct-25 https://www.affarsvarlden.se/artikel/affarsjuristerna-gar-starkt-finns-fler-bolag-i-ipo-pipelinen ;</t>
         </is>
       </c>
     </row>
     <row r="38">
       <c r="A38" s="45" t="inlineStr">
         <is>
-          <t>Realtid 1-Sep-26 https://www.realtid.se/juridik/setterwalls-malmokontor-gar-till-riskkapitalagda-agrd/ ; Affärsvärlden 5-Oct-26 (Schjødt) https://www.affarsvarlden.se/artikel/schjdt-vaxer-snabbast--men-konkurrensen-hardnar ;</t>
+          <t>Realtid 7-Aug-26 https://www.realtid.se/juridik/vinge-tappar-mark-mannheimer-swartling-drar-ifran/ ; Realtid 26-Apr-26 https://www.realtid.se/juridik/affarsjuridiken-vaxer-men-sprickorna-syns/ ; Realtid 27-Nov-25 https://www.realtid.se/juridik/white-case-dubblade-omsattningen-var-styrka/ ;</t>
         </is>
       </c>
     </row>
     <row r="39">
       <c r="A39" s="45" t="inlineStr">
         <is>
+          <t>Realtid 1-Sep-26 https://www.realtid.se/juridik/setterwalls-malmokontor-gar-till-riskkapitalagda-agrd/ ; Affärsvärlden 5-Oct-26 (Schjødt) https://www.affarsvarlden.se/artikel/schjdt-vaxer-snabbast--men-konkurrensen-hardnar ;</t>
+        </is>
+      </c>
+    </row>
+    <row r="40">
+      <c r="A40" s="45" t="inlineStr">
+        <is>
           <t>company accounts via https://www.allabolag.se/{org.nr} ; Chambers Europe 2026 firm profiles (firm-supplied "top figures"); firm websites.</t>
         </is>
       </c>
     </row>
   </sheetData>
   <mergeCells count="1">
-    <mergeCell ref="A2:N2"/>
+    <mergeCell ref="A2:O2"/>
   </mergeCells>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Add niche firms tab (ranked independents incl. PE-owned and Legal 500 firms to watch) and directory headcount data
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01Tu61bPEQej1E6sErbEFanY
</commit_message>
<xml_diff>
--- a/research/swedish_legal_market.xlsx
+++ b/research/swedish_legal_market.xlsx
@@ -10,11 +10,12 @@
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="A. Market size" sheetId="1" state="visible" r:id="rId1"/>
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="A. Firms" sheetId="2" state="visible" r:id="rId2"/>
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="A. Growth drivers" sheetId="3" state="visible" r:id="rId3"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="B. Practice rankings" sheetId="4" state="visible" r:id="rId4"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="B. Rankings raw" sheetId="5" state="visible" r:id="rId5"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="A. Niche firms" sheetId="4" state="visible" r:id="rId4"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="B. Practice rankings" sheetId="5" state="visible" r:id="rId5"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="B. Rankings raw" sheetId="6" state="visible" r:id="rId6"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="4" hidden="1">'B. Rankings raw'!$A$1:$E$661</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="5" hidden="1">'B. Rankings raw'!$A$1:$E$661</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -286,7 +287,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="67">
+  <cellXfs count="74">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
@@ -450,6 +451,27 @@
       <alignment vertical="top"/>
     </xf>
     <xf numFmtId="9" fontId="0" fillId="0" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="top"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="7" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="top"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="7" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="5" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="top"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="5" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="6" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="top"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="6" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0" hidden="0"/>
@@ -3174,6 +3196,1979 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
+  <dimension ref="A1:K59"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="26" customWidth="1" min="1" max="1"/>
+    <col width="30" customWidth="1" min="2" max="2"/>
+    <col width="10" customWidth="1" min="3" max="3"/>
+    <col width="10" customWidth="1" min="4" max="4"/>
+    <col width="10" customWidth="1" min="5" max="5"/>
+    <col width="9" customWidth="1" min="6" max="6"/>
+    <col width="36" customWidth="1" min="7" max="7"/>
+    <col width="28" customWidth="1" min="8" max="8"/>
+    <col width="9" customWidth="1" min="9" max="9"/>
+    <col width="9" customWidth="1" min="10" max="10"/>
+    <col width="28" customWidth="1" min="11" max="11"/>
+  </cols>
+  <sheetData>
+    <row r="1">
+      <c r="A1" s="1" t="inlineStr">
+        <is>
+          <t>A5. Niche / independent Swedish law firms ranked by Chambers or Legal 500</t>
+        </is>
+      </c>
+    </row>
+    <row r="2" ht="60" customHeight="1">
+      <c r="A2" s="2" t="inlineStr">
+        <is>
+          <t>Universe: firm-level rankings in Chambers Europe 2026 (Sweden) and Legal 500 EMEA (Sweden), incl. Legal 500 "firms to watch". Excludes international firms and the nine largest Swedish full-service firms. Counts: 45 ranked independents (incl. PE-owned AGRD firms) + 2 firms to watch only = 47; +5 borderline mid-size firms = 52. Partner/lawyer counts are firm-supplied to Legal 500 / Chambers (2026), blank where not published.</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" s="52" t="inlineStr">
+        <is>
+          <t>Firm</t>
+        </is>
+      </c>
+      <c r="B4" s="52" t="inlineStr">
+        <is>
+          <t>Category</t>
+        </is>
+      </c>
+      <c r="C4" s="52" t="inlineStr">
+        <is>
+          <t># Chambers rankings</t>
+        </is>
+      </c>
+      <c r="D4" s="52" t="inlineStr">
+        <is>
+          <t># Legal 500 rankings</t>
+        </is>
+      </c>
+      <c r="E4" s="52" t="inlineStr">
+        <is>
+          <t># L500 firm-to-watch</t>
+        </is>
+      </c>
+      <c r="F4" s="52" t="inlineStr">
+        <is>
+          <t>Best band/tier</t>
+        </is>
+      </c>
+      <c r="G4" s="52" t="inlineStr">
+        <is>
+          <t>Practice area(s) at best band/tier</t>
+        </is>
+      </c>
+      <c r="H4" s="52" t="inlineStr">
+        <is>
+          <t>Firm-to-watch areas</t>
+        </is>
+      </c>
+      <c r="I4" s="52" t="inlineStr">
+        <is>
+          <t>Partners</t>
+        </is>
+      </c>
+      <c r="J4" s="52" t="inlineStr">
+        <is>
+          <t>Lawyers</t>
+        </is>
+      </c>
+      <c r="K4" s="52" t="inlineStr">
+        <is>
+          <t>Headcount source</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" s="67" t="inlineStr">
+        <is>
+          <t>Hellström</t>
+        </is>
+      </c>
+      <c r="B5" s="49" t="inlineStr">
+        <is>
+          <t>Ranked independent</t>
+        </is>
+      </c>
+      <c r="C5" s="67" t="n">
+        <v>1</v>
+      </c>
+      <c r="D5" s="67" t="n">
+        <v>7</v>
+      </c>
+      <c r="E5" s="67" t="n">
+        <v>0</v>
+      </c>
+      <c r="F5" s="67" t="n">
+        <v>2</v>
+      </c>
+      <c r="G5" s="49" t="inlineStr">
+        <is>
+          <t>Data protection</t>
+        </is>
+      </c>
+      <c r="H5" s="49" t="n"/>
+      <c r="I5" s="67" t="n">
+        <v>22</v>
+      </c>
+      <c r="J5" s="67" t="n">
+        <v>49</v>
+      </c>
+      <c r="K5" s="49" t="inlineStr">
+        <is>
+          <t>L500 (22 partners, 10 senior assoc., 17 assoc.)</t>
+        </is>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" s="67" t="inlineStr">
+        <is>
+          <t>TIME DANOWSKY Advokatbyrå AB</t>
+        </is>
+      </c>
+      <c r="B6" s="49" t="inlineStr">
+        <is>
+          <t>Ranked independent</t>
+        </is>
+      </c>
+      <c r="C6" s="67" t="n">
+        <v>3</v>
+      </c>
+      <c r="D6" s="67" t="n">
+        <v>4</v>
+      </c>
+      <c r="E6" s="67" t="n">
+        <v>0</v>
+      </c>
+      <c r="F6" s="67" t="n">
+        <v>2</v>
+      </c>
+      <c r="G6" s="49" t="inlineStr">
+        <is>
+          <t>Data protection; IT / TMT</t>
+        </is>
+      </c>
+      <c r="H6" s="49" t="n"/>
+      <c r="I6" s="67" t="n"/>
+      <c r="J6" s="67" t="n">
+        <v>22</v>
+      </c>
+      <c r="K6" s="49" t="inlineStr">
+        <is>
+          <t>L500</t>
+        </is>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" s="67" t="inlineStr">
+        <is>
+          <t>Kastell</t>
+        </is>
+      </c>
+      <c r="B7" s="49" t="inlineStr">
+        <is>
+          <t>Ranked independent</t>
+        </is>
+      </c>
+      <c r="C7" s="67" t="n">
+        <v>3</v>
+      </c>
+      <c r="D7" s="67" t="n">
+        <v>3</v>
+      </c>
+      <c r="E7" s="67" t="n">
+        <v>0</v>
+      </c>
+      <c r="F7" s="67" t="n">
+        <v>2</v>
+      </c>
+      <c r="G7" s="49" t="inlineStr">
+        <is>
+          <t>Competition / EU; Public procurement</t>
+        </is>
+      </c>
+      <c r="H7" s="49" t="n"/>
+      <c r="I7" s="67" t="n">
+        <v>9</v>
+      </c>
+      <c r="J7" s="67" t="n">
+        <v>19</v>
+      </c>
+      <c r="K7" s="49" t="inlineStr">
+        <is>
+          <t>Chambers</t>
+        </is>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" s="67" t="inlineStr">
+        <is>
+          <t>Westerberg &amp; Partners</t>
+        </is>
+      </c>
+      <c r="B8" s="49" t="inlineStr">
+        <is>
+          <t>Ranked independent</t>
+        </is>
+      </c>
+      <c r="C8" s="67" t="n">
+        <v>2</v>
+      </c>
+      <c r="D8" s="67" t="n">
+        <v>4</v>
+      </c>
+      <c r="E8" s="67" t="n">
+        <v>0</v>
+      </c>
+      <c r="F8" s="67" t="n">
+        <v>1</v>
+      </c>
+      <c r="G8" s="49" t="inlineStr">
+        <is>
+          <t>IP; Insurance</t>
+        </is>
+      </c>
+      <c r="H8" s="49" t="n"/>
+      <c r="I8" s="67" t="n">
+        <v>12</v>
+      </c>
+      <c r="J8" s="67" t="n"/>
+      <c r="K8" s="49" t="inlineStr">
+        <is>
+          <t>Chambers</t>
+        </is>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" s="67" t="inlineStr">
+        <is>
+          <t>Kahn Pedersen</t>
+        </is>
+      </c>
+      <c r="B9" s="49" t="inlineStr">
+        <is>
+          <t>Ranked independent</t>
+        </is>
+      </c>
+      <c r="C9" s="67" t="n">
+        <v>2</v>
+      </c>
+      <c r="D9" s="67" t="n">
+        <v>3</v>
+      </c>
+      <c r="E9" s="67" t="n">
+        <v>0</v>
+      </c>
+      <c r="F9" s="67" t="n">
+        <v>1</v>
+      </c>
+      <c r="G9" s="49" t="inlineStr">
+        <is>
+          <t>Data protection; IT / TMT; Public procurement</t>
+        </is>
+      </c>
+      <c r="H9" s="49" t="n"/>
+      <c r="I9" s="67" t="n">
+        <v>6</v>
+      </c>
+      <c r="J9" s="67" t="n">
+        <v>19</v>
+      </c>
+      <c r="K9" s="49" t="inlineStr">
+        <is>
+          <t>L500/Chambers</t>
+        </is>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" s="67" t="inlineStr">
+        <is>
+          <t>Nordia Law</t>
+        </is>
+      </c>
+      <c r="B10" s="49" t="inlineStr">
+        <is>
+          <t>Ranked independent</t>
+        </is>
+      </c>
+      <c r="C10" s="67" t="n">
+        <v>1</v>
+      </c>
+      <c r="D10" s="67" t="n">
+        <v>4</v>
+      </c>
+      <c r="E10" s="67" t="n">
+        <v>0</v>
+      </c>
+      <c r="F10" s="67" t="n">
+        <v>2</v>
+      </c>
+      <c r="G10" s="49" t="inlineStr">
+        <is>
+          <t>Insurance</t>
+        </is>
+      </c>
+      <c r="H10" s="49" t="n"/>
+      <c r="I10" s="67" t="n"/>
+      <c r="J10" s="67" t="n"/>
+      <c r="K10" s="49" t="n"/>
+    </row>
+    <row r="11">
+      <c r="A11" s="67" t="inlineStr">
+        <is>
+          <t>AG Advokat</t>
+        </is>
+      </c>
+      <c r="B11" s="49" t="inlineStr">
+        <is>
+          <t>Ranked independent</t>
+        </is>
+      </c>
+      <c r="C11" s="67" t="n">
+        <v>1</v>
+      </c>
+      <c r="D11" s="67" t="n">
+        <v>3</v>
+      </c>
+      <c r="E11" s="67" t="n">
+        <v>0</v>
+      </c>
+      <c r="F11" s="67" t="n">
+        <v>1</v>
+      </c>
+      <c r="G11" s="49" t="inlineStr">
+        <is>
+          <t>Real estate</t>
+        </is>
+      </c>
+      <c r="H11" s="49" t="n"/>
+      <c r="I11" s="67" t="n"/>
+      <c r="J11" s="67" t="n">
+        <v>41</v>
+      </c>
+      <c r="K11" s="49" t="inlineStr">
+        <is>
+          <t>L500</t>
+        </is>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" s="67" t="inlineStr">
+        <is>
+          <t>Bokwall Rislund</t>
+        </is>
+      </c>
+      <c r="B12" s="49" t="inlineStr">
+        <is>
+          <t>Ranked independent</t>
+        </is>
+      </c>
+      <c r="C12" s="67" t="n">
+        <v>2</v>
+      </c>
+      <c r="D12" s="67" t="n">
+        <v>2</v>
+      </c>
+      <c r="E12" s="67" t="n">
+        <v>0</v>
+      </c>
+      <c r="F12" s="67" t="n">
+        <v>1</v>
+      </c>
+      <c r="G12" s="49" t="inlineStr">
+        <is>
+          <t>Competition / EU; Public procurement</t>
+        </is>
+      </c>
+      <c r="H12" s="49" t="n"/>
+      <c r="I12" s="67" t="n"/>
+      <c r="J12" s="67" t="n"/>
+      <c r="K12" s="49" t="n"/>
+    </row>
+    <row r="13">
+      <c r="A13" s="67" t="inlineStr">
+        <is>
+          <t>Sandart &amp; Partners</t>
+        </is>
+      </c>
+      <c r="B13" s="49" t="inlineStr">
+        <is>
+          <t>Ranked independent</t>
+        </is>
+      </c>
+      <c r="C13" s="67" t="n">
+        <v>2</v>
+      </c>
+      <c r="D13" s="67" t="n">
+        <v>2</v>
+      </c>
+      <c r="E13" s="67" t="n">
+        <v>0</v>
+      </c>
+      <c r="F13" s="67" t="n">
+        <v>1</v>
+      </c>
+      <c r="G13" s="49" t="inlineStr">
+        <is>
+          <t>IP</t>
+        </is>
+      </c>
+      <c r="H13" s="49" t="n"/>
+      <c r="I13" s="67" t="n">
+        <v>10</v>
+      </c>
+      <c r="J13" s="67" t="n">
+        <v>12</v>
+      </c>
+      <c r="K13" s="49" t="inlineStr">
+        <is>
+          <t>L500</t>
+        </is>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" s="67" t="inlineStr">
+        <is>
+          <t>Brick</t>
+        </is>
+      </c>
+      <c r="B14" s="49" t="inlineStr">
+        <is>
+          <t>Ranked independent</t>
+        </is>
+      </c>
+      <c r="C14" s="67" t="n">
+        <v>1</v>
+      </c>
+      <c r="D14" s="67" t="n">
+        <v>2</v>
+      </c>
+      <c r="E14" s="67" t="n">
+        <v>0</v>
+      </c>
+      <c r="F14" s="67" t="n">
+        <v>2</v>
+      </c>
+      <c r="G14" s="49" t="inlineStr">
+        <is>
+          <t>Real estate</t>
+        </is>
+      </c>
+      <c r="H14" s="49" t="n"/>
+      <c r="I14" s="67" t="n"/>
+      <c r="J14" s="67" t="n"/>
+      <c r="K14" s="49" t="n"/>
+    </row>
+    <row r="15">
+      <c r="A15" s="67" t="inlineStr">
+        <is>
+          <t>Kompass</t>
+        </is>
+      </c>
+      <c r="B15" s="49" t="inlineStr">
+        <is>
+          <t>Ranked independent</t>
+        </is>
+      </c>
+      <c r="C15" s="67" t="n">
+        <v>2</v>
+      </c>
+      <c r="D15" s="67" t="n">
+        <v>1</v>
+      </c>
+      <c r="E15" s="67" t="n">
+        <v>0</v>
+      </c>
+      <c r="F15" s="67" t="n">
+        <v>3</v>
+      </c>
+      <c r="G15" s="49" t="inlineStr">
+        <is>
+          <t>Insurance</t>
+        </is>
+      </c>
+      <c r="H15" s="49" t="n"/>
+      <c r="I15" s="67" t="n">
+        <v>4</v>
+      </c>
+      <c r="J15" s="67" t="n">
+        <v>15</v>
+      </c>
+      <c r="K15" s="49" t="inlineStr">
+        <is>
+          <t>L500</t>
+        </is>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" s="67" t="inlineStr">
+        <is>
+          <t>A1 Advokater</t>
+        </is>
+      </c>
+      <c r="B16" s="49" t="inlineStr">
+        <is>
+          <t>Ranked independent</t>
+        </is>
+      </c>
+      <c r="C16" s="67" t="n">
+        <v>1</v>
+      </c>
+      <c r="D16" s="67" t="n">
+        <v>1</v>
+      </c>
+      <c r="E16" s="67" t="n">
+        <v>0</v>
+      </c>
+      <c r="F16" s="67" t="n">
+        <v>4</v>
+      </c>
+      <c r="G16" s="49" t="inlineStr">
+        <is>
+          <t>Dispute resolution</t>
+        </is>
+      </c>
+      <c r="H16" s="49" t="n"/>
+      <c r="I16" s="67" t="n"/>
+      <c r="J16" s="67" t="n"/>
+      <c r="K16" s="49" t="inlineStr">
+        <is>
+          <t>Chambers: 17 staff</t>
+        </is>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" s="67" t="inlineStr">
+        <is>
+          <t>Elmzell</t>
+        </is>
+      </c>
+      <c r="B17" s="49" t="inlineStr">
+        <is>
+          <t>Ranked independent</t>
+        </is>
+      </c>
+      <c r="C17" s="67" t="n">
+        <v>1</v>
+      </c>
+      <c r="D17" s="67" t="n">
+        <v>1</v>
+      </c>
+      <c r="E17" s="67" t="n">
+        <v>0</v>
+      </c>
+      <c r="F17" s="67" t="n">
+        <v>2</v>
+      </c>
+      <c r="G17" s="49" t="inlineStr">
+        <is>
+          <t>Employment</t>
+        </is>
+      </c>
+      <c r="H17" s="49" t="n"/>
+      <c r="I17" s="67" t="n"/>
+      <c r="J17" s="67" t="n"/>
+      <c r="K17" s="49" t="n"/>
+    </row>
+    <row r="18">
+      <c r="A18" s="67" t="inlineStr">
+        <is>
+          <t>Fröberg &amp; Lundholm</t>
+        </is>
+      </c>
+      <c r="B18" s="49" t="inlineStr">
+        <is>
+          <t>Ranked independent</t>
+        </is>
+      </c>
+      <c r="C18" s="67" t="n">
+        <v>1</v>
+      </c>
+      <c r="D18" s="67" t="n">
+        <v>1</v>
+      </c>
+      <c r="E18" s="67" t="n">
+        <v>0</v>
+      </c>
+      <c r="F18" s="67" t="n">
+        <v>1</v>
+      </c>
+      <c r="G18" s="49" t="inlineStr">
+        <is>
+          <t>Environment</t>
+        </is>
+      </c>
+      <c r="H18" s="49" t="n"/>
+      <c r="I18" s="67" t="n"/>
+      <c r="J18" s="67" t="n"/>
+      <c r="K18" s="49" t="n"/>
+    </row>
+    <row r="19">
+      <c r="A19" s="67" t="inlineStr">
+        <is>
+          <t>Gulliksson</t>
+        </is>
+      </c>
+      <c r="B19" s="49" t="inlineStr">
+        <is>
+          <t>Ranked independent</t>
+        </is>
+      </c>
+      <c r="C19" s="67" t="n">
+        <v>1</v>
+      </c>
+      <c r="D19" s="67" t="n">
+        <v>1</v>
+      </c>
+      <c r="E19" s="67" t="n">
+        <v>0</v>
+      </c>
+      <c r="F19" s="67" t="n">
+        <v>2</v>
+      </c>
+      <c r="G19" s="49" t="inlineStr">
+        <is>
+          <t>IP</t>
+        </is>
+      </c>
+      <c r="H19" s="49" t="n"/>
+      <c r="I19" s="67" t="n"/>
+      <c r="J19" s="67" t="n">
+        <v>41</v>
+      </c>
+      <c r="K19" s="49" t="inlineStr">
+        <is>
+          <t>L500</t>
+        </is>
+      </c>
+    </row>
+    <row r="20">
+      <c r="A20" s="67" t="inlineStr">
+        <is>
+          <t>Harvest</t>
+        </is>
+      </c>
+      <c r="B20" s="49" t="inlineStr">
+        <is>
+          <t>Ranked independent</t>
+        </is>
+      </c>
+      <c r="C20" s="67" t="n">
+        <v>0</v>
+      </c>
+      <c r="D20" s="67" t="n">
+        <v>2</v>
+      </c>
+      <c r="E20" s="67" t="n">
+        <v>0</v>
+      </c>
+      <c r="F20" s="67" t="n">
+        <v>3</v>
+      </c>
+      <c r="G20" s="49" t="inlineStr">
+        <is>
+          <t>Banking &amp; finance; Fintech</t>
+        </is>
+      </c>
+      <c r="H20" s="49" t="n"/>
+      <c r="I20" s="67" t="n"/>
+      <c r="J20" s="67" t="n"/>
+      <c r="K20" s="49" t="n"/>
+    </row>
+    <row r="21">
+      <c r="A21" s="67" t="inlineStr">
+        <is>
+          <t>Norburg &amp; Scherp</t>
+        </is>
+      </c>
+      <c r="B21" s="49" t="inlineStr">
+        <is>
+          <t>Ranked independent</t>
+        </is>
+      </c>
+      <c r="C21" s="67" t="n">
+        <v>1</v>
+      </c>
+      <c r="D21" s="67" t="n">
+        <v>1</v>
+      </c>
+      <c r="E21" s="67" t="n">
+        <v>0</v>
+      </c>
+      <c r="F21" s="67" t="n">
+        <v>3</v>
+      </c>
+      <c r="G21" s="49" t="inlineStr">
+        <is>
+          <t>Dispute resolution</t>
+        </is>
+      </c>
+      <c r="H21" s="49" t="n"/>
+      <c r="I21" s="67" t="n"/>
+      <c r="J21" s="67" t="n">
+        <v>18</v>
+      </c>
+      <c r="K21" s="49" t="inlineStr">
+        <is>
+          <t>L500</t>
+        </is>
+      </c>
+    </row>
+    <row r="22">
+      <c r="A22" s="67" t="inlineStr">
+        <is>
+          <t>Norma</t>
+        </is>
+      </c>
+      <c r="B22" s="49" t="inlineStr">
+        <is>
+          <t>Ranked independent</t>
+        </is>
+      </c>
+      <c r="C22" s="67" t="n">
+        <v>0</v>
+      </c>
+      <c r="D22" s="67" t="n">
+        <v>2</v>
+      </c>
+      <c r="E22" s="67" t="n">
+        <v>0</v>
+      </c>
+      <c r="F22" s="67" t="n">
+        <v>4</v>
+      </c>
+      <c r="G22" s="49" t="inlineStr">
+        <is>
+          <t>Real estate</t>
+        </is>
+      </c>
+      <c r="H22" s="49" t="n"/>
+      <c r="I22" s="67" t="n"/>
+      <c r="J22" s="67" t="n"/>
+      <c r="K22" s="49" t="n"/>
+    </row>
+    <row r="23">
+      <c r="A23" s="67" t="inlineStr">
+        <is>
+          <t>RE:FI STHLM</t>
+        </is>
+      </c>
+      <c r="B23" s="49" t="inlineStr">
+        <is>
+          <t>Ranked independent</t>
+        </is>
+      </c>
+      <c r="C23" s="67" t="n">
+        <v>1</v>
+      </c>
+      <c r="D23" s="67" t="n">
+        <v>1</v>
+      </c>
+      <c r="E23" s="67" t="n">
+        <v>0</v>
+      </c>
+      <c r="F23" s="67" t="n">
+        <v>3</v>
+      </c>
+      <c r="G23" s="49" t="inlineStr">
+        <is>
+          <t>Banking &amp; finance</t>
+        </is>
+      </c>
+      <c r="H23" s="49" t="n"/>
+      <c r="I23" s="67" t="n"/>
+      <c r="J23" s="67" t="n"/>
+      <c r="K23" s="49" t="n"/>
+    </row>
+    <row r="24">
+      <c r="A24" s="67" t="inlineStr">
+        <is>
+          <t>REAL Advokatbyrå</t>
+        </is>
+      </c>
+      <c r="B24" s="49" t="inlineStr">
+        <is>
+          <t>Ranked independent</t>
+        </is>
+      </c>
+      <c r="C24" s="67" t="n">
+        <v>1</v>
+      </c>
+      <c r="D24" s="67" t="n">
+        <v>1</v>
+      </c>
+      <c r="E24" s="67" t="n">
+        <v>0</v>
+      </c>
+      <c r="F24" s="67" t="n">
+        <v>2</v>
+      </c>
+      <c r="G24" s="49" t="inlineStr">
+        <is>
+          <t>Real estate</t>
+        </is>
+      </c>
+      <c r="H24" s="49" t="n"/>
+      <c r="I24" s="67" t="n">
+        <v>5</v>
+      </c>
+      <c r="J24" s="67" t="n">
+        <v>20</v>
+      </c>
+      <c r="K24" s="49" t="inlineStr">
+        <is>
+          <t>L500/Chambers</t>
+        </is>
+      </c>
+    </row>
+    <row r="25">
+      <c r="A25" s="67" t="inlineStr">
+        <is>
+          <t>Skierfe</t>
+        </is>
+      </c>
+      <c r="B25" s="49" t="inlineStr">
+        <is>
+          <t>Ranked independent</t>
+        </is>
+      </c>
+      <c r="C25" s="67" t="n">
+        <v>1</v>
+      </c>
+      <c r="D25" s="67" t="n">
+        <v>1</v>
+      </c>
+      <c r="E25" s="67" t="n">
+        <v>0</v>
+      </c>
+      <c r="F25" s="67" t="n">
+        <v>3</v>
+      </c>
+      <c r="G25" s="49" t="inlineStr">
+        <is>
+          <t>Real estate</t>
+        </is>
+      </c>
+      <c r="H25" s="49" t="n"/>
+      <c r="I25" s="67" t="n"/>
+      <c r="J25" s="67" t="n"/>
+      <c r="K25" s="49" t="n"/>
+    </row>
+    <row r="26">
+      <c r="A26" s="67" t="inlineStr">
+        <is>
+          <t>Ström</t>
+        </is>
+      </c>
+      <c r="B26" s="49" t="inlineStr">
+        <is>
+          <t>Ranked independent</t>
+        </is>
+      </c>
+      <c r="C26" s="67" t="n">
+        <v>1</v>
+      </c>
+      <c r="D26" s="67" t="n">
+        <v>1</v>
+      </c>
+      <c r="E26" s="67" t="n">
+        <v>0</v>
+      </c>
+      <c r="F26" s="67" t="n">
+        <v>2</v>
+      </c>
+      <c r="G26" s="49" t="inlineStr">
+        <is>
+          <t>IP</t>
+        </is>
+      </c>
+      <c r="H26" s="49" t="n"/>
+      <c r="I26" s="67" t="n">
+        <v>5</v>
+      </c>
+      <c r="J26" s="67" t="n"/>
+      <c r="K26" s="49" t="inlineStr">
+        <is>
+          <t>Chambers</t>
+        </is>
+      </c>
+    </row>
+    <row r="27">
+      <c r="A27" s="67" t="inlineStr">
+        <is>
+          <t>Ulfsdotter</t>
+        </is>
+      </c>
+      <c r="B27" s="49" t="inlineStr">
+        <is>
+          <t>Ranked independent</t>
+        </is>
+      </c>
+      <c r="C27" s="67" t="n">
+        <v>1</v>
+      </c>
+      <c r="D27" s="67" t="n">
+        <v>1</v>
+      </c>
+      <c r="E27" s="67" t="n">
+        <v>0</v>
+      </c>
+      <c r="F27" s="67" t="n">
+        <v>2</v>
+      </c>
+      <c r="G27" s="49" t="inlineStr">
+        <is>
+          <t>Public procurement</t>
+        </is>
+      </c>
+      <c r="H27" s="49" t="n"/>
+      <c r="I27" s="67" t="n"/>
+      <c r="J27" s="67" t="n"/>
+      <c r="K27" s="49" t="n"/>
+    </row>
+    <row r="28">
+      <c r="A28" s="67" t="inlineStr">
+        <is>
+          <t>Wallin &amp; Partners</t>
+        </is>
+      </c>
+      <c r="B28" s="49" t="inlineStr">
+        <is>
+          <t>Ranked independent</t>
+        </is>
+      </c>
+      <c r="C28" s="67" t="n">
+        <v>1</v>
+      </c>
+      <c r="D28" s="67" t="n">
+        <v>1</v>
+      </c>
+      <c r="E28" s="67" t="n">
+        <v>0</v>
+      </c>
+      <c r="F28" s="67" t="n">
+        <v>3</v>
+      </c>
+      <c r="G28" s="49" t="inlineStr">
+        <is>
+          <t>Dispute resolution</t>
+        </is>
+      </c>
+      <c r="H28" s="49" t="n"/>
+      <c r="I28" s="67" t="n"/>
+      <c r="J28" s="67" t="n"/>
+      <c r="K28" s="49" t="n"/>
+    </row>
+    <row r="29">
+      <c r="A29" s="67" t="inlineStr">
+        <is>
+          <t>edpLaw</t>
+        </is>
+      </c>
+      <c r="B29" s="49" t="inlineStr">
+        <is>
+          <t>Ranked independent</t>
+        </is>
+      </c>
+      <c r="C29" s="67" t="n">
+        <v>0</v>
+      </c>
+      <c r="D29" s="67" t="n">
+        <v>2</v>
+      </c>
+      <c r="E29" s="67" t="n">
+        <v>0</v>
+      </c>
+      <c r="F29" s="67" t="n">
+        <v>2</v>
+      </c>
+      <c r="G29" s="49" t="inlineStr">
+        <is>
+          <t>Data protection</t>
+        </is>
+      </c>
+      <c r="H29" s="49" t="n"/>
+      <c r="I29" s="67" t="n"/>
+      <c r="J29" s="67" t="n"/>
+      <c r="K29" s="49" t="n"/>
+    </row>
+    <row r="30">
+      <c r="A30" s="67" t="inlineStr">
+        <is>
+          <t>AWA</t>
+        </is>
+      </c>
+      <c r="B30" s="49" t="inlineStr">
+        <is>
+          <t>Ranked independent</t>
+        </is>
+      </c>
+      <c r="C30" s="67" t="n">
+        <v>0</v>
+      </c>
+      <c r="D30" s="67" t="n">
+        <v>1</v>
+      </c>
+      <c r="E30" s="67" t="n">
+        <v>0</v>
+      </c>
+      <c r="F30" s="67" t="n">
+        <v>2</v>
+      </c>
+      <c r="G30" s="49" t="inlineStr">
+        <is>
+          <t>IP</t>
+        </is>
+      </c>
+      <c r="H30" s="49" t="n"/>
+      <c r="I30" s="67" t="n"/>
+      <c r="J30" s="67" t="n"/>
+      <c r="K30" s="49" t="n"/>
+    </row>
+    <row r="31">
+      <c r="A31" s="67" t="inlineStr">
+        <is>
+          <t>Advokatfirman Malmstedt Law AB</t>
+        </is>
+      </c>
+      <c r="B31" s="49" t="inlineStr">
+        <is>
+          <t>Ranked independent</t>
+        </is>
+      </c>
+      <c r="C31" s="67" t="n">
+        <v>0</v>
+      </c>
+      <c r="D31" s="67" t="n">
+        <v>1</v>
+      </c>
+      <c r="E31" s="67" t="n">
+        <v>0</v>
+      </c>
+      <c r="F31" s="67" t="n">
+        <v>3</v>
+      </c>
+      <c r="G31" s="49" t="inlineStr">
+        <is>
+          <t>IP</t>
+        </is>
+      </c>
+      <c r="H31" s="49" t="n"/>
+      <c r="I31" s="67" t="n"/>
+      <c r="J31" s="67" t="n"/>
+      <c r="K31" s="49" t="n"/>
+    </row>
+    <row r="32">
+      <c r="A32" s="67" t="inlineStr">
+        <is>
+          <t>Advokatfirman MarLaw AB</t>
+        </is>
+      </c>
+      <c r="B32" s="49" t="inlineStr">
+        <is>
+          <t>Ranked independent</t>
+        </is>
+      </c>
+      <c r="C32" s="67" t="n">
+        <v>0</v>
+      </c>
+      <c r="D32" s="67" t="n">
+        <v>1</v>
+      </c>
+      <c r="E32" s="67" t="n">
+        <v>0</v>
+      </c>
+      <c r="F32" s="67" t="n">
+        <v>4</v>
+      </c>
+      <c r="G32" s="49" t="inlineStr">
+        <is>
+          <t>IP</t>
+        </is>
+      </c>
+      <c r="H32" s="49" t="n"/>
+      <c r="I32" s="67" t="n"/>
+      <c r="J32" s="67" t="n"/>
+      <c r="K32" s="49" t="n"/>
+    </row>
+    <row r="33">
+      <c r="A33" s="67" t="inlineStr">
+        <is>
+          <t>Advokatfirman Åberg &amp; Co AB</t>
+        </is>
+      </c>
+      <c r="B33" s="49" t="inlineStr">
+        <is>
+          <t>Ranked independent</t>
+        </is>
+      </c>
+      <c r="C33" s="67" t="n">
+        <v>1</v>
+      </c>
+      <c r="D33" s="67" t="n">
+        <v>0</v>
+      </c>
+      <c r="E33" s="67" t="n">
+        <v>0</v>
+      </c>
+      <c r="F33" s="67" t="n">
+        <v>3</v>
+      </c>
+      <c r="G33" s="49" t="inlineStr">
+        <is>
+          <t>Environment</t>
+        </is>
+      </c>
+      <c r="H33" s="49" t="n"/>
+      <c r="I33" s="67" t="n"/>
+      <c r="J33" s="67" t="n"/>
+      <c r="K33" s="49" t="n"/>
+    </row>
+    <row r="34">
+      <c r="A34" s="67" t="inlineStr">
+        <is>
+          <t>Affärsadvokaterna i Sverige AB</t>
+        </is>
+      </c>
+      <c r="B34" s="49" t="inlineStr">
+        <is>
+          <t>Ranked independent</t>
+        </is>
+      </c>
+      <c r="C34" s="67" t="n">
+        <v>0</v>
+      </c>
+      <c r="D34" s="67" t="n">
+        <v>1</v>
+      </c>
+      <c r="E34" s="67" t="n">
+        <v>1</v>
+      </c>
+      <c r="F34" s="67" t="n">
+        <v>4</v>
+      </c>
+      <c r="G34" s="49" t="inlineStr">
+        <is>
+          <t>IT / TMT</t>
+        </is>
+      </c>
+      <c r="H34" s="49" t="inlineStr">
+        <is>
+          <t>Data protection</t>
+        </is>
+      </c>
+      <c r="I34" s="67" t="n"/>
+      <c r="J34" s="67" t="n"/>
+      <c r="K34" s="49" t="n"/>
+    </row>
+    <row r="35">
+      <c r="A35" s="67" t="inlineStr">
+        <is>
+          <t>Alrutz' Advokatbyrå</t>
+        </is>
+      </c>
+      <c r="B35" s="49" t="inlineStr">
+        <is>
+          <t>Ranked independent</t>
+        </is>
+      </c>
+      <c r="C35" s="67" t="n">
+        <v>1</v>
+      </c>
+      <c r="D35" s="67" t="n">
+        <v>0</v>
+      </c>
+      <c r="E35" s="67" t="n">
+        <v>0</v>
+      </c>
+      <c r="F35" s="67" t="n">
+        <v>3</v>
+      </c>
+      <c r="G35" s="49" t="inlineStr">
+        <is>
+          <t>Environment</t>
+        </is>
+      </c>
+      <c r="H35" s="49" t="n"/>
+      <c r="I35" s="67" t="n"/>
+      <c r="J35" s="67" t="n"/>
+      <c r="K35" s="49" t="n"/>
+    </row>
+    <row r="36">
+      <c r="A36" s="67" t="inlineStr">
+        <is>
+          <t>Andulf</t>
+        </is>
+      </c>
+      <c r="B36" s="49" t="inlineStr">
+        <is>
+          <t>Ranked independent</t>
+        </is>
+      </c>
+      <c r="C36" s="67" t="n">
+        <v>1</v>
+      </c>
+      <c r="D36" s="67" t="n">
+        <v>0</v>
+      </c>
+      <c r="E36" s="67" t="n">
+        <v>0</v>
+      </c>
+      <c r="F36" s="67" t="n">
+        <v>1</v>
+      </c>
+      <c r="G36" s="49" t="inlineStr">
+        <is>
+          <t>PE fund formation</t>
+        </is>
+      </c>
+      <c r="H36" s="49" t="n"/>
+      <c r="I36" s="67" t="n"/>
+      <c r="J36" s="67" t="n"/>
+      <c r="K36" s="49" t="n"/>
+    </row>
+    <row r="37">
+      <c r="A37" s="67" t="inlineStr">
+        <is>
+          <t>Carler</t>
+        </is>
+      </c>
+      <c r="B37" s="49" t="inlineStr">
+        <is>
+          <t>Ranked independent</t>
+        </is>
+      </c>
+      <c r="C37" s="67" t="n">
+        <v>1</v>
+      </c>
+      <c r="D37" s="67" t="n">
+        <v>0</v>
+      </c>
+      <c r="E37" s="67" t="n">
+        <v>0</v>
+      </c>
+      <c r="F37" s="67" t="n">
+        <v>3</v>
+      </c>
+      <c r="G37" s="49" t="inlineStr">
+        <is>
+          <t>Insolvency trustees</t>
+        </is>
+      </c>
+      <c r="H37" s="49" t="n"/>
+      <c r="I37" s="67" t="n">
+        <v>7</v>
+      </c>
+      <c r="J37" s="67" t="n"/>
+      <c r="K37" s="49" t="inlineStr">
+        <is>
+          <t>Chambers</t>
+        </is>
+      </c>
+    </row>
+    <row r="38">
+      <c r="A38" s="67" t="inlineStr">
+        <is>
+          <t>DE Advokatbyrå AB</t>
+        </is>
+      </c>
+      <c r="B38" s="49" t="inlineStr">
+        <is>
+          <t>Ranked independent</t>
+        </is>
+      </c>
+      <c r="C38" s="67" t="n">
+        <v>0</v>
+      </c>
+      <c r="D38" s="67" t="n">
+        <v>1</v>
+      </c>
+      <c r="E38" s="67" t="n">
+        <v>0</v>
+      </c>
+      <c r="F38" s="67" t="n">
+        <v>3</v>
+      </c>
+      <c r="G38" s="49" t="inlineStr">
+        <is>
+          <t>Construction</t>
+        </is>
+      </c>
+      <c r="H38" s="49" t="n"/>
+      <c r="I38" s="67" t="n"/>
+      <c r="J38" s="67" t="n"/>
+      <c r="K38" s="49" t="n"/>
+    </row>
+    <row r="39">
+      <c r="A39" s="67" t="inlineStr">
+        <is>
+          <t>Edel</t>
+        </is>
+      </c>
+      <c r="B39" s="49" t="inlineStr">
+        <is>
+          <t>Ranked independent</t>
+        </is>
+      </c>
+      <c r="C39" s="67" t="n">
+        <v>1</v>
+      </c>
+      <c r="D39" s="67" t="n">
+        <v>0</v>
+      </c>
+      <c r="E39" s="67" t="n">
+        <v>0</v>
+      </c>
+      <c r="F39" s="67" t="n">
+        <v>4</v>
+      </c>
+      <c r="G39" s="49" t="inlineStr">
+        <is>
+          <t>Real estate</t>
+        </is>
+      </c>
+      <c r="H39" s="49" t="n"/>
+      <c r="I39" s="67" t="n"/>
+      <c r="J39" s="67" t="n"/>
+      <c r="K39" s="49" t="n"/>
+    </row>
+    <row r="40">
+      <c r="A40" s="67" t="inlineStr">
+        <is>
+          <t>Forssander Sonander Advokat</t>
+        </is>
+      </c>
+      <c r="B40" s="49" t="inlineStr">
+        <is>
+          <t>Ranked independent</t>
+        </is>
+      </c>
+      <c r="C40" s="67" t="n">
+        <v>0</v>
+      </c>
+      <c r="D40" s="67" t="n">
+        <v>1</v>
+      </c>
+      <c r="E40" s="67" t="n">
+        <v>0</v>
+      </c>
+      <c r="F40" s="67" t="n">
+        <v>3</v>
+      </c>
+      <c r="G40" s="49" t="inlineStr">
+        <is>
+          <t>Employment</t>
+        </is>
+      </c>
+      <c r="H40" s="49" t="n"/>
+      <c r="I40" s="67" t="n"/>
+      <c r="J40" s="67" t="n"/>
+      <c r="K40" s="49" t="n"/>
+    </row>
+    <row r="41">
+      <c r="A41" s="67" t="inlineStr">
+        <is>
+          <t>Merino</t>
+        </is>
+      </c>
+      <c r="B41" s="49" t="inlineStr">
+        <is>
+          <t>Ranked independent</t>
+        </is>
+      </c>
+      <c r="C41" s="67" t="n">
+        <v>0</v>
+      </c>
+      <c r="D41" s="67" t="n">
+        <v>1</v>
+      </c>
+      <c r="E41" s="67" t="n">
+        <v>0</v>
+      </c>
+      <c r="F41" s="67" t="n">
+        <v>4</v>
+      </c>
+      <c r="G41" s="49" t="inlineStr">
+        <is>
+          <t>Restructuring / insolvency</t>
+        </is>
+      </c>
+      <c r="H41" s="49" t="n"/>
+      <c r="I41" s="67" t="n"/>
+      <c r="J41" s="67" t="n"/>
+      <c r="K41" s="49" t="n"/>
+    </row>
+    <row r="42">
+      <c r="A42" s="67" t="inlineStr">
+        <is>
+          <t>Wimert Lundgren Advokatbyrå</t>
+        </is>
+      </c>
+      <c r="B42" s="49" t="inlineStr">
+        <is>
+          <t>Ranked independent</t>
+        </is>
+      </c>
+      <c r="C42" s="67" t="n">
+        <v>0</v>
+      </c>
+      <c r="D42" s="67" t="n">
+        <v>1</v>
+      </c>
+      <c r="E42" s="67" t="n">
+        <v>0</v>
+      </c>
+      <c r="F42" s="67" t="n">
+        <v>4</v>
+      </c>
+      <c r="G42" s="49" t="inlineStr">
+        <is>
+          <t>Construction</t>
+        </is>
+      </c>
+      <c r="H42" s="49" t="n"/>
+      <c r="I42" s="67" t="n"/>
+      <c r="J42" s="67" t="n"/>
+      <c r="K42" s="49" t="n"/>
+    </row>
+    <row r="43">
+      <c r="A43" s="67" t="inlineStr">
+        <is>
+          <t>Zacco</t>
+        </is>
+      </c>
+      <c r="B43" s="49" t="inlineStr">
+        <is>
+          <t>Ranked independent</t>
+        </is>
+      </c>
+      <c r="C43" s="67" t="n">
+        <v>0</v>
+      </c>
+      <c r="D43" s="67" t="n">
+        <v>1</v>
+      </c>
+      <c r="E43" s="67" t="n">
+        <v>0</v>
+      </c>
+      <c r="F43" s="67" t="n">
+        <v>3</v>
+      </c>
+      <c r="G43" s="49" t="inlineStr">
+        <is>
+          <t>IP</t>
+        </is>
+      </c>
+      <c r="H43" s="49" t="n"/>
+      <c r="I43" s="67" t="n"/>
+      <c r="J43" s="67" t="n"/>
+      <c r="K43" s="49" t="n"/>
+    </row>
+    <row r="44">
+      <c r="A44" s="68" t="inlineStr">
+        <is>
+          <t>TM &amp; Partners</t>
+        </is>
+      </c>
+      <c r="B44" s="69" t="inlineStr">
+        <is>
+          <t>Ranked independent: PE-owned (AGRD / Axcel)</t>
+        </is>
+      </c>
+      <c r="C44" s="68" t="n">
+        <v>5</v>
+      </c>
+      <c r="D44" s="68" t="n">
+        <v>11</v>
+      </c>
+      <c r="E44" s="68" t="n">
+        <v>0</v>
+      </c>
+      <c r="F44" s="68" t="n">
+        <v>2</v>
+      </c>
+      <c r="G44" s="69" t="inlineStr">
+        <is>
+          <t>Employment</t>
+        </is>
+      </c>
+      <c r="H44" s="69" t="n"/>
+      <c r="I44" s="68" t="n"/>
+      <c r="J44" s="68" t="n">
+        <v>60</v>
+      </c>
+      <c r="K44" s="69" t="inlineStr">
+        <is>
+          <t>L500</t>
+        </is>
+      </c>
+    </row>
+    <row r="45">
+      <c r="A45" s="68" t="inlineStr">
+        <is>
+          <t>Morris Law</t>
+        </is>
+      </c>
+      <c r="B45" s="69" t="inlineStr">
+        <is>
+          <t>Ranked independent: PE-owned (AGRD / Axcel)</t>
+        </is>
+      </c>
+      <c r="C45" s="68" t="n">
+        <v>2</v>
+      </c>
+      <c r="D45" s="68" t="n">
+        <v>9</v>
+      </c>
+      <c r="E45" s="68" t="n">
+        <v>0</v>
+      </c>
+      <c r="F45" s="68" t="n">
+        <v>2</v>
+      </c>
+      <c r="G45" s="69" t="inlineStr">
+        <is>
+          <t>Employment; Environment</t>
+        </is>
+      </c>
+      <c r="H45" s="69" t="n"/>
+      <c r="I45" s="68" t="n"/>
+      <c r="J45" s="68" t="n">
+        <v>56</v>
+      </c>
+      <c r="K45" s="69" t="inlineStr">
+        <is>
+          <t>L500</t>
+        </is>
+      </c>
+    </row>
+    <row r="46">
+      <c r="A46" s="68" t="inlineStr">
+        <is>
+          <t>Synch</t>
+        </is>
+      </c>
+      <c r="B46" s="69" t="inlineStr">
+        <is>
+          <t>Ranked independent: PE-owned (AGRD / Axcel)</t>
+        </is>
+      </c>
+      <c r="C46" s="68" t="n">
+        <v>2</v>
+      </c>
+      <c r="D46" s="68" t="n">
+        <v>7</v>
+      </c>
+      <c r="E46" s="68" t="n">
+        <v>0</v>
+      </c>
+      <c r="F46" s="68" t="n">
+        <v>2</v>
+      </c>
+      <c r="G46" s="69" t="inlineStr">
+        <is>
+          <t>IP</t>
+        </is>
+      </c>
+      <c r="H46" s="69" t="n"/>
+      <c r="I46" s="68" t="n"/>
+      <c r="J46" s="68" t="n"/>
+      <c r="K46" s="69" t="n"/>
+    </row>
+    <row r="47">
+      <c r="A47" s="68" t="inlineStr">
+        <is>
+          <t>Next Law</t>
+        </is>
+      </c>
+      <c r="B47" s="69" t="inlineStr">
+        <is>
+          <t>Ranked independent: PE-owned (AGRD / Axcel)</t>
+        </is>
+      </c>
+      <c r="C47" s="68" t="n">
+        <v>1</v>
+      </c>
+      <c r="D47" s="68" t="n">
+        <v>4</v>
+      </c>
+      <c r="E47" s="68" t="n">
+        <v>0</v>
+      </c>
+      <c r="F47" s="68" t="n">
+        <v>2</v>
+      </c>
+      <c r="G47" s="69" t="inlineStr">
+        <is>
+          <t>Shipping</t>
+        </is>
+      </c>
+      <c r="H47" s="69" t="n"/>
+      <c r="I47" s="68" t="n"/>
+      <c r="J47" s="68" t="n"/>
+      <c r="K47" s="69" t="n"/>
+    </row>
+    <row r="48">
+      <c r="A48" s="68" t="inlineStr">
+        <is>
+          <t>Born</t>
+        </is>
+      </c>
+      <c r="B48" s="69" t="inlineStr">
+        <is>
+          <t>Ranked independent: PE-owned (AGRD / Axcel)</t>
+        </is>
+      </c>
+      <c r="C48" s="68" t="n">
+        <v>1</v>
+      </c>
+      <c r="D48" s="68" t="n">
+        <v>1</v>
+      </c>
+      <c r="E48" s="68" t="n">
+        <v>0</v>
+      </c>
+      <c r="F48" s="68" t="n">
+        <v>3</v>
+      </c>
+      <c r="G48" s="69" t="inlineStr">
+        <is>
+          <t>Real estate</t>
+        </is>
+      </c>
+      <c r="H48" s="69" t="n"/>
+      <c r="I48" s="68" t="n"/>
+      <c r="J48" s="68" t="n"/>
+      <c r="K48" s="69" t="n"/>
+    </row>
+    <row r="49">
+      <c r="A49" s="68" t="inlineStr">
+        <is>
+          <t>Allié</t>
+        </is>
+      </c>
+      <c r="B49" s="69" t="inlineStr">
+        <is>
+          <t>Ranked independent: PE-owned (AGRD / Axcel)</t>
+        </is>
+      </c>
+      <c r="C49" s="68" t="n">
+        <v>0</v>
+      </c>
+      <c r="D49" s="68" t="n">
+        <v>1</v>
+      </c>
+      <c r="E49" s="68" t="n">
+        <v>0</v>
+      </c>
+      <c r="F49" s="68" t="n">
+        <v>4</v>
+      </c>
+      <c r="G49" s="69" t="inlineStr">
+        <is>
+          <t>Real estate</t>
+        </is>
+      </c>
+      <c r="H49" s="69" t="n"/>
+      <c r="I49" s="68" t="n"/>
+      <c r="J49" s="68" t="n"/>
+      <c r="K49" s="69" t="n"/>
+    </row>
+    <row r="50">
+      <c r="A50" s="70" t="inlineStr">
+        <is>
+          <t>Hammarskiöld</t>
+        </is>
+      </c>
+      <c r="B50" s="71" t="inlineStr">
+        <is>
+          <t>Borderline: Mid-size full-service</t>
+        </is>
+      </c>
+      <c r="C50" s="70" t="n">
+        <v>4</v>
+      </c>
+      <c r="D50" s="70" t="n">
+        <v>10</v>
+      </c>
+      <c r="E50" s="70" t="n">
+        <v>0</v>
+      </c>
+      <c r="F50" s="70" t="n">
+        <v>2</v>
+      </c>
+      <c r="G50" s="71" t="inlineStr">
+        <is>
+          <t>Banking &amp; finance; Healthcare / life sciences</t>
+        </is>
+      </c>
+      <c r="H50" s="71" t="n"/>
+      <c r="I50" s="70" t="n"/>
+      <c r="J50" s="70" t="n">
+        <v>47</v>
+      </c>
+      <c r="K50" s="71" t="inlineStr">
+        <is>
+          <t>Chambers</t>
+        </is>
+      </c>
+    </row>
+    <row r="51">
+      <c r="A51" s="70" t="inlineStr">
+        <is>
+          <t>Wigge &amp; Partners</t>
+        </is>
+      </c>
+      <c r="B51" s="71" t="inlineStr">
+        <is>
+          <t>Borderline: Mid-size corporate</t>
+        </is>
+      </c>
+      <c r="C51" s="70" t="n">
+        <v>5</v>
+      </c>
+      <c r="D51" s="70" t="n">
+        <v>3</v>
+      </c>
+      <c r="E51" s="70" t="n">
+        <v>0</v>
+      </c>
+      <c r="F51" s="70" t="n">
+        <v>1</v>
+      </c>
+      <c r="G51" s="71" t="inlineStr">
+        <is>
+          <t>Real estate</t>
+        </is>
+      </c>
+      <c r="H51" s="71" t="n"/>
+      <c r="I51" s="70" t="n">
+        <v>10</v>
+      </c>
+      <c r="J51" s="70" t="n">
+        <v>40</v>
+      </c>
+      <c r="K51" s="71" t="inlineStr">
+        <is>
+          <t>L500 (10 partners, 30 associates)</t>
+        </is>
+      </c>
+    </row>
+    <row r="52">
+      <c r="A52" s="70" t="inlineStr">
+        <is>
+          <t>Fylgia</t>
+        </is>
+      </c>
+      <c r="B52" s="71" t="inlineStr">
+        <is>
+          <t>Borderline: Mid-size full-service</t>
+        </is>
+      </c>
+      <c r="C52" s="70" t="n">
+        <v>1</v>
+      </c>
+      <c r="D52" s="70" t="n">
+        <v>6</v>
+      </c>
+      <c r="E52" s="70" t="n">
+        <v>0</v>
+      </c>
+      <c r="F52" s="70" t="n">
+        <v>2</v>
+      </c>
+      <c r="G52" s="71" t="inlineStr">
+        <is>
+          <t>Public procurement; Restructuring / insolvency</t>
+        </is>
+      </c>
+      <c r="H52" s="71" t="n"/>
+      <c r="I52" s="70" t="n">
+        <v>19</v>
+      </c>
+      <c r="J52" s="70" t="n">
+        <v>30</v>
+      </c>
+      <c r="K52" s="71" t="inlineStr">
+        <is>
+          <t>Chambers (lawyers excl. partners?)</t>
+        </is>
+      </c>
+    </row>
+    <row r="53">
+      <c r="A53" s="70" t="inlineStr">
+        <is>
+          <t>Foyen</t>
+        </is>
+      </c>
+      <c r="B53" s="71" t="inlineStr">
+        <is>
+          <t>Borderline: Mid-size full-service</t>
+        </is>
+      </c>
+      <c r="C53" s="70" t="n">
+        <v>0</v>
+      </c>
+      <c r="D53" s="70" t="n">
+        <v>6</v>
+      </c>
+      <c r="E53" s="70" t="n">
+        <v>0</v>
+      </c>
+      <c r="F53" s="70" t="n">
+        <v>2</v>
+      </c>
+      <c r="G53" s="71" t="inlineStr">
+        <is>
+          <t>Construction; Energy; Environment</t>
+        </is>
+      </c>
+      <c r="H53" s="71" t="n"/>
+      <c r="I53" s="70" t="n"/>
+      <c r="J53" s="70" t="n">
+        <v>75</v>
+      </c>
+      <c r="K53" s="71" t="inlineStr">
+        <is>
+          <t>L500</t>
+        </is>
+      </c>
+    </row>
+    <row r="54">
+      <c r="A54" s="70" t="inlineStr">
+        <is>
+          <t>Kanter</t>
+        </is>
+      </c>
+      <c r="B54" s="71" t="inlineStr">
+        <is>
+          <t>Borderline: Mid-size corporate</t>
+        </is>
+      </c>
+      <c r="C54" s="70" t="n">
+        <v>3</v>
+      </c>
+      <c r="D54" s="70" t="n">
+        <v>0</v>
+      </c>
+      <c r="E54" s="70" t="n">
+        <v>0</v>
+      </c>
+      <c r="F54" s="70" t="n">
+        <v>4</v>
+      </c>
+      <c r="G54" s="71" t="inlineStr">
+        <is>
+          <t>IP; Private equity</t>
+        </is>
+      </c>
+      <c r="H54" s="71" t="n"/>
+      <c r="I54" s="70" t="n">
+        <v>13</v>
+      </c>
+      <c r="J54" s="70" t="n">
+        <v>39</v>
+      </c>
+      <c r="K54" s="71" t="inlineStr">
+        <is>
+          <t>Chambers</t>
+        </is>
+      </c>
+    </row>
+    <row r="55">
+      <c r="A55" s="72" t="inlineStr">
+        <is>
+          <t>HC Advokat AB</t>
+        </is>
+      </c>
+      <c r="B55" s="73" t="inlineStr">
+        <is>
+          <t>Legal 500 firm to watch only</t>
+        </is>
+      </c>
+      <c r="C55" s="72" t="n">
+        <v>0</v>
+      </c>
+      <c r="D55" s="72" t="n">
+        <v>0</v>
+      </c>
+      <c r="E55" s="72" t="n">
+        <v>1</v>
+      </c>
+      <c r="F55" s="72" t="n"/>
+      <c r="G55" s="73" t="n"/>
+      <c r="H55" s="73" t="inlineStr">
+        <is>
+          <t>Construction</t>
+        </is>
+      </c>
+      <c r="I55" s="72" t="n"/>
+      <c r="J55" s="72" t="n"/>
+      <c r="K55" s="73" t="n"/>
+    </row>
+    <row r="56">
+      <c r="A56" s="72" t="inlineStr">
+        <is>
+          <t>Pogona Advokatbyrå AB</t>
+        </is>
+      </c>
+      <c r="B56" s="73" t="inlineStr">
+        <is>
+          <t>Legal 500 firm to watch only</t>
+        </is>
+      </c>
+      <c r="C56" s="72" t="n">
+        <v>0</v>
+      </c>
+      <c r="D56" s="72" t="n">
+        <v>0</v>
+      </c>
+      <c r="E56" s="72" t="n">
+        <v>1</v>
+      </c>
+      <c r="F56" s="72" t="n"/>
+      <c r="G56" s="73" t="n"/>
+      <c r="H56" s="73" t="inlineStr">
+        <is>
+          <t>Environment</t>
+        </is>
+      </c>
+      <c r="I56" s="72" t="n"/>
+      <c r="J56" s="72" t="n"/>
+      <c r="K56" s="73" t="n"/>
+    </row>
+    <row r="58">
+      <c r="A58" s="45" t="inlineStr">
+        <is>
+          <t>Best band/tier: 1 = top (Chambers band or Legal 500 tier, whichever is better). Yellow = PE-owned (AGRD, Axcel-backed roll-up formed Aug-2025); green = Legal 500 firm to watch only; grey = borderline mid-size firms.</t>
+        </is>
+      </c>
+    </row>
+    <row r="59">
+      <c r="A59" s="45" t="inlineStr">
+        <is>
+          <t>Excluded (international): BAHR, Baker McKenzie, Barker Brettell LLP, Bird &amp; Bird, CMS Wistrand, DLA Piper, Ernst &amp; Young AB, Eversheds Sutherland, Kilpatrick Townsend &amp; Stockton Advokat KB, Linklaters, Magnusson, Potter Clarkson LLP, Roschier, Schjødt, Snellman, White &amp; Case. Excluded (large Swedish full-service): Cederquist, Cirio, Delphi, Gernandt &amp; Danielsson, Lindahl, MAQS, Mannheimer Swartling, Setterwalls, Vinge.</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+  <mergeCells count="1">
+    <mergeCell ref="A2:K2"/>
+  </mergeCells>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
   <dimension ref="A1:BB66"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
@@ -10081,7 +12076,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
     <outlinePr summaryBelow="1" summaryRight="1"/>

</xml_diff>

<commit_message>
Add Section D rate card comparison and Word briefing on charging rates
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01Tu61bPEQej1E6sErbEFanY
</commit_message>
<xml_diff>
--- a/research/swedish_legal_market.xlsx
+++ b/research/swedish_legal_market.xlsx
@@ -13,6 +13,7 @@
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="A. Niche firms" sheetId="4" state="visible" r:id="rId4"/>
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="B. Practice rankings" sheetId="5" state="visible" r:id="rId5"/>
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="B. Rankings raw" sheetId="6" state="visible" r:id="rId6"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="D. Rate cards" sheetId="7" state="visible" r:id="rId7"/>
   </sheets>
   <definedNames>
     <definedName name="_xlnm._FilterDatabase" localSheetId="5" hidden="1">'B. Rankings raw'!$A$1:$E$661</definedName>
@@ -23,10 +24,11 @@
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <numFmts count="1">
+  <numFmts count="2">
     <numFmt numFmtId="164" formatCode="0.0"/>
+    <numFmt numFmtId="165" formatCode="+0%;-0%"/>
   </numFmts>
-  <fonts count="8">
+  <fonts count="9">
     <font>
       <name val="Calibri"/>
       <family val="2"/>
@@ -57,6 +59,10 @@
     <font>
       <b val="1"/>
       <sz val="11"/>
+    </font>
+    <font>
+      <b val="1"/>
+      <sz val="9"/>
     </font>
   </fonts>
   <fills count="10">
@@ -107,7 +113,7 @@
       </patternFill>
     </fill>
   </fills>
-  <borders count="13">
+  <borders count="19">
     <border>
       <left/>
       <right/>
@@ -283,11 +289,77 @@
         <color rgb="00C00000"/>
       </bottom>
     </border>
+    <border>
+      <left/>
+      <right/>
+      <top style="thin">
+        <color rgb="00BFBFBF"/>
+      </top>
+      <bottom/>
+      <diagonal/>
+    </border>
+    <border>
+      <left/>
+      <right style="thin">
+        <color rgb="00BFBFBF"/>
+      </right>
+      <top style="thin">
+        <color rgb="00BFBFBF"/>
+      </top>
+      <bottom/>
+      <diagonal/>
+    </border>
+    <border>
+      <left/>
+      <right style="thin">
+        <color rgb="00BFBFBF"/>
+      </right>
+      <top style="thin">
+        <color rgb="00BFBFBF"/>
+      </top>
+      <bottom style="thin">
+        <color rgb="00BFBFBF"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left style="thin">
+        <color rgb="00BFBFBF"/>
+      </left>
+      <right/>
+      <top/>
+      <bottom/>
+      <diagonal/>
+    </border>
+    <border>
+      <left style="thin">
+        <color rgb="00BFBFBF"/>
+      </left>
+      <right style="thin">
+        <color rgb="00BFBFBF"/>
+      </right>
+      <top/>
+      <bottom/>
+      <diagonal/>
+    </border>
+    <border>
+      <left style="thin">
+        <color rgb="00BFBFBF"/>
+      </left>
+      <right style="thin">
+        <color rgb="00BFBFBF"/>
+      </right>
+      <top/>
+      <bottom style="thin">
+        <color rgb="00BFBFBF"/>
+      </bottom>
+      <diagonal/>
+    </border>
   </borders>
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="84">
+  <cellXfs count="90">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
@@ -501,6 +573,20 @@
     </xf>
     <xf numFmtId="0" fontId="0" fillId="5" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="top"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="15" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="18" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="8" fillId="3" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="3" fontId="0" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="164" fontId="0" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="165" fontId="0" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
   </cellXfs>
   <cellStyles count="1">
@@ -3579,7 +3665,7 @@
       </c>
     </row>
     <row r="5">
-      <c r="A5" s="77" t="inlineStr">
+      <c r="A5" s="81" t="inlineStr">
         <is>
           <t>Hellström</t>
         </is>
@@ -3589,16 +3675,16 @@
           <t>Ranked independent</t>
         </is>
       </c>
-      <c r="C5" s="77" t="n">
+      <c r="C5" s="81" t="n">
         <v>1</v>
       </c>
-      <c r="D5" s="77" t="n">
+      <c r="D5" s="81" t="n">
         <v>7</v>
       </c>
-      <c r="E5" s="77" t="n">
+      <c r="E5" s="81" t="n">
         <v>0</v>
       </c>
-      <c r="F5" s="77" t="n">
+      <c r="F5" s="81" t="n">
         <v>2</v>
       </c>
       <c r="G5" s="49" t="inlineStr">
@@ -3607,10 +3693,10 @@
         </is>
       </c>
       <c r="H5" s="49" t="n"/>
-      <c r="I5" s="77" t="n">
+      <c r="I5" s="81" t="n">
         <v>22</v>
       </c>
-      <c r="J5" s="77" t="n">
+      <c r="J5" s="81" t="n">
         <v>49</v>
       </c>
       <c r="K5" s="49" t="inlineStr">
@@ -3620,7 +3706,7 @@
       </c>
     </row>
     <row r="6">
-      <c r="A6" s="77" t="inlineStr">
+      <c r="A6" s="81" t="inlineStr">
         <is>
           <t>TIME DANOWSKY Advokatbyrå AB</t>
         </is>
@@ -3630,16 +3716,16 @@
           <t>Ranked independent</t>
         </is>
       </c>
-      <c r="C6" s="77" t="n">
+      <c r="C6" s="81" t="n">
         <v>3</v>
       </c>
-      <c r="D6" s="77" t="n">
+      <c r="D6" s="81" t="n">
         <v>4</v>
       </c>
-      <c r="E6" s="77" t="n">
+      <c r="E6" s="81" t="n">
         <v>0</v>
       </c>
-      <c r="F6" s="77" t="n">
+      <c r="F6" s="81" t="n">
         <v>2</v>
       </c>
       <c r="G6" s="49" t="inlineStr">
@@ -3648,8 +3734,8 @@
         </is>
       </c>
       <c r="H6" s="49" t="n"/>
-      <c r="I6" s="77" t="n"/>
-      <c r="J6" s="77" t="n">
+      <c r="I6" s="81" t="n"/>
+      <c r="J6" s="81" t="n">
         <v>22</v>
       </c>
       <c r="K6" s="49" t="inlineStr">
@@ -3659,7 +3745,7 @@
       </c>
     </row>
     <row r="7">
-      <c r="A7" s="77" t="inlineStr">
+      <c r="A7" s="81" t="inlineStr">
         <is>
           <t>Kastell</t>
         </is>
@@ -3669,16 +3755,16 @@
           <t>Ranked independent</t>
         </is>
       </c>
-      <c r="C7" s="77" t="n">
+      <c r="C7" s="81" t="n">
         <v>3</v>
       </c>
-      <c r="D7" s="77" t="n">
+      <c r="D7" s="81" t="n">
         <v>3</v>
       </c>
-      <c r="E7" s="77" t="n">
+      <c r="E7" s="81" t="n">
         <v>0</v>
       </c>
-      <c r="F7" s="77" t="n">
+      <c r="F7" s="81" t="n">
         <v>2</v>
       </c>
       <c r="G7" s="49" t="inlineStr">
@@ -3687,10 +3773,10 @@
         </is>
       </c>
       <c r="H7" s="49" t="n"/>
-      <c r="I7" s="77" t="n">
+      <c r="I7" s="81" t="n">
         <v>9</v>
       </c>
-      <c r="J7" s="77" t="n">
+      <c r="J7" s="81" t="n">
         <v>18</v>
       </c>
       <c r="K7" s="49" t="inlineStr">
@@ -3700,7 +3786,7 @@
       </c>
     </row>
     <row r="8">
-      <c r="A8" s="77" t="inlineStr">
+      <c r="A8" s="81" t="inlineStr">
         <is>
           <t>Westerberg &amp; Partners</t>
         </is>
@@ -3710,16 +3796,16 @@
           <t>Ranked independent</t>
         </is>
       </c>
-      <c r="C8" s="77" t="n">
+      <c r="C8" s="81" t="n">
         <v>2</v>
       </c>
-      <c r="D8" s="77" t="n">
+      <c r="D8" s="81" t="n">
         <v>4</v>
       </c>
-      <c r="E8" s="77" t="n">
+      <c r="E8" s="81" t="n">
         <v>0</v>
       </c>
-      <c r="F8" s="77" t="n">
+      <c r="F8" s="81" t="n">
         <v>1</v>
       </c>
       <c r="G8" s="49" t="inlineStr">
@@ -3728,10 +3814,10 @@
         </is>
       </c>
       <c r="H8" s="49" t="n"/>
-      <c r="I8" s="77" t="n">
+      <c r="I8" s="81" t="n">
         <v>12</v>
       </c>
-      <c r="J8" s="77" t="n">
+      <c r="J8" s="81" t="n">
         <v>24</v>
       </c>
       <c r="K8" s="49" t="inlineStr">
@@ -3741,7 +3827,7 @@
       </c>
     </row>
     <row r="9">
-      <c r="A9" s="77" t="inlineStr">
+      <c r="A9" s="81" t="inlineStr">
         <is>
           <t>Kahn Pedersen</t>
         </is>
@@ -3751,16 +3837,16 @@
           <t>Ranked independent</t>
         </is>
       </c>
-      <c r="C9" s="77" t="n">
+      <c r="C9" s="81" t="n">
         <v>2</v>
       </c>
-      <c r="D9" s="77" t="n">
+      <c r="D9" s="81" t="n">
         <v>3</v>
       </c>
-      <c r="E9" s="77" t="n">
+      <c r="E9" s="81" t="n">
         <v>0</v>
       </c>
-      <c r="F9" s="77" t="n">
+      <c r="F9" s="81" t="n">
         <v>1</v>
       </c>
       <c r="G9" s="49" t="inlineStr">
@@ -3769,10 +3855,10 @@
         </is>
       </c>
       <c r="H9" s="49" t="n"/>
-      <c r="I9" s="77" t="n">
+      <c r="I9" s="81" t="n">
         <v>6</v>
       </c>
-      <c r="J9" s="77" t="n">
+      <c r="J9" s="81" t="n">
         <v>19</v>
       </c>
       <c r="K9" s="49" t="inlineStr">
@@ -3782,7 +3868,7 @@
       </c>
     </row>
     <row r="10">
-      <c r="A10" s="77" t="inlineStr">
+      <c r="A10" s="81" t="inlineStr">
         <is>
           <t>Nordia Law</t>
         </is>
@@ -3792,16 +3878,16 @@
           <t>Ranked independent</t>
         </is>
       </c>
-      <c r="C10" s="77" t="n">
+      <c r="C10" s="81" t="n">
         <v>1</v>
       </c>
-      <c r="D10" s="77" t="n">
+      <c r="D10" s="81" t="n">
         <v>4</v>
       </c>
-      <c r="E10" s="77" t="n">
+      <c r="E10" s="81" t="n">
         <v>0</v>
       </c>
-      <c r="F10" s="77" t="n">
+      <c r="F10" s="81" t="n">
         <v>2</v>
       </c>
       <c r="G10" s="49" t="inlineStr">
@@ -3810,12 +3896,12 @@
         </is>
       </c>
       <c r="H10" s="49" t="n"/>
-      <c r="I10" s="77" t="n"/>
-      <c r="J10" s="77" t="n"/>
+      <c r="I10" s="81" t="n"/>
+      <c r="J10" s="81" t="n"/>
       <c r="K10" s="49" t="n"/>
     </row>
     <row r="11">
-      <c r="A11" s="77" t="inlineStr">
+      <c r="A11" s="81" t="inlineStr">
         <is>
           <t>AG Advokat</t>
         </is>
@@ -3825,16 +3911,16 @@
           <t>Ranked independent</t>
         </is>
       </c>
-      <c r="C11" s="77" t="n">
+      <c r="C11" s="81" t="n">
         <v>1</v>
       </c>
-      <c r="D11" s="77" t="n">
+      <c r="D11" s="81" t="n">
         <v>3</v>
       </c>
-      <c r="E11" s="77" t="n">
+      <c r="E11" s="81" t="n">
         <v>0</v>
       </c>
-      <c r="F11" s="77" t="n">
+      <c r="F11" s="81" t="n">
         <v>1</v>
       </c>
       <c r="G11" s="49" t="inlineStr">
@@ -3843,8 +3929,8 @@
         </is>
       </c>
       <c r="H11" s="49" t="n"/>
-      <c r="I11" s="77" t="n"/>
-      <c r="J11" s="77" t="n">
+      <c r="I11" s="81" t="n"/>
+      <c r="J11" s="81" t="n">
         <v>41</v>
       </c>
       <c r="K11" s="49" t="inlineStr">
@@ -3854,7 +3940,7 @@
       </c>
     </row>
     <row r="12">
-      <c r="A12" s="77" t="inlineStr">
+      <c r="A12" s="81" t="inlineStr">
         <is>
           <t>Bokwall Rislund</t>
         </is>
@@ -3864,16 +3950,16 @@
           <t>Ranked independent</t>
         </is>
       </c>
-      <c r="C12" s="77" t="n">
+      <c r="C12" s="81" t="n">
         <v>2</v>
       </c>
-      <c r="D12" s="77" t="n">
+      <c r="D12" s="81" t="n">
         <v>2</v>
       </c>
-      <c r="E12" s="77" t="n">
+      <c r="E12" s="81" t="n">
         <v>0</v>
       </c>
-      <c r="F12" s="77" t="n">
+      <c r="F12" s="81" t="n">
         <v>1</v>
       </c>
       <c r="G12" s="49" t="inlineStr">
@@ -3882,12 +3968,12 @@
         </is>
       </c>
       <c r="H12" s="49" t="n"/>
-      <c r="I12" s="77" t="n"/>
-      <c r="J12" s="77" t="n"/>
+      <c r="I12" s="81" t="n"/>
+      <c r="J12" s="81" t="n"/>
       <c r="K12" s="49" t="n"/>
     </row>
     <row r="13">
-      <c r="A13" s="77" t="inlineStr">
+      <c r="A13" s="81" t="inlineStr">
         <is>
           <t>Sandart &amp; Partners</t>
         </is>
@@ -3897,16 +3983,16 @@
           <t>Ranked independent</t>
         </is>
       </c>
-      <c r="C13" s="77" t="n">
+      <c r="C13" s="81" t="n">
         <v>2</v>
       </c>
-      <c r="D13" s="77" t="n">
+      <c r="D13" s="81" t="n">
         <v>2</v>
       </c>
-      <c r="E13" s="77" t="n">
+      <c r="E13" s="81" t="n">
         <v>0</v>
       </c>
-      <c r="F13" s="77" t="n">
+      <c r="F13" s="81" t="n">
         <v>1</v>
       </c>
       <c r="G13" s="49" t="inlineStr">
@@ -3915,10 +4001,10 @@
         </is>
       </c>
       <c r="H13" s="49" t="n"/>
-      <c r="I13" s="77" t="n">
+      <c r="I13" s="81" t="n">
         <v>10</v>
       </c>
-      <c r="J13" s="77" t="n">
+      <c r="J13" s="81" t="n">
         <v>12</v>
       </c>
       <c r="K13" s="49" t="inlineStr">
@@ -3928,7 +4014,7 @@
       </c>
     </row>
     <row r="14">
-      <c r="A14" s="77" t="inlineStr">
+      <c r="A14" s="81" t="inlineStr">
         <is>
           <t>Brick</t>
         </is>
@@ -3938,16 +4024,16 @@
           <t>Ranked independent</t>
         </is>
       </c>
-      <c r="C14" s="77" t="n">
+      <c r="C14" s="81" t="n">
         <v>1</v>
       </c>
-      <c r="D14" s="77" t="n">
+      <c r="D14" s="81" t="n">
         <v>2</v>
       </c>
-      <c r="E14" s="77" t="n">
+      <c r="E14" s="81" t="n">
         <v>0</v>
       </c>
-      <c r="F14" s="77" t="n">
+      <c r="F14" s="81" t="n">
         <v>2</v>
       </c>
       <c r="G14" s="49" t="inlineStr">
@@ -3956,12 +4042,12 @@
         </is>
       </c>
       <c r="H14" s="49" t="n"/>
-      <c r="I14" s="77" t="n"/>
-      <c r="J14" s="77" t="n"/>
+      <c r="I14" s="81" t="n"/>
+      <c r="J14" s="81" t="n"/>
       <c r="K14" s="49" t="n"/>
     </row>
     <row r="15">
-      <c r="A15" s="77" t="inlineStr">
+      <c r="A15" s="81" t="inlineStr">
         <is>
           <t>Kompass</t>
         </is>
@@ -3971,16 +4057,16 @@
           <t>Ranked independent</t>
         </is>
       </c>
-      <c r="C15" s="77" t="n">
+      <c r="C15" s="81" t="n">
         <v>2</v>
       </c>
-      <c r="D15" s="77" t="n">
+      <c r="D15" s="81" t="n">
         <v>1</v>
       </c>
-      <c r="E15" s="77" t="n">
+      <c r="E15" s="81" t="n">
         <v>0</v>
       </c>
-      <c r="F15" s="77" t="n">
+      <c r="F15" s="81" t="n">
         <v>3</v>
       </c>
       <c r="G15" s="49" t="inlineStr">
@@ -3989,10 +4075,10 @@
         </is>
       </c>
       <c r="H15" s="49" t="n"/>
-      <c r="I15" s="77" t="n">
+      <c r="I15" s="81" t="n">
         <v>4</v>
       </c>
-      <c r="J15" s="77" t="n">
+      <c r="J15" s="81" t="n">
         <v>15</v>
       </c>
       <c r="K15" s="49" t="inlineStr">
@@ -4002,7 +4088,7 @@
       </c>
     </row>
     <row r="16">
-      <c r="A16" s="77" t="inlineStr">
+      <c r="A16" s="81" t="inlineStr">
         <is>
           <t>A1 Advokater</t>
         </is>
@@ -4012,16 +4098,16 @@
           <t>Ranked independent</t>
         </is>
       </c>
-      <c r="C16" s="77" t="n">
+      <c r="C16" s="81" t="n">
         <v>1</v>
       </c>
-      <c r="D16" s="77" t="n">
+      <c r="D16" s="81" t="n">
         <v>1</v>
       </c>
-      <c r="E16" s="77" t="n">
+      <c r="E16" s="81" t="n">
         <v>0</v>
       </c>
-      <c r="F16" s="77" t="n">
+      <c r="F16" s="81" t="n">
         <v>4</v>
       </c>
       <c r="G16" s="49" t="inlineStr">
@@ -4030,8 +4116,8 @@
         </is>
       </c>
       <c r="H16" s="49" t="n"/>
-      <c r="I16" s="77" t="n"/>
-      <c r="J16" s="77" t="n"/>
+      <c r="I16" s="81" t="n"/>
+      <c r="J16" s="81" t="n"/>
       <c r="K16" s="49" t="inlineStr">
         <is>
           <t>Chambers: 17 staff</t>
@@ -4039,7 +4125,7 @@
       </c>
     </row>
     <row r="17">
-      <c r="A17" s="77" t="inlineStr">
+      <c r="A17" s="81" t="inlineStr">
         <is>
           <t>Elmzell</t>
         </is>
@@ -4049,16 +4135,16 @@
           <t>Ranked independent</t>
         </is>
       </c>
-      <c r="C17" s="77" t="n">
+      <c r="C17" s="81" t="n">
         <v>1</v>
       </c>
-      <c r="D17" s="77" t="n">
+      <c r="D17" s="81" t="n">
         <v>1</v>
       </c>
-      <c r="E17" s="77" t="n">
+      <c r="E17" s="81" t="n">
         <v>0</v>
       </c>
-      <c r="F17" s="77" t="n">
+      <c r="F17" s="81" t="n">
         <v>2</v>
       </c>
       <c r="G17" s="49" t="inlineStr">
@@ -4067,12 +4153,12 @@
         </is>
       </c>
       <c r="H17" s="49" t="n"/>
-      <c r="I17" s="77" t="n"/>
-      <c r="J17" s="77" t="n"/>
+      <c r="I17" s="81" t="n"/>
+      <c r="J17" s="81" t="n"/>
       <c r="K17" s="49" t="n"/>
     </row>
     <row r="18">
-      <c r="A18" s="77" t="inlineStr">
+      <c r="A18" s="81" t="inlineStr">
         <is>
           <t>Fröberg &amp; Lundholm</t>
         </is>
@@ -4082,16 +4168,16 @@
           <t>Ranked independent</t>
         </is>
       </c>
-      <c r="C18" s="77" t="n">
+      <c r="C18" s="81" t="n">
         <v>1</v>
       </c>
-      <c r="D18" s="77" t="n">
+      <c r="D18" s="81" t="n">
         <v>1</v>
       </c>
-      <c r="E18" s="77" t="n">
+      <c r="E18" s="81" t="n">
         <v>0</v>
       </c>
-      <c r="F18" s="77" t="n">
+      <c r="F18" s="81" t="n">
         <v>1</v>
       </c>
       <c r="G18" s="49" t="inlineStr">
@@ -4100,12 +4186,12 @@
         </is>
       </c>
       <c r="H18" s="49" t="n"/>
-      <c r="I18" s="77" t="n"/>
-      <c r="J18" s="77" t="n"/>
+      <c r="I18" s="81" t="n"/>
+      <c r="J18" s="81" t="n"/>
       <c r="K18" s="49" t="n"/>
     </row>
     <row r="19">
-      <c r="A19" s="77" t="inlineStr">
+      <c r="A19" s="81" t="inlineStr">
         <is>
           <t>Gulliksson</t>
         </is>
@@ -4115,16 +4201,16 @@
           <t>Ranked independent</t>
         </is>
       </c>
-      <c r="C19" s="77" t="n">
+      <c r="C19" s="81" t="n">
         <v>1</v>
       </c>
-      <c r="D19" s="77" t="n">
+      <c r="D19" s="81" t="n">
         <v>1</v>
       </c>
-      <c r="E19" s="77" t="n">
+      <c r="E19" s="81" t="n">
         <v>0</v>
       </c>
-      <c r="F19" s="77" t="n">
+      <c r="F19" s="81" t="n">
         <v>2</v>
       </c>
       <c r="G19" s="49" t="inlineStr">
@@ -4133,8 +4219,8 @@
         </is>
       </c>
       <c r="H19" s="49" t="n"/>
-      <c r="I19" s="77" t="n"/>
-      <c r="J19" s="77" t="n">
+      <c r="I19" s="81" t="n"/>
+      <c r="J19" s="81" t="n">
         <v>41</v>
       </c>
       <c r="K19" s="49" t="inlineStr">
@@ -4144,7 +4230,7 @@
       </c>
     </row>
     <row r="20">
-      <c r="A20" s="77" t="inlineStr">
+      <c r="A20" s="81" t="inlineStr">
         <is>
           <t>Harvest</t>
         </is>
@@ -4154,16 +4240,16 @@
           <t>Ranked independent</t>
         </is>
       </c>
-      <c r="C20" s="77" t="n">
+      <c r="C20" s="81" t="n">
         <v>0</v>
       </c>
-      <c r="D20" s="77" t="n">
+      <c r="D20" s="81" t="n">
         <v>2</v>
       </c>
-      <c r="E20" s="77" t="n">
+      <c r="E20" s="81" t="n">
         <v>0</v>
       </c>
-      <c r="F20" s="77" t="n">
+      <c r="F20" s="81" t="n">
         <v>3</v>
       </c>
       <c r="G20" s="49" t="inlineStr">
@@ -4172,10 +4258,10 @@
         </is>
       </c>
       <c r="H20" s="49" t="n"/>
-      <c r="I20" s="77" t="n">
+      <c r="I20" s="81" t="n">
         <v>5</v>
       </c>
-      <c r="J20" s="77" t="n">
+      <c r="J20" s="81" t="n">
         <v>27</v>
       </c>
       <c r="K20" s="49" t="inlineStr">
@@ -4185,7 +4271,7 @@
       </c>
     </row>
     <row r="21">
-      <c r="A21" s="77" t="inlineStr">
+      <c r="A21" s="81" t="inlineStr">
         <is>
           <t>Norburg &amp; Scherp</t>
         </is>
@@ -4195,16 +4281,16 @@
           <t>Ranked independent</t>
         </is>
       </c>
-      <c r="C21" s="77" t="n">
+      <c r="C21" s="81" t="n">
         <v>1</v>
       </c>
-      <c r="D21" s="77" t="n">
+      <c r="D21" s="81" t="n">
         <v>1</v>
       </c>
-      <c r="E21" s="77" t="n">
+      <c r="E21" s="81" t="n">
         <v>0</v>
       </c>
-      <c r="F21" s="77" t="n">
+      <c r="F21" s="81" t="n">
         <v>3</v>
       </c>
       <c r="G21" s="49" t="inlineStr">
@@ -4213,8 +4299,8 @@
         </is>
       </c>
       <c r="H21" s="49" t="n"/>
-      <c r="I21" s="77" t="n"/>
-      <c r="J21" s="77" t="n">
+      <c r="I21" s="81" t="n"/>
+      <c r="J21" s="81" t="n">
         <v>18</v>
       </c>
       <c r="K21" s="49" t="inlineStr">
@@ -4224,7 +4310,7 @@
       </c>
     </row>
     <row r="22">
-      <c r="A22" s="77" t="inlineStr">
+      <c r="A22" s="81" t="inlineStr">
         <is>
           <t>Norma</t>
         </is>
@@ -4234,16 +4320,16 @@
           <t>Ranked independent</t>
         </is>
       </c>
-      <c r="C22" s="77" t="n">
+      <c r="C22" s="81" t="n">
         <v>0</v>
       </c>
-      <c r="D22" s="77" t="n">
+      <c r="D22" s="81" t="n">
         <v>2</v>
       </c>
-      <c r="E22" s="77" t="n">
+      <c r="E22" s="81" t="n">
         <v>0</v>
       </c>
-      <c r="F22" s="77" t="n">
+      <c r="F22" s="81" t="n">
         <v>4</v>
       </c>
       <c r="G22" s="49" t="inlineStr">
@@ -4252,12 +4338,12 @@
         </is>
       </c>
       <c r="H22" s="49" t="n"/>
-      <c r="I22" s="77" t="n"/>
-      <c r="J22" s="77" t="n"/>
+      <c r="I22" s="81" t="n"/>
+      <c r="J22" s="81" t="n"/>
       <c r="K22" s="49" t="n"/>
     </row>
     <row r="23">
-      <c r="A23" s="77" t="inlineStr">
+      <c r="A23" s="81" t="inlineStr">
         <is>
           <t>RE:FI STHLM</t>
         </is>
@@ -4267,16 +4353,16 @@
           <t>Ranked independent</t>
         </is>
       </c>
-      <c r="C23" s="77" t="n">
+      <c r="C23" s="81" t="n">
         <v>1</v>
       </c>
-      <c r="D23" s="77" t="n">
+      <c r="D23" s="81" t="n">
         <v>1</v>
       </c>
-      <c r="E23" s="77" t="n">
+      <c r="E23" s="81" t="n">
         <v>0</v>
       </c>
-      <c r="F23" s="77" t="n">
+      <c r="F23" s="81" t="n">
         <v>3</v>
       </c>
       <c r="G23" s="49" t="inlineStr">
@@ -4285,12 +4371,12 @@
         </is>
       </c>
       <c r="H23" s="49" t="n"/>
-      <c r="I23" s="77" t="n"/>
-      <c r="J23" s="77" t="n"/>
+      <c r="I23" s="81" t="n"/>
+      <c r="J23" s="81" t="n"/>
       <c r="K23" s="49" t="n"/>
     </row>
     <row r="24">
-      <c r="A24" s="77" t="inlineStr">
+      <c r="A24" s="81" t="inlineStr">
         <is>
           <t>REAL Advokatbyrå</t>
         </is>
@@ -4300,16 +4386,16 @@
           <t>Ranked independent</t>
         </is>
       </c>
-      <c r="C24" s="77" t="n">
+      <c r="C24" s="81" t="n">
         <v>1</v>
       </c>
-      <c r="D24" s="77" t="n">
+      <c r="D24" s="81" t="n">
         <v>1</v>
       </c>
-      <c r="E24" s="77" t="n">
+      <c r="E24" s="81" t="n">
         <v>0</v>
       </c>
-      <c r="F24" s="77" t="n">
+      <c r="F24" s="81" t="n">
         <v>2</v>
       </c>
       <c r="G24" s="49" t="inlineStr">
@@ -4318,10 +4404,10 @@
         </is>
       </c>
       <c r="H24" s="49" t="n"/>
-      <c r="I24" s="77" t="n">
+      <c r="I24" s="81" t="n">
         <v>5</v>
       </c>
-      <c r="J24" s="77" t="n">
+      <c r="J24" s="81" t="n">
         <v>20</v>
       </c>
       <c r="K24" s="49" t="inlineStr">
@@ -4331,7 +4417,7 @@
       </c>
     </row>
     <row r="25">
-      <c r="A25" s="77" t="inlineStr">
+      <c r="A25" s="81" t="inlineStr">
         <is>
           <t>Skierfe</t>
         </is>
@@ -4341,16 +4427,16 @@
           <t>Ranked independent</t>
         </is>
       </c>
-      <c r="C25" s="77" t="n">
+      <c r="C25" s="81" t="n">
         <v>1</v>
       </c>
-      <c r="D25" s="77" t="n">
+      <c r="D25" s="81" t="n">
         <v>1</v>
       </c>
-      <c r="E25" s="77" t="n">
+      <c r="E25" s="81" t="n">
         <v>0</v>
       </c>
-      <c r="F25" s="77" t="n">
+      <c r="F25" s="81" t="n">
         <v>3</v>
       </c>
       <c r="G25" s="49" t="inlineStr">
@@ -4359,12 +4445,12 @@
         </is>
       </c>
       <c r="H25" s="49" t="n"/>
-      <c r="I25" s="77" t="n"/>
-      <c r="J25" s="77" t="n"/>
+      <c r="I25" s="81" t="n"/>
+      <c r="J25" s="81" t="n"/>
       <c r="K25" s="49" t="n"/>
     </row>
     <row r="26">
-      <c r="A26" s="77" t="inlineStr">
+      <c r="A26" s="81" t="inlineStr">
         <is>
           <t>Ström</t>
         </is>
@@ -4374,16 +4460,16 @@
           <t>Ranked independent</t>
         </is>
       </c>
-      <c r="C26" s="77" t="n">
+      <c r="C26" s="81" t="n">
         <v>1</v>
       </c>
-      <c r="D26" s="77" t="n">
+      <c r="D26" s="81" t="n">
         <v>1</v>
       </c>
-      <c r="E26" s="77" t="n">
+      <c r="E26" s="81" t="n">
         <v>0</v>
       </c>
-      <c r="F26" s="77" t="n">
+      <c r="F26" s="81" t="n">
         <v>2</v>
       </c>
       <c r="G26" s="49" t="inlineStr">
@@ -4392,10 +4478,10 @@
         </is>
       </c>
       <c r="H26" s="49" t="n"/>
-      <c r="I26" s="77" t="n">
+      <c r="I26" s="81" t="n">
         <v>5</v>
       </c>
-      <c r="J26" s="77" t="n"/>
+      <c r="J26" s="81" t="n"/>
       <c r="K26" s="49" t="inlineStr">
         <is>
           <t>Chambers</t>
@@ -4403,7 +4489,7 @@
       </c>
     </row>
     <row r="27">
-      <c r="A27" s="77" t="inlineStr">
+      <c r="A27" s="81" t="inlineStr">
         <is>
           <t>Ulfsdotter</t>
         </is>
@@ -4413,16 +4499,16 @@
           <t>Ranked independent</t>
         </is>
       </c>
-      <c r="C27" s="77" t="n">
+      <c r="C27" s="81" t="n">
         <v>1</v>
       </c>
-      <c r="D27" s="77" t="n">
+      <c r="D27" s="81" t="n">
         <v>1</v>
       </c>
-      <c r="E27" s="77" t="n">
+      <c r="E27" s="81" t="n">
         <v>0</v>
       </c>
-      <c r="F27" s="77" t="n">
+      <c r="F27" s="81" t="n">
         <v>2</v>
       </c>
       <c r="G27" s="49" t="inlineStr">
@@ -4431,12 +4517,12 @@
         </is>
       </c>
       <c r="H27" s="49" t="n"/>
-      <c r="I27" s="77" t="n"/>
-      <c r="J27" s="77" t="n"/>
+      <c r="I27" s="81" t="n"/>
+      <c r="J27" s="81" t="n"/>
       <c r="K27" s="49" t="n"/>
     </row>
     <row r="28">
-      <c r="A28" s="77" t="inlineStr">
+      <c r="A28" s="81" t="inlineStr">
         <is>
           <t>Wallin &amp; Partners</t>
         </is>
@@ -4446,16 +4532,16 @@
           <t>Ranked independent</t>
         </is>
       </c>
-      <c r="C28" s="77" t="n">
+      <c r="C28" s="81" t="n">
         <v>1</v>
       </c>
-      <c r="D28" s="77" t="n">
+      <c r="D28" s="81" t="n">
         <v>1</v>
       </c>
-      <c r="E28" s="77" t="n">
+      <c r="E28" s="81" t="n">
         <v>0</v>
       </c>
-      <c r="F28" s="77" t="n">
+      <c r="F28" s="81" t="n">
         <v>3</v>
       </c>
       <c r="G28" s="49" t="inlineStr">
@@ -4464,12 +4550,12 @@
         </is>
       </c>
       <c r="H28" s="49" t="n"/>
-      <c r="I28" s="77" t="n"/>
-      <c r="J28" s="77" t="n"/>
+      <c r="I28" s="81" t="n"/>
+      <c r="J28" s="81" t="n"/>
       <c r="K28" s="49" t="n"/>
     </row>
     <row r="29">
-      <c r="A29" s="77" t="inlineStr">
+      <c r="A29" s="81" t="inlineStr">
         <is>
           <t>edpLaw</t>
         </is>
@@ -4479,16 +4565,16 @@
           <t>Ranked independent</t>
         </is>
       </c>
-      <c r="C29" s="77" t="n">
+      <c r="C29" s="81" t="n">
         <v>0</v>
       </c>
-      <c r="D29" s="77" t="n">
+      <c r="D29" s="81" t="n">
         <v>2</v>
       </c>
-      <c r="E29" s="77" t="n">
+      <c r="E29" s="81" t="n">
         <v>0</v>
       </c>
-      <c r="F29" s="77" t="n">
+      <c r="F29" s="81" t="n">
         <v>2</v>
       </c>
       <c r="G29" s="49" t="inlineStr">
@@ -4497,12 +4583,12 @@
         </is>
       </c>
       <c r="H29" s="49" t="n"/>
-      <c r="I29" s="77" t="n"/>
-      <c r="J29" s="77" t="n"/>
+      <c r="I29" s="81" t="n"/>
+      <c r="J29" s="81" t="n"/>
       <c r="K29" s="49" t="n"/>
     </row>
     <row r="30">
-      <c r="A30" s="77" t="inlineStr">
+      <c r="A30" s="81" t="inlineStr">
         <is>
           <t>AWA</t>
         </is>
@@ -4512,16 +4598,16 @@
           <t>Ranked independent</t>
         </is>
       </c>
-      <c r="C30" s="77" t="n">
+      <c r="C30" s="81" t="n">
         <v>0</v>
       </c>
-      <c r="D30" s="77" t="n">
+      <c r="D30" s="81" t="n">
         <v>1</v>
       </c>
-      <c r="E30" s="77" t="n">
+      <c r="E30" s="81" t="n">
         <v>0</v>
       </c>
-      <c r="F30" s="77" t="n">
+      <c r="F30" s="81" t="n">
         <v>2</v>
       </c>
       <c r="G30" s="49" t="inlineStr">
@@ -4530,12 +4616,12 @@
         </is>
       </c>
       <c r="H30" s="49" t="n"/>
-      <c r="I30" s="77" t="n"/>
-      <c r="J30" s="77" t="n"/>
+      <c r="I30" s="81" t="n"/>
+      <c r="J30" s="81" t="n"/>
       <c r="K30" s="49" t="n"/>
     </row>
     <row r="31">
-      <c r="A31" s="77" t="inlineStr">
+      <c r="A31" s="81" t="inlineStr">
         <is>
           <t>Advokatfirman Malmstedt Law AB</t>
         </is>
@@ -4545,16 +4631,16 @@
           <t>Ranked independent</t>
         </is>
       </c>
-      <c r="C31" s="77" t="n">
+      <c r="C31" s="81" t="n">
         <v>0</v>
       </c>
-      <c r="D31" s="77" t="n">
+      <c r="D31" s="81" t="n">
         <v>1</v>
       </c>
-      <c r="E31" s="77" t="n">
+      <c r="E31" s="81" t="n">
         <v>0</v>
       </c>
-      <c r="F31" s="77" t="n">
+      <c r="F31" s="81" t="n">
         <v>3</v>
       </c>
       <c r="G31" s="49" t="inlineStr">
@@ -4563,12 +4649,12 @@
         </is>
       </c>
       <c r="H31" s="49" t="n"/>
-      <c r="I31" s="77" t="n"/>
-      <c r="J31" s="77" t="n"/>
+      <c r="I31" s="81" t="n"/>
+      <c r="J31" s="81" t="n"/>
       <c r="K31" s="49" t="n"/>
     </row>
     <row r="32">
-      <c r="A32" s="77" t="inlineStr">
+      <c r="A32" s="81" t="inlineStr">
         <is>
           <t>Advokatfirman MarLaw AB</t>
         </is>
@@ -4578,16 +4664,16 @@
           <t>Ranked independent</t>
         </is>
       </c>
-      <c r="C32" s="77" t="n">
+      <c r="C32" s="81" t="n">
         <v>0</v>
       </c>
-      <c r="D32" s="77" t="n">
+      <c r="D32" s="81" t="n">
         <v>1</v>
       </c>
-      <c r="E32" s="77" t="n">
+      <c r="E32" s="81" t="n">
         <v>0</v>
       </c>
-      <c r="F32" s="77" t="n">
+      <c r="F32" s="81" t="n">
         <v>4</v>
       </c>
       <c r="G32" s="49" t="inlineStr">
@@ -4596,12 +4682,12 @@
         </is>
       </c>
       <c r="H32" s="49" t="n"/>
-      <c r="I32" s="77" t="n"/>
-      <c r="J32" s="77" t="n"/>
+      <c r="I32" s="81" t="n"/>
+      <c r="J32" s="81" t="n"/>
       <c r="K32" s="49" t="n"/>
     </row>
     <row r="33">
-      <c r="A33" s="77" t="inlineStr">
+      <c r="A33" s="81" t="inlineStr">
         <is>
           <t>Advokatfirman Åberg &amp; Co AB</t>
         </is>
@@ -4611,16 +4697,16 @@
           <t>Ranked independent</t>
         </is>
       </c>
-      <c r="C33" s="77" t="n">
+      <c r="C33" s="81" t="n">
         <v>1</v>
       </c>
-      <c r="D33" s="77" t="n">
+      <c r="D33" s="81" t="n">
         <v>0</v>
       </c>
-      <c r="E33" s="77" t="n">
+      <c r="E33" s="81" t="n">
         <v>0</v>
       </c>
-      <c r="F33" s="77" t="n">
+      <c r="F33" s="81" t="n">
         <v>3</v>
       </c>
       <c r="G33" s="49" t="inlineStr">
@@ -4629,12 +4715,12 @@
         </is>
       </c>
       <c r="H33" s="49" t="n"/>
-      <c r="I33" s="77" t="n"/>
-      <c r="J33" s="77" t="n"/>
+      <c r="I33" s="81" t="n"/>
+      <c r="J33" s="81" t="n"/>
       <c r="K33" s="49" t="n"/>
     </row>
     <row r="34">
-      <c r="A34" s="77" t="inlineStr">
+      <c r="A34" s="81" t="inlineStr">
         <is>
           <t>Affärsadvokaterna i Sverige AB</t>
         </is>
@@ -4644,16 +4730,16 @@
           <t>Ranked independent</t>
         </is>
       </c>
-      <c r="C34" s="77" t="n">
+      <c r="C34" s="81" t="n">
         <v>0</v>
       </c>
-      <c r="D34" s="77" t="n">
+      <c r="D34" s="81" t="n">
         <v>1</v>
       </c>
-      <c r="E34" s="77" t="n">
+      <c r="E34" s="81" t="n">
         <v>1</v>
       </c>
-      <c r="F34" s="77" t="n">
+      <c r="F34" s="81" t="n">
         <v>4</v>
       </c>
       <c r="G34" s="49" t="inlineStr">
@@ -4666,12 +4752,12 @@
           <t>Data protection</t>
         </is>
       </c>
-      <c r="I34" s="77" t="n"/>
-      <c r="J34" s="77" t="n"/>
+      <c r="I34" s="81" t="n"/>
+      <c r="J34" s="81" t="n"/>
       <c r="K34" s="49" t="n"/>
     </row>
     <row r="35">
-      <c r="A35" s="77" t="inlineStr">
+      <c r="A35" s="81" t="inlineStr">
         <is>
           <t>Alrutz' Advokatbyrå</t>
         </is>
@@ -4681,16 +4767,16 @@
           <t>Ranked independent</t>
         </is>
       </c>
-      <c r="C35" s="77" t="n">
+      <c r="C35" s="81" t="n">
         <v>1</v>
       </c>
-      <c r="D35" s="77" t="n">
+      <c r="D35" s="81" t="n">
         <v>0</v>
       </c>
-      <c r="E35" s="77" t="n">
+      <c r="E35" s="81" t="n">
         <v>0</v>
       </c>
-      <c r="F35" s="77" t="n">
+      <c r="F35" s="81" t="n">
         <v>3</v>
       </c>
       <c r="G35" s="49" t="inlineStr">
@@ -4699,12 +4785,12 @@
         </is>
       </c>
       <c r="H35" s="49" t="n"/>
-      <c r="I35" s="77" t="n"/>
-      <c r="J35" s="77" t="n"/>
+      <c r="I35" s="81" t="n"/>
+      <c r="J35" s="81" t="n"/>
       <c r="K35" s="49" t="n"/>
     </row>
     <row r="36">
-      <c r="A36" s="77" t="inlineStr">
+      <c r="A36" s="81" t="inlineStr">
         <is>
           <t>Andulf</t>
         </is>
@@ -4714,16 +4800,16 @@
           <t>Ranked independent</t>
         </is>
       </c>
-      <c r="C36" s="77" t="n">
+      <c r="C36" s="81" t="n">
         <v>1</v>
       </c>
-      <c r="D36" s="77" t="n">
+      <c r="D36" s="81" t="n">
         <v>0</v>
       </c>
-      <c r="E36" s="77" t="n">
+      <c r="E36" s="81" t="n">
         <v>0</v>
       </c>
-      <c r="F36" s="77" t="n">
+      <c r="F36" s="81" t="n">
         <v>1</v>
       </c>
       <c r="G36" s="49" t="inlineStr">
@@ -4732,12 +4818,12 @@
         </is>
       </c>
       <c r="H36" s="49" t="n"/>
-      <c r="I36" s="77" t="n"/>
-      <c r="J36" s="77" t="n"/>
+      <c r="I36" s="81" t="n"/>
+      <c r="J36" s="81" t="n"/>
       <c r="K36" s="49" t="n"/>
     </row>
     <row r="37">
-      <c r="A37" s="77" t="inlineStr">
+      <c r="A37" s="81" t="inlineStr">
         <is>
           <t>Carler</t>
         </is>
@@ -4747,16 +4833,16 @@
           <t>Ranked independent</t>
         </is>
       </c>
-      <c r="C37" s="77" t="n">
+      <c r="C37" s="81" t="n">
         <v>1</v>
       </c>
-      <c r="D37" s="77" t="n">
+      <c r="D37" s="81" t="n">
         <v>0</v>
       </c>
-      <c r="E37" s="77" t="n">
+      <c r="E37" s="81" t="n">
         <v>0</v>
       </c>
-      <c r="F37" s="77" t="n">
+      <c r="F37" s="81" t="n">
         <v>3</v>
       </c>
       <c r="G37" s="49" t="inlineStr">
@@ -4765,10 +4851,10 @@
         </is>
       </c>
       <c r="H37" s="49" t="n"/>
-      <c r="I37" s="77" t="n">
+      <c r="I37" s="81" t="n">
         <v>7</v>
       </c>
-      <c r="J37" s="77" t="n"/>
+      <c r="J37" s="81" t="n"/>
       <c r="K37" s="49" t="inlineStr">
         <is>
           <t>Chambers</t>
@@ -4776,7 +4862,7 @@
       </c>
     </row>
     <row r="38">
-      <c r="A38" s="77" t="inlineStr">
+      <c r="A38" s="81" t="inlineStr">
         <is>
           <t>DE Advokatbyrå AB</t>
         </is>
@@ -4786,16 +4872,16 @@
           <t>Ranked independent</t>
         </is>
       </c>
-      <c r="C38" s="77" t="n">
+      <c r="C38" s="81" t="n">
         <v>0</v>
       </c>
-      <c r="D38" s="77" t="n">
+      <c r="D38" s="81" t="n">
         <v>1</v>
       </c>
-      <c r="E38" s="77" t="n">
+      <c r="E38" s="81" t="n">
         <v>0</v>
       </c>
-      <c r="F38" s="77" t="n">
+      <c r="F38" s="81" t="n">
         <v>3</v>
       </c>
       <c r="G38" s="49" t="inlineStr">
@@ -4804,12 +4890,12 @@
         </is>
       </c>
       <c r="H38" s="49" t="n"/>
-      <c r="I38" s="77" t="n"/>
-      <c r="J38" s="77" t="n"/>
+      <c r="I38" s="81" t="n"/>
+      <c r="J38" s="81" t="n"/>
       <c r="K38" s="49" t="n"/>
     </row>
     <row r="39">
-      <c r="A39" s="77" t="inlineStr">
+      <c r="A39" s="81" t="inlineStr">
         <is>
           <t>Edel</t>
         </is>
@@ -4819,16 +4905,16 @@
           <t>Ranked independent</t>
         </is>
       </c>
-      <c r="C39" s="77" t="n">
+      <c r="C39" s="81" t="n">
         <v>1</v>
       </c>
-      <c r="D39" s="77" t="n">
+      <c r="D39" s="81" t="n">
         <v>0</v>
       </c>
-      <c r="E39" s="77" t="n">
+      <c r="E39" s="81" t="n">
         <v>0</v>
       </c>
-      <c r="F39" s="77" t="n">
+      <c r="F39" s="81" t="n">
         <v>4</v>
       </c>
       <c r="G39" s="49" t="inlineStr">
@@ -4837,12 +4923,12 @@
         </is>
       </c>
       <c r="H39" s="49" t="n"/>
-      <c r="I39" s="77" t="n"/>
-      <c r="J39" s="77" t="n"/>
+      <c r="I39" s="81" t="n"/>
+      <c r="J39" s="81" t="n"/>
       <c r="K39" s="49" t="n"/>
     </row>
     <row r="40">
-      <c r="A40" s="77" t="inlineStr">
+      <c r="A40" s="81" t="inlineStr">
         <is>
           <t>Forssander Sonander Advokat</t>
         </is>
@@ -4852,16 +4938,16 @@
           <t>Ranked independent</t>
         </is>
       </c>
-      <c r="C40" s="77" t="n">
+      <c r="C40" s="81" t="n">
         <v>0</v>
       </c>
-      <c r="D40" s="77" t="n">
+      <c r="D40" s="81" t="n">
         <v>1</v>
       </c>
-      <c r="E40" s="77" t="n">
+      <c r="E40" s="81" t="n">
         <v>0</v>
       </c>
-      <c r="F40" s="77" t="n">
+      <c r="F40" s="81" t="n">
         <v>3</v>
       </c>
       <c r="G40" s="49" t="inlineStr">
@@ -4870,12 +4956,12 @@
         </is>
       </c>
       <c r="H40" s="49" t="n"/>
-      <c r="I40" s="77" t="n"/>
-      <c r="J40" s="77" t="n"/>
+      <c r="I40" s="81" t="n"/>
+      <c r="J40" s="81" t="n"/>
       <c r="K40" s="49" t="n"/>
     </row>
     <row r="41">
-      <c r="A41" s="77" t="inlineStr">
+      <c r="A41" s="81" t="inlineStr">
         <is>
           <t>Merino</t>
         </is>
@@ -4885,16 +4971,16 @@
           <t>Ranked independent</t>
         </is>
       </c>
-      <c r="C41" s="77" t="n">
+      <c r="C41" s="81" t="n">
         <v>0</v>
       </c>
-      <c r="D41" s="77" t="n">
+      <c r="D41" s="81" t="n">
         <v>1</v>
       </c>
-      <c r="E41" s="77" t="n">
+      <c r="E41" s="81" t="n">
         <v>0</v>
       </c>
-      <c r="F41" s="77" t="n">
+      <c r="F41" s="81" t="n">
         <v>4</v>
       </c>
       <c r="G41" s="49" t="inlineStr">
@@ -4903,12 +4989,12 @@
         </is>
       </c>
       <c r="H41" s="49" t="n"/>
-      <c r="I41" s="77" t="n"/>
-      <c r="J41" s="77" t="n"/>
+      <c r="I41" s="81" t="n"/>
+      <c r="J41" s="81" t="n"/>
       <c r="K41" s="49" t="n"/>
     </row>
     <row r="42">
-      <c r="A42" s="77" t="inlineStr">
+      <c r="A42" s="81" t="inlineStr">
         <is>
           <t>Wimert Lundgren Advokatbyrå</t>
         </is>
@@ -4918,16 +5004,16 @@
           <t>Ranked independent</t>
         </is>
       </c>
-      <c r="C42" s="77" t="n">
+      <c r="C42" s="81" t="n">
         <v>0</v>
       </c>
-      <c r="D42" s="77" t="n">
+      <c r="D42" s="81" t="n">
         <v>1</v>
       </c>
-      <c r="E42" s="77" t="n">
+      <c r="E42" s="81" t="n">
         <v>0</v>
       </c>
-      <c r="F42" s="77" t="n">
+      <c r="F42" s="81" t="n">
         <v>4</v>
       </c>
       <c r="G42" s="49" t="inlineStr">
@@ -4936,12 +5022,12 @@
         </is>
       </c>
       <c r="H42" s="49" t="n"/>
-      <c r="I42" s="77" t="n"/>
-      <c r="J42" s="77" t="n"/>
+      <c r="I42" s="81" t="n"/>
+      <c r="J42" s="81" t="n"/>
       <c r="K42" s="49" t="n"/>
     </row>
     <row r="43">
-      <c r="A43" s="77" t="inlineStr">
+      <c r="A43" s="81" t="inlineStr">
         <is>
           <t>Zacco</t>
         </is>
@@ -4951,16 +5037,16 @@
           <t>Ranked independent</t>
         </is>
       </c>
-      <c r="C43" s="77" t="n">
+      <c r="C43" s="81" t="n">
         <v>0</v>
       </c>
-      <c r="D43" s="77" t="n">
+      <c r="D43" s="81" t="n">
         <v>1</v>
       </c>
-      <c r="E43" s="77" t="n">
+      <c r="E43" s="81" t="n">
         <v>0</v>
       </c>
-      <c r="F43" s="77" t="n">
+      <c r="F43" s="81" t="n">
         <v>3</v>
       </c>
       <c r="G43" s="49" t="inlineStr">
@@ -4969,8 +5055,8 @@
         </is>
       </c>
       <c r="H43" s="49" t="n"/>
-      <c r="I43" s="77" t="n"/>
-      <c r="J43" s="77" t="n"/>
+      <c r="I43" s="81" t="n"/>
+      <c r="J43" s="81" t="n"/>
       <c r="K43" s="49" t="n"/>
     </row>
     <row r="44">
@@ -5202,7 +5288,7 @@
       <c r="K49" s="69" t="n"/>
     </row>
     <row r="50">
-      <c r="A50" s="79" t="inlineStr">
+      <c r="A50" s="83" t="inlineStr">
         <is>
           <t>Hammarskiöld</t>
         </is>
@@ -5212,16 +5298,16 @@
           <t>Borderline: Mid-size full-service</t>
         </is>
       </c>
-      <c r="C50" s="79" t="n">
+      <c r="C50" s="83" t="n">
         <v>4</v>
       </c>
-      <c r="D50" s="79" t="n">
+      <c r="D50" s="83" t="n">
         <v>10</v>
       </c>
-      <c r="E50" s="79" t="n">
+      <c r="E50" s="83" t="n">
         <v>0</v>
       </c>
-      <c r="F50" s="79" t="n">
+      <c r="F50" s="83" t="n">
         <v>2</v>
       </c>
       <c r="G50" s="71" t="inlineStr">
@@ -5230,8 +5316,8 @@
         </is>
       </c>
       <c r="H50" s="71" t="n"/>
-      <c r="I50" s="79" t="n"/>
-      <c r="J50" s="79" t="n">
+      <c r="I50" s="83" t="n"/>
+      <c r="J50" s="83" t="n">
         <v>47</v>
       </c>
       <c r="K50" s="71" t="inlineStr">
@@ -5241,7 +5327,7 @@
       </c>
     </row>
     <row r="51">
-      <c r="A51" s="79" t="inlineStr">
+      <c r="A51" s="83" t="inlineStr">
         <is>
           <t>Wigge &amp; Partners</t>
         </is>
@@ -5251,16 +5337,16 @@
           <t>Borderline: Mid-size corporate</t>
         </is>
       </c>
-      <c r="C51" s="79" t="n">
+      <c r="C51" s="83" t="n">
         <v>5</v>
       </c>
-      <c r="D51" s="79" t="n">
+      <c r="D51" s="83" t="n">
         <v>3</v>
       </c>
-      <c r="E51" s="79" t="n">
+      <c r="E51" s="83" t="n">
         <v>0</v>
       </c>
-      <c r="F51" s="79" t="n">
+      <c r="F51" s="83" t="n">
         <v>1</v>
       </c>
       <c r="G51" s="71" t="inlineStr">
@@ -5269,10 +5355,10 @@
         </is>
       </c>
       <c r="H51" s="71" t="n"/>
-      <c r="I51" s="79" t="n">
+      <c r="I51" s="83" t="n">
         <v>11</v>
       </c>
-      <c r="J51" s="79" t="n">
+      <c r="J51" s="83" t="n">
         <v>40</v>
       </c>
       <c r="K51" s="71" t="inlineStr">
@@ -5282,7 +5368,7 @@
       </c>
     </row>
     <row r="52">
-      <c r="A52" s="79" t="inlineStr">
+      <c r="A52" s="83" t="inlineStr">
         <is>
           <t>Fylgia</t>
         </is>
@@ -5292,16 +5378,16 @@
           <t>Borderline: Mid-size full-service</t>
         </is>
       </c>
-      <c r="C52" s="79" t="n">
+      <c r="C52" s="83" t="n">
         <v>1</v>
       </c>
-      <c r="D52" s="79" t="n">
+      <c r="D52" s="83" t="n">
         <v>6</v>
       </c>
-      <c r="E52" s="79" t="n">
+      <c r="E52" s="83" t="n">
         <v>0</v>
       </c>
-      <c r="F52" s="79" t="n">
+      <c r="F52" s="83" t="n">
         <v>2</v>
       </c>
       <c r="G52" s="71" t="inlineStr">
@@ -5310,10 +5396,10 @@
         </is>
       </c>
       <c r="H52" s="71" t="n"/>
-      <c r="I52" s="79" t="n">
+      <c r="I52" s="83" t="n">
         <v>21</v>
       </c>
-      <c r="J52" s="79" t="n">
+      <c r="J52" s="83" t="n">
         <v>35</v>
       </c>
       <c r="K52" s="71" t="inlineStr">
@@ -5323,7 +5409,7 @@
       </c>
     </row>
     <row r="53">
-      <c r="A53" s="79" t="inlineStr">
+      <c r="A53" s="83" t="inlineStr">
         <is>
           <t>Foyen</t>
         </is>
@@ -5333,16 +5419,16 @@
           <t>Borderline: Mid-size full-service</t>
         </is>
       </c>
-      <c r="C53" s="79" t="n">
+      <c r="C53" s="83" t="n">
         <v>0</v>
       </c>
-      <c r="D53" s="79" t="n">
+      <c r="D53" s="83" t="n">
         <v>6</v>
       </c>
-      <c r="E53" s="79" t="n">
+      <c r="E53" s="83" t="n">
         <v>0</v>
       </c>
-      <c r="F53" s="79" t="n">
+      <c r="F53" s="83" t="n">
         <v>2</v>
       </c>
       <c r="G53" s="71" t="inlineStr">
@@ -5351,10 +5437,10 @@
         </is>
       </c>
       <c r="H53" s="71" t="n"/>
-      <c r="I53" s="79" t="n">
+      <c r="I53" s="83" t="n">
         <v>23</v>
       </c>
-      <c r="J53" s="79" t="n">
+      <c r="J53" s="83" t="n">
         <v>73</v>
       </c>
       <c r="K53" s="71" t="inlineStr">
@@ -5364,7 +5450,7 @@
       </c>
     </row>
     <row r="54">
-      <c r="A54" s="79" t="inlineStr">
+      <c r="A54" s="83" t="inlineStr">
         <is>
           <t>Kanter</t>
         </is>
@@ -5374,16 +5460,16 @@
           <t>Borderline: Mid-size corporate</t>
         </is>
       </c>
-      <c r="C54" s="79" t="n">
+      <c r="C54" s="83" t="n">
         <v>3</v>
       </c>
-      <c r="D54" s="79" t="n">
+      <c r="D54" s="83" t="n">
         <v>0</v>
       </c>
-      <c r="E54" s="79" t="n">
+      <c r="E54" s="83" t="n">
         <v>0</v>
       </c>
-      <c r="F54" s="79" t="n">
+      <c r="F54" s="83" t="n">
         <v>4</v>
       </c>
       <c r="G54" s="71" t="inlineStr">
@@ -5392,10 +5478,10 @@
         </is>
       </c>
       <c r="H54" s="71" t="n"/>
-      <c r="I54" s="79" t="n">
+      <c r="I54" s="83" t="n">
         <v>13</v>
       </c>
-      <c r="J54" s="79" t="n">
+      <c r="J54" s="83" t="n">
         <v>39</v>
       </c>
       <c r="K54" s="71" t="inlineStr">
@@ -30268,4 +30354,1767 @@
   <autoFilter ref="A1:E661"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
+</file>
+
+<file path=xl/worksheets/sheet7.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:R55"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="26" customWidth="1" min="1" max="1"/>
+    <col width="20" customWidth="1" min="2" max="2"/>
+    <col width="28" customWidth="1" min="3" max="3"/>
+    <col width="10" customWidth="1" min="4" max="4"/>
+    <col width="10" customWidth="1" min="5" max="5"/>
+    <col width="12" customWidth="1" min="6" max="6"/>
+    <col width="12" customWidth="1" min="7" max="7"/>
+    <col width="10" customWidth="1" min="8" max="8"/>
+    <col width="10" customWidth="1" min="9" max="9"/>
+    <col width="10" customWidth="1" min="10" max="10"/>
+    <col width="10" customWidth="1" min="11" max="11"/>
+    <col width="10" customWidth="1" min="12" max="12"/>
+    <col width="10" customWidth="1" min="13" max="13"/>
+    <col width="10" customWidth="1" min="14" max="14"/>
+    <col width="10" customWidth="1" min="15" max="15"/>
+    <col width="13" customWidth="1" min="16" max="16"/>
+    <col width="40" customWidth="1" min="17" max="17"/>
+    <col width="40" customWidth="1" min="18" max="18"/>
+  </cols>
+  <sheetData>
+    <row r="1">
+      <c r="A1" s="1" t="inlineStr">
+        <is>
+          <t>Section D. Rate card comparison: Swedish business law firms (SEK per hour, excl. VAT)</t>
+        </is>
+      </c>
+    </row>
+    <row r="2" ht="45" customHeight="1">
+      <c r="A2" s="2" t="inlineStr">
+        <is>
+          <t>Rates are only comparable when dated: Swedish firms typically revise rates annually on 1 January. Public-sector price annexes are usually confidential (Kammarrätten i Stockholm, 2017, Vinge / E-hälsomyndigheten), so firm-level rate cards are scarce. Source type matters: list price (rate card) &gt; court/Chapter 11 filings (actual billed) &gt; public tender (discounted).</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" s="47" t="inlineStr">
+        <is>
+          <t>D1. Rate cards by level (list prices)</t>
+        </is>
+      </c>
+    </row>
+    <row r="5" ht="42" customHeight="1">
+      <c r="A5" s="52" t="inlineStr">
+        <is>
+          <t>Firm</t>
+        </is>
+      </c>
+      <c r="B5" s="52" t="inlineStr">
+        <is>
+          <t>Rate date</t>
+        </is>
+      </c>
+      <c r="C5" s="52" t="inlineStr">
+        <is>
+          <t>Source</t>
+        </is>
+      </c>
+      <c r="D5" s="52" t="inlineStr">
+        <is>
+          <t>Partner</t>
+        </is>
+      </c>
+      <c r="E5" s="84" t="n"/>
+      <c r="F5" s="52" t="inlineStr">
+        <is>
+          <t>Counsel / Senior associate</t>
+        </is>
+      </c>
+      <c r="G5" s="84" t="n"/>
+      <c r="H5" s="52" t="inlineStr">
+        <is>
+          <t>Associate</t>
+        </is>
+      </c>
+      <c r="I5" s="84" t="n"/>
+      <c r="J5" s="52" t="inlineStr">
+        <is>
+          <t>Junior associate</t>
+        </is>
+      </c>
+      <c r="K5" s="84" t="n"/>
+      <c r="L5" s="52" t="inlineStr">
+        <is>
+          <t>Paralegal</t>
+        </is>
+      </c>
+      <c r="M5" s="52" t="inlineStr">
+        <is>
+          <t>Partner mid</t>
+        </is>
+      </c>
+      <c r="N5" s="52" t="inlineStr">
+        <is>
+          <t>Junior mid</t>
+        </is>
+      </c>
+      <c r="O5" s="52" t="inlineStr">
+        <is>
+          <t>Partner / junior (x)</t>
+        </is>
+      </c>
+      <c r="P5" s="52" t="inlineStr">
+        <is>
+          <t>Partner mid vs legal-aid norm 2025 (x)</t>
+        </is>
+      </c>
+      <c r="Q5" s="52" t="inlineStr">
+        <is>
+          <t>Level definitions in source</t>
+        </is>
+      </c>
+      <c r="R5" s="52" t="inlineStr">
+        <is>
+          <t>Notes</t>
+        </is>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" s="85" t="n"/>
+      <c r="B6" s="85" t="n"/>
+      <c r="C6" s="85" t="n"/>
+      <c r="D6" s="86" t="inlineStr">
+        <is>
+          <t>Low</t>
+        </is>
+      </c>
+      <c r="E6" s="86" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
+      <c r="F6" s="86" t="inlineStr">
+        <is>
+          <t>Low</t>
+        </is>
+      </c>
+      <c r="G6" s="86" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
+      <c r="H6" s="86" t="inlineStr">
+        <is>
+          <t>Low</t>
+        </is>
+      </c>
+      <c r="I6" s="86" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
+      <c r="J6" s="86" t="inlineStr">
+        <is>
+          <t>Low</t>
+        </is>
+      </c>
+      <c r="K6" s="86" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
+      <c r="L6" s="85" t="n"/>
+      <c r="M6" s="85" t="n"/>
+      <c r="N6" s="85" t="n"/>
+      <c r="O6" s="85" t="n"/>
+      <c r="P6" s="85" t="n"/>
+      <c r="Q6" s="85" t="n"/>
+      <c r="R6" s="85" t="n"/>
+    </row>
+    <row r="7" ht="60" customHeight="1">
+      <c r="A7" s="49" t="inlineStr">
+        <is>
+          <t>Mannheimer Swartling</t>
+        </is>
+      </c>
+      <c r="B7" s="49" t="inlineStr">
+        <is>
+          <t>Not stated (provided by colleague, Oct-26)</t>
+        </is>
+      </c>
+      <c r="C7" s="49" t="inlineStr">
+        <is>
+          <t>Firm rate card (client-provided snip)</t>
+        </is>
+      </c>
+      <c r="D7" s="87" t="n">
+        <v>6000</v>
+      </c>
+      <c r="E7" s="87" t="n">
+        <v>10000</v>
+      </c>
+      <c r="F7" s="87" t="n">
+        <v>4550</v>
+      </c>
+      <c r="G7" s="87" t="n">
+        <v>8000</v>
+      </c>
+      <c r="H7" s="87" t="n">
+        <v>3650</v>
+      </c>
+      <c r="I7" s="87" t="n">
+        <v>4150</v>
+      </c>
+      <c r="J7" s="87" t="n">
+        <v>2750</v>
+      </c>
+      <c r="K7" s="87" t="n">
+        <v>3350</v>
+      </c>
+      <c r="L7" s="87" t="n"/>
+      <c r="M7" s="87">
+        <f>AVERAGE(D7:E7)</f>
+        <v/>
+      </c>
+      <c r="N7" s="87">
+        <f>AVERAGE(J7:K7)</f>
+        <v/>
+      </c>
+      <c r="O7" s="88">
+        <f>M7/N7</f>
+        <v/>
+      </c>
+      <c r="P7" s="88">
+        <f>M7/1586</f>
+        <v/>
+      </c>
+      <c r="Q7" s="49" t="inlineStr">
+        <is>
+          <t>Junior Assoc 0-24 months; Associates 25-59 months; Senior Assoc / PDL / Specialist Counsel 60+ months; Partners / Senior Advisor</t>
+        </is>
+      </c>
+      <c r="R7" s="49" t="inlineStr">
+        <is>
+          <t>Counsel band (4,550-8,000) overlaps partner band. Date to be confirmed.</t>
+        </is>
+      </c>
+    </row>
+    <row r="8" ht="60" customHeight="1">
+      <c r="A8" s="49" t="inlineStr">
+        <is>
+          <t>Cederquist</t>
+        </is>
+      </c>
+      <c r="B8" s="49" t="inlineStr">
+        <is>
+          <t>2025 (revised annually 1 Jan)</t>
+        </is>
+      </c>
+      <c r="C8" s="49" t="inlineStr">
+        <is>
+          <t>Firm cost estimate / fee structure (client-provided snip)</t>
+        </is>
+      </c>
+      <c r="D8" s="87" t="n">
+        <v>6500</v>
+      </c>
+      <c r="E8" s="87" t="n">
+        <v>8000</v>
+      </c>
+      <c r="F8" s="87" t="n">
+        <v>4500</v>
+      </c>
+      <c r="G8" s="87" t="n">
+        <v>5800</v>
+      </c>
+      <c r="H8" s="87" t="n">
+        <v>3600</v>
+      </c>
+      <c r="I8" s="87" t="n">
+        <v>4100</v>
+      </c>
+      <c r="J8" s="87" t="n">
+        <v>2300</v>
+      </c>
+      <c r="K8" s="87" t="n">
+        <v>3100</v>
+      </c>
+      <c r="L8" s="87" t="n">
+        <v>1500</v>
+      </c>
+      <c r="M8" s="87">
+        <f>AVERAGE(D8:E8)</f>
+        <v/>
+      </c>
+      <c r="N8" s="87">
+        <f>AVERAGE(J8:K8)</f>
+        <v/>
+      </c>
+      <c r="O8" s="88">
+        <f>M8/N8</f>
+        <v/>
+      </c>
+      <c r="P8" s="88">
+        <f>M8/1586</f>
+        <v/>
+      </c>
+      <c r="Q8" s="49" t="inlineStr">
+        <is>
+          <t>Partners; Senior Associates; Associates; Junior Associates; Paralegals</t>
+        </is>
+      </c>
+      <c r="R8" s="49" t="inlineStr">
+        <is>
+          <t>Time-incurred basis; open to alternative fee arrangements per project.</t>
+        </is>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" s="46" t="inlineStr">
+        <is>
+          <t>Difference: Mannheimer Swartling vs Cederquist (mid-points)</t>
+        </is>
+      </c>
+      <c r="D9" s="89">
+        <f>AVERAGE(D7:E7)/AVERAGE(D8:E8)-1</f>
+        <v/>
+      </c>
+      <c r="F9" s="89">
+        <f>AVERAGE(F7:G7)/AVERAGE(F8:G8)-1</f>
+        <v/>
+      </c>
+      <c r="H9" s="89">
+        <f>AVERAGE(H7:I7)/AVERAGE(H8:I8)-1</f>
+        <v/>
+      </c>
+      <c r="J9" s="89">
+        <f>AVERAGE(J7:K7)/AVERAGE(J8:K8)-1</f>
+        <v/>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" s="47" t="inlineStr">
+        <is>
+          <t>D2. Indicative firm-wide hourly ranges (third-party directory, low reliability)</t>
+        </is>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" s="52" t="inlineStr">
+        <is>
+          <t>Firm</t>
+        </is>
+      </c>
+      <c r="B12" s="52" t="inlineStr">
+        <is>
+          <t>Accessed</t>
+        </is>
+      </c>
+      <c r="C12" s="52" t="inlineStr">
+        <is>
+          <t>Source</t>
+        </is>
+      </c>
+      <c r="D12" s="52" t="inlineStr">
+        <is>
+          <t>Low (~associate)</t>
+        </is>
+      </c>
+      <c r="E12" s="52" t="inlineStr">
+        <is>
+          <t>High (~partner)</t>
+        </is>
+      </c>
+      <c r="F12" s="52" t="inlineStr">
+        <is>
+          <t>Mid</t>
+        </is>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" s="49" t="inlineStr">
+        <is>
+          <t>Mannheimer Swartling</t>
+        </is>
+      </c>
+      <c r="B13" s="49" t="inlineStr">
+        <is>
+          <t>Oct-2026 (undated on site)</t>
+        </is>
+      </c>
+      <c r="C13" s="49" t="inlineStr">
+        <is>
+          <t>skatterätt.se firm pages (tax practice; no level split, no source)</t>
+        </is>
+      </c>
+      <c r="D13" s="87" t="n">
+        <v>4500</v>
+      </c>
+      <c r="E13" s="87" t="n">
+        <v>8000</v>
+      </c>
+      <c r="F13" s="87">
+        <f>AVERAGE(D13:E13)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" s="49" t="inlineStr">
+        <is>
+          <t>Roschier</t>
+        </is>
+      </c>
+      <c r="B14" s="49" t="inlineStr">
+        <is>
+          <t>Oct-2026 (undated on site)</t>
+        </is>
+      </c>
+      <c r="C14" s="49" t="inlineStr">
+        <is>
+          <t>skatterätt.se firm pages (tax practice; no level split, no source)</t>
+        </is>
+      </c>
+      <c r="D14" s="87" t="n">
+        <v>4200</v>
+      </c>
+      <c r="E14" s="87" t="n">
+        <v>7000</v>
+      </c>
+      <c r="F14" s="87">
+        <f>AVERAGE(D14:E14)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" s="49" t="inlineStr">
+        <is>
+          <t>Vinge</t>
+        </is>
+      </c>
+      <c r="B15" s="49" t="inlineStr">
+        <is>
+          <t>Oct-2026 (undated on site)</t>
+        </is>
+      </c>
+      <c r="C15" s="49" t="inlineStr">
+        <is>
+          <t>skatterätt.se firm pages (tax practice; no level split, no source)</t>
+        </is>
+      </c>
+      <c r="D15" s="87" t="n">
+        <v>4000</v>
+      </c>
+      <c r="E15" s="87" t="n">
+        <v>7000</v>
+      </c>
+      <c r="F15" s="87">
+        <f>AVERAGE(D15:E15)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" s="49" t="inlineStr">
+        <is>
+          <t>DLA Piper</t>
+        </is>
+      </c>
+      <c r="B16" s="49" t="inlineStr">
+        <is>
+          <t>Oct-2026 (undated on site)</t>
+        </is>
+      </c>
+      <c r="C16" s="49" t="inlineStr">
+        <is>
+          <t>skatterätt.se firm pages (tax practice; no level split, no source)</t>
+        </is>
+      </c>
+      <c r="D16" s="87" t="n">
+        <v>4000</v>
+      </c>
+      <c r="E16" s="87" t="n">
+        <v>7000</v>
+      </c>
+      <c r="F16" s="87">
+        <f>AVERAGE(D16:E16)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" s="49" t="inlineStr">
+        <is>
+          <t>Schjødt</t>
+        </is>
+      </c>
+      <c r="B17" s="49" t="inlineStr">
+        <is>
+          <t>Oct-2026 (undated on site)</t>
+        </is>
+      </c>
+      <c r="C17" s="49" t="inlineStr">
+        <is>
+          <t>skatterätt.se firm pages (tax practice; no level split, no source)</t>
+        </is>
+      </c>
+      <c r="D17" s="87" t="n">
+        <v>3800</v>
+      </c>
+      <c r="E17" s="87" t="n">
+        <v>6500</v>
+      </c>
+      <c r="F17" s="87">
+        <f>AVERAGE(D17:E17)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="18">
+      <c r="A18" s="49" t="inlineStr">
+        <is>
+          <t>Cederquist</t>
+        </is>
+      </c>
+      <c r="B18" s="49" t="inlineStr">
+        <is>
+          <t>Oct-2026 (undated on site)</t>
+        </is>
+      </c>
+      <c r="C18" s="49" t="inlineStr">
+        <is>
+          <t>skatterätt.se firm pages (tax practice; no level split, no source)</t>
+        </is>
+      </c>
+      <c r="D18" s="87" t="n">
+        <v>3800</v>
+      </c>
+      <c r="E18" s="87" t="n">
+        <v>6500</v>
+      </c>
+      <c r="F18" s="87">
+        <f>AVERAGE(D18:E18)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="19">
+      <c r="A19" s="49" t="inlineStr">
+        <is>
+          <t>Setterwalls</t>
+        </is>
+      </c>
+      <c r="B19" s="49" t="inlineStr">
+        <is>
+          <t>Oct-2026 (undated on site)</t>
+        </is>
+      </c>
+      <c r="C19" s="49" t="inlineStr">
+        <is>
+          <t>skatterätt.se firm pages (tax practice; no level split, no source)</t>
+        </is>
+      </c>
+      <c r="D19" s="87" t="n">
+        <v>3500</v>
+      </c>
+      <c r="E19" s="87" t="n">
+        <v>6000</v>
+      </c>
+      <c r="F19" s="87">
+        <f>AVERAGE(D19:E19)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="20">
+      <c r="A20" s="49" t="inlineStr">
+        <is>
+          <t>Bird &amp; Bird</t>
+        </is>
+      </c>
+      <c r="B20" s="49" t="inlineStr">
+        <is>
+          <t>Oct-2026 (undated on site)</t>
+        </is>
+      </c>
+      <c r="C20" s="49" t="inlineStr">
+        <is>
+          <t>skatterätt.se firm pages (tax practice; no level split, no source)</t>
+        </is>
+      </c>
+      <c r="D20" s="87" t="n">
+        <v>3500</v>
+      </c>
+      <c r="E20" s="87" t="n">
+        <v>6000</v>
+      </c>
+      <c r="F20" s="87">
+        <f>AVERAGE(D20:E20)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="21">
+      <c r="A21" s="49" t="inlineStr">
+        <is>
+          <t>Delphi</t>
+        </is>
+      </c>
+      <c r="B21" s="49" t="inlineStr">
+        <is>
+          <t>Oct-2026 (undated on site)</t>
+        </is>
+      </c>
+      <c r="C21" s="49" t="inlineStr">
+        <is>
+          <t>skatterätt.se firm pages (tax practice; no level split, no source)</t>
+        </is>
+      </c>
+      <c r="D21" s="87" t="n">
+        <v>3200</v>
+      </c>
+      <c r="E21" s="87" t="n">
+        <v>5500</v>
+      </c>
+      <c r="F21" s="87">
+        <f>AVERAGE(D21:E21)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="22">
+      <c r="A22" s="49" t="inlineStr">
+        <is>
+          <t>Lindahl</t>
+        </is>
+      </c>
+      <c r="B22" s="49" t="inlineStr">
+        <is>
+          <t>Oct-2026 (undated on site)</t>
+        </is>
+      </c>
+      <c r="C22" s="49" t="inlineStr">
+        <is>
+          <t>skatterätt.se firm pages (tax practice; no level split, no source)</t>
+        </is>
+      </c>
+      <c r="D22" s="87" t="n">
+        <v>3000</v>
+      </c>
+      <c r="E22" s="87" t="n">
+        <v>5500</v>
+      </c>
+      <c r="F22" s="87">
+        <f>AVERAGE(D22:E22)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="23">
+      <c r="A23" s="45" t="inlineStr">
+        <is>
+          <t>Example: https://www.xn--skattertt-12a.se/byra/vinge-skatt/ (Vinge: "Timarvode 4 000 till 7 000 kr"). Ranges may be estimates; use only for relative positioning.</t>
+        </is>
+      </c>
+    </row>
+    <row r="25">
+      <c r="A25" s="47" t="inlineStr">
+        <is>
+          <t>D3. Dated rate data points: invoices, court filings, tenders, market commentary</t>
+        </is>
+      </c>
+    </row>
+    <row r="26">
+      <c r="A26" s="52" t="inlineStr">
+        <is>
+          <t>Firm</t>
+        </is>
+      </c>
+      <c r="B26" s="52" t="inlineStr">
+        <is>
+          <t>Rate date</t>
+        </is>
+      </c>
+      <c r="C26" s="52" t="inlineStr">
+        <is>
+          <t>Level (as stated)</t>
+        </is>
+      </c>
+      <c r="D26" s="52" t="inlineStr">
+        <is>
+          <t>Mapped level</t>
+        </is>
+      </c>
+      <c r="E26" s="52" t="inlineStr">
+        <is>
+          <t>Rate low</t>
+        </is>
+      </c>
+      <c r="F26" s="52" t="inlineStr">
+        <is>
+          <t>Rate high</t>
+        </is>
+      </c>
+      <c r="G26" s="52" t="inlineStr">
+        <is>
+          <t>Context / client</t>
+        </is>
+      </c>
+      <c r="H26" s="52" t="inlineStr">
+        <is>
+          <t>Source type</t>
+        </is>
+      </c>
+      <c r="I26" s="52" t="inlineStr">
+        <is>
+          <t>Discounted / public?</t>
+        </is>
+      </c>
+      <c r="J26" s="52" t="inlineStr">
+        <is>
+          <t>Source</t>
+        </is>
+      </c>
+    </row>
+    <row r="27">
+      <c r="A27" s="49" t="inlineStr">
+        <is>
+          <t>Mannheimer Swartling</t>
+        </is>
+      </c>
+      <c r="B27" s="49" t="inlineStr">
+        <is>
+          <t>Nov-2010</t>
+        </is>
+      </c>
+      <c r="C27" s="49" t="inlineStr">
+        <is>
+          <t>Delägare</t>
+        </is>
+      </c>
+      <c r="D27" s="49" t="inlineStr">
+        <is>
+          <t>Partner</t>
+        </is>
+      </c>
+      <c r="E27" s="87" t="n">
+        <v>3150</v>
+      </c>
+      <c r="F27" s="87" t="n">
+        <v>3150</v>
+      </c>
+      <c r="G27" s="49" t="inlineStr">
+        <is>
+          <t>SL (Stockholm public transport), C30 metro procurement</t>
+        </is>
+      </c>
+      <c r="H27" s="49" t="inlineStr">
+        <is>
+          <t>Invoice (press)</t>
+        </is>
+      </c>
+      <c r="I27" s="49" t="inlineStr">
+        <is>
+          <t>Yes: SL framework + 10% invoice discount</t>
+        </is>
+      </c>
+      <c r="J27" s="49" t="inlineStr">
+        <is>
+          <t>https://www.realtid.se/bors-finans/mannheimers-taxa-till-sl-1906-krh/</t>
+        </is>
+      </c>
+    </row>
+    <row r="28">
+      <c r="A28" s="49" t="inlineStr">
+        <is>
+          <t>Mannheimer Swartling</t>
+        </is>
+      </c>
+      <c r="B28" s="49" t="inlineStr">
+        <is>
+          <t>Nov-2010</t>
+        </is>
+      </c>
+      <c r="C28" s="49" t="inlineStr">
+        <is>
+          <t>Biträdande jurist (advokat)</t>
+        </is>
+      </c>
+      <c r="D28" s="49" t="inlineStr">
+        <is>
+          <t>Associate / Senior associate</t>
+        </is>
+      </c>
+      <c r="E28" s="87" t="n">
+        <v>2150</v>
+      </c>
+      <c r="F28" s="87" t="n">
+        <v>2150</v>
+      </c>
+      <c r="G28" s="49" t="inlineStr">
+        <is>
+          <t>SL</t>
+        </is>
+      </c>
+      <c r="H28" s="49" t="inlineStr">
+        <is>
+          <t>Invoice (press)</t>
+        </is>
+      </c>
+      <c r="I28" s="49" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="J28" s="49" t="inlineStr">
+        <is>
+          <t>https://www.realtid.se/bors-finans/mannheimers-taxa-till-sl-1906-krh/</t>
+        </is>
+      </c>
+    </row>
+    <row r="29">
+      <c r="A29" s="49" t="inlineStr">
+        <is>
+          <t>Mannheimer Swartling</t>
+        </is>
+      </c>
+      <c r="B29" s="49" t="inlineStr">
+        <is>
+          <t>Nov-2010</t>
+        </is>
+      </c>
+      <c r="C29" s="49" t="inlineStr">
+        <is>
+          <t>Junior biträdande jurist</t>
+        </is>
+      </c>
+      <c r="D29" s="49" t="inlineStr">
+        <is>
+          <t>Junior associate</t>
+        </is>
+      </c>
+      <c r="E29" s="87" t="n">
+        <v>1550</v>
+      </c>
+      <c r="F29" s="87" t="n">
+        <v>1550</v>
+      </c>
+      <c r="G29" s="49" t="inlineStr">
+        <is>
+          <t>SL; blended 2,118 (1,906 after discount)</t>
+        </is>
+      </c>
+      <c r="H29" s="49" t="inlineStr">
+        <is>
+          <t>Invoice (press)</t>
+        </is>
+      </c>
+      <c r="I29" s="49" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="J29" s="49" t="inlineStr">
+        <is>
+          <t>https://www.realtid.se/bors-finans/mannheimers-taxa-till-sl-1906-krh/</t>
+        </is>
+      </c>
+    </row>
+    <row r="30">
+      <c r="A30" s="49" t="inlineStr">
+        <is>
+          <t>Mannheimer Swartling</t>
+        </is>
+      </c>
+      <c r="B30" s="49" t="inlineStr">
+        <is>
+          <t>Oct-2009</t>
+        </is>
+      </c>
+      <c r="C30" s="49" t="inlineStr">
+        <is>
+          <t>Partner (chairman)</t>
+        </is>
+      </c>
+      <c r="D30" s="49" t="inlineStr">
+        <is>
+          <t>Partner</t>
+        </is>
+      </c>
+      <c r="E30" s="87" t="n">
+        <v>3200</v>
+      </c>
+      <c r="F30" s="87" t="n">
+        <v>3200</v>
+      </c>
+      <c r="G30" s="49" t="inlineStr">
+        <is>
+          <t>Försvarsmakten, Projekt PRIO</t>
+        </is>
+      </c>
+      <c r="H30" s="49" t="inlineStr">
+        <is>
+          <t>Invoice (press)</t>
+        </is>
+      </c>
+      <c r="I30" s="49" t="inlineStr">
+        <is>
+          <t>Public client; discount unknown</t>
+        </is>
+      </c>
+      <c r="J30" s="49" t="inlineStr">
+        <is>
+          <t>https://www.realtid.se/sa-hog-ar-mannheimers-timtaxa-mot-forsvarsmakten/</t>
+        </is>
+      </c>
+    </row>
+    <row r="31">
+      <c r="A31" s="49" t="inlineStr">
+        <is>
+          <t>Mannheimer Swartling</t>
+        </is>
+      </c>
+      <c r="B31" s="49" t="inlineStr">
+        <is>
+          <t>Jan-2010</t>
+        </is>
+      </c>
+      <c r="C31" s="49" t="inlineStr">
+        <is>
+          <t>Not stated (partner-led team)</t>
+        </is>
+      </c>
+      <c r="D31" s="49" t="inlineStr">
+        <is>
+          <t>Partner / blended</t>
+        </is>
+      </c>
+      <c r="E31" s="87" t="n">
+        <v>3800</v>
+      </c>
+      <c r="F31" s="87" t="n">
+        <v>3800</v>
+      </c>
+      <c r="G31" s="49" t="inlineStr">
+        <is>
+          <t>Riksgälden, Carnegie valuation dispute</t>
+        </is>
+      </c>
+      <c r="H31" s="49" t="inlineStr">
+        <is>
+          <t>Invoice (press)</t>
+        </is>
+      </c>
+      <c r="I31" s="49" t="inlineStr">
+        <is>
+          <t>Public client; direct award</t>
+        </is>
+      </c>
+      <c r="J31" s="49" t="inlineStr">
+        <is>
+          <t>https://www.realtid.se/bors-finans/bo-lundgrens-advokatnota-21-mkr/</t>
+        </is>
+      </c>
+    </row>
+    <row r="32">
+      <c r="A32" s="49" t="inlineStr">
+        <is>
+          <t>DLA Piper Sweden</t>
+        </is>
+      </c>
+      <c r="B32" s="49" t="inlineStr">
+        <is>
+          <t>2012-2017 (claimed Jun-2017)</t>
+        </is>
+      </c>
+      <c r="C32" s="49" t="inlineStr">
+        <is>
+          <t>Ombud (counsel team)</t>
+        </is>
+      </c>
+      <c r="D32" s="49" t="inlineStr">
+        <is>
+          <t>Partner / senior</t>
+        </is>
+      </c>
+      <c r="E32" s="87" t="n">
+        <v>3400</v>
+      </c>
+      <c r="F32" s="87" t="n">
+        <v>3900</v>
+      </c>
+      <c r="G32" s="49" t="inlineStr">
+        <is>
+          <t>HQ AB v. former directors, Stockholm District Court</t>
+        </is>
+      </c>
+      <c r="H32" s="49" t="inlineStr">
+        <is>
+          <t>Court cost claim</t>
+        </is>
+      </c>
+      <c r="I32" s="49" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="J32" s="49" t="inlineStr">
+        <is>
+          <t>https://www.realtid.se/bors-finans/hq-processens-prislapp-441-miljoner-kronor/</t>
+        </is>
+      </c>
+    </row>
+    <row r="33">
+      <c r="A33" s="49" t="inlineStr">
+        <is>
+          <t>Roschier</t>
+        </is>
+      </c>
+      <c r="B33" s="49" t="inlineStr">
+        <is>
+          <t>2012-2017 (claimed 2017)</t>
+        </is>
+      </c>
+      <c r="C33" s="49" t="inlineStr">
+        <is>
+          <t>Implied blended (SEK 17.5m / 5,207 h)</t>
+        </is>
+      </c>
+      <c r="D33" s="49" t="inlineStr">
+        <is>
+          <t>Blended</t>
+        </is>
+      </c>
+      <c r="E33" s="87" t="n">
+        <v>3360</v>
+      </c>
+      <c r="F33" s="87" t="n">
+        <v>3360</v>
+      </c>
+      <c r="G33" s="49" t="inlineStr">
+        <is>
+          <t>HQ AB (claimant)</t>
+        </is>
+      </c>
+      <c r="H33" s="49" t="inlineStr">
+        <is>
+          <t>Court cost claim (calc.)</t>
+        </is>
+      </c>
+      <c r="I33" s="49" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="J33" s="49" t="inlineStr">
+        <is>
+          <t>https://www.realtid.se/bors-finans/hq-processens-prislapp-441-miljoner-kronor/</t>
+        </is>
+      </c>
+    </row>
+    <row r="34">
+      <c r="A34" s="49" t="inlineStr">
+        <is>
+          <t>Mannheimer Swartling</t>
+        </is>
+      </c>
+      <c r="B34" s="49" t="inlineStr">
+        <is>
+          <t>Nov-2024 to Mar-2025</t>
+        </is>
+      </c>
+      <c r="C34" s="49" t="inlineStr">
+        <is>
+          <t>Average across team (~6,000 h, SEK 32m)</t>
+        </is>
+      </c>
+      <c r="D34" s="49" t="inlineStr">
+        <is>
+          <t>Blended</t>
+        </is>
+      </c>
+      <c r="E34" s="87" t="n">
+        <v>4000</v>
+      </c>
+      <c r="F34" s="87" t="n">
+        <v>4000</v>
+      </c>
+      <c r="G34" s="49" t="inlineStr">
+        <is>
+          <t>Northvolt US Chapter 11 (Swedish counsel); lowest average of advisers</t>
+        </is>
+      </c>
+      <c r="H34" s="49" t="inlineStr">
+        <is>
+          <t>Chapter 11 filing (press)</t>
+        </is>
+      </c>
+      <c r="I34" s="49" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="J34" s="49" t="inlineStr">
+        <is>
+          <t>https://www.affarsvarlden.se/artikel/sa-dyrt-blev-northvolts-raddningsforsok-i-usa-debiteras-47-000-timmar</t>
+        </is>
+      </c>
+    </row>
+    <row r="35">
+      <c r="A35" s="49" t="inlineStr">
+        <is>
+          <t>Kirkland &amp; Ellis (comparison)</t>
+        </is>
+      </c>
+      <c r="B35" s="49" t="inlineStr">
+        <is>
+          <t>Nov-Dec-2024</t>
+        </is>
+      </c>
+      <c r="C35" s="49" t="inlineStr">
+        <is>
+          <t>Average / top rate</t>
+        </is>
+      </c>
+      <c r="D35" s="49" t="inlineStr">
+        <is>
+          <t>Blended / top partner</t>
+        </is>
+      </c>
+      <c r="E35" s="87" t="n">
+        <v>14300</v>
+      </c>
+      <c r="F35" s="87" t="n">
+        <v>25500</v>
+      </c>
+      <c r="G35" s="49" t="inlineStr">
+        <is>
+          <t>Northvolt Chapter 11 (US lead counsel)</t>
+        </is>
+      </c>
+      <c r="H35" s="49" t="inlineStr">
+        <is>
+          <t>Chapter 11 filing (press)</t>
+        </is>
+      </c>
+      <c r="I35" s="49" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="J35" s="49" t="inlineStr">
+        <is>
+          <t>https://www.affarsvarlden.se/artikel/northvolts-nota-over-100-miljoner-i-manaden-pa-advokater-och-radgivare</t>
+        </is>
+      </c>
+    </row>
+    <row r="36">
+      <c r="A36" s="49" t="inlineStr">
+        <is>
+          <t>Front Advokater</t>
+        </is>
+      </c>
+      <c r="B36" s="49" t="inlineStr">
+        <is>
+          <t>2016-2020</t>
+        </is>
+      </c>
+      <c r="C36" s="49" t="inlineStr">
+        <is>
+          <t>Junior / Jurist / Senior (&gt;=2/5/10 yrs)</t>
+        </is>
+      </c>
+      <c r="D36" s="49" t="inlineStr">
+        <is>
+          <t>Junior / Associate / Senior</t>
+        </is>
+      </c>
+      <c r="E36" s="87" t="n">
+        <v>953</v>
+      </c>
+      <c r="F36" s="87" t="n">
+        <v>1588</v>
+      </c>
+      <c r="G36" s="49" t="inlineStr">
+        <is>
+          <t>City of Gothenburg legal services framework (area A: 953/1,270/1,588; area B: 833/1,110/1,388)</t>
+        </is>
+      </c>
+      <c r="H36" s="49" t="inlineStr">
+        <is>
+          <t>Public tender (court judgment)</t>
+        </is>
+      </c>
+      <c r="I36" s="49" t="inlineStr">
+        <is>
+          <t>Yes: aggressive tender pricing</t>
+        </is>
+      </c>
+      <c r="J36" s="49" t="inlineStr">
+        <is>
+          <t>https://upphandling24.se/wp-content/uploads/2024/03/goteborgs-tr-t-20148-21-dom-2024-02-21.pdf</t>
+        </is>
+      </c>
+    </row>
+    <row r="37">
+      <c r="A37" s="49" t="inlineStr">
+        <is>
+          <t>7 unnamed firms</t>
+        </is>
+      </c>
+      <c r="B37" s="49" t="inlineStr">
+        <is>
+          <t>2007</t>
+        </is>
+      </c>
+      <c r="C37" s="49" t="inlineStr">
+        <is>
+          <t>Tender price</t>
+        </is>
+      </c>
+      <c r="D37" s="49" t="inlineStr">
+        <is>
+          <t>Blended</t>
+        </is>
+      </c>
+      <c r="E37" s="87" t="n">
+        <v>1800</v>
+      </c>
+      <c r="F37" s="87" t="n">
+        <v>2800</v>
+      </c>
+      <c r="G37" s="49" t="inlineStr">
+        <is>
+          <t>State tender: advisers for divesting state-owned companies</t>
+        </is>
+      </c>
+      <c r="H37" s="49" t="inlineStr">
+        <is>
+          <t>Public tender (press)</t>
+        </is>
+      </c>
+      <c r="I37" s="49" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="J37" s="49" t="inlineStr">
+        <is>
+          <t>https://www.realtid.se/bors-finans/det-blir-13000-kronor-tack-per-timme/</t>
+        </is>
+      </c>
+    </row>
+    <row r="38">
+      <c r="A38" s="49" t="inlineStr">
+        <is>
+          <t>Unnamed external advokat</t>
+        </is>
+      </c>
+      <c r="B38" s="49" t="inlineStr">
+        <is>
+          <t>Dec-2024</t>
+        </is>
+      </c>
+      <c r="C38" s="49" t="inlineStr">
+        <is>
+          <t>Advokat</t>
+        </is>
+      </c>
+      <c r="D38" s="49" t="inlineStr">
+        <is>
+          <t>Partner</t>
+        </is>
+      </c>
+      <c r="E38" s="87" t="n">
+        <v>4500</v>
+      </c>
+      <c r="F38" s="87" t="n">
+        <v>4500</v>
+      </c>
+      <c r="G38" s="49" t="inlineStr">
+        <is>
+          <t>Botkyrka municipality</t>
+        </is>
+      </c>
+      <c r="H38" s="49" t="inlineStr">
+        <is>
+          <t>Press</t>
+        </is>
+      </c>
+      <c r="I38" s="49" t="inlineStr">
+        <is>
+          <t>Public client</t>
+        </is>
+      </c>
+      <c r="J38" s="49" t="inlineStr">
+        <is>
+          <t>https://www.svt.se/nyheter/lokalt/stockholm/botkyrka-tar-in-extern-advokat-for-4-500-kronor-i-timmen</t>
+        </is>
+      </c>
+    </row>
+    <row r="39">
+      <c r="A39" s="49" t="inlineStr">
+        <is>
+          <t>Law firm (unnamed)</t>
+        </is>
+      </c>
+      <c r="B39" s="49" t="inlineStr">
+        <is>
+          <t>Apr-2026</t>
+        </is>
+      </c>
+      <c r="C39" s="49" t="inlineStr">
+        <is>
+          <t>Hourly rate held reasonable</t>
+        </is>
+      </c>
+      <c r="D39" s="49" t="inlineStr">
+        <is>
+          <t>n/a</t>
+        </is>
+      </c>
+      <c r="E39" s="87" t="n">
+        <v>4000</v>
+      </c>
+      <c r="F39" s="87" t="n">
+        <v>4000</v>
+      </c>
+      <c r="G39" s="49" t="inlineStr">
+        <is>
+          <t>Luleå tingsrätt cost ruling</t>
+        </is>
+      </c>
+      <c r="H39" s="49" t="inlineStr">
+        <is>
+          <t>Court ruling (press)</t>
+        </is>
+      </c>
+      <c r="I39" s="49" t="inlineStr">
+        <is>
+          <t>n/a</t>
+        </is>
+      </c>
+      <c r="J39" s="49" t="inlineStr">
+        <is>
+          <t>https://www.realtid.se/juridik/ratten-om-timarvoden-4-000-kronor-i-timmen-ar-ok/</t>
+        </is>
+      </c>
+    </row>
+    <row r="40">
+      <c r="A40" s="49" t="inlineStr">
+        <is>
+          <t>Top-tier firms (market)</t>
+        </is>
+      </c>
+      <c r="B40" s="49" t="inlineStr">
+        <is>
+          <t>2026</t>
+        </is>
+      </c>
+      <c r="C40" s="49" t="inlineStr">
+        <is>
+          <t>Partner</t>
+        </is>
+      </c>
+      <c r="D40" s="49" t="inlineStr">
+        <is>
+          <t>Partner</t>
+        </is>
+      </c>
+      <c r="E40" s="87" t="n">
+        <v>7000</v>
+      </c>
+      <c r="F40" s="87" t="n">
+        <v>9000</v>
+      </c>
+      <c r="G40" s="49" t="inlineStr">
+        <is>
+          <t>Olle Flygt (ex-Vinge/MSA partner): partners bill 7,000-9,000; associates ~3,000</t>
+        </is>
+      </c>
+      <c r="H40" s="49" t="inlineStr">
+        <is>
+          <t>Market commentary</t>
+        </is>
+      </c>
+      <c r="I40" s="49" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="J40" s="49" t="inlineStr">
+        <is>
+          <t>https://www.realtid.se/perfectweekend/affarsjuridikens-karna-det-har-blivit-for-mycket-fokus-pa-pengar/</t>
+        </is>
+      </c>
+    </row>
+    <row r="41">
+      <c r="A41" s="49" t="inlineStr">
+        <is>
+          <t>Top-tier firms (market)</t>
+        </is>
+      </c>
+      <c r="B41" s="49" t="inlineStr">
+        <is>
+          <t>2026</t>
+        </is>
+      </c>
+      <c r="C41" s="49" t="inlineStr">
+        <is>
+          <t>Associate</t>
+        </is>
+      </c>
+      <c r="D41" s="49" t="inlineStr">
+        <is>
+          <t>Associate</t>
+        </is>
+      </c>
+      <c r="E41" s="87" t="n">
+        <v>3000</v>
+      </c>
+      <c r="F41" s="87" t="n">
+        <v>3000</v>
+      </c>
+      <c r="G41" s="49" t="inlineStr">
+        <is>
+          <t>As above</t>
+        </is>
+      </c>
+      <c r="H41" s="49" t="inlineStr">
+        <is>
+          <t>Market commentary</t>
+        </is>
+      </c>
+      <c r="I41" s="49" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="J41" s="49" t="inlineStr">
+        <is>
+          <t>https://www.realtid.se/perfectweekend/affarsjuridikens-karna-det-har-blivit-for-mycket-fokus-pa-pengar/</t>
+        </is>
+      </c>
+    </row>
+    <row r="42">
+      <c r="A42" s="49" t="inlineStr">
+        <is>
+          <t>Mannheimer Swartling</t>
+        </is>
+      </c>
+      <c r="B42" s="49" t="inlineStr">
+        <is>
+          <t>Final years before 2025 (not specified)</t>
+        </is>
+      </c>
+      <c r="C42" s="49" t="inlineStr">
+        <is>
+          <t>Partner (Olle Flygt)</t>
+        </is>
+      </c>
+      <c r="D42" s="49" t="inlineStr">
+        <is>
+          <t>Partner</t>
+        </is>
+      </c>
+      <c r="E42" s="87" t="n">
+        <v>7000</v>
+      </c>
+      <c r="F42" s="87" t="n">
+        <v>8000</v>
+      </c>
+      <c r="G42" s="49" t="inlineStr">
+        <is>
+          <t>Own billing rate</t>
+        </is>
+      </c>
+      <c r="H42" s="49" t="inlineStr">
+        <is>
+          <t>Market commentary</t>
+        </is>
+      </c>
+      <c r="I42" s="49" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="J42" s="49" t="inlineStr">
+        <is>
+          <t>https://www.realtid.se/juridik/affarsjuridiken-vaxer-men-sprickorna-syns/</t>
+        </is>
+      </c>
+    </row>
+    <row r="44">
+      <c r="A44" s="47" t="inlineStr">
+        <is>
+          <t>D4. Benchmarks</t>
+        </is>
+      </c>
+    </row>
+    <row r="45">
+      <c r="A45" s="52" t="inlineStr">
+        <is>
+          <t>Benchmark</t>
+        </is>
+      </c>
+      <c r="B45" s="52" t="inlineStr">
+        <is>
+          <t>Period</t>
+        </is>
+      </c>
+      <c r="C45" s="52" t="inlineStr">
+        <is>
+          <t>Rate</t>
+        </is>
+      </c>
+      <c r="D45" s="52" t="inlineStr">
+        <is>
+          <t>Currency</t>
+        </is>
+      </c>
+      <c r="E45" s="52" t="inlineStr">
+        <is>
+          <t>Notes</t>
+        </is>
+      </c>
+      <c r="F45" s="52" t="inlineStr">
+        <is>
+          <t>Source</t>
+        </is>
+      </c>
+    </row>
+    <row r="46">
+      <c r="A46" s="49" t="inlineStr">
+        <is>
+          <t>Legal-aid hourly norm (timkostnadsnorm), F-skatt</t>
+        </is>
+      </c>
+      <c r="B46" s="49" t="inlineStr">
+        <is>
+          <t>2025</t>
+        </is>
+      </c>
+      <c r="C46" s="87" t="n">
+        <v>1586</v>
+      </c>
+      <c r="D46" s="49" t="inlineStr">
+        <is>
+          <t>SEK</t>
+        </is>
+      </c>
+      <c r="E46" s="49" t="inlineStr">
+        <is>
+          <t>SFS 2024:913</t>
+        </is>
+      </c>
+      <c r="F46" s="49" t="inlineStr">
+        <is>
+          <t>https://www.svenskforfattningssamling.se/sites/default/files/sfs/2024-10/SFS2024-913.pdf</t>
+        </is>
+      </c>
+    </row>
+    <row r="47">
+      <c r="A47" s="49" t="inlineStr">
+        <is>
+          <t>Legal-aid hourly norm (timkostnadsnorm), F-skatt</t>
+        </is>
+      </c>
+      <c r="B47" s="49" t="inlineStr">
+        <is>
+          <t>2026</t>
+        </is>
+      </c>
+      <c r="C47" s="87" t="n">
+        <v>1626</v>
+      </c>
+      <c r="D47" s="49" t="inlineStr">
+        <is>
+          <t>SEK</t>
+        </is>
+      </c>
+      <c r="E47" s="49" t="inlineStr">
+        <is>
+          <t>SFS 2025:919 (+2.5%). Bar Association: business lawyers bill "at least three times" this</t>
+        </is>
+      </c>
+      <c r="F47" s="49" t="inlineStr">
+        <is>
+          <t>https://xn--svenskfrfattningssamling-roc.se/sites/default/files/sfs/2025-10/SFS2025-919.pdf</t>
+        </is>
+      </c>
+    </row>
+    <row r="48">
+      <c r="A48" s="49" t="inlineStr">
+        <is>
+          <t>Affärsvärlden fee income per lawyer (56-63 firms)</t>
+        </is>
+      </c>
+      <c r="B48" s="49" t="inlineStr">
+        <is>
+          <t>2024</t>
+        </is>
+      </c>
+      <c r="C48" s="87" t="n">
+        <v>4130000</v>
+      </c>
+      <c r="D48" s="49" t="inlineStr">
+        <is>
+          <t>SEK p.a.</t>
+        </is>
+      </c>
+      <c r="E48" s="49" t="inlineStr">
+        <is>
+          <t>~SEK 2,580/h at 1,600 billable hours (illustrative)</t>
+        </is>
+      </c>
+      <c r="F48" s="49" t="inlineStr">
+        <is>
+          <t>https://www.realtid.se/affarer/154-miljarder-sa-klarade-affarsjuristerna-tullchocken/</t>
+        </is>
+      </c>
+    </row>
+    <row r="49">
+      <c r="A49" s="49" t="inlineStr">
+        <is>
+          <t>Affärsvärlden fee income per lawyer</t>
+        </is>
+      </c>
+      <c r="B49" s="49" t="inlineStr">
+        <is>
+          <t>2023</t>
+        </is>
+      </c>
+      <c r="C49" s="87" t="n">
+        <v>4220000</v>
+      </c>
+      <c r="D49" s="49" t="inlineStr">
+        <is>
+          <t>SEK p.a.</t>
+        </is>
+      </c>
+      <c r="E49" s="49" t="inlineStr"/>
+      <c r="F49" s="49" t="inlineStr">
+        <is>
+          <t>https://www.affarsvarlden.se/artikel/affarsjuristerna-om-trenden-pe-bolagen-kommer-vara-motorn</t>
+        </is>
+      </c>
+    </row>
+    <row r="50">
+      <c r="A50" s="49" t="inlineStr">
+        <is>
+          <t>Denmark: Kammeradvokaten state agreement, partner</t>
+        </is>
+      </c>
+      <c r="B50" s="49" t="inlineStr">
+        <is>
+          <t>From Jan-2024</t>
+        </is>
+      </c>
+      <c r="C50" s="87" t="n">
+        <v>2790</v>
+      </c>
+      <c r="D50" s="49" t="inlineStr">
+        <is>
+          <t>DKK</t>
+        </is>
+      </c>
+      <c r="E50" s="49" t="inlineStr">
+        <is>
+          <t>Advokat &gt;3 yrs 2,263; &lt;3 yrs 1,891; fuldmægtig 1,395 (snippet only)</t>
+        </is>
+      </c>
+      <c r="F50" s="49" t="inlineStr">
+        <is>
+          <t>https://ft.dk/samling/20241/almdel/reu/bilag/88/2953293.pdf</t>
+        </is>
+      </c>
+    </row>
+    <row r="51">
+      <c r="A51" s="49" t="inlineStr">
+        <is>
+          <t>Norway: public legal-aid rate (salærsats)</t>
+        </is>
+      </c>
+      <c r="B51" s="49" t="inlineStr">
+        <is>
+          <t>2026</t>
+        </is>
+      </c>
+      <c r="C51" s="87" t="n">
+        <v>1375</v>
+      </c>
+      <c r="D51" s="49" t="inlineStr">
+        <is>
+          <t>NOK</t>
+        </is>
+      </c>
+      <c r="E51" s="49" t="inlineStr">
+        <is>
+          <t>2025: NOK 1,315</t>
+        </is>
+      </c>
+      <c r="F51" s="49" t="inlineStr">
+        <is>
+          <t>https://www.advokatforeningen.no/contentassets/770460b5483c4bd0acb76ff98d2ad3fa/vedlegg-1--salarradets-anbefaling-for-2026.pdf</t>
+        </is>
+      </c>
+    </row>
+    <row r="52">
+      <c r="A52" s="49" t="inlineStr">
+        <is>
+          <t>UK top-10 firms average hourly rate</t>
+        </is>
+      </c>
+      <c r="B52" s="49" t="inlineStr">
+        <is>
+          <t>2024</t>
+        </is>
+      </c>
+      <c r="C52" s="87" t="n">
+        <v>449</v>
+      </c>
+      <c r="D52" s="49" t="inlineStr">
+        <is>
+          <t>GBP</t>
+        </is>
+      </c>
+      <c r="E52" s="49" t="inlineStr">
+        <is>
+          <t>2019: GBP 321; firms 11-25: GBP 325 (PwC, snippet only)</t>
+        </is>
+      </c>
+      <c r="F52" s="49" t="inlineStr">
+        <is>
+          <t>https://www.legalcheek.com/2025/04/the-2000-per-hour-solicitor</t>
+        </is>
+      </c>
+    </row>
+    <row r="54">
+      <c r="A54" s="45" t="inlineStr">
+        <is>
+          <t>Gaps: no published rate cards found for Vinge, White &amp; Case, Setterwalls, Lindahl, Gernandt &amp; Danielsson, CMS Wistrand, Cirio, MAQS, Baker McKenzie, Snellman, Foyen, Glimstedt, Eversheds, Fylgia, Hammarskiöld, Magnusson, Kahn Pedersen, Wigge, Kastell, Westerberg or TM &amp; Partners.</t>
+        </is>
+      </c>
+    </row>
+    <row r="55">
+      <c r="A55" s="45" t="inlineStr">
+        <is>
+          <t>Routes to fill: (1) US Chapter 11 fee statements (PACER) for SAS (S.D.N.Y. 22-10925) and Northvolt (S.D. Tex. 24-90577) list per-timekeeper rates for Mannheimer Swartling 2022-25; (2) FOI requests to public buyers (price annexes often withheld); (3) client invoices (e.g. Axo, requested).</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+  <mergeCells count="15">
+    <mergeCell ref="A5:A6"/>
+    <mergeCell ref="O5:O6"/>
+    <mergeCell ref="N5:N6"/>
+    <mergeCell ref="P5:P6"/>
+    <mergeCell ref="Q5:Q6"/>
+    <mergeCell ref="R5:R6"/>
+    <mergeCell ref="J5:K5"/>
+    <mergeCell ref="A2:R2"/>
+    <mergeCell ref="L5:L6"/>
+    <mergeCell ref="F5:G5"/>
+    <mergeCell ref="D5:E5"/>
+    <mergeCell ref="H5:I5"/>
+    <mergeCell ref="M5:M6"/>
+    <mergeCell ref="B5:B6"/>
+    <mergeCell ref="C5:C6"/>
+  </mergeCells>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
 </file>
</xml_diff>

<commit_message>
Add Section E: partner compensation from filed accounts and SCB wage data
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01Tu61bPEQej1E6sErbEFanY
</commit_message>
<xml_diff>
--- a/research/swedish_legal_market.xlsx
+++ b/research/swedish_legal_market.xlsx
@@ -14,6 +14,7 @@
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="B. Practice rankings" sheetId="5" state="visible" r:id="rId5"/>
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="B. Rankings raw" sheetId="6" state="visible" r:id="rId6"/>
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="D. Rate cards" sheetId="7" state="visible" r:id="rId7"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="E. Partner compensation" sheetId="8" state="visible" r:id="rId8"/>
   </sheets>
   <definedNames>
     <definedName name="_xlnm._FilterDatabase" localSheetId="5" hidden="1">'B. Rankings raw'!$A$1:$E$661</definedName>
@@ -24,9 +25,10 @@
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <numFmts count="2">
+  <numFmts count="3">
     <numFmt numFmtId="164" formatCode="0.0"/>
     <numFmt numFmtId="165" formatCode="+0%;-0%"/>
+    <numFmt numFmtId="166" formatCode="#,##0.0"/>
   </numFmts>
   <fonts count="9">
     <font>
@@ -359,7 +361,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="90">
+  <cellXfs count="101">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
@@ -587,6 +589,39 @@
     </xf>
     <xf numFmtId="165" fontId="0" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="166" fontId="0" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="164" fontId="0" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="2" fontId="0" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="7" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="166" fontId="0" fillId="7" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="164" fontId="0" fillId="7" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="2" fontId="0" fillId="7" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="5" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="2" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="3" fontId="0" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="top" wrapText="1"/>
     </xf>
   </cellXfs>
   <cellStyles count="1">
@@ -32117,4 +32152,1453 @@
   </mergeCells>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
+</file>
+
+<file path=xl/worksheets/sheet8.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:P35"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="24" customWidth="1" min="1" max="1"/>
+    <col width="22" customWidth="1" min="2" max="2"/>
+    <col width="12" customWidth="1" min="3" max="3"/>
+    <col width="10" customWidth="1" min="4" max="4"/>
+    <col width="11" customWidth="1" min="5" max="5"/>
+    <col width="11" customWidth="1" min="6" max="6"/>
+    <col width="11" customWidth="1" min="7" max="7"/>
+    <col width="9" customWidth="1" min="8" max="8"/>
+    <col width="22" customWidth="1" min="9" max="9"/>
+    <col width="11" customWidth="1" min="10" max="10"/>
+    <col width="11" customWidth="1" min="11" max="11"/>
+    <col width="13" customWidth="1" min="12" max="12"/>
+    <col width="10" customWidth="1" min="13" max="13"/>
+    <col width="11" customWidth="1" min="14" max="14"/>
+    <col width="10" customWidth="1" min="15" max="15"/>
+    <col width="50" customWidth="1" min="16" max="16"/>
+  </cols>
+  <sheetData>
+    <row r="1">
+      <c r="A1" s="1" t="inlineStr">
+        <is>
+          <t>Section E. Partner compensation: profit pool per partner from filed annual reports</t>
+        </is>
+      </c>
+    </row>
+    <row r="2" ht="75" customHeight="1">
+      <c r="A2" s="2" t="inlineStr">
+        <is>
+          <t>Source: annual reports filed with Bolagsverket, read via allabolag.se (Oct-2026); amounts SEK m. Swedish law firms pay partners mainly through the profit of the firm company (dividends to partners or their holding companies) plus any salary. "Profit pool per partner" = profit before tax (+ disclosed board/CEO salaries, typically partners) / partners: a proxy for AVERAGE equity-partner compensation before personal tax. It understates pay where partners are also on the payroll (salaries are not split out) and overstates local partner pay where profits flow to an international or cross-border partnership (amber rows). Limited partnerships (KB: Gernandt &amp; Danielsson, DLA Piper, Baker McKenzie, CMS Wistrand, Magnusson) do not file public accounts.</t>
+        </is>
+      </c>
+    </row>
+    <row r="4" ht="45" customHeight="1">
+      <c r="A4" s="52" t="inlineStr">
+        <is>
+          <t>Firm</t>
+        </is>
+      </c>
+      <c r="B4" s="52" t="inlineStr">
+        <is>
+          <t>Entities included (org.nr)</t>
+        </is>
+      </c>
+      <c r="C4" s="52" t="inlineStr">
+        <is>
+          <t>FY</t>
+        </is>
+      </c>
+      <c r="D4" s="52" t="inlineStr">
+        <is>
+          <t>Revenue</t>
+        </is>
+      </c>
+      <c r="E4" s="52" t="inlineStr">
+        <is>
+          <t>Profit before tax</t>
+        </is>
+      </c>
+      <c r="F4" s="52" t="inlineStr">
+        <is>
+          <t>Board / CEO salaries</t>
+        </is>
+      </c>
+      <c r="G4" s="52" t="inlineStr">
+        <is>
+          <t>Proposed dividend</t>
+        </is>
+      </c>
+      <c r="H4" s="52" t="inlineStr">
+        <is>
+          <t>Partners</t>
+        </is>
+      </c>
+      <c r="I4" s="52" t="inlineStr">
+        <is>
+          <t>Partner source</t>
+        </is>
+      </c>
+      <c r="J4" s="52" t="inlineStr">
+        <is>
+          <t>Profit pool / partner</t>
+        </is>
+      </c>
+      <c r="K4" s="52" t="inlineStr">
+        <is>
+          <t>Dividend / partner</t>
+        </is>
+      </c>
+      <c r="L4" s="52" t="inlineStr">
+        <is>
+          <t>Illustrative senior partner (1.4x avg)</t>
+        </is>
+      </c>
+      <c r="M4" s="52" t="inlineStr">
+        <is>
+          <t>Employees</t>
+        </is>
+      </c>
+      <c r="N4" s="52" t="inlineStr">
+        <is>
+          <t>Staff salaries / employee</t>
+        </is>
+      </c>
+      <c r="O4" s="52" t="inlineStr">
+        <is>
+          <t>Reliability</t>
+        </is>
+      </c>
+      <c r="P4" s="52" t="inlineStr">
+        <is>
+          <t>Notes</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" s="49" t="inlineStr">
+        <is>
+          <t>Mannheimer Swartling</t>
+        </is>
+      </c>
+      <c r="B5" s="49" t="inlineStr">
+        <is>
+          <t>5563994499</t>
+        </is>
+      </c>
+      <c r="C5" s="90" t="inlineStr">
+        <is>
+          <t>2025</t>
+        </is>
+      </c>
+      <c r="D5" s="91" t="n">
+        <v>2002.2</v>
+      </c>
+      <c r="E5" s="91" t="n">
+        <v>797.4</v>
+      </c>
+      <c r="F5" s="91" t="n"/>
+      <c r="G5" s="91" t="n">
+        <v>617</v>
+      </c>
+      <c r="H5" s="90" t="n">
+        <v>92</v>
+      </c>
+      <c r="I5" s="49" t="inlineStr">
+        <is>
+          <t>DJ via Realtid (dividend split)</t>
+        </is>
+      </c>
+      <c r="J5" s="92">
+        <f>(E5+N(F5))/H5</f>
+        <v/>
+      </c>
+      <c r="K5" s="92">
+        <f>G5/H5</f>
+        <v/>
+      </c>
+      <c r="L5" s="92">
+        <f>J5*1.4</f>
+        <v/>
+      </c>
+      <c r="M5" s="90" t="n">
+        <v>649</v>
+      </c>
+      <c r="N5" s="93">
+        <f>496.0/M5</f>
+        <v/>
+      </c>
+      <c r="O5" s="49" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
+      <c r="P5" s="49" t="inlineStr">
+        <is>
+          <t>Pure lockstep. Dividend SEK 617m per Dagens Juridik/Realtid (allabolag shows none). 2024: PBT 789.6, dividend 582.</t>
+        </is>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" s="49" t="inlineStr">
+        <is>
+          <t>Vinge</t>
+        </is>
+      </c>
+      <c r="B6" s="49" t="inlineStr">
+        <is>
+          <t>5566907100, 5566866108, 5566886551</t>
+        </is>
+      </c>
+      <c r="C6" s="90" t="inlineStr">
+        <is>
+          <t>2025</t>
+        </is>
+      </c>
+      <c r="D6" s="91" t="n">
+        <v>1446.6</v>
+      </c>
+      <c r="E6" s="91" t="n">
+        <v>445.3</v>
+      </c>
+      <c r="F6" s="91" t="n">
+        <v>52.3</v>
+      </c>
+      <c r="G6" s="91" t="n">
+        <v>294</v>
+      </c>
+      <c r="H6" s="90" t="n">
+        <v>71</v>
+      </c>
+      <c r="I6" s="49" t="inlineStr">
+        <is>
+          <t>Firm website, Oct-26</t>
+        </is>
+      </c>
+      <c r="J6" s="92">
+        <f>(E6+N(F6))/H6</f>
+        <v/>
+      </c>
+      <c r="K6" s="92">
+        <f>G6/H6</f>
+        <v/>
+      </c>
+      <c r="L6" s="92">
+        <f>J6*1.4</f>
+        <v/>
+      </c>
+      <c r="M6" s="90" t="n">
+        <v>529</v>
+      </c>
+      <c r="N6" s="93">
+        <f>775.9/M6</f>
+        <v/>
+      </c>
+      <c r="O6" s="49" t="inlineStr">
+        <is>
+          <t>Medium</t>
+        </is>
+      </c>
+      <c r="P6" s="49" t="inlineStr">
+        <is>
+          <t>Stockholm + Malmö + Göteborg ABs. Realtid: Stockholm dividend 273m to 49 partners (SEK 5.5m each), Malmö 32m to 14. Partners may also draw salary (not split out).</t>
+        </is>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" s="69" t="inlineStr">
+        <is>
+          <t>Roschier (Sweden)</t>
+        </is>
+      </c>
+      <c r="B7" s="69" t="inlineStr">
+        <is>
+          <t>5566865670</t>
+        </is>
+      </c>
+      <c r="C7" s="94" t="inlineStr">
+        <is>
+          <t>FY Jun25-May26</t>
+        </is>
+      </c>
+      <c r="D7" s="95" t="n">
+        <v>1304.1</v>
+      </c>
+      <c r="E7" s="95" t="n">
+        <v>646.4</v>
+      </c>
+      <c r="F7" s="95" t="n">
+        <v>6</v>
+      </c>
+      <c r="G7" s="95" t="n">
+        <v>508.9</v>
+      </c>
+      <c r="H7" s="94" t="n">
+        <v>26</v>
+      </c>
+      <c r="I7" s="69" t="inlineStr">
+        <is>
+          <t>Firm website (Stockholm), Oct-26</t>
+        </is>
+      </c>
+      <c r="J7" s="96">
+        <f>(E7+N(F7))/H7</f>
+        <v/>
+      </c>
+      <c r="K7" s="96">
+        <f>G7/H7</f>
+        <v/>
+      </c>
+      <c r="L7" s="96">
+        <f>J7*1.4</f>
+        <v/>
+      </c>
+      <c r="M7" s="94" t="n">
+        <v>220</v>
+      </c>
+      <c r="N7" s="97">
+        <f>234.9/M7</f>
+        <v/>
+      </c>
+      <c r="O7" s="69" t="inlineStr">
+        <is>
+          <t>Low</t>
+        </is>
+      </c>
+      <c r="P7" s="69" t="inlineStr">
+        <is>
+          <t>Profit likely pooled with Finnish practice (group 52 partners): SEK 12.4m per group partner on the same basis.</t>
+        </is>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" s="69" t="inlineStr">
+        <is>
+          <t>White &amp; Case (Stockholm)</t>
+        </is>
+      </c>
+      <c r="B8" s="69" t="inlineStr">
+        <is>
+          <t>5562323922</t>
+        </is>
+      </c>
+      <c r="C8" s="94" t="inlineStr">
+        <is>
+          <t>2025</t>
+        </is>
+      </c>
+      <c r="D8" s="95" t="n">
+        <v>1107.8</v>
+      </c>
+      <c r="E8" s="95" t="n">
+        <v>239</v>
+      </c>
+      <c r="F8" s="95" t="n">
+        <v>0.8</v>
+      </c>
+      <c r="G8" s="95" t="n">
+        <v>198.1</v>
+      </c>
+      <c r="H8" s="94" t="n">
+        <v>16</v>
+      </c>
+      <c r="I8" s="69" t="inlineStr">
+        <is>
+          <t>Implied (DJ)</t>
+        </is>
+      </c>
+      <c r="J8" s="96">
+        <f>(E8+N(F8))/H8</f>
+        <v/>
+      </c>
+      <c r="K8" s="96">
+        <f>G8/H8</f>
+        <v/>
+      </c>
+      <c r="L8" s="96">
+        <f>J8*1.4</f>
+        <v/>
+      </c>
+      <c r="M8" s="94" t="n">
+        <v>120</v>
+      </c>
+      <c r="N8" s="97">
+        <f>105.3/M8</f>
+        <v/>
+      </c>
+      <c r="O8" s="69" t="inlineStr">
+        <is>
+          <t>Low</t>
+        </is>
+      </c>
+      <c r="P8" s="69" t="inlineStr">
+        <is>
+          <t>Global LLP: entity profit likely flows to the international partnership, not equal to local partner pay.</t>
+        </is>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" s="49" t="inlineStr">
+        <is>
+          <t>Setterwalls</t>
+        </is>
+      </c>
+      <c r="B9" s="49" t="inlineStr">
+        <is>
+          <t>5568743230, 5565943221</t>
+        </is>
+      </c>
+      <c r="C9" s="90" t="inlineStr">
+        <is>
+          <t>2025</t>
+        </is>
+      </c>
+      <c r="D9" s="91" t="n">
+        <v>705</v>
+      </c>
+      <c r="E9" s="91" t="n">
+        <v>272.6</v>
+      </c>
+      <c r="F9" s="91" t="n"/>
+      <c r="G9" s="91" t="n">
+        <v>215.2</v>
+      </c>
+      <c r="H9" s="90" t="n">
+        <v>38</v>
+      </c>
+      <c r="I9" s="49" t="inlineStr">
+        <is>
+          <t>Firm website, Oct-26</t>
+        </is>
+      </c>
+      <c r="J9" s="92">
+        <f>(E9+N(F9))/H9</f>
+        <v/>
+      </c>
+      <c r="K9" s="92">
+        <f>G9/H9</f>
+        <v/>
+      </c>
+      <c r="L9" s="92">
+        <f>J9*1.4</f>
+        <v/>
+      </c>
+      <c r="M9" s="90" t="n">
+        <v>217</v>
+      </c>
+      <c r="N9" s="93">
+        <f>193.6/M9</f>
+        <v/>
+      </c>
+      <c r="O9" s="49" t="inlineStr">
+        <is>
+          <t>Medium</t>
+        </is>
+      </c>
+      <c r="P9" s="49" t="inlineStr">
+        <is>
+          <t>Stockholm + Göteborg operating ABs (parent AB is a pass-through). Malmö office excluded (left Sep-26).</t>
+        </is>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" s="49" t="inlineStr">
+        <is>
+          <t>Cederquist</t>
+        </is>
+      </c>
+      <c r="B10" s="49" t="inlineStr">
+        <is>
+          <t>5569891277</t>
+        </is>
+      </c>
+      <c r="C10" s="90" t="inlineStr">
+        <is>
+          <t>2025</t>
+        </is>
+      </c>
+      <c r="D10" s="91" t="n"/>
+      <c r="E10" s="91" t="n">
+        <v>134.1</v>
+      </c>
+      <c r="F10" s="91" t="n">
+        <v>0</v>
+      </c>
+      <c r="G10" s="91" t="n">
+        <v>105.1</v>
+      </c>
+      <c r="H10" s="90" t="n">
+        <v>26</v>
+      </c>
+      <c r="I10" s="49" t="inlineStr">
+        <is>
+          <t>Legal 500 (firm-supplied)</t>
+        </is>
+      </c>
+      <c r="J10" s="92">
+        <f>(E10+N(F10))/H10</f>
+        <v/>
+      </c>
+      <c r="K10" s="92">
+        <f>G10/H10</f>
+        <v/>
+      </c>
+      <c r="L10" s="92">
+        <f>J10*1.4</f>
+        <v/>
+      </c>
+      <c r="M10" s="90" t="n"/>
+      <c r="N10" s="98" t="n"/>
+      <c r="O10" s="49" t="inlineStr">
+        <is>
+          <t>Low</t>
+        </is>
+      </c>
+      <c r="P10" s="49" t="inlineStr">
+        <is>
+          <t>AB is a partner in the operating KB (profit share); may not capture all partners.</t>
+        </is>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" s="49" t="inlineStr">
+        <is>
+          <t>Cirio</t>
+        </is>
+      </c>
+      <c r="B11" s="49" t="inlineStr">
+        <is>
+          <t>5569530008</t>
+        </is>
+      </c>
+      <c r="C11" s="90" t="inlineStr">
+        <is>
+          <t>2025</t>
+        </is>
+      </c>
+      <c r="D11" s="91" t="n">
+        <v>430.6</v>
+      </c>
+      <c r="E11" s="91" t="n">
+        <v>124.8</v>
+      </c>
+      <c r="F11" s="91" t="n">
+        <v>6.5</v>
+      </c>
+      <c r="G11" s="91" t="n">
+        <v>98</v>
+      </c>
+      <c r="H11" s="90" t="n">
+        <v>27</v>
+      </c>
+      <c r="I11" s="49" t="inlineStr">
+        <is>
+          <t>Legal 500 (firm-supplied)</t>
+        </is>
+      </c>
+      <c r="J11" s="92">
+        <f>(E11+N(F11))/H11</f>
+        <v/>
+      </c>
+      <c r="K11" s="92">
+        <f>G11/H11</f>
+        <v/>
+      </c>
+      <c r="L11" s="92">
+        <f>J11*1.4</f>
+        <v/>
+      </c>
+      <c r="M11" s="90" t="n">
+        <v>127</v>
+      </c>
+      <c r="N11" s="93">
+        <f>121.7/M11</f>
+        <v/>
+      </c>
+      <c r="O11" s="49" t="inlineStr">
+        <is>
+          <t>Medium</t>
+        </is>
+      </c>
+      <c r="P11" s="49" t="inlineStr">
+        <is>
+          <t>2024: PBT 122.9, dividend 96.7.</t>
+        </is>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" s="49" t="inlineStr">
+        <is>
+          <t>Snellman (Sweden)</t>
+        </is>
+      </c>
+      <c r="B12" s="49" t="inlineStr">
+        <is>
+          <t>5567572101</t>
+        </is>
+      </c>
+      <c r="C12" s="90" t="inlineStr">
+        <is>
+          <t>2025</t>
+        </is>
+      </c>
+      <c r="D12" s="91" t="n">
+        <v>279.4</v>
+      </c>
+      <c r="E12" s="91" t="n">
+        <v>88.8</v>
+      </c>
+      <c r="F12" s="91" t="n">
+        <v>4.2</v>
+      </c>
+      <c r="G12" s="91" t="n">
+        <v>74.3</v>
+      </c>
+      <c r="H12" s="90" t="n">
+        <v>17</v>
+      </c>
+      <c r="I12" s="49" t="inlineStr">
+        <is>
+          <t>Legal 500 (stale)</t>
+        </is>
+      </c>
+      <c r="J12" s="92">
+        <f>(E12+N(F12))/H12</f>
+        <v/>
+      </c>
+      <c r="K12" s="92">
+        <f>G12/H12</f>
+        <v/>
+      </c>
+      <c r="L12" s="92">
+        <f>J12*1.4</f>
+        <v/>
+      </c>
+      <c r="M12" s="90" t="n">
+        <v>107</v>
+      </c>
+      <c r="N12" s="93">
+        <f>76.3/M12</f>
+        <v/>
+      </c>
+      <c r="O12" s="49" t="inlineStr">
+        <is>
+          <t>Low</t>
+        </is>
+      </c>
+      <c r="P12" s="49" t="inlineStr">
+        <is>
+          <t>Partner count unverified.</t>
+        </is>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" s="49" t="inlineStr">
+        <is>
+          <t>Delphi</t>
+        </is>
+      </c>
+      <c r="B13" s="49" t="inlineStr">
+        <is>
+          <t>5566623293, 5566438163, 5563262913</t>
+        </is>
+      </c>
+      <c r="C13" s="90" t="inlineStr">
+        <is>
+          <t>2025</t>
+        </is>
+      </c>
+      <c r="D13" s="91" t="n">
+        <v>355.8</v>
+      </c>
+      <c r="E13" s="91" t="n">
+        <v>82.90000000000001</v>
+      </c>
+      <c r="F13" s="91" t="n"/>
+      <c r="G13" s="91" t="n">
+        <v>49</v>
+      </c>
+      <c r="H13" s="90" t="n">
+        <v>49</v>
+      </c>
+      <c r="I13" s="49" t="inlineStr">
+        <is>
+          <t>Chambers (firm-supplied)</t>
+        </is>
+      </c>
+      <c r="J13" s="92">
+        <f>(E13+N(F13))/H13</f>
+        <v/>
+      </c>
+      <c r="K13" s="92">
+        <f>G13/H13</f>
+        <v/>
+      </c>
+      <c r="L13" s="92">
+        <f>J13*1.4</f>
+        <v/>
+      </c>
+      <c r="M13" s="90" t="n">
+        <v>126</v>
+      </c>
+      <c r="N13" s="93">
+        <f>70.9/M13</f>
+        <v/>
+      </c>
+      <c r="O13" s="49" t="inlineStr">
+        <is>
+          <t>Low</t>
+        </is>
+      </c>
+      <c r="P13" s="49" t="inlineStr">
+        <is>
+          <t>Stockholm, Göteborg, Malmö ABs only (Östergötland missing). Low PBT relative to revenue suggests partners are paid largely via salary.</t>
+        </is>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" s="49" t="inlineStr">
+        <is>
+          <t>MAQS</t>
+        </is>
+      </c>
+      <c r="B14" s="49" t="inlineStr">
+        <is>
+          <t>5569507733</t>
+        </is>
+      </c>
+      <c r="C14" s="90" t="inlineStr">
+        <is>
+          <t>2025</t>
+        </is>
+      </c>
+      <c r="D14" s="91" t="n">
+        <v>324.3</v>
+      </c>
+      <c r="E14" s="91" t="n">
+        <v>96.40000000000001</v>
+      </c>
+      <c r="F14" s="91" t="n"/>
+      <c r="G14" s="91" t="n">
+        <v>0</v>
+      </c>
+      <c r="H14" s="90" t="n">
+        <v>48</v>
+      </c>
+      <c r="I14" s="49" t="inlineStr">
+        <is>
+          <t>Firm website, Oct-26</t>
+        </is>
+      </c>
+      <c r="J14" s="92">
+        <f>(E14+N(F14))/H14</f>
+        <v/>
+      </c>
+      <c r="K14" s="92">
+        <f>G14/H14</f>
+        <v/>
+      </c>
+      <c r="L14" s="92">
+        <f>J14*1.4</f>
+        <v/>
+      </c>
+      <c r="M14" s="90" t="n">
+        <v>121</v>
+      </c>
+      <c r="N14" s="93">
+        <f>97.2/M14</f>
+        <v/>
+      </c>
+      <c r="O14" s="49" t="inlineStr">
+        <is>
+          <t>Low</t>
+        </is>
+      </c>
+      <c r="P14" s="49" t="inlineStr">
+        <is>
+          <t>Main AB only (~78% of Afv revenue). 2024 dividend 73.7. Partners likely partly salaried.</t>
+        </is>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" s="49" t="inlineStr">
+        <is>
+          <t>Hammarskiöld</t>
+        </is>
+      </c>
+      <c r="B15" s="49" t="inlineStr">
+        <is>
+          <t>5565471637</t>
+        </is>
+      </c>
+      <c r="C15" s="90" t="inlineStr">
+        <is>
+          <t>2025</t>
+        </is>
+      </c>
+      <c r="D15" s="91" t="n">
+        <v>178.3</v>
+      </c>
+      <c r="E15" s="91" t="n">
+        <v>49.8</v>
+      </c>
+      <c r="F15" s="91" t="n"/>
+      <c r="G15" s="91" t="n">
+        <v>38.4</v>
+      </c>
+      <c r="H15" s="90" t="n"/>
+      <c r="I15" s="49" t="inlineStr"/>
+      <c r="J15" s="98" t="n"/>
+      <c r="K15" s="98" t="n"/>
+      <c r="L15" s="98" t="n"/>
+      <c r="M15" s="90" t="n">
+        <v>63</v>
+      </c>
+      <c r="N15" s="93">
+        <f>58.6/M15</f>
+        <v/>
+      </c>
+      <c r="O15" s="49" t="inlineStr">
+        <is>
+          <t>n/a</t>
+        </is>
+      </c>
+      <c r="P15" s="49" t="inlineStr">
+        <is>
+          <t>Partner count not found.</t>
+        </is>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" s="49" t="inlineStr">
+        <is>
+          <t>Foyen</t>
+        </is>
+      </c>
+      <c r="B16" s="49" t="inlineStr">
+        <is>
+          <t>5565837134</t>
+        </is>
+      </c>
+      <c r="C16" s="90" t="inlineStr">
+        <is>
+          <t>2025</t>
+        </is>
+      </c>
+      <c r="D16" s="91" t="n">
+        <v>172.5</v>
+      </c>
+      <c r="E16" s="91" t="n">
+        <v>46.1</v>
+      </c>
+      <c r="F16" s="91" t="n">
+        <v>6</v>
+      </c>
+      <c r="G16" s="91" t="n">
+        <v>35.9</v>
+      </c>
+      <c r="H16" s="90" t="n">
+        <v>23</v>
+      </c>
+      <c r="I16" s="49" t="inlineStr">
+        <is>
+          <t>Firm website, Oct-26</t>
+        </is>
+      </c>
+      <c r="J16" s="92">
+        <f>(E16+N(F16))/H16</f>
+        <v/>
+      </c>
+      <c r="K16" s="92">
+        <f>G16/H16</f>
+        <v/>
+      </c>
+      <c r="L16" s="92">
+        <f>J16*1.4</f>
+        <v/>
+      </c>
+      <c r="M16" s="90" t="n">
+        <v>104</v>
+      </c>
+      <c r="N16" s="93">
+        <f>72.3/M16</f>
+        <v/>
+      </c>
+      <c r="O16" s="49" t="inlineStr">
+        <is>
+          <t>Medium</t>
+        </is>
+      </c>
+      <c r="P16" s="49" t="inlineStr">
+        <is>
+          <t>Main Swedish AB.</t>
+        </is>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" s="49" t="inlineStr">
+        <is>
+          <t>Moll Wendén</t>
+        </is>
+      </c>
+      <c r="B17" s="49" t="inlineStr">
+        <is>
+          <t>5566487939</t>
+        </is>
+      </c>
+      <c r="C17" s="90" t="inlineStr">
+        <is>
+          <t>2025</t>
+        </is>
+      </c>
+      <c r="D17" s="91" t="n">
+        <v>101.3</v>
+      </c>
+      <c r="E17" s="91" t="n">
+        <v>30.2</v>
+      </c>
+      <c r="F17" s="91" t="n"/>
+      <c r="G17" s="91" t="n">
+        <v>23.8</v>
+      </c>
+      <c r="H17" s="90" t="n">
+        <v>8</v>
+      </c>
+      <c r="I17" s="49" t="inlineStr">
+        <is>
+          <t>Firm website, Oct-26</t>
+        </is>
+      </c>
+      <c r="J17" s="92">
+        <f>(E17+N(F17))/H17</f>
+        <v/>
+      </c>
+      <c r="K17" s="92">
+        <f>G17/H17</f>
+        <v/>
+      </c>
+      <c r="L17" s="92">
+        <f>J17*1.4</f>
+        <v/>
+      </c>
+      <c r="M17" s="90" t="n">
+        <v>44</v>
+      </c>
+      <c r="N17" s="98" t="n"/>
+      <c r="O17" s="49" t="inlineStr">
+        <is>
+          <t>Medium</t>
+        </is>
+      </c>
+      <c r="P17" s="49" t="inlineStr"/>
+    </row>
+    <row r="18">
+      <c r="A18" s="49" t="inlineStr">
+        <is>
+          <t>TM &amp; Partners</t>
+        </is>
+      </c>
+      <c r="B18" s="49" t="inlineStr">
+        <is>
+          <t>5566947163</t>
+        </is>
+      </c>
+      <c r="C18" s="90" t="inlineStr">
+        <is>
+          <t>2025</t>
+        </is>
+      </c>
+      <c r="D18" s="91" t="n">
+        <v>102.5</v>
+      </c>
+      <c r="E18" s="91" t="n">
+        <v>30.1</v>
+      </c>
+      <c r="F18" s="91" t="n">
+        <v>4.6</v>
+      </c>
+      <c r="G18" s="91" t="n">
+        <v>0</v>
+      </c>
+      <c r="H18" s="90" t="n">
+        <v>18</v>
+      </c>
+      <c r="I18" s="49" t="inlineStr">
+        <is>
+          <t>Firm website, Oct-26</t>
+        </is>
+      </c>
+      <c r="J18" s="92">
+        <f>(E18+N(F18))/H18</f>
+        <v/>
+      </c>
+      <c r="K18" s="92">
+        <f>G18/H18</f>
+        <v/>
+      </c>
+      <c r="L18" s="92">
+        <f>J18*1.4</f>
+        <v/>
+      </c>
+      <c r="M18" s="90" t="n">
+        <v>73</v>
+      </c>
+      <c r="N18" s="93">
+        <f>54.2/M18</f>
+        <v/>
+      </c>
+      <c r="O18" s="49" t="inlineStr">
+        <is>
+          <t>Low</t>
+        </is>
+      </c>
+      <c r="P18" s="49" t="inlineStr">
+        <is>
+          <t>Part of AGRD (PE-owned) since 2025; post-deal economics differ.</t>
+        </is>
+      </c>
+    </row>
+    <row r="19">
+      <c r="A19" s="49" t="inlineStr">
+        <is>
+          <t>Westerberg &amp; Partners</t>
+        </is>
+      </c>
+      <c r="B19" s="49" t="inlineStr">
+        <is>
+          <t>5591623268</t>
+        </is>
+      </c>
+      <c r="C19" s="90" t="inlineStr">
+        <is>
+          <t>2025</t>
+        </is>
+      </c>
+      <c r="D19" s="91" t="n">
+        <v>106.5</v>
+      </c>
+      <c r="E19" s="91" t="n">
+        <v>24.7</v>
+      </c>
+      <c r="F19" s="91" t="n">
+        <v>5</v>
+      </c>
+      <c r="G19" s="91" t="n">
+        <v>19.3</v>
+      </c>
+      <c r="H19" s="90" t="n">
+        <v>12</v>
+      </c>
+      <c r="I19" s="49" t="inlineStr">
+        <is>
+          <t>Firm website, Oct-26</t>
+        </is>
+      </c>
+      <c r="J19" s="92">
+        <f>(E19+N(F19))/H19</f>
+        <v/>
+      </c>
+      <c r="K19" s="92">
+        <f>G19/H19</f>
+        <v/>
+      </c>
+      <c r="L19" s="92">
+        <f>J19*1.4</f>
+        <v/>
+      </c>
+      <c r="M19" s="90" t="n">
+        <v>35</v>
+      </c>
+      <c r="N19" s="93">
+        <f>22.7/M19</f>
+        <v/>
+      </c>
+      <c r="O19" s="49" t="inlineStr">
+        <is>
+          <t>Medium</t>
+        </is>
+      </c>
+      <c r="P19" s="49" t="inlineStr"/>
+    </row>
+    <row r="20">
+      <c r="A20" s="49" t="inlineStr">
+        <is>
+          <t>Harvest</t>
+        </is>
+      </c>
+      <c r="B20" s="49" t="inlineStr">
+        <is>
+          <t>5590700224</t>
+        </is>
+      </c>
+      <c r="C20" s="90" t="inlineStr">
+        <is>
+          <t>2025</t>
+        </is>
+      </c>
+      <c r="D20" s="91" t="n">
+        <v>82.3</v>
+      </c>
+      <c r="E20" s="91" t="n">
+        <v>22.9</v>
+      </c>
+      <c r="F20" s="91" t="n"/>
+      <c r="G20" s="91" t="n">
+        <v>17.8</v>
+      </c>
+      <c r="H20" s="90" t="n">
+        <v>5</v>
+      </c>
+      <c r="I20" s="49" t="inlineStr">
+        <is>
+          <t>Firm website, Oct-26</t>
+        </is>
+      </c>
+      <c r="J20" s="92">
+        <f>(E20+N(F20))/H20</f>
+        <v/>
+      </c>
+      <c r="K20" s="92">
+        <f>G20/H20</f>
+        <v/>
+      </c>
+      <c r="L20" s="92">
+        <f>J20*1.4</f>
+        <v/>
+      </c>
+      <c r="M20" s="90" t="n">
+        <v>27</v>
+      </c>
+      <c r="N20" s="98" t="n"/>
+      <c r="O20" s="49" t="inlineStr">
+        <is>
+          <t>Medium</t>
+        </is>
+      </c>
+      <c r="P20" s="49" t="inlineStr"/>
+    </row>
+    <row r="21">
+      <c r="A21" s="49" t="inlineStr">
+        <is>
+          <t>Synch</t>
+        </is>
+      </c>
+      <c r="B21" s="49" t="inlineStr">
+        <is>
+          <t>5569556656</t>
+        </is>
+      </c>
+      <c r="C21" s="90" t="inlineStr">
+        <is>
+          <t>2025</t>
+        </is>
+      </c>
+      <c r="D21" s="91" t="n">
+        <v>81.40000000000001</v>
+      </c>
+      <c r="E21" s="91" t="n">
+        <v>20.3</v>
+      </c>
+      <c r="F21" s="91" t="n"/>
+      <c r="G21" s="91" t="n">
+        <v>0</v>
+      </c>
+      <c r="H21" s="90" t="n">
+        <v>9</v>
+      </c>
+      <c r="I21" s="49" t="inlineStr">
+        <is>
+          <t>Firm website, Oct-26</t>
+        </is>
+      </c>
+      <c r="J21" s="92">
+        <f>(E21+N(F21))/H21</f>
+        <v/>
+      </c>
+      <c r="K21" s="92">
+        <f>G21/H21</f>
+        <v/>
+      </c>
+      <c r="L21" s="92">
+        <f>J21*1.4</f>
+        <v/>
+      </c>
+      <c r="M21" s="90" t="n">
+        <v>38</v>
+      </c>
+      <c r="N21" s="98" t="n"/>
+      <c r="O21" s="49" t="inlineStr">
+        <is>
+          <t>Low</t>
+        </is>
+      </c>
+      <c r="P21" s="49" t="inlineStr">
+        <is>
+          <t>Part of AGRD (PE-owned) since 2025.</t>
+        </is>
+      </c>
+    </row>
+    <row r="22">
+      <c r="A22" s="49" t="inlineStr">
+        <is>
+          <t>Kastell</t>
+        </is>
+      </c>
+      <c r="B22" s="49" t="inlineStr">
+        <is>
+          <t>5568116494</t>
+        </is>
+      </c>
+      <c r="C22" s="90" t="inlineStr">
+        <is>
+          <t>2025</t>
+        </is>
+      </c>
+      <c r="D22" s="91" t="n">
+        <v>79.59999999999999</v>
+      </c>
+      <c r="E22" s="91" t="n">
+        <v>16.9</v>
+      </c>
+      <c r="F22" s="91" t="n"/>
+      <c r="G22" s="91" t="n">
+        <v>15.2</v>
+      </c>
+      <c r="H22" s="90" t="n">
+        <v>9</v>
+      </c>
+      <c r="I22" s="49" t="inlineStr">
+        <is>
+          <t>Firm website, Oct-26</t>
+        </is>
+      </c>
+      <c r="J22" s="92">
+        <f>(E22+N(F22))/H22</f>
+        <v/>
+      </c>
+      <c r="K22" s="92">
+        <f>G22/H22</f>
+        <v/>
+      </c>
+      <c r="L22" s="92">
+        <f>J22*1.4</f>
+        <v/>
+      </c>
+      <c r="M22" s="90" t="n">
+        <v>21</v>
+      </c>
+      <c r="N22" s="98" t="n"/>
+      <c r="O22" s="49" t="inlineStr">
+        <is>
+          <t>Medium</t>
+        </is>
+      </c>
+      <c r="P22" s="49" t="inlineStr"/>
+    </row>
+    <row r="23">
+      <c r="A23" s="49" t="inlineStr">
+        <is>
+          <t>Eversheds Sutherland</t>
+        </is>
+      </c>
+      <c r="B23" s="49" t="inlineStr">
+        <is>
+          <t>5568782774</t>
+        </is>
+      </c>
+      <c r="C23" s="90" t="inlineStr">
+        <is>
+          <t>2025</t>
+        </is>
+      </c>
+      <c r="D23" s="91" t="n">
+        <v>165.5</v>
+      </c>
+      <c r="E23" s="91" t="n">
+        <v>21.1</v>
+      </c>
+      <c r="F23" s="91" t="n"/>
+      <c r="G23" s="91" t="n">
+        <v>16.5</v>
+      </c>
+      <c r="H23" s="90" t="n"/>
+      <c r="I23" s="49" t="inlineStr"/>
+      <c r="J23" s="98" t="n"/>
+      <c r="K23" s="98" t="n"/>
+      <c r="L23" s="98" t="n"/>
+      <c r="M23" s="90" t="n">
+        <v>59</v>
+      </c>
+      <c r="N23" s="93">
+        <f>49.4/M23</f>
+        <v/>
+      </c>
+      <c r="O23" s="49" t="inlineStr">
+        <is>
+          <t>n/a</t>
+        </is>
+      </c>
+      <c r="P23" s="49" t="inlineStr">
+        <is>
+          <t>Partner count not found.</t>
+        </is>
+      </c>
+    </row>
+    <row r="25">
+      <c r="A25" s="45" t="inlineStr">
+        <is>
+          <t>Reading the table: e.g. Mannheimer Swartling SEK 797m profit before tax / 92 partners = SEK 8.7m average per partner before corporate and personal tax; dividend SEK 6.7m per partner (after 20.6% corporate tax).</t>
+        </is>
+      </c>
+    </row>
+    <row r="26">
+      <c r="A26" s="45" t="inlineStr">
+        <is>
+          <t>Senior partner: Mannheimer Swartling operates a pure lockstep (profit shares rise with seniority to a plateau). Individual point scales are not published. The illustrative column assumes a top-of-ladder partner earns ~1.4x the average (consistent with a 1:2.5 entry-to-top lockstep ladder); this is an assumption, not reported data.</t>
+        </is>
+      </c>
+    </row>
+    <row r="27">
+      <c r="A27" s="45" t="inlineStr">
+        <is>
+          <t>Tax treatment: partners owning &lt;4% of the firm company have nearly all of their profit share taxed as salary income (rule since 2014, per Advokaten), so profit-pool figures are pre-personal-tax.</t>
+        </is>
+      </c>
+    </row>
+    <row r="28">
+      <c r="A28" s="45" t="inlineStr">
+        <is>
+          <t>Individual taxed income is public in Sweden (Skatteverket), but compiling named individuals' income is personal data processing under GDPR; this sheet uses firm-level filed accounts only.</t>
+        </is>
+      </c>
+    </row>
+    <row r="29">
+      <c r="A29" s="45" t="inlineStr">
+        <is>
+          <t>Staff salaries / employee = "Löner övriga" / average employees (SEK m): an average across associates and support staff (and partners where on payroll).</t>
+        </is>
+      </c>
+    </row>
+    <row r="31">
+      <c r="A31" s="47" t="inlineStr">
+        <is>
+          <t>Context: SCB salary statistics, private-sector employees, monthly salary (SEK), 2025</t>
+        </is>
+      </c>
+    </row>
+    <row r="32">
+      <c r="A32" s="99" t="inlineStr">
+        <is>
+          <t>Occupation (SSYK 2012)</t>
+        </is>
+      </c>
+      <c r="B32" s="99" t="inlineStr">
+        <is>
+          <t>Mean</t>
+        </is>
+      </c>
+      <c r="C32" s="99" t="inlineStr">
+        <is>
+          <t>P10</t>
+        </is>
+      </c>
+      <c r="D32" s="99" t="inlineStr">
+        <is>
+          <t>P25</t>
+        </is>
+      </c>
+      <c r="E32" s="99" t="inlineStr">
+        <is>
+          <t>Median</t>
+        </is>
+      </c>
+      <c r="F32" s="99" t="inlineStr">
+        <is>
+          <t>P75</t>
+        </is>
+      </c>
+      <c r="G32" s="99" t="inlineStr">
+        <is>
+          <t>P90</t>
+        </is>
+      </c>
+      <c r="H32" s="99" t="inlineStr">
+        <is>
+          <t>P90 annualised (x12)</t>
+        </is>
+      </c>
+    </row>
+    <row r="33">
+      <c r="A33" s="6" t="inlineStr">
+        <is>
+          <t>2611 Advokater</t>
+        </is>
+      </c>
+      <c r="B33" s="100" t="n">
+        <v>70200</v>
+      </c>
+      <c r="C33" s="100" t="n">
+        <v>47200</v>
+      </c>
+      <c r="D33" s="100" t="n">
+        <v>54800</v>
+      </c>
+      <c r="E33" s="100" t="n">
+        <v>66000</v>
+      </c>
+      <c r="F33" s="100" t="n">
+        <v>80000</v>
+      </c>
+      <c r="G33" s="100" t="n">
+        <v>100000</v>
+      </c>
+      <c r="H33" s="100">
+        <f>G33*12</f>
+        <v/>
+      </c>
+    </row>
+    <row r="34">
+      <c r="A34" s="6" t="inlineStr">
+        <is>
+          <t>2614 Business &amp; corporate lawyers</t>
+        </is>
+      </c>
+      <c r="B34" s="100" t="n">
+        <v>73000</v>
+      </c>
+      <c r="C34" s="100" t="n">
+        <v>40700</v>
+      </c>
+      <c r="D34" s="100" t="n">
+        <v>50000</v>
+      </c>
+      <c r="E34" s="100" t="n">
+        <v>67800</v>
+      </c>
+      <c r="F34" s="100" t="n">
+        <v>86400</v>
+      </c>
+      <c r="G34" s="100" t="n">
+        <v>109100</v>
+      </c>
+      <c r="H34" s="100">
+        <f>G34*12</f>
+        <v/>
+      </c>
+    </row>
+    <row r="35">
+      <c r="A35" s="45" t="inlineStr">
+        <is>
+          <t>SCB table AM0110A/LoneSpridSektYrk4AN (salaried employees only; equity partners paid via profit shares are not captured). 2611 mean rose from 58,600 (2023) to 70,200 (2025).</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+  <mergeCells count="1">
+    <mergeCell ref="A2:P2"/>
+  </mergeCells>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
 </file>
</xml_diff>

<commit_message>
Add Section C: top-30 benchmarking with revenue per partner/employee/lawyer and leverage ratios
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01Tu61bPEQej1E6sErbEFanY
</commit_message>
<xml_diff>
--- a/research/swedish_legal_market.xlsx
+++ b/research/swedish_legal_market.xlsx
@@ -13,8 +13,9 @@
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="A. Niche firms" sheetId="4" state="visible" r:id="rId4"/>
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="B. Practice rankings" sheetId="5" state="visible" r:id="rId5"/>
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="B. Rankings raw" sheetId="6" state="visible" r:id="rId6"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="D. Rate cards" sheetId="7" state="visible" r:id="rId7"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="E. Partner compensation" sheetId="8" state="visible" r:id="rId8"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="C. Benchmarking" sheetId="7" state="visible" r:id="rId7"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="D. Rate cards" sheetId="8" state="visible" r:id="rId8"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="E. Partner compensation" sheetId="9" state="visible" r:id="rId9"/>
   </sheets>
   <definedNames>
     <definedName name="_xlnm._FilterDatabase" localSheetId="5" hidden="1">'B. Rankings raw'!$A$1:$E$661</definedName>
@@ -361,7 +362,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="101">
+  <cellXfs count="105">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
@@ -621,6 +622,18 @@
       <alignment horizontal="center" vertical="top" wrapText="1"/>
     </xf>
     <xf numFmtId="3" fontId="0" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="9" fontId="0" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="164" fontId="5" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="2" fontId="5" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="9" fontId="5" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="top" wrapText="1"/>
     </xf>
   </cellXfs>
@@ -30397,6 +30410,2170 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
+  <dimension ref="A1:R43"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="5" customWidth="1" min="1" max="1"/>
+    <col width="26" customWidth="1" min="2" max="2"/>
+    <col width="11" customWidth="1" min="3" max="3"/>
+    <col width="10" customWidth="1" min="4" max="4"/>
+    <col width="9" customWidth="1" min="5" max="5"/>
+    <col width="10" customWidth="1" min="6" max="6"/>
+    <col width="26" customWidth="1" min="7" max="7"/>
+    <col width="9" customWidth="1" min="8" max="8"/>
+    <col width="10" customWidth="1" min="9" max="9"/>
+    <col width="10" customWidth="1" min="10" max="10"/>
+    <col width="30" customWidth="1" min="11" max="11"/>
+    <col width="10" customWidth="1" min="12" max="12"/>
+    <col width="10" customWidth="1" min="13" max="13"/>
+    <col width="10" customWidth="1" min="14" max="14"/>
+    <col width="12" customWidth="1" min="15" max="15"/>
+    <col width="12" customWidth="1" min="16" max="16"/>
+    <col width="10" customWidth="1" min="17" max="17"/>
+    <col width="40" customWidth="1" min="18" max="18"/>
+  </cols>
+  <sheetData>
+    <row r="1">
+      <c r="A1" s="1" t="inlineStr">
+        <is>
+          <t>Section C. Benchmarking: top 30 Swedish business law firms</t>
+        </is>
+      </c>
+    </row>
+    <row r="2" ht="45" customHeight="1">
+      <c r="A2" s="2" t="inlineStr">
+        <is>
+          <t>Ranking: Affärsvärlden fee income FY2024 (revised table, 3 Oct 2025; split-year firms on FY24/25). Ratios use the latest available revenue (FY2025 where published, else FY2024; basis shown) against current headcount (mostly Oct-2026), so they are indicative. Leverage (requested) = partners / total employees; partners / lawyers shown alongside. Grey = not available.</t>
+        </is>
+      </c>
+    </row>
+    <row r="4" ht="48" customHeight="1">
+      <c r="A4" s="52" t="inlineStr">
+        <is>
+          <t>#</t>
+        </is>
+      </c>
+      <c r="B4" s="52" t="inlineStr">
+        <is>
+          <t>Firm</t>
+        </is>
+      </c>
+      <c r="C4" s="52" t="inlineStr">
+        <is>
+          <t>Afv fee income FY2024</t>
+        </is>
+      </c>
+      <c r="D4" s="52" t="inlineStr">
+        <is>
+          <t>Afv FY2023</t>
+        </is>
+      </c>
+      <c r="E4" s="52" t="inlineStr">
+        <is>
+          <t>Growth FY24</t>
+        </is>
+      </c>
+      <c r="F4" s="52" t="inlineStr">
+        <is>
+          <t>Latest revenue</t>
+        </is>
+      </c>
+      <c r="G4" s="52" t="inlineStr">
+        <is>
+          <t>Latest revenue basis</t>
+        </is>
+      </c>
+      <c r="H4" s="52" t="inlineStr">
+        <is>
+          <t>Partners</t>
+        </is>
+      </c>
+      <c r="I4" s="52" t="inlineStr">
+        <is>
+          <t>Lawyers (incl. partners)</t>
+        </is>
+      </c>
+      <c r="J4" s="52" t="inlineStr">
+        <is>
+          <t>Total employees</t>
+        </is>
+      </c>
+      <c r="K4" s="52" t="inlineStr">
+        <is>
+          <t>Headcount source</t>
+        </is>
+      </c>
+      <c r="L4" s="52" t="inlineStr">
+        <is>
+          <t>Rev / partner</t>
+        </is>
+      </c>
+      <c r="M4" s="52" t="inlineStr">
+        <is>
+          <t>Rev / employee</t>
+        </is>
+      </c>
+      <c r="N4" s="52" t="inlineStr">
+        <is>
+          <t>Rev / lawyer</t>
+        </is>
+      </c>
+      <c r="O4" s="52" t="inlineStr">
+        <is>
+          <t>Leverage: partners / employees</t>
+        </is>
+      </c>
+      <c r="P4" s="52" t="inlineStr">
+        <is>
+          <t>Leverage: partners / lawyers</t>
+        </is>
+      </c>
+      <c r="Q4" s="52" t="inlineStr">
+        <is>
+          <t>Employees per partner</t>
+        </is>
+      </c>
+      <c r="R4" s="52" t="inlineStr">
+        <is>
+          <t>Notes</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" s="90" t="n">
+        <v>1</v>
+      </c>
+      <c r="B5" s="49" t="inlineStr">
+        <is>
+          <t>Vinge</t>
+        </is>
+      </c>
+      <c r="C5" s="100" t="n">
+        <v>2085</v>
+      </c>
+      <c r="D5" s="100" t="n">
+        <v>1751</v>
+      </c>
+      <c r="E5" s="101">
+        <f>C5/D5-1</f>
+        <v/>
+      </c>
+      <c r="F5" s="100" t="n">
+        <v>2036</v>
+      </c>
+      <c r="G5" s="49" t="inlineStr">
+        <is>
+          <t>FY2025 group (annual reports, DJ)</t>
+        </is>
+      </c>
+      <c r="H5" s="90" t="n">
+        <v>71</v>
+      </c>
+      <c r="I5" s="90" t="n">
+        <v>389</v>
+      </c>
+      <c r="J5" s="90" t="n">
+        <v>529</v>
+      </c>
+      <c r="K5" s="49" t="inlineStr">
+        <is>
+          <t>Firm website count Oct-26; employees: 3 ABs 2025 accounts</t>
+        </is>
+      </c>
+      <c r="L5" s="92">
+        <f>F5/H5</f>
+        <v/>
+      </c>
+      <c r="M5" s="93">
+        <f>F5/J5</f>
+        <v/>
+      </c>
+      <c r="N5" s="93">
+        <f>F5/I5</f>
+        <v/>
+      </c>
+      <c r="O5" s="101">
+        <f>H5/J5</f>
+        <v/>
+      </c>
+      <c r="P5" s="101">
+        <f>H5/I5</f>
+        <v/>
+      </c>
+      <c r="Q5" s="92">
+        <f>J5/H5</f>
+        <v/>
+      </c>
+      <c r="R5" s="49" t="inlineStr">
+        <is>
+          <t>Lawyers incl. ~46 on leave</t>
+        </is>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" s="90" t="n">
+        <v>2</v>
+      </c>
+      <c r="B6" s="49" t="inlineStr">
+        <is>
+          <t>Mannheimer Swartling</t>
+        </is>
+      </c>
+      <c r="C6" s="100" t="n">
+        <v>1911</v>
+      </c>
+      <c r="D6" s="100" t="n">
+        <v>1807</v>
+      </c>
+      <c r="E6" s="101">
+        <f>C6/D6-1</f>
+        <v/>
+      </c>
+      <c r="F6" s="100" t="n">
+        <v>2002</v>
+      </c>
+      <c r="G6" s="49" t="inlineStr">
+        <is>
+          <t>FY2025 (annual report)</t>
+        </is>
+      </c>
+      <c r="H6" s="90" t="n">
+        <v>92</v>
+      </c>
+      <c r="I6" s="90" t="n">
+        <v>430</v>
+      </c>
+      <c r="J6" s="90" t="n">
+        <v>649</v>
+      </c>
+      <c r="K6" s="49" t="inlineStr">
+        <is>
+          <t>DJ/Chambers 2026; employees 2025 accounts</t>
+        </is>
+      </c>
+      <c r="L6" s="92">
+        <f>F6/H6</f>
+        <v/>
+      </c>
+      <c r="M6" s="93">
+        <f>F6/J6</f>
+        <v/>
+      </c>
+      <c r="N6" s="93">
+        <f>F6/I6</f>
+        <v/>
+      </c>
+      <c r="O6" s="101">
+        <f>H6/J6</f>
+        <v/>
+      </c>
+      <c r="P6" s="101">
+        <f>H6/I6</f>
+        <v/>
+      </c>
+      <c r="Q6" s="92">
+        <f>J6/H6</f>
+        <v/>
+      </c>
+      <c r="R6" s="49" t="inlineStr"/>
+    </row>
+    <row r="7">
+      <c r="A7" s="90" t="n">
+        <v>3</v>
+      </c>
+      <c r="B7" s="49" t="inlineStr">
+        <is>
+          <t>Roschier (Sweden)</t>
+        </is>
+      </c>
+      <c r="C7" s="100" t="n">
+        <v>1254</v>
+      </c>
+      <c r="D7" s="100" t="n">
+        <v>1026</v>
+      </c>
+      <c r="E7" s="101">
+        <f>C7/D7-1</f>
+        <v/>
+      </c>
+      <c r="F7" s="100" t="n">
+        <v>1304</v>
+      </c>
+      <c r="G7" s="49" t="inlineStr">
+        <is>
+          <t>FY Jun25-May26 net sales (AB)</t>
+        </is>
+      </c>
+      <c r="H7" s="90" t="n">
+        <v>26</v>
+      </c>
+      <c r="I7" s="90" t="n">
+        <v>181</v>
+      </c>
+      <c r="J7" s="90" t="n">
+        <v>220</v>
+      </c>
+      <c r="K7" s="49" t="inlineStr">
+        <is>
+          <t>Firm website count Oct-26 (Stockholm); employees AB accounts</t>
+        </is>
+      </c>
+      <c r="L7" s="92">
+        <f>F7/H7</f>
+        <v/>
+      </c>
+      <c r="M7" s="93">
+        <f>F7/J7</f>
+        <v/>
+      </c>
+      <c r="N7" s="93">
+        <f>F7/I7</f>
+        <v/>
+      </c>
+      <c r="O7" s="101">
+        <f>H7/J7</f>
+        <v/>
+      </c>
+      <c r="P7" s="101">
+        <f>H7/I7</f>
+        <v/>
+      </c>
+      <c r="Q7" s="92">
+        <f>J7/H7</f>
+        <v/>
+      </c>
+      <c r="R7" s="49" t="inlineStr">
+        <is>
+          <t>Split year; Afv FY24 = FY Jun24-May25</t>
+        </is>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" s="90" t="n">
+        <v>4</v>
+      </c>
+      <c r="B8" s="49" t="inlineStr">
+        <is>
+          <t>Setterwalls</t>
+        </is>
+      </c>
+      <c r="C8" s="100" t="n">
+        <v>918</v>
+      </c>
+      <c r="D8" s="100" t="n">
+        <v>899</v>
+      </c>
+      <c r="E8" s="101">
+        <f>C8/D8-1</f>
+        <v/>
+      </c>
+      <c r="F8" s="100" t="n">
+        <v>1000</v>
+      </c>
+      <c r="G8" s="49" t="inlineStr">
+        <is>
+          <t>FY2025 (Afv "&gt;1bn")</t>
+        </is>
+      </c>
+      <c r="H8" s="90" t="n">
+        <v>38</v>
+      </c>
+      <c r="I8" s="90" t="n">
+        <v>177</v>
+      </c>
+      <c r="J8" s="90" t="n">
+        <v>306</v>
+      </c>
+      <c r="K8" s="49" t="inlineStr">
+        <is>
+          <t>Firm website count Oct-26; employees 3 entities 2025</t>
+        </is>
+      </c>
+      <c r="L8" s="92">
+        <f>F8/H8</f>
+        <v/>
+      </c>
+      <c r="M8" s="93">
+        <f>F8/J8</f>
+        <v/>
+      </c>
+      <c r="N8" s="93">
+        <f>F8/I8</f>
+        <v/>
+      </c>
+      <c r="O8" s="101">
+        <f>H8/J8</f>
+        <v/>
+      </c>
+      <c r="P8" s="101">
+        <f>H8/I8</f>
+        <v/>
+      </c>
+      <c r="Q8" s="92">
+        <f>J8/H8</f>
+        <v/>
+      </c>
+      <c r="R8" s="49" t="inlineStr">
+        <is>
+          <t>Revenue/employees incl. Malmö (left Sep-26); partners/lawyers exclude it</t>
+        </is>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" s="90" t="n">
+        <v>5</v>
+      </c>
+      <c r="B9" s="49" t="inlineStr">
+        <is>
+          <t>Lindahl</t>
+        </is>
+      </c>
+      <c r="C9" s="100" t="n">
+        <v>737</v>
+      </c>
+      <c r="D9" s="100" t="n">
+        <v>707</v>
+      </c>
+      <c r="E9" s="101">
+        <f>C9/D9-1</f>
+        <v/>
+      </c>
+      <c r="F9" s="100" t="n">
+        <v>737</v>
+      </c>
+      <c r="G9" s="49" t="inlineStr">
+        <is>
+          <t>FY2024 (Afv)</t>
+        </is>
+      </c>
+      <c r="H9" s="90" t="n">
+        <v>68</v>
+      </c>
+      <c r="I9" s="90" t="n">
+        <v>220</v>
+      </c>
+      <c r="J9" s="90" t="n">
+        <v>300</v>
+      </c>
+      <c r="K9" s="49" t="inlineStr">
+        <is>
+          <t>Legal 500 / Chambers (firm-supplied)</t>
+        </is>
+      </c>
+      <c r="L9" s="92">
+        <f>F9/H9</f>
+        <v/>
+      </c>
+      <c r="M9" s="93">
+        <f>F9/J9</f>
+        <v/>
+      </c>
+      <c r="N9" s="93">
+        <f>F9/I9</f>
+        <v/>
+      </c>
+      <c r="O9" s="101">
+        <f>H9/J9</f>
+        <v/>
+      </c>
+      <c r="P9" s="101">
+        <f>H9/I9</f>
+        <v/>
+      </c>
+      <c r="Q9" s="92">
+        <f>J9/H9</f>
+        <v/>
+      </c>
+      <c r="R9" s="49" t="inlineStr"/>
+    </row>
+    <row r="10">
+      <c r="A10" s="90" t="n">
+        <v>6</v>
+      </c>
+      <c r="B10" s="49" t="inlineStr">
+        <is>
+          <t>Gernandt &amp; Danielsson</t>
+        </is>
+      </c>
+      <c r="C10" s="100" t="n">
+        <v>676</v>
+      </c>
+      <c r="D10" s="100" t="n">
+        <v>601</v>
+      </c>
+      <c r="E10" s="101">
+        <f>C10/D10-1</f>
+        <v/>
+      </c>
+      <c r="F10" s="100" t="n">
+        <v>676</v>
+      </c>
+      <c r="G10" s="49" t="inlineStr">
+        <is>
+          <t>FY24/25 (Afv)</t>
+        </is>
+      </c>
+      <c r="H10" s="90" t="n">
+        <v>20</v>
+      </c>
+      <c r="I10" s="90" t="n">
+        <v>91</v>
+      </c>
+      <c r="J10" s="90" t="n">
+        <v>150</v>
+      </c>
+      <c r="K10" s="49" t="inlineStr">
+        <is>
+          <t>Firm website count Oct-26; employees firm website</t>
+        </is>
+      </c>
+      <c r="L10" s="92">
+        <f>F10/H10</f>
+        <v/>
+      </c>
+      <c r="M10" s="93">
+        <f>F10/J10</f>
+        <v/>
+      </c>
+      <c r="N10" s="93">
+        <f>F10/I10</f>
+        <v/>
+      </c>
+      <c r="O10" s="101">
+        <f>H10/J10</f>
+        <v/>
+      </c>
+      <c r="P10" s="101">
+        <f>H10/I10</f>
+        <v/>
+      </c>
+      <c r="Q10" s="92">
+        <f>J10/H10</f>
+        <v/>
+      </c>
+      <c r="R10" s="49" t="inlineStr">
+        <is>
+          <t>KB - no public accounts</t>
+        </is>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" s="90" t="n">
+        <v>7</v>
+      </c>
+      <c r="B11" s="49" t="inlineStr">
+        <is>
+          <t>DLA Piper (Sweden)</t>
+        </is>
+      </c>
+      <c r="C11" s="100" t="n">
+        <v>602</v>
+      </c>
+      <c r="D11" s="100" t="n">
+        <v>660</v>
+      </c>
+      <c r="E11" s="101">
+        <f>C11/D11-1</f>
+        <v/>
+      </c>
+      <c r="F11" s="100" t="n">
+        <v>602</v>
+      </c>
+      <c r="G11" s="49" t="inlineStr">
+        <is>
+          <t>FY24/25 (Afv)</t>
+        </is>
+      </c>
+      <c r="H11" s="90" t="n">
+        <v>37</v>
+      </c>
+      <c r="I11" s="90" t="n">
+        <v>148</v>
+      </c>
+      <c r="J11" s="98" t="n"/>
+      <c r="K11" s="49" t="inlineStr">
+        <is>
+          <t>Firm website count Oct-26</t>
+        </is>
+      </c>
+      <c r="L11" s="92">
+        <f>F11/H11</f>
+        <v/>
+      </c>
+      <c r="M11" s="98" t="n"/>
+      <c r="N11" s="93">
+        <f>F11/I11</f>
+        <v/>
+      </c>
+      <c r="O11" s="98" t="n"/>
+      <c r="P11" s="101">
+        <f>H11/I11</f>
+        <v/>
+      </c>
+      <c r="Q11" s="98" t="n"/>
+      <c r="R11" s="49" t="inlineStr">
+        <is>
+          <t>Employees: allabolag band 200-499 only</t>
+        </is>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" s="90" t="n">
+        <v>8</v>
+      </c>
+      <c r="B12" s="49" t="inlineStr">
+        <is>
+          <t>CMS Wistrand</t>
+        </is>
+      </c>
+      <c r="C12" s="100" t="n">
+        <v>558</v>
+      </c>
+      <c r="D12" s="100" t="n">
+        <v>529</v>
+      </c>
+      <c r="E12" s="101">
+        <f>C12/D12-1</f>
+        <v/>
+      </c>
+      <c r="F12" s="100" t="n">
+        <v>558</v>
+      </c>
+      <c r="G12" s="49" t="inlineStr">
+        <is>
+          <t>FY2024 (Afv)</t>
+        </is>
+      </c>
+      <c r="H12" s="90" t="n">
+        <v>51</v>
+      </c>
+      <c r="I12" s="90" t="n">
+        <v>150</v>
+      </c>
+      <c r="J12" s="90" t="n">
+        <v>220</v>
+      </c>
+      <c r="K12" s="49" t="inlineStr">
+        <is>
+          <t>Firm statement / Chambers 2026 ("&gt;220")</t>
+        </is>
+      </c>
+      <c r="L12" s="92">
+        <f>F12/H12</f>
+        <v/>
+      </c>
+      <c r="M12" s="93">
+        <f>F12/J12</f>
+        <v/>
+      </c>
+      <c r="N12" s="93">
+        <f>F12/I12</f>
+        <v/>
+      </c>
+      <c r="O12" s="101">
+        <f>H12/J12</f>
+        <v/>
+      </c>
+      <c r="P12" s="101">
+        <f>H12/I12</f>
+        <v/>
+      </c>
+      <c r="Q12" s="92">
+        <f>J12/H12</f>
+        <v/>
+      </c>
+      <c r="R12" s="49" t="inlineStr"/>
+    </row>
+    <row r="13">
+      <c r="A13" s="90" t="n">
+        <v>9</v>
+      </c>
+      <c r="B13" s="49" t="inlineStr">
+        <is>
+          <t>Delphi</t>
+        </is>
+      </c>
+      <c r="C13" s="100" t="n">
+        <v>516</v>
+      </c>
+      <c r="D13" s="100" t="n">
+        <v>505</v>
+      </c>
+      <c r="E13" s="101">
+        <f>C13/D13-1</f>
+        <v/>
+      </c>
+      <c r="F13" s="100" t="n">
+        <v>516</v>
+      </c>
+      <c r="G13" s="49" t="inlineStr">
+        <is>
+          <t>FY2024 (Afv)</t>
+        </is>
+      </c>
+      <c r="H13" s="90" t="n">
+        <v>49</v>
+      </c>
+      <c r="I13" s="90" t="n">
+        <v>150</v>
+      </c>
+      <c r="J13" s="90" t="n">
+        <v>220</v>
+      </c>
+      <c r="K13" s="49" t="inlineStr">
+        <is>
+          <t>Chambers 2026 / firm website</t>
+        </is>
+      </c>
+      <c r="L13" s="92">
+        <f>F13/H13</f>
+        <v/>
+      </c>
+      <c r="M13" s="93">
+        <f>F13/J13</f>
+        <v/>
+      </c>
+      <c r="N13" s="93">
+        <f>F13/I13</f>
+        <v/>
+      </c>
+      <c r="O13" s="101">
+        <f>H13/J13</f>
+        <v/>
+      </c>
+      <c r="P13" s="101">
+        <f>H13/I13</f>
+        <v/>
+      </c>
+      <c r="Q13" s="92">
+        <f>J13/H13</f>
+        <v/>
+      </c>
+      <c r="R13" s="49" t="inlineStr"/>
+    </row>
+    <row r="14">
+      <c r="A14" s="90" t="n">
+        <v>10</v>
+      </c>
+      <c r="B14" s="49" t="inlineStr">
+        <is>
+          <t>Cederquist</t>
+        </is>
+      </c>
+      <c r="C14" s="100" t="n">
+        <v>500</v>
+      </c>
+      <c r="D14" s="100" t="n">
+        <v>472</v>
+      </c>
+      <c r="E14" s="101">
+        <f>C14/D14-1</f>
+        <v/>
+      </c>
+      <c r="F14" s="100" t="n">
+        <v>500</v>
+      </c>
+      <c r="G14" s="49" t="inlineStr">
+        <is>
+          <t>FY2024 (Afv)</t>
+        </is>
+      </c>
+      <c r="H14" s="90" t="n">
+        <v>26</v>
+      </c>
+      <c r="I14" s="90" t="n">
+        <v>124</v>
+      </c>
+      <c r="J14" s="98" t="n"/>
+      <c r="K14" s="49" t="inlineStr">
+        <is>
+          <t>Legal 500 (firm-supplied)</t>
+        </is>
+      </c>
+      <c r="L14" s="92">
+        <f>F14/H14</f>
+        <v/>
+      </c>
+      <c r="M14" s="98" t="n"/>
+      <c r="N14" s="93">
+        <f>F14/I14</f>
+        <v/>
+      </c>
+      <c r="O14" s="98" t="n"/>
+      <c r="P14" s="101">
+        <f>H14/I14</f>
+        <v/>
+      </c>
+      <c r="Q14" s="98" t="n"/>
+      <c r="R14" s="49" t="inlineStr">
+        <is>
+          <t>KB - no public accounts; Chambers 120 lawyers</t>
+        </is>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" s="90" t="n">
+        <v>11</v>
+      </c>
+      <c r="B15" s="49" t="inlineStr">
+        <is>
+          <t>Schjødt (Sweden)</t>
+        </is>
+      </c>
+      <c r="C15" s="100" t="n">
+        <v>427</v>
+      </c>
+      <c r="D15" s="100" t="n">
+        <v>343</v>
+      </c>
+      <c r="E15" s="101">
+        <f>C15/D15-1</f>
+        <v/>
+      </c>
+      <c r="F15" s="100" t="n">
+        <v>534</v>
+      </c>
+      <c r="G15" s="49" t="inlineStr">
+        <is>
+          <t>FY2025 est. ("&gt;0.5bn", +25%)</t>
+        </is>
+      </c>
+      <c r="H15" s="90" t="n">
+        <v>20</v>
+      </c>
+      <c r="I15" s="90" t="n">
+        <v>65</v>
+      </c>
+      <c r="J15" s="98" t="n"/>
+      <c r="K15" s="49" t="inlineStr">
+        <is>
+          <t>Firm website count Oct-26 (Stockholm)</t>
+        </is>
+      </c>
+      <c r="L15" s="92">
+        <f>F15/H15</f>
+        <v/>
+      </c>
+      <c r="M15" s="98" t="n"/>
+      <c r="N15" s="93">
+        <f>F15/I15</f>
+        <v/>
+      </c>
+      <c r="O15" s="98" t="n"/>
+      <c r="P15" s="101">
+        <f>H15/I15</f>
+        <v/>
+      </c>
+      <c r="Q15" s="98" t="n"/>
+      <c r="R15" s="49" t="inlineStr">
+        <is>
+          <t>May include leavers to BAHR; branch band 50-99 employees</t>
+        </is>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" s="90" t="n">
+        <v>12</v>
+      </c>
+      <c r="B16" s="49" t="inlineStr">
+        <is>
+          <t>MAQS</t>
+        </is>
+      </c>
+      <c r="C16" s="100" t="n">
+        <v>417</v>
+      </c>
+      <c r="D16" s="100" t="n">
+        <v>346</v>
+      </c>
+      <c r="E16" s="101">
+        <f>C16/D16-1</f>
+        <v/>
+      </c>
+      <c r="F16" s="100" t="n">
+        <v>417</v>
+      </c>
+      <c r="G16" s="49" t="inlineStr">
+        <is>
+          <t>FY2024 (Afv)</t>
+        </is>
+      </c>
+      <c r="H16" s="90" t="n">
+        <v>48</v>
+      </c>
+      <c r="I16" s="90" t="n">
+        <v>144</v>
+      </c>
+      <c r="J16" s="90" t="n">
+        <v>180</v>
+      </c>
+      <c r="K16" s="49" t="inlineStr">
+        <is>
+          <t>Firm website count Oct-26; employees Chambers 2026</t>
+        </is>
+      </c>
+      <c r="L16" s="92">
+        <f>F16/H16</f>
+        <v/>
+      </c>
+      <c r="M16" s="93">
+        <f>F16/J16</f>
+        <v/>
+      </c>
+      <c r="N16" s="93">
+        <f>F16/I16</f>
+        <v/>
+      </c>
+      <c r="O16" s="101">
+        <f>H16/J16</f>
+        <v/>
+      </c>
+      <c r="P16" s="101">
+        <f>H16/I16</f>
+        <v/>
+      </c>
+      <c r="Q16" s="92">
+        <f>J16/H16</f>
+        <v/>
+      </c>
+      <c r="R16" s="49" t="inlineStr">
+        <is>
+          <t>Splitting from 1 Jan 2027: Malmö (MAQS KB) vs Sthlm/Gbg/Sundsvall (MAQS AB)</t>
+        </is>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" s="90" t="n">
+        <v>13</v>
+      </c>
+      <c r="B17" s="49" t="inlineStr">
+        <is>
+          <t>Cirio</t>
+        </is>
+      </c>
+      <c r="C17" s="100" t="n">
+        <v>363</v>
+      </c>
+      <c r="D17" s="100" t="n">
+        <v>317</v>
+      </c>
+      <c r="E17" s="101">
+        <f>C17/D17-1</f>
+        <v/>
+      </c>
+      <c r="F17" s="100" t="n">
+        <v>431</v>
+      </c>
+      <c r="G17" s="49" t="inlineStr">
+        <is>
+          <t>FY2025 net sales (AB)</t>
+        </is>
+      </c>
+      <c r="H17" s="90" t="n">
+        <v>27</v>
+      </c>
+      <c r="I17" s="90" t="n">
+        <v>76</v>
+      </c>
+      <c r="J17" s="90" t="n">
+        <v>127</v>
+      </c>
+      <c r="K17" s="49" t="inlineStr">
+        <is>
+          <t>Legal 500; employees 2025 accounts</t>
+        </is>
+      </c>
+      <c r="L17" s="92">
+        <f>F17/H17</f>
+        <v/>
+      </c>
+      <c r="M17" s="93">
+        <f>F17/J17</f>
+        <v/>
+      </c>
+      <c r="N17" s="93">
+        <f>F17/I17</f>
+        <v/>
+      </c>
+      <c r="O17" s="101">
+        <f>H17/J17</f>
+        <v/>
+      </c>
+      <c r="P17" s="101">
+        <f>H17/I17</f>
+        <v/>
+      </c>
+      <c r="Q17" s="92">
+        <f>J17/H17</f>
+        <v/>
+      </c>
+      <c r="R17" s="49" t="inlineStr"/>
+    </row>
+    <row r="18">
+      <c r="A18" s="90" t="n">
+        <v>14</v>
+      </c>
+      <c r="B18" s="49" t="inlineStr">
+        <is>
+          <t>Snellman (Sweden)</t>
+        </is>
+      </c>
+      <c r="C18" s="100" t="n">
+        <v>295</v>
+      </c>
+      <c r="D18" s="100" t="n">
+        <v>300</v>
+      </c>
+      <c r="E18" s="101">
+        <f>C18/D18-1</f>
+        <v/>
+      </c>
+      <c r="F18" s="100" t="n">
+        <v>279</v>
+      </c>
+      <c r="G18" s="49" t="inlineStr">
+        <is>
+          <t>FY2025 net sales (AB)</t>
+        </is>
+      </c>
+      <c r="H18" s="90" t="n">
+        <v>17</v>
+      </c>
+      <c r="I18" s="98" t="n"/>
+      <c r="J18" s="90" t="n">
+        <v>107</v>
+      </c>
+      <c r="K18" s="49" t="inlineStr">
+        <is>
+          <t>Legal 500 (stale); employees 2025 accounts</t>
+        </is>
+      </c>
+      <c r="L18" s="92">
+        <f>F18/H18</f>
+        <v/>
+      </c>
+      <c r="M18" s="93">
+        <f>F18/J18</f>
+        <v/>
+      </c>
+      <c r="N18" s="98" t="n"/>
+      <c r="O18" s="101">
+        <f>H18/J18</f>
+        <v/>
+      </c>
+      <c r="P18" s="98" t="n"/>
+      <c r="Q18" s="92">
+        <f>J18/H18</f>
+        <v/>
+      </c>
+      <c r="R18" s="49" t="inlineStr">
+        <is>
+          <t>Partner count unverified</t>
+        </is>
+      </c>
+    </row>
+    <row r="19">
+      <c r="A19" s="90" t="n">
+        <v>15</v>
+      </c>
+      <c r="B19" s="49" t="inlineStr">
+        <is>
+          <t>Foyen</t>
+        </is>
+      </c>
+      <c r="C19" s="100" t="n">
+        <v>277</v>
+      </c>
+      <c r="D19" s="100" t="n">
+        <v>263</v>
+      </c>
+      <c r="E19" s="101">
+        <f>C19/D19-1</f>
+        <v/>
+      </c>
+      <c r="F19" s="100" t="n">
+        <v>277</v>
+      </c>
+      <c r="G19" s="49" t="inlineStr">
+        <is>
+          <t>FY2024 (Afv)</t>
+        </is>
+      </c>
+      <c r="H19" s="90" t="n">
+        <v>23</v>
+      </c>
+      <c r="I19" s="90" t="n">
+        <v>73</v>
+      </c>
+      <c r="J19" s="90" t="n">
+        <v>106</v>
+      </c>
+      <c r="K19" s="49" t="inlineStr">
+        <is>
+          <t>Firm website count Oct-26; employees AB accounts</t>
+        </is>
+      </c>
+      <c r="L19" s="92">
+        <f>F19/H19</f>
+        <v/>
+      </c>
+      <c r="M19" s="93">
+        <f>F19/J19</f>
+        <v/>
+      </c>
+      <c r="N19" s="93">
+        <f>F19/I19</f>
+        <v/>
+      </c>
+      <c r="O19" s="101">
+        <f>H19/J19</f>
+        <v/>
+      </c>
+      <c r="P19" s="101">
+        <f>H19/I19</f>
+        <v/>
+      </c>
+      <c r="Q19" s="92">
+        <f>J19/H19</f>
+        <v/>
+      </c>
+      <c r="R19" s="49" t="inlineStr"/>
+    </row>
+    <row r="20">
+      <c r="A20" s="90" t="n">
+        <v>16</v>
+      </c>
+      <c r="B20" s="49" t="inlineStr">
+        <is>
+          <t>AG Advokat</t>
+        </is>
+      </c>
+      <c r="C20" s="100" t="n">
+        <v>198</v>
+      </c>
+      <c r="D20" s="100" t="n">
+        <v>228</v>
+      </c>
+      <c r="E20" s="101">
+        <f>C20/D20-1</f>
+        <v/>
+      </c>
+      <c r="F20" s="100" t="n">
+        <v>198</v>
+      </c>
+      <c r="G20" s="49" t="inlineStr">
+        <is>
+          <t>FY2024 (Afv)</t>
+        </is>
+      </c>
+      <c r="H20" s="98" t="n"/>
+      <c r="I20" s="90" t="n">
+        <v>41</v>
+      </c>
+      <c r="J20" s="98" t="n"/>
+      <c r="K20" s="49" t="inlineStr">
+        <is>
+          <t>Legal 500</t>
+        </is>
+      </c>
+      <c r="L20" s="98" t="n"/>
+      <c r="M20" s="98" t="n"/>
+      <c r="N20" s="93">
+        <f>F20/I20</f>
+        <v/>
+      </c>
+      <c r="O20" s="98" t="n"/>
+      <c r="P20" s="98" t="n"/>
+      <c r="Q20" s="98" t="n"/>
+      <c r="R20" s="49" t="inlineStr">
+        <is>
+          <t>Lost 12-person team to Cirio (Jan-25)</t>
+        </is>
+      </c>
+    </row>
+    <row r="21">
+      <c r="A21" s="90" t="n">
+        <v>17</v>
+      </c>
+      <c r="B21" s="49" t="inlineStr">
+        <is>
+          <t>Glimstedt</t>
+        </is>
+      </c>
+      <c r="C21" s="100" t="n">
+        <v>196</v>
+      </c>
+      <c r="D21" s="100" t="n">
+        <v>174</v>
+      </c>
+      <c r="E21" s="101">
+        <f>C21/D21-1</f>
+        <v/>
+      </c>
+      <c r="F21" s="100" t="n">
+        <v>196</v>
+      </c>
+      <c r="G21" s="49" t="inlineStr">
+        <is>
+          <t>FY2024 (Afv)</t>
+        </is>
+      </c>
+      <c r="H21" s="90" t="n">
+        <v>41</v>
+      </c>
+      <c r="I21" s="90" t="n">
+        <v>78</v>
+      </c>
+      <c r="J21" s="98" t="n"/>
+      <c r="K21" s="49" t="inlineStr">
+        <is>
+          <t>Firm website count Oct-26 (Sweden)</t>
+        </is>
+      </c>
+      <c r="L21" s="92">
+        <f>F21/H21</f>
+        <v/>
+      </c>
+      <c r="M21" s="98" t="n"/>
+      <c r="N21" s="93">
+        <f>F21/I21</f>
+        <v/>
+      </c>
+      <c r="O21" s="98" t="n"/>
+      <c r="P21" s="101">
+        <f>H21/I21</f>
+        <v/>
+      </c>
+      <c r="Q21" s="98" t="n"/>
+      <c r="R21" s="49" t="inlineStr">
+        <is>
+          <t>~200 staff incl. Baltics (not used)</t>
+        </is>
+      </c>
+    </row>
+    <row r="22">
+      <c r="A22" s="90" t="n">
+        <v>18</v>
+      </c>
+      <c r="B22" s="49" t="inlineStr">
+        <is>
+          <t>TM &amp; Partners</t>
+        </is>
+      </c>
+      <c r="C22" s="100" t="n">
+        <v>188</v>
+      </c>
+      <c r="D22" s="100" t="n">
+        <v>175</v>
+      </c>
+      <c r="E22" s="101">
+        <f>C22/D22-1</f>
+        <v/>
+      </c>
+      <c r="F22" s="100" t="n">
+        <v>188</v>
+      </c>
+      <c r="G22" s="49" t="inlineStr">
+        <is>
+          <t>FY2024 (Afv)</t>
+        </is>
+      </c>
+      <c r="H22" s="90" t="n">
+        <v>18</v>
+      </c>
+      <c r="I22" s="90" t="n">
+        <v>63</v>
+      </c>
+      <c r="J22" s="98" t="n"/>
+      <c r="K22" s="49" t="inlineStr">
+        <is>
+          <t>Firm website count Oct-26</t>
+        </is>
+      </c>
+      <c r="L22" s="92">
+        <f>F22/H22</f>
+        <v/>
+      </c>
+      <c r="M22" s="98" t="n"/>
+      <c r="N22" s="93">
+        <f>F22/I22</f>
+        <v/>
+      </c>
+      <c r="O22" s="98" t="n"/>
+      <c r="P22" s="101">
+        <f>H22/I22</f>
+        <v/>
+      </c>
+      <c r="Q22" s="98" t="n"/>
+      <c r="R22" s="49" t="inlineStr">
+        <is>
+          <t>Part of AGRD since 2025; AB (73 staff) is partial</t>
+        </is>
+      </c>
+    </row>
+    <row r="23">
+      <c r="A23" s="90" t="n">
+        <v>19</v>
+      </c>
+      <c r="B23" s="49" t="inlineStr">
+        <is>
+          <t>WSA</t>
+        </is>
+      </c>
+      <c r="C23" s="100" t="n">
+        <v>165</v>
+      </c>
+      <c r="D23" s="100" t="n">
+        <v>164</v>
+      </c>
+      <c r="E23" s="101">
+        <f>C23/D23-1</f>
+        <v/>
+      </c>
+      <c r="F23" s="100" t="n">
+        <v>165</v>
+      </c>
+      <c r="G23" s="49" t="inlineStr">
+        <is>
+          <t>FY2024 (Afv)</t>
+        </is>
+      </c>
+      <c r="H23" s="98" t="n"/>
+      <c r="I23" s="98" t="n"/>
+      <c r="J23" s="98" t="n"/>
+      <c r="K23" s="49" t="inlineStr"/>
+      <c r="L23" s="98" t="n"/>
+      <c r="M23" s="98" t="n"/>
+      <c r="N23" s="98" t="n"/>
+      <c r="O23" s="98" t="n"/>
+      <c r="P23" s="98" t="n"/>
+      <c r="Q23" s="98" t="n"/>
+      <c r="R23" s="49" t="inlineStr">
+        <is>
+          <t>Headcount not researched</t>
+        </is>
+      </c>
+    </row>
+    <row r="24">
+      <c r="A24" s="90" t="n">
+        <v>20</v>
+      </c>
+      <c r="B24" s="49" t="inlineStr">
+        <is>
+          <t>Morris Law</t>
+        </is>
+      </c>
+      <c r="C24" s="100" t="n">
+        <v>163</v>
+      </c>
+      <c r="D24" s="100" t="n">
+        <v>151</v>
+      </c>
+      <c r="E24" s="101">
+        <f>C24/D24-1</f>
+        <v/>
+      </c>
+      <c r="F24" s="100" t="n">
+        <v>163</v>
+      </c>
+      <c r="G24" s="49" t="inlineStr">
+        <is>
+          <t>FY2024 (Afv)</t>
+        </is>
+      </c>
+      <c r="H24" s="98" t="n"/>
+      <c r="I24" s="90" t="n">
+        <v>56</v>
+      </c>
+      <c r="J24" s="98" t="n"/>
+      <c r="K24" s="49" t="inlineStr">
+        <is>
+          <t>Legal 500</t>
+        </is>
+      </c>
+      <c r="L24" s="98" t="n"/>
+      <c r="M24" s="98" t="n"/>
+      <c r="N24" s="93">
+        <f>F24/I24</f>
+        <v/>
+      </c>
+      <c r="O24" s="98" t="n"/>
+      <c r="P24" s="98" t="n"/>
+      <c r="Q24" s="98" t="n"/>
+      <c r="R24" s="49" t="inlineStr">
+        <is>
+          <t>Part of AGRD since 2025</t>
+        </is>
+      </c>
+    </row>
+    <row r="25">
+      <c r="A25" s="90" t="n">
+        <v>21</v>
+      </c>
+      <c r="B25" s="49" t="inlineStr">
+        <is>
+          <t>Hammarskiöld</t>
+        </is>
+      </c>
+      <c r="C25" s="100" t="n">
+        <v>158</v>
+      </c>
+      <c r="D25" s="100" t="n">
+        <v>133</v>
+      </c>
+      <c r="E25" s="101">
+        <f>C25/D25-1</f>
+        <v/>
+      </c>
+      <c r="F25" s="100" t="n">
+        <v>178</v>
+      </c>
+      <c r="G25" s="49" t="inlineStr">
+        <is>
+          <t>FY2025 net sales (AB)</t>
+        </is>
+      </c>
+      <c r="H25" s="98" t="n"/>
+      <c r="I25" s="90" t="n">
+        <v>47</v>
+      </c>
+      <c r="J25" s="90" t="n">
+        <v>63</v>
+      </c>
+      <c r="K25" s="49" t="inlineStr">
+        <is>
+          <t>Chambers 2026; employees 2025 accounts</t>
+        </is>
+      </c>
+      <c r="L25" s="98" t="n"/>
+      <c r="M25" s="93">
+        <f>F25/J25</f>
+        <v/>
+      </c>
+      <c r="N25" s="93">
+        <f>F25/I25</f>
+        <v/>
+      </c>
+      <c r="O25" s="98" t="n"/>
+      <c r="P25" s="98" t="n"/>
+      <c r="Q25" s="98" t="n"/>
+      <c r="R25" s="49" t="inlineStr"/>
+    </row>
+    <row r="26">
+      <c r="A26" s="90" t="n">
+        <v>22</v>
+      </c>
+      <c r="B26" s="49" t="inlineStr">
+        <is>
+          <t>Wigge &amp; Partners</t>
+        </is>
+      </c>
+      <c r="C26" s="100" t="n">
+        <v>146</v>
+      </c>
+      <c r="D26" s="100" t="n">
+        <v>122</v>
+      </c>
+      <c r="E26" s="101">
+        <f>C26/D26-1</f>
+        <v/>
+      </c>
+      <c r="F26" s="100" t="n">
+        <v>146</v>
+      </c>
+      <c r="G26" s="49" t="inlineStr">
+        <is>
+          <t>FY2024 (Afv)</t>
+        </is>
+      </c>
+      <c r="H26" s="90" t="n">
+        <v>11</v>
+      </c>
+      <c r="I26" s="90" t="n">
+        <v>40</v>
+      </c>
+      <c r="J26" s="98" t="n"/>
+      <c r="K26" s="49" t="inlineStr">
+        <is>
+          <t>Firm website count Oct-26</t>
+        </is>
+      </c>
+      <c r="L26" s="92">
+        <f>F26/H26</f>
+        <v/>
+      </c>
+      <c r="M26" s="98" t="n"/>
+      <c r="N26" s="93">
+        <f>F26/I26</f>
+        <v/>
+      </c>
+      <c r="O26" s="98" t="n"/>
+      <c r="P26" s="101">
+        <f>H26/I26</f>
+        <v/>
+      </c>
+      <c r="Q26" s="98" t="n"/>
+      <c r="R26" s="49" t="inlineStr">
+        <is>
+          <t>Service AB (53 staff) is partial; joined AGRD Jan-26</t>
+        </is>
+      </c>
+    </row>
+    <row r="27">
+      <c r="A27" s="90" t="n">
+        <v>23</v>
+      </c>
+      <c r="B27" s="49" t="inlineStr">
+        <is>
+          <t>Gulliksson</t>
+        </is>
+      </c>
+      <c r="C27" s="100" t="n">
+        <v>141</v>
+      </c>
+      <c r="D27" s="100" t="n">
+        <v>117</v>
+      </c>
+      <c r="E27" s="101">
+        <f>C27/D27-1</f>
+        <v/>
+      </c>
+      <c r="F27" s="100" t="n">
+        <v>141</v>
+      </c>
+      <c r="G27" s="49" t="inlineStr">
+        <is>
+          <t>FY2024 (Afv)</t>
+        </is>
+      </c>
+      <c r="H27" s="98" t="n"/>
+      <c r="I27" s="90" t="n">
+        <v>41</v>
+      </c>
+      <c r="J27" s="98" t="n"/>
+      <c r="K27" s="49" t="inlineStr">
+        <is>
+          <t>Legal 500</t>
+        </is>
+      </c>
+      <c r="L27" s="98" t="n"/>
+      <c r="M27" s="98" t="n"/>
+      <c r="N27" s="93">
+        <f>F27/I27</f>
+        <v/>
+      </c>
+      <c r="O27" s="98" t="n"/>
+      <c r="P27" s="98" t="n"/>
+      <c r="Q27" s="98" t="n"/>
+      <c r="R27" s="49" t="inlineStr"/>
+    </row>
+    <row r="28">
+      <c r="A28" s="90" t="n">
+        <v>24</v>
+      </c>
+      <c r="B28" s="49" t="inlineStr">
+        <is>
+          <t>Eversheds Sutherland</t>
+        </is>
+      </c>
+      <c r="C28" s="100" t="n">
+        <v>140</v>
+      </c>
+      <c r="D28" s="100" t="n">
+        <v>148</v>
+      </c>
+      <c r="E28" s="101">
+        <f>C28/D28-1</f>
+        <v/>
+      </c>
+      <c r="F28" s="100" t="n">
+        <v>166</v>
+      </c>
+      <c r="G28" s="49" t="inlineStr">
+        <is>
+          <t>FY2025 net sales (AB)</t>
+        </is>
+      </c>
+      <c r="H28" s="98" t="n"/>
+      <c r="I28" s="98" t="n"/>
+      <c r="J28" s="90" t="n">
+        <v>59</v>
+      </c>
+      <c r="K28" s="49" t="inlineStr">
+        <is>
+          <t>2025 accounts</t>
+        </is>
+      </c>
+      <c r="L28" s="98" t="n"/>
+      <c r="M28" s="93">
+        <f>F28/J28</f>
+        <v/>
+      </c>
+      <c r="N28" s="98" t="n"/>
+      <c r="O28" s="98" t="n"/>
+      <c r="P28" s="98" t="n"/>
+      <c r="Q28" s="98" t="n"/>
+      <c r="R28" s="49" t="inlineStr"/>
+    </row>
+    <row r="29">
+      <c r="A29" s="90" t="n">
+        <v>25</v>
+      </c>
+      <c r="B29" s="49" t="inlineStr">
+        <is>
+          <t>Fylgia</t>
+        </is>
+      </c>
+      <c r="C29" s="100" t="n">
+        <v>131</v>
+      </c>
+      <c r="D29" s="100" t="n">
+        <v>120</v>
+      </c>
+      <c r="E29" s="101">
+        <f>C29/D29-1</f>
+        <v/>
+      </c>
+      <c r="F29" s="100" t="n">
+        <v>131</v>
+      </c>
+      <c r="G29" s="49" t="inlineStr">
+        <is>
+          <t>FY2024 (Afv)</t>
+        </is>
+      </c>
+      <c r="H29" s="90" t="n">
+        <v>21</v>
+      </c>
+      <c r="I29" s="90" t="n">
+        <v>35</v>
+      </c>
+      <c r="J29" s="98" t="n"/>
+      <c r="K29" s="49" t="inlineStr">
+        <is>
+          <t>Firm website count Oct-26</t>
+        </is>
+      </c>
+      <c r="L29" s="92">
+        <f>F29/H29</f>
+        <v/>
+      </c>
+      <c r="M29" s="98" t="n"/>
+      <c r="N29" s="93">
+        <f>F29/I29</f>
+        <v/>
+      </c>
+      <c r="O29" s="98" t="n"/>
+      <c r="P29" s="101">
+        <f>H29/I29</f>
+        <v/>
+      </c>
+      <c r="Q29" s="98" t="n"/>
+      <c r="R29" s="49" t="inlineStr">
+        <is>
+          <t>KB band 20-49 employees</t>
+        </is>
+      </c>
+    </row>
+    <row r="30">
+      <c r="A30" s="90" t="n">
+        <v>26</v>
+      </c>
+      <c r="B30" s="49" t="inlineStr">
+        <is>
+          <t>Kilpatrick Townsend</t>
+        </is>
+      </c>
+      <c r="C30" s="100" t="n">
+        <v>130</v>
+      </c>
+      <c r="D30" s="100" t="n">
+        <v>114</v>
+      </c>
+      <c r="E30" s="101">
+        <f>C30/D30-1</f>
+        <v/>
+      </c>
+      <c r="F30" s="100" t="n">
+        <v>130</v>
+      </c>
+      <c r="G30" s="49" t="inlineStr">
+        <is>
+          <t>FY2024 (Afv)</t>
+        </is>
+      </c>
+      <c r="H30" s="98" t="n"/>
+      <c r="I30" s="98" t="n"/>
+      <c r="J30" s="98" t="n"/>
+      <c r="K30" s="49" t="inlineStr"/>
+      <c r="L30" s="98" t="n"/>
+      <c r="M30" s="98" t="n"/>
+      <c r="N30" s="98" t="n"/>
+      <c r="O30" s="98" t="n"/>
+      <c r="P30" s="98" t="n"/>
+      <c r="Q30" s="98" t="n"/>
+      <c r="R30" s="49" t="inlineStr">
+        <is>
+          <t>AB (49 staff) is partial</t>
+        </is>
+      </c>
+    </row>
+    <row r="31">
+      <c r="A31" s="90" t="n">
+        <v>27</v>
+      </c>
+      <c r="B31" s="49" t="inlineStr">
+        <is>
+          <t>Nordia Law</t>
+        </is>
+      </c>
+      <c r="C31" s="100" t="n">
+        <v>126</v>
+      </c>
+      <c r="D31" s="100" t="n">
+        <v>126</v>
+      </c>
+      <c r="E31" s="101">
+        <f>C31/D31-1</f>
+        <v/>
+      </c>
+      <c r="F31" s="100" t="n">
+        <v>126</v>
+      </c>
+      <c r="G31" s="49" t="inlineStr">
+        <is>
+          <t>FY2024 (Afv)</t>
+        </is>
+      </c>
+      <c r="H31" s="98" t="n"/>
+      <c r="I31" s="98" t="n"/>
+      <c r="J31" s="90" t="n">
+        <v>96</v>
+      </c>
+      <c r="K31" s="49" t="inlineStr">
+        <is>
+          <t>Legal 500 ("number of staff")</t>
+        </is>
+      </c>
+      <c r="L31" s="98" t="n"/>
+      <c r="M31" s="93">
+        <f>F31/J31</f>
+        <v/>
+      </c>
+      <c r="N31" s="98" t="n"/>
+      <c r="O31" s="98" t="n"/>
+      <c r="P31" s="98" t="n"/>
+      <c r="Q31" s="98" t="n"/>
+      <c r="R31" s="49" t="inlineStr"/>
+    </row>
+    <row r="32">
+      <c r="A32" s="90" t="n">
+        <v>28</v>
+      </c>
+      <c r="B32" s="49" t="inlineStr">
+        <is>
+          <t>Kaiding</t>
+        </is>
+      </c>
+      <c r="C32" s="100" t="n">
+        <v>122</v>
+      </c>
+      <c r="D32" s="100" t="n">
+        <v>117</v>
+      </c>
+      <c r="E32" s="101">
+        <f>C32/D32-1</f>
+        <v/>
+      </c>
+      <c r="F32" s="100" t="n">
+        <v>122</v>
+      </c>
+      <c r="G32" s="49" t="inlineStr">
+        <is>
+          <t>FY24/25 (Afv)</t>
+        </is>
+      </c>
+      <c r="H32" s="98" t="n"/>
+      <c r="I32" s="98" t="n"/>
+      <c r="J32" s="98" t="n"/>
+      <c r="K32" s="49" t="inlineStr"/>
+      <c r="L32" s="98" t="n"/>
+      <c r="M32" s="98" t="n"/>
+      <c r="N32" s="98" t="n"/>
+      <c r="O32" s="98" t="n"/>
+      <c r="P32" s="98" t="n"/>
+      <c r="Q32" s="98" t="n"/>
+      <c r="R32" s="49" t="inlineStr">
+        <is>
+          <t>Headcount not researched</t>
+        </is>
+      </c>
+    </row>
+    <row r="33">
+      <c r="A33" s="90" t="n">
+        <v>29</v>
+      </c>
+      <c r="B33" s="49" t="inlineStr">
+        <is>
+          <t>Magnusson (Sweden)</t>
+        </is>
+      </c>
+      <c r="C33" s="100" t="n">
+        <v>112</v>
+      </c>
+      <c r="D33" s="100" t="n">
+        <v>124</v>
+      </c>
+      <c r="E33" s="101">
+        <f>C33/D33-1</f>
+        <v/>
+      </c>
+      <c r="F33" s="100" t="n">
+        <v>125</v>
+      </c>
+      <c r="G33" s="49" t="inlineStr">
+        <is>
+          <t>FY2025 net sales (AB)</t>
+        </is>
+      </c>
+      <c r="H33" s="90" t="n">
+        <v>13</v>
+      </c>
+      <c r="I33" s="90" t="n">
+        <v>47</v>
+      </c>
+      <c r="J33" s="90" t="n">
+        <v>46</v>
+      </c>
+      <c r="K33" s="49" t="inlineStr">
+        <is>
+          <t>Firm website count Oct-26; employees 2025 accounts</t>
+        </is>
+      </c>
+      <c r="L33" s="92">
+        <f>F33/H33</f>
+        <v/>
+      </c>
+      <c r="M33" s="93">
+        <f>F33/J33</f>
+        <v/>
+      </c>
+      <c r="N33" s="93">
+        <f>F33/I33</f>
+        <v/>
+      </c>
+      <c r="O33" s="101">
+        <f>H33/J33</f>
+        <v/>
+      </c>
+      <c r="P33" s="101">
+        <f>H33/I33</f>
+        <v/>
+      </c>
+      <c r="Q33" s="92">
+        <f>J33/H33</f>
+        <v/>
+      </c>
+      <c r="R33" s="49" t="inlineStr">
+        <is>
+          <t>Merged with Gro Advokatbyrå 1 Oct 2026 (~SEK 20m)</t>
+        </is>
+      </c>
+    </row>
+    <row r="34">
+      <c r="A34" s="90" t="n">
+        <v>30</v>
+      </c>
+      <c r="B34" s="49" t="inlineStr">
+        <is>
+          <t>Moll Wendén</t>
+        </is>
+      </c>
+      <c r="C34" s="100" t="n">
+        <v>108</v>
+      </c>
+      <c r="D34" s="100" t="n">
+        <v>89</v>
+      </c>
+      <c r="E34" s="101">
+        <f>C34/D34-1</f>
+        <v/>
+      </c>
+      <c r="F34" s="100" t="n">
+        <v>101</v>
+      </c>
+      <c r="G34" s="49" t="inlineStr">
+        <is>
+          <t>FY2025 net sales (AB)</t>
+        </is>
+      </c>
+      <c r="H34" s="90" t="n">
+        <v>8</v>
+      </c>
+      <c r="I34" s="90" t="n">
+        <v>37</v>
+      </c>
+      <c r="J34" s="90" t="n">
+        <v>44</v>
+      </c>
+      <c r="K34" s="49" t="inlineStr">
+        <is>
+          <t>Firm website count Oct-26; employees 2025 accounts</t>
+        </is>
+      </c>
+      <c r="L34" s="92">
+        <f>F34/H34</f>
+        <v/>
+      </c>
+      <c r="M34" s="93">
+        <f>F34/J34</f>
+        <v/>
+      </c>
+      <c r="N34" s="93">
+        <f>F34/I34</f>
+        <v/>
+      </c>
+      <c r="O34" s="101">
+        <f>H34/J34</f>
+        <v/>
+      </c>
+      <c r="P34" s="101">
+        <f>H34/I34</f>
+        <v/>
+      </c>
+      <c r="Q34" s="92">
+        <f>J34/H34</f>
+        <v/>
+      </c>
+      <c r="R34" s="49" t="inlineStr">
+        <is>
+          <t>Joined AGRD May-26</t>
+        </is>
+      </c>
+    </row>
+    <row r="35">
+      <c r="A35" s="90" t="inlineStr">
+        <is>
+          <t>n/r</t>
+        </is>
+      </c>
+      <c r="B35" s="49" t="inlineStr">
+        <is>
+          <t>Baker McKenzie (Stockholm)</t>
+        </is>
+      </c>
+      <c r="C35" s="100" t="n">
+        <v>334</v>
+      </c>
+      <c r="D35" s="100" t="n">
+        <v>323</v>
+      </c>
+      <c r="E35" s="101">
+        <f>C35/D35-1</f>
+        <v/>
+      </c>
+      <c r="F35" s="100" t="n">
+        <v>334</v>
+      </c>
+      <c r="G35" s="49" t="inlineStr">
+        <is>
+          <t>FY23/24 (Afv Apr-25; not in revised table)</t>
+        </is>
+      </c>
+      <c r="H35" s="90" t="n">
+        <v>12</v>
+      </c>
+      <c r="I35" s="90" t="n">
+        <v>73</v>
+      </c>
+      <c r="J35" s="90" t="n">
+        <v>125</v>
+      </c>
+      <c r="K35" s="49" t="inlineStr">
+        <is>
+          <t>Firm website count Oct-26; "~125 professionals" (Mar-26)</t>
+        </is>
+      </c>
+      <c r="L35" s="92">
+        <f>F35/H35</f>
+        <v/>
+      </c>
+      <c r="M35" s="93">
+        <f>F35/J35</f>
+        <v/>
+      </c>
+      <c r="N35" s="93">
+        <f>F35/I35</f>
+        <v/>
+      </c>
+      <c r="O35" s="101">
+        <f>H35/J35</f>
+        <v/>
+      </c>
+      <c r="P35" s="101">
+        <f>H35/I35</f>
+        <v/>
+      </c>
+      <c r="Q35" s="92">
+        <f>J35/H35</f>
+        <v/>
+      </c>
+      <c r="R35" s="49" t="inlineStr">
+        <is>
+          <t>Would rank ~14</t>
+        </is>
+      </c>
+    </row>
+    <row r="36">
+      <c r="A36" s="90" t="inlineStr">
+        <is>
+          <t>n/r</t>
+        </is>
+      </c>
+      <c r="B36" s="49" t="inlineStr">
+        <is>
+          <t>Linklaters (Stockholm)</t>
+        </is>
+      </c>
+      <c r="C36" s="100" t="n">
+        <v>195</v>
+      </c>
+      <c r="D36" s="100" t="n">
+        <v>199</v>
+      </c>
+      <c r="E36" s="101">
+        <f>C36/D36-1</f>
+        <v/>
+      </c>
+      <c r="F36" s="100" t="n">
+        <v>195</v>
+      </c>
+      <c r="G36" s="49" t="inlineStr">
+        <is>
+          <t>FY23/24 (Afv Apr-25; not in revised table)</t>
+        </is>
+      </c>
+      <c r="H36" s="98" t="n"/>
+      <c r="I36" s="98" t="n"/>
+      <c r="J36" s="90" t="n">
+        <v>75</v>
+      </c>
+      <c r="K36" s="49" t="inlineStr">
+        <is>
+          <t>AB accounts FY24/25</t>
+        </is>
+      </c>
+      <c r="L36" s="98" t="n"/>
+      <c r="M36" s="93">
+        <f>F36/J36</f>
+        <v/>
+      </c>
+      <c r="N36" s="98" t="n"/>
+      <c r="O36" s="98" t="n"/>
+      <c r="P36" s="98" t="n"/>
+      <c r="Q36" s="98" t="n"/>
+      <c r="R36" s="49" t="inlineStr">
+        <is>
+          <t>AB net sales 376 (basis unclear)</t>
+        </is>
+      </c>
+    </row>
+    <row r="37">
+      <c r="B37" s="46" t="inlineStr">
+        <is>
+          <t>Median (top 30)</t>
+        </is>
+      </c>
+      <c r="L37" s="102">
+        <f>MEDIAN(L5:L34)</f>
+        <v/>
+      </c>
+      <c r="M37" s="103">
+        <f>MEDIAN(M5:M34)</f>
+        <v/>
+      </c>
+      <c r="N37" s="103">
+        <f>MEDIAN(N5:N34)</f>
+        <v/>
+      </c>
+      <c r="O37" s="104">
+        <f>MEDIAN(O5:O34)</f>
+        <v/>
+      </c>
+      <c r="P37" s="104">
+        <f>MEDIAN(P5:P34)</f>
+        <v/>
+      </c>
+      <c r="Q37" s="102">
+        <f>MEDIAN(Q5:Q34)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="38">
+      <c r="B38" s="46" t="inlineStr">
+        <is>
+          <t>Top-30 total fee income FY2024</t>
+        </is>
+      </c>
+      <c r="C38" s="58">
+        <f>SUM(C5:C34)</f>
+        <v/>
+      </c>
+      <c r="D38" s="58">
+        <f>SUM(D5:D34)</f>
+        <v/>
+      </c>
+      <c r="E38" s="59">
+        <f>C38/D38-1</f>
+        <v/>
+      </c>
+    </row>
+    <row r="39">
+      <c r="B39" t="inlineStr">
+        <is>
+          <t>Share of Afv panel total (SEK 15,455m)</t>
+        </is>
+      </c>
+      <c r="C39" s="59">
+        <f>C38/15455</f>
+        <v/>
+      </c>
+    </row>
+    <row r="41">
+      <c r="A41" s="45" t="inlineStr">
+        <is>
+          <t>Units: SEK m; ratios in SEK m per head. Revenue per partner/employee/lawyer uses "Latest revenue" (column F).</t>
+        </is>
+      </c>
+    </row>
+    <row r="42">
+      <c r="A42" s="45" t="inlineStr">
+        <is>
+          <t>Sources: Affärsvärlden 3 Oct 2025 https://www.affarsvarlden.se/artikel/affarsjuristerna-gar-starkt-finns-fler-bolag-i-ipo-pipelinen (FY2024 table) and 12 Apr 2025 (original); company accounts via allabolag.se (Bolagsverket filings); firm websites (counted Oct-2026); Legal 500 and Chambers Europe 2026 firm-supplied figures.</t>
+        </is>
+      </c>
+    </row>
+    <row r="43">
+      <c r="A43" s="45" t="inlineStr">
+        <is>
+          <t>Gaps: total employees not found for DLA Piper, Cederquist, Schjødt (Sweden), Glimstedt (Sweden only), TM &amp; Partners, Wigge, Fylgia, AG Advokat; partner counts missing for 9 firms. Limited partnerships (KB) file no public accounts.</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+  <mergeCells count="1">
+    <mergeCell ref="A2:R2"/>
+  </mergeCells>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet8.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
   <dimension ref="A1:R55"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
@@ -32154,7 +34331,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet8.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet9.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
     <outlinePr summaryBelow="1" summaryRight="1"/>

</xml_diff>

<commit_message>
Add Section F: M&A, PE roll-ups and team lifts 2020-2026; correct G&D team move date
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01Tu61bPEQej1E6sErbEFanY
</commit_message>
<xml_diff>
--- a/research/swedish_legal_market.xlsx
+++ b/research/swedish_legal_market.xlsx
@@ -16,6 +16,7 @@
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="C. Benchmarking" sheetId="7" state="visible" r:id="rId7"/>
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="D. Rate cards" sheetId="8" state="visible" r:id="rId8"/>
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="E. Partner compensation" sheetId="9" state="visible" r:id="rId9"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="F. M&amp;A &amp; team lifts" sheetId="10" state="visible" r:id="rId10"/>
   </sheets>
   <definedNames>
     <definedName name="_xlnm._FilterDatabase" localSheetId="5" hidden="1">'B. Rankings raw'!$A$1:$E$661</definedName>
@@ -68,7 +69,7 @@
       <sz val="9"/>
     </font>
   </fonts>
-  <fills count="10">
+  <fills count="11">
     <fill>
       <patternFill/>
     </fill>
@@ -113,6 +114,11 @@
     <fill>
       <patternFill patternType="solid">
         <fgColor rgb="00F2F2F2"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="00DDEBF7"/>
       </patternFill>
     </fill>
   </fills>
@@ -362,7 +368,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="105">
+  <cellXfs count="112">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
@@ -635,6 +641,25 @@
     </xf>
     <xf numFmtId="9" fontId="5" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="10" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="8" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="top"/>
+    </xf>
+    <xf numFmtId="3" fontId="0" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="top"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="5" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="top"/>
     </xf>
   </cellXfs>
   <cellStyles count="1">
@@ -1004,11 +1029,11 @@
   <dimension ref="A1:E24"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
-    <col width="58" customWidth="1" min="1" max="1"/>
-    <col width="40" customWidth="1" min="2" max="2"/>
-    <col width="20" customWidth="1" min="3" max="3"/>
-    <col width="24" customWidth="1" min="4" max="4"/>
-    <col width="20" customWidth="1" min="5" max="5"/>
+    <col width="58" customWidth="1" style="108" min="1" max="1"/>
+    <col width="40" customWidth="1" style="108" min="2" max="2"/>
+    <col width="20" customWidth="1" style="108" min="3" max="3"/>
+    <col width="24" customWidth="1" style="108" min="4" max="4"/>
+    <col width="20" customWidth="1" style="108" min="5" max="5"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -1395,6 +1420,2249 @@
       </c>
     </row>
   </sheetData>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet10.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:J91"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="18" customWidth="1" style="108" min="1" max="1"/>
+    <col width="22" customWidth="1" style="108" min="2" max="2"/>
+    <col width="26" customWidth="1" style="108" min="3" max="3"/>
+    <col width="28" customWidth="1" style="108" min="4" max="4"/>
+    <col width="14" customWidth="1" style="108" min="5" max="5"/>
+    <col width="22" customWidth="1" style="108" min="6" max="6"/>
+    <col width="26" customWidth="1" style="108" min="7" max="7"/>
+    <col width="40" customWidth="1" style="108" min="8" max="8"/>
+    <col width="50" customWidth="1" style="108" min="9" max="9"/>
+  </cols>
+  <sheetData>
+    <row r="1">
+      <c r="A1" s="1" t="inlineStr">
+        <is>
+          <t>Section F. Consolidation and team lifts: Swedish business law, Jan 2020 - Oct 2026</t>
+        </is>
+      </c>
+    </row>
+    <row r="2" ht="45" customHeight="1" s="108">
+      <c r="A2" s="2" t="inlineStr">
+        <is>
+          <t>Team lift = 2+ partners or 5+ lawyers moving together from one firm within ~12 months. Dates from article metadata (search-index dates are unreliable). Sources: Realtid, Dagens Juridik (paywalled: headline/lead only), Affärsvärlden, Advokatbladet, Legal 500 2026 firm pages, firm press releases. "1-src" = single source. Coverage of 2020-2023 is thinner (Legal 500 reflects ~2024-26; international legal press paywalled).</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" s="47" t="inlineStr">
+        <is>
+          <t>F1. Mergers, acquisitions, PE roll-ups, market entries and splits</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" s="52" t="inlineStr">
+        <is>
+          <t>Date (announced / effective)</t>
+        </is>
+      </c>
+      <c r="B5" s="52" t="inlineStr">
+        <is>
+          <t>Type</t>
+        </is>
+      </c>
+      <c r="C5" s="52" t="inlineStr">
+        <is>
+          <t>Acquirer / surviving firm</t>
+        </is>
+      </c>
+      <c r="D5" s="52" t="inlineStr">
+        <is>
+          <t>Target / source</t>
+        </is>
+      </c>
+      <c r="E5" s="52" t="inlineStr">
+        <is>
+          <t>Partners</t>
+        </is>
+      </c>
+      <c r="F5" s="52" t="inlineStr">
+        <is>
+          <t>People</t>
+        </is>
+      </c>
+      <c r="G5" s="52" t="inlineStr">
+        <is>
+          <t>Practice / office</t>
+        </is>
+      </c>
+      <c r="H5" s="52" t="inlineStr">
+        <is>
+          <t>Notes</t>
+        </is>
+      </c>
+      <c r="I5" s="52" t="inlineStr">
+        <is>
+          <t>Source</t>
+        </is>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" s="105" t="inlineStr">
+        <is>
+          <t>Oct-2019 / Jan-2020</t>
+        </is>
+      </c>
+      <c r="B6" s="105" t="inlineStr">
+        <is>
+          <t>Market entry (merger)</t>
+        </is>
+      </c>
+      <c r="C6" s="105" t="inlineStr">
+        <is>
+          <t>Schjødt (Norway)</t>
+        </is>
+      </c>
+      <c r="D6" s="105" t="inlineStr">
+        <is>
+          <t>Hamilton Advokatbyrå</t>
+        </is>
+      </c>
+      <c r="E6" s="105" t="inlineStr"/>
+      <c r="F6" s="105" t="inlineStr">
+        <is>
+          <t>~65 lawyers</t>
+        </is>
+      </c>
+      <c r="G6" s="105" t="inlineStr">
+        <is>
+          <t>Full service, Stockholm</t>
+        </is>
+      </c>
+      <c r="H6" s="105" t="inlineStr">
+        <is>
+          <t>Hamilton 2018 revenue SEK 215m; Norwegian-Swedish one-stop shop</t>
+        </is>
+      </c>
+      <c r="I6" s="105" t="inlineStr">
+        <is>
+          <t>realtid.se/bors-finans/hamilton-gar-ihop-med-norska-byran-schjodt/</t>
+        </is>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" s="49" t="inlineStr">
+        <is>
+          <t>Jan-2020</t>
+        </is>
+      </c>
+      <c r="B7" s="49" t="inlineStr">
+        <is>
+          <t>Merger</t>
+        </is>
+      </c>
+      <c r="C7" s="49" t="inlineStr">
+        <is>
+          <t>Time Danowsky</t>
+        </is>
+      </c>
+      <c r="D7" s="49" t="inlineStr">
+        <is>
+          <t>Time Advokatbyrå + Danowsky &amp; Partners</t>
+        </is>
+      </c>
+      <c r="E7" s="49" t="inlineStr"/>
+      <c r="F7" s="49" t="inlineStr">
+        <is>
+          <t>27 staff combined</t>
+        </is>
+      </c>
+      <c r="G7" s="49" t="inlineStr">
+        <is>
+          <t>Tech, media</t>
+        </is>
+      </c>
+      <c r="H7" s="49" t="inlineStr">
+        <is>
+          <t>1-src</t>
+        </is>
+      </c>
+      <c r="I7" s="49" t="inlineStr">
+        <is>
+          <t>realtid.se/bors-finans/advokatbyran-time-danowsky-bildas-efter-sammanslagning/</t>
+        </is>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" s="106" t="inlineStr">
+        <is>
+          <t>Nov-2021 / Jan-2022</t>
+        </is>
+      </c>
+      <c r="B8" s="106" t="inlineStr">
+        <is>
+          <t>Split / exit</t>
+        </is>
+      </c>
+      <c r="C8" s="106" t="inlineStr">
+        <is>
+          <t>Born Advokater (Sthlm); Norma Advokater (Gbg)</t>
+        </is>
+      </c>
+      <c r="D8" s="106" t="inlineStr">
+        <is>
+          <t>Glimstedt Stockholm and Göteborg offices</t>
+        </is>
+      </c>
+      <c r="E8" s="106" t="inlineStr"/>
+      <c r="F8" s="106" t="inlineStr"/>
+      <c r="G8" s="106" t="inlineStr">
+        <is>
+          <t>Banking &amp; finance, real estate, M&amp;A</t>
+        </is>
+      </c>
+      <c r="H8" s="106" t="inlineStr">
+        <is>
+          <t>Offices left Glimstedt brand; Born later a founding AGRD firm. 1-src</t>
+        </is>
+      </c>
+      <c r="I8" s="106" t="inlineStr">
+        <is>
+          <t>realtid.se/bors-finans/glimstedt-renodlar-verksamheten/</t>
+        </is>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" s="105" t="inlineStr">
+        <is>
+          <t>Nov-2023 / Mar-2024</t>
+        </is>
+      </c>
+      <c r="B9" s="105" t="inlineStr">
+        <is>
+          <t>Market entry (membership)</t>
+        </is>
+      </c>
+      <c r="C9" s="105" t="inlineStr">
+        <is>
+          <t>CMS</t>
+        </is>
+      </c>
+      <c r="D9" s="105" t="inlineStr">
+        <is>
+          <t>Wistrand (now CMS Wistrand)</t>
+        </is>
+      </c>
+      <c r="E9" s="105" t="inlineStr"/>
+      <c r="F9" s="105" t="inlineStr">
+        <is>
+          <t>~150 lawyers</t>
+        </is>
+      </c>
+      <c r="G9" s="105" t="inlineStr">
+        <is>
+          <t>Stockholm, Göteborg; full service</t>
+        </is>
+      </c>
+      <c r="H9" s="105" t="inlineStr">
+        <is>
+          <t>Joins 5,800-lawyer network; cross-border deal growth</t>
+        </is>
+      </c>
+      <c r="I9" s="105" t="inlineStr">
+        <is>
+          <t>dagensjuridik.se/nyheter/wistrand-blir-en-del-av-cms-gar-fran-150-jurister-till-5-800-varlden-over/</t>
+        </is>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" s="49" t="inlineStr">
+        <is>
+          <t>Feb-2024</t>
+        </is>
+      </c>
+      <c r="B10" s="49" t="inlineStr">
+        <is>
+          <t>Merger</t>
+        </is>
+      </c>
+      <c r="C10" s="49" t="inlineStr">
+        <is>
+          <t>Carthiel</t>
+        </is>
+      </c>
+      <c r="D10" s="49" t="inlineStr">
+        <is>
+          <t>Grey Advokatbyrå</t>
+        </is>
+      </c>
+      <c r="E10" s="49" t="inlineStr"/>
+      <c r="F10" s="49" t="inlineStr">
+        <is>
+          <t>~10 staff combined</t>
+        </is>
+      </c>
+      <c r="G10" s="49" t="inlineStr">
+        <is>
+          <t>Disputes added</t>
+        </is>
+      </c>
+      <c r="H10" s="49" t="inlineStr">
+        <is>
+          <t>Carthiel grew +155% (FY2024). Firm release only (1-src)</t>
+        </is>
+      </c>
+      <c r="I10" s="49" t="inlineStr">
+        <is>
+          <t>carthiel.se/post/advokatfirman-carthiel-går-ihop-med-grey-advokatbyrå</t>
+        </is>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" s="106" t="inlineStr">
+        <is>
+          <t>Feb / Mar-2024</t>
+        </is>
+      </c>
+      <c r="B11" s="106" t="inlineStr">
+        <is>
+          <t>Split / exit</t>
+        </is>
+      </c>
+      <c r="C11" s="106" t="inlineStr">
+        <is>
+          <t>Hannes Snellman Sweden (now "Snellman")</t>
+        </is>
+      </c>
+      <c r="D11" s="106" t="inlineStr">
+        <is>
+          <t>Hannes Snellman group (Finland)</t>
+        </is>
+      </c>
+      <c r="E11" s="106" t="inlineStr"/>
+      <c r="F11" s="106" t="inlineStr">
+        <is>
+          <t>&gt;80 lawyers (Sthlm)</t>
+        </is>
+      </c>
+      <c r="G11" s="106" t="inlineStr">
+        <is>
+          <t>Stockholm</t>
+        </is>
+      </c>
+      <c r="H11" s="106" t="inlineStr">
+        <is>
+          <t>Helsinki and Stockholm strategies diverged</t>
+        </is>
+      </c>
+      <c r="I11" s="106" t="inlineStr">
+        <is>
+          <t>dagensjuridik.se/nyheter/snellmans-nya-mp-stora-strategiska-fragor-for-branschen/</t>
+        </is>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" s="106" t="inlineStr">
+        <is>
+          <t>Mar-2024</t>
+        </is>
+      </c>
+      <c r="B12" s="106" t="inlineStr">
+        <is>
+          <t>Split / exit</t>
+        </is>
+      </c>
+      <c r="C12" s="106" t="inlineStr">
+        <is>
+          <t>(bankruptcy)</t>
+        </is>
+      </c>
+      <c r="D12" s="106" t="inlineStr">
+        <is>
+          <t>Front Advokater</t>
+        </is>
+      </c>
+      <c r="E12" s="106" t="inlineStr"/>
+      <c r="F12" s="106" t="inlineStr"/>
+      <c r="G12" s="106" t="inlineStr">
+        <is>
+          <t>Göteborg</t>
+        </is>
+      </c>
+      <c r="H12" s="106" t="inlineStr">
+        <is>
+          <t>Bankrupt after losing case vs City of Göteborg. 1-src</t>
+        </is>
+      </c>
+      <c r="I12" s="106" t="inlineStr">
+        <is>
+          <t>dagensjuridik.se/nyheter/efter-forlusten-i-domstol-front-advokater-i-konkurs/</t>
+        </is>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" s="69" t="inlineStr">
+        <is>
+          <t>Aug-2025</t>
+        </is>
+      </c>
+      <c r="B13" s="69" t="inlineStr">
+        <is>
+          <t>PE roll-up (formation)</t>
+        </is>
+      </c>
+      <c r="C13" s="69" t="inlineStr">
+        <is>
+          <t>AGRD Partners (Axcel)</t>
+        </is>
+      </c>
+      <c r="D13" s="69" t="inlineStr">
+        <is>
+          <t>Allié, Born, Morris Law, Next, Synch, TM &amp; Partners</t>
+        </is>
+      </c>
+      <c r="E13" s="69" t="inlineStr"/>
+      <c r="F13" s="69" t="inlineStr">
+        <is>
+          <t>~250 staff, 8 offices; ~100-130 advokater left the Bar</t>
+        </is>
+      </c>
+      <c r="G13" s="69" t="inlineStr">
+        <is>
+          <t>Business law</t>
+        </is>
+      </c>
+      <c r="H13" s="69" t="inlineStr">
+        <is>
+          <t>Revenue ~SEK 660m (top-10). Firms keep names. CEO Maria-Pia Hope (ex-Vinge)</t>
+        </is>
+      </c>
+      <c r="I13" s="69" t="inlineStr">
+        <is>
+          <t>realtid.se/juridik/massavhopp-fran-advokatsamfundet-nar-ny-jattebyra-bildas/</t>
+        </is>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" s="105" t="inlineStr">
+        <is>
+          <t>Oct-2025 / Jan-2026</t>
+        </is>
+      </c>
+      <c r="B14" s="105" t="inlineStr">
+        <is>
+          <t>Market entry (team lift)</t>
+        </is>
+      </c>
+      <c r="C14" s="105" t="inlineStr">
+        <is>
+          <t>BAHR (Norway)</t>
+        </is>
+      </c>
+      <c r="D14" s="105" t="inlineStr">
+        <is>
+          <t>Schjødt (Oslo and Stockholm)</t>
+        </is>
+      </c>
+      <c r="E14" s="105" t="inlineStr">
+        <is>
+          <t>8 (Sweden); 23 group-wide</t>
+        </is>
+      </c>
+      <c r="F14" s="105" t="inlineStr">
+        <is>
+          <t>~20 of ~30 Stockholm opening staff; 54 people group-wide</t>
+        </is>
+      </c>
+      <c r="G14" s="105" t="inlineStr">
+        <is>
+          <t>M&amp;A, banking, capital markets</t>
+        </is>
+      </c>
+      <c r="H14" s="105" t="inlineStr">
+        <is>
+          <t>Targets 100+ lawyers in Stockholm; ~50 Stockholm staff by Feb-2026</t>
+        </is>
+      </c>
+      <c r="I14" s="105" t="inlineStr">
+        <is>
+          <t>dagensjuridik.se/nyheter/schjodt-skakas-av-avhopp-atta-i-stockholm-lamnar/</t>
+        </is>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" s="69" t="inlineStr">
+        <is>
+          <t>Jan-2026</t>
+        </is>
+      </c>
+      <c r="B15" s="69" t="inlineStr">
+        <is>
+          <t>PE roll-up (add-on)</t>
+        </is>
+      </c>
+      <c r="C15" s="69" t="inlineStr">
+        <is>
+          <t>AGRD Partners</t>
+        </is>
+      </c>
+      <c r="D15" s="69" t="inlineStr">
+        <is>
+          <t>Wigge &amp; Partners; Bokwall Rislund</t>
+        </is>
+      </c>
+      <c r="E15" s="69" t="inlineStr"/>
+      <c r="F15" s="69" t="inlineStr"/>
+      <c r="G15" s="69" t="inlineStr">
+        <is>
+          <t>Transactions/PE; competition &amp; procurement</t>
+        </is>
+      </c>
+      <c r="H15" s="69" t="inlineStr">
+        <is>
+          <t>First add-ons; both left the Bar</t>
+        </is>
+      </c>
+      <c r="I15" s="69" t="inlineStr">
+        <is>
+          <t>dagensjuridik.se/nyheter/agrd-vaxer-tva-nya-byraer-gar-med/</t>
+        </is>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" s="69" t="inlineStr">
+        <is>
+          <t>May-2026</t>
+        </is>
+      </c>
+      <c r="B16" s="69" t="inlineStr">
+        <is>
+          <t>PE roll-up (add-on)</t>
+        </is>
+      </c>
+      <c r="C16" s="69" t="inlineStr">
+        <is>
+          <t>AGRD Partners</t>
+        </is>
+      </c>
+      <c r="D16" s="69" t="inlineStr">
+        <is>
+          <t>BBA//Fjeldco (Iceland)</t>
+        </is>
+      </c>
+      <c r="E16" s="69" t="inlineStr"/>
+      <c r="F16" s="69" t="inlineStr"/>
+      <c r="G16" s="69" t="inlineStr">
+        <is>
+          <t>Iceland</t>
+        </is>
+      </c>
+      <c r="H16" s="69" t="inlineStr">
+        <is>
+          <t>First non-Swedish investment (context)</t>
+        </is>
+      </c>
+      <c r="I16" s="69" t="inlineStr">
+        <is>
+          <t>dagensjuridik.se/nyheter/agrd-expanderar-till-island/</t>
+        </is>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" s="69" t="inlineStr">
+        <is>
+          <t>May-2026</t>
+        </is>
+      </c>
+      <c r="B17" s="69" t="inlineStr">
+        <is>
+          <t>PE roll-up (add-on)</t>
+        </is>
+      </c>
+      <c r="C17" s="69" t="inlineStr">
+        <is>
+          <t>AGRD Partners</t>
+        </is>
+      </c>
+      <c r="D17" s="69" t="inlineStr">
+        <is>
+          <t>Moll Wendén (Malmö)</t>
+        </is>
+      </c>
+      <c r="E17" s="69" t="inlineStr">
+        <is>
+          <t>8</t>
+        </is>
+      </c>
+      <c r="F17" s="69" t="inlineStr">
+        <is>
+          <t>~47 staff</t>
+        </is>
+      </c>
+      <c r="G17" s="69" t="inlineStr">
+        <is>
+          <t>Malmö, 15 practice areas</t>
+        </is>
+      </c>
+      <c r="H17" s="69" t="inlineStr">
+        <is>
+          <t>First deal in southern Sweden; Öresund strategy</t>
+        </is>
+      </c>
+      <c r="I17" s="69" t="inlineStr">
+        <is>
+          <t>dagensjuridik.se/nyheter/moll-wenden-gar-in-i-agrd/</t>
+        </is>
+      </c>
+    </row>
+    <row r="18">
+      <c r="A18" s="106" t="inlineStr">
+        <is>
+          <t>Aug-2026 / Jan-2027</t>
+        </is>
+      </c>
+      <c r="B18" s="106" t="inlineStr">
+        <is>
+          <t>Split / exit</t>
+        </is>
+      </c>
+      <c r="C18" s="106" t="inlineStr">
+        <is>
+          <t>MAQS KB (Malmö, keeps brand) / Keelion Law (Sthlm, Gbg, Sundsvall)</t>
+        </is>
+      </c>
+      <c r="D18" s="106" t="inlineStr">
+        <is>
+          <t>MAQS</t>
+        </is>
+      </c>
+      <c r="E18" s="106" t="inlineStr"/>
+      <c r="F18" s="106" t="inlineStr"/>
+      <c r="G18" s="106" t="inlineStr">
+        <is>
+          <t>Malmö vs northern offices</t>
+        </is>
+      </c>
+      <c r="H18" s="106" t="inlineStr">
+        <is>
+          <t>Amicable; Malmö plans AI-forward premium firm</t>
+        </is>
+      </c>
+      <c r="I18" s="106" t="inlineStr">
+        <is>
+          <t>realtid.se/juridik/advokatbyra-delas-malmo-bryter-sig-loss/</t>
+        </is>
+      </c>
+    </row>
+    <row r="19">
+      <c r="A19" s="69" t="inlineStr">
+        <is>
+          <t>Aug-2026</t>
+        </is>
+      </c>
+      <c r="B19" s="69" t="inlineStr">
+        <is>
+          <t>PE roll-up (add-on)</t>
+        </is>
+      </c>
+      <c r="C19" s="69" t="inlineStr">
+        <is>
+          <t>Synch (AGRD)</t>
+        </is>
+      </c>
+      <c r="D19" s="69" t="inlineStr">
+        <is>
+          <t>Qap Legal Advisors</t>
+        </is>
+      </c>
+      <c r="E19" s="69" t="inlineStr"/>
+      <c r="F19" s="69" t="inlineStr">
+        <is>
+          <t>All Qap staff</t>
+        </is>
+      </c>
+      <c r="G19" s="69" t="inlineStr">
+        <is>
+          <t>Stockholm boutique</t>
+        </is>
+      </c>
+      <c r="H19" s="69" t="inlineStr">
+        <is>
+          <t>Synch "open to more acquisitions". 1-src</t>
+        </is>
+      </c>
+      <c r="I19" s="69" t="inlineStr">
+        <is>
+          <t>dagensjuridik.se/nyheter/synch-och-qap-legal-gar-ihop/</t>
+        </is>
+      </c>
+    </row>
+    <row r="20">
+      <c r="A20" s="49" t="inlineStr">
+        <is>
+          <t>Aug-2026</t>
+        </is>
+      </c>
+      <c r="B20" s="49" t="inlineStr">
+        <is>
+          <t>Merger</t>
+        </is>
+      </c>
+      <c r="C20" s="49" t="inlineStr">
+        <is>
+          <t>MAQS Malmö</t>
+        </is>
+      </c>
+      <c r="D20" s="49" t="inlineStr">
+        <is>
+          <t>Fredersen Advokatbyrå</t>
+        </is>
+      </c>
+      <c r="E20" s="49" t="inlineStr"/>
+      <c r="F20" s="49" t="inlineStr"/>
+      <c r="G20" s="49" t="inlineStr">
+        <is>
+          <t>Malmö</t>
+        </is>
+      </c>
+      <c r="H20" s="49" t="inlineStr">
+        <is>
+          <t>Ahead of MAQS separation. 1-src</t>
+        </is>
+      </c>
+      <c r="I20" s="49" t="inlineStr">
+        <is>
+          <t>dagensjuridik.se/nyheter/fredersen-gar-ihop-med-maqs-i-malmo/</t>
+        </is>
+      </c>
+    </row>
+    <row r="21">
+      <c r="A21" s="69" t="inlineStr">
+        <is>
+          <t>Sep-2026</t>
+        </is>
+      </c>
+      <c r="B21" s="69" t="inlineStr">
+        <is>
+          <t>PE roll-up (add-on)</t>
+        </is>
+      </c>
+      <c r="C21" s="69" t="inlineStr">
+        <is>
+          <t>AGRD Partners (as Ascente Law)</t>
+        </is>
+      </c>
+      <c r="D21" s="69" t="inlineStr">
+        <is>
+          <t>Setterwalls Malmö office</t>
+        </is>
+      </c>
+      <c r="E21" s="69" t="inlineStr">
+        <is>
+          <t>12</t>
+        </is>
+      </c>
+      <c r="F21" s="69" t="inlineStr">
+        <is>
+          <t>~100 people</t>
+        </is>
+      </c>
+      <c r="G21" s="69" t="inlineStr">
+        <is>
+          <t>Malmö; corporate, energy, patent litigation</t>
+        </is>
+      </c>
+      <c r="H21" s="69" t="inlineStr">
+        <is>
+          <t>AGRD's largest deal; office leaves the Bar (~SEK 305m revenue in 2025)</t>
+        </is>
+      </c>
+      <c r="I21" s="69" t="inlineStr">
+        <is>
+          <t>realtid.se/juridik/setterwalls-malmokontor-gar-till-riskkapitalagda-agrd/</t>
+        </is>
+      </c>
+    </row>
+    <row r="22">
+      <c r="A22" s="49" t="inlineStr">
+        <is>
+          <t>Sep / Oct-2026</t>
+        </is>
+      </c>
+      <c r="B22" s="49" t="inlineStr">
+        <is>
+          <t>Merger</t>
+        </is>
+      </c>
+      <c r="C22" s="49" t="inlineStr">
+        <is>
+          <t>Magnusson</t>
+        </is>
+      </c>
+      <c r="D22" s="49" t="inlineStr">
+        <is>
+          <t>Gro Advokatbyrå</t>
+        </is>
+      </c>
+      <c r="E22" s="49" t="inlineStr"/>
+      <c r="F22" s="49" t="inlineStr">
+        <is>
+          <t>&lt;10 staff, ~SEK 20m revenue</t>
+        </is>
+      </c>
+      <c r="G22" s="49" t="inlineStr">
+        <is>
+          <t>VC, tech, data protection; Stockholm</t>
+        </is>
+      </c>
+      <c r="H22" s="49" t="inlineStr">
+        <is>
+          <t>Positioned as a commitment to the advokat model (vs AGRD)</t>
+        </is>
+      </c>
+      <c r="I22" s="49" t="inlineStr">
+        <is>
+          <t>realtid.se/juridik/byraer-gar-samman-fortsatter-satsa-pa-advokatmodellen/</t>
+        </is>
+      </c>
+    </row>
+    <row r="23">
+      <c r="A23" s="49" t="inlineStr">
+        <is>
+          <t>Oct-2026 / Jan-2027</t>
+        </is>
+      </c>
+      <c r="B23" s="49" t="inlineStr">
+        <is>
+          <t>Merger</t>
+        </is>
+      </c>
+      <c r="C23" s="49" t="inlineStr">
+        <is>
+          <t>Walthon Ramberg</t>
+        </is>
+      </c>
+      <c r="D23" s="49" t="inlineStr">
+        <is>
+          <t>Walthon Advokater + Ramberg Advokater</t>
+        </is>
+      </c>
+      <c r="E23" s="49" t="inlineStr"/>
+      <c r="F23" s="49" t="inlineStr">
+        <is>
+          <t>~40 lawyers</t>
+        </is>
+      </c>
+      <c r="G23" s="49" t="inlineStr">
+        <is>
+          <t>Transactions, disputes, insolvency; Stockholm</t>
+        </is>
+      </c>
+      <c r="H23" s="49" t="inlineStr">
+        <is>
+          <t>1-src outlet</t>
+        </is>
+      </c>
+      <c r="I23" s="49" t="inlineStr">
+        <is>
+          <t>dagensjuridik.se/nyheter/walthon-och-ramberg-gar-ihop-samlar-40-jurister/</t>
+        </is>
+      </c>
+    </row>
+    <row r="24">
+      <c r="A24" s="45" t="inlineStr">
+        <is>
+          <t>Colour: yellow = PE roll-up; blue = market entry; orange = split / exit. Context: Schjødt merged with Norrbom Vinding (Denmark, Jan-2026); Advokatsamfundet reviewing its ownership rules after AGRD.</t>
+        </is>
+      </c>
+    </row>
+    <row r="26">
+      <c r="A26" s="47" t="inlineStr">
+        <is>
+          <t>F2. Team lifts (2+ partners or 5+ lawyers)</t>
+        </is>
+      </c>
+    </row>
+    <row r="27">
+      <c r="A27" s="52" t="inlineStr">
+        <is>
+          <t>Date</t>
+        </is>
+      </c>
+      <c r="B27" s="52" t="inlineStr">
+        <is>
+          <t>Hiring firm</t>
+        </is>
+      </c>
+      <c r="C27" s="52" t="inlineStr">
+        <is>
+          <t>Source firm</t>
+        </is>
+      </c>
+      <c r="D27" s="52" t="inlineStr">
+        <is>
+          <t>Partners</t>
+        </is>
+      </c>
+      <c r="E27" s="52" t="inlineStr">
+        <is>
+          <t>Other lawyers / staff</t>
+        </is>
+      </c>
+      <c r="F27" s="52" t="inlineStr">
+        <is>
+          <t>Practice</t>
+        </is>
+      </c>
+      <c r="G27" s="52" t="inlineStr">
+        <is>
+          <t>Partner names</t>
+        </is>
+      </c>
+      <c r="H27" s="52" t="inlineStr">
+        <is>
+          <t>Confidence</t>
+        </is>
+      </c>
+      <c r="I27" s="52" t="inlineStr">
+        <is>
+          <t>Source</t>
+        </is>
+      </c>
+    </row>
+    <row r="28">
+      <c r="A28" s="49" t="inlineStr">
+        <is>
+          <t>Feb-2020</t>
+        </is>
+      </c>
+      <c r="B28" s="49" t="inlineStr">
+        <is>
+          <t>Lindahl (new Stockholm office)</t>
+        </is>
+      </c>
+      <c r="C28" s="49" t="inlineStr">
+        <is>
+          <t>Westermark Anjou</t>
+        </is>
+      </c>
+      <c r="D28" s="49" t="n">
+        <v>2</v>
+      </c>
+      <c r="E28" s="49" t="n">
+        <v>2</v>
+      </c>
+      <c r="F28" s="49" t="inlineStr">
+        <is>
+          <t>Capital markets / public M&amp;A</t>
+        </is>
+      </c>
+      <c r="G28" s="49" t="inlineStr">
+        <is>
+          <t>Monica Lagercrantz, Dennis Westermark</t>
+        </is>
+      </c>
+      <c r="H28" s="49" t="inlineStr">
+        <is>
+          <t>Medium (firm release)</t>
+        </is>
+      </c>
+      <c r="I28" s="49" t="inlineStr">
+        <is>
+          <t>dagensjuridik.se/pressrum/lindahl/advokatfirman-lindahl-vaxer-i-stockholm-tva-nya-delagare-och-tva-jurister-2/</t>
+        </is>
+      </c>
+    </row>
+    <row r="29">
+      <c r="A29" s="49" t="inlineStr">
+        <is>
+          <t>Jan-Mar-2020</t>
+        </is>
+      </c>
+      <c r="B29" s="49" t="inlineStr">
+        <is>
+          <t>Fylgia</t>
+        </is>
+      </c>
+      <c r="C29" s="49" t="inlineStr">
+        <is>
+          <t>Setterwalls</t>
+        </is>
+      </c>
+      <c r="D29" s="49" t="inlineStr">
+        <is>
+          <t>1+</t>
+        </is>
+      </c>
+      <c r="E29" s="49" t="n">
+        <v>3</v>
+      </c>
+      <c r="F29" s="49" t="inlineStr">
+        <is>
+          <t>Insolvency / restructuring</t>
+        </is>
+      </c>
+      <c r="G29" s="49" t="inlineStr">
+        <is>
+          <t>Mathias Winge (+3, titles unstated)</t>
+        </is>
+      </c>
+      <c r="H29" s="49" t="inlineStr">
+        <is>
+          <t>Medium (1-src; borderline)</t>
+        </is>
+      </c>
+      <c r="I29" s="49" t="inlineStr">
+        <is>
+          <t>realtid.se/bors-finans/fylgia-tar-over-obestandsavdelningen-fran-setterwalls/</t>
+        </is>
+      </c>
+    </row>
+    <row r="30">
+      <c r="A30" s="49" t="inlineStr">
+        <is>
+          <t>Jan-2024</t>
+        </is>
+      </c>
+      <c r="B30" s="49" t="inlineStr">
+        <is>
+          <t>MAQS</t>
+        </is>
+      </c>
+      <c r="C30" s="49" t="inlineStr">
+        <is>
+          <t>Delphi</t>
+        </is>
+      </c>
+      <c r="D30" s="49" t="n">
+        <v>3</v>
+      </c>
+      <c r="E30" s="49" t="inlineStr"/>
+      <c r="F30" s="49" t="inlineStr">
+        <is>
+          <t>M&amp;A</t>
+        </is>
+      </c>
+      <c r="G30" s="49" t="inlineStr">
+        <is>
+          <t>Anders Lindström, Per Lagerkvist, Fredrik Mörner</t>
+        </is>
+      </c>
+      <c r="H30" s="49" t="inlineStr">
+        <is>
+          <t>Medium (1-src)</t>
+        </is>
+      </c>
+      <c r="I30" s="49" t="inlineStr">
+        <is>
+          <t>realtid.se/juridik/tre-nya-delagare-inom-ma-ansluter-till-maqs/</t>
+        </is>
+      </c>
+    </row>
+    <row r="31">
+      <c r="A31" s="49" t="inlineStr">
+        <is>
+          <t>Apr-2024</t>
+        </is>
+      </c>
+      <c r="B31" s="49" t="inlineStr">
+        <is>
+          <t>RE:FI STHLM (new boutique)</t>
+        </is>
+      </c>
+      <c r="C31" s="49" t="inlineStr">
+        <is>
+          <t>Cederquist</t>
+        </is>
+      </c>
+      <c r="D31" s="49" t="inlineStr">
+        <is>
+          <t>1+ (4 partners at new firm)</t>
+        </is>
+      </c>
+      <c r="E31" s="49" t="inlineStr">
+        <is>
+          <t>3</t>
+        </is>
+      </c>
+      <c r="F31" s="49" t="inlineStr">
+        <is>
+          <t>Banking / finance / restructuring</t>
+        </is>
+      </c>
+      <c r="G31" s="49" t="inlineStr">
+        <is>
+          <t>Johan Lundberg (ex-MP)</t>
+        </is>
+      </c>
+      <c r="H31" s="49" t="inlineStr">
+        <is>
+          <t>Medium</t>
+        </is>
+      </c>
+      <c r="I31" s="49" t="inlineStr">
+        <is>
+          <t>dagensjuridik.se/nyheter/finansieringsexpert-pa-cederquist-lanserar-egen-specialistbyra/</t>
+        </is>
+      </c>
+    </row>
+    <row r="32">
+      <c r="A32" s="49" t="inlineStr">
+        <is>
+          <t>Jun-2024</t>
+        </is>
+      </c>
+      <c r="B32" s="49" t="inlineStr">
+        <is>
+          <t>Gernandt &amp; Danielsson</t>
+        </is>
+      </c>
+      <c r="C32" s="49" t="inlineStr">
+        <is>
+          <t>Linklaters Stockholm</t>
+        </is>
+      </c>
+      <c r="D32" s="49" t="n">
+        <v>2</v>
+      </c>
+      <c r="E32" s="49" t="n">
+        <v>5</v>
+      </c>
+      <c r="F32" s="49" t="inlineStr">
+        <is>
+          <t>Real estate transactions</t>
+        </is>
+      </c>
+      <c r="G32" s="49" t="inlineStr">
+        <is>
+          <t>Magnus Lidman, Anna Eriksson</t>
+        </is>
+      </c>
+      <c r="H32" s="49" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
+      <c r="I32" s="49" t="inlineStr">
+        <is>
+          <t>mynewsdesk.com/se/gernandtdanielsson</t>
+        </is>
+      </c>
+    </row>
+    <row r="33">
+      <c r="A33" s="49" t="inlineStr">
+        <is>
+          <t>Jan-2025</t>
+        </is>
+      </c>
+      <c r="B33" s="49" t="inlineStr">
+        <is>
+          <t>Cirio</t>
+        </is>
+      </c>
+      <c r="C33" s="49" t="inlineStr">
+        <is>
+          <t>AG Advokat</t>
+        </is>
+      </c>
+      <c r="D33" s="49" t="n">
+        <v>3</v>
+      </c>
+      <c r="E33" s="49" t="n">
+        <v>9</v>
+      </c>
+      <c r="F33" s="49" t="inlineStr">
+        <is>
+          <t>Real estate / construction disputes</t>
+        </is>
+      </c>
+      <c r="G33" s="49" t="inlineStr">
+        <is>
+          <t>Johan Lindberg, Johan Rosén, Måns Derk</t>
+        </is>
+      </c>
+      <c r="H33" s="49" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
+      <c r="I33" s="49" t="inlineStr">
+        <is>
+          <t>realtid.se/juridik/cirio-expanderar-inom-fastighets-och-entreprenadjuridik/</t>
+        </is>
+      </c>
+    </row>
+    <row r="34">
+      <c r="A34" s="49" t="inlineStr">
+        <is>
+          <t>Oct-2025 / Feb-2026</t>
+        </is>
+      </c>
+      <c r="B34" s="49" t="inlineStr">
+        <is>
+          <t>BAHR (new Stockholm office)</t>
+        </is>
+      </c>
+      <c r="C34" s="49" t="inlineStr">
+        <is>
+          <t>Schjødt Sweden</t>
+        </is>
+      </c>
+      <c r="D34" s="49" t="n">
+        <v>8</v>
+      </c>
+      <c r="E34" s="49" t="inlineStr">
+        <is>
+          <t>~12</t>
+        </is>
+      </c>
+      <c r="F34" s="49" t="inlineStr">
+        <is>
+          <t>M&amp;A, banking, capital markets</t>
+        </is>
+      </c>
+      <c r="G34" s="49" t="inlineStr">
+        <is>
+          <t>Ola Hansson, Eric Halvarsson, Emil Hedberg, Peter Svanqvist, Kristoffer Stråth, Frida Lantoft, Karl Klackenberg, Tom Wehtje</t>
+        </is>
+      </c>
+      <c r="H34" s="49" t="inlineStr">
+        <is>
+          <t>High (count); medium (names)</t>
+        </is>
+      </c>
+      <c r="I34" s="49" t="inlineStr">
+        <is>
+          <t>dagensjuridik.se/nyheter/schjodt-skakas-av-avhopp-atta-i-stockholm-lamnar/</t>
+        </is>
+      </c>
+    </row>
+    <row r="35">
+      <c r="A35" s="49" t="inlineStr">
+        <is>
+          <t>Sep-2026</t>
+        </is>
+      </c>
+      <c r="B35" s="49" t="inlineStr">
+        <is>
+          <t>Ascente Law (AGRD)</t>
+        </is>
+      </c>
+      <c r="C35" s="49" t="inlineStr">
+        <is>
+          <t>Setterwalls Malmö</t>
+        </is>
+      </c>
+      <c r="D35" s="49" t="n">
+        <v>12</v>
+      </c>
+      <c r="E35" s="49" t="inlineStr">
+        <is>
+          <t>~88</t>
+        </is>
+      </c>
+      <c r="F35" s="49" t="inlineStr">
+        <is>
+          <t>Full service</t>
+        </is>
+      </c>
+      <c r="G35" s="49" t="inlineStr">
+        <is>
+          <t>Marc Tullgren (MP); others not named</t>
+        </is>
+      </c>
+      <c r="H35" s="49" t="inlineStr">
+        <is>
+          <t>High (event)</t>
+        </is>
+      </c>
+      <c r="I35" s="49" t="inlineStr">
+        <is>
+          <t>realtid.se/juridik/setterwalls-malmokontor-gar-till-riskkapitalagda-agrd/</t>
+        </is>
+      </c>
+    </row>
+    <row r="36">
+      <c r="A36" s="45" t="inlineStr">
+        <is>
+          <t>Below threshold: AG Advokat -&gt; MAQS (Elin Schedin + 1, Jan-2025); Lindahl -&gt; Foyen (Jan Berg + 3, Dec-2025).</t>
+        </is>
+      </c>
+    </row>
+    <row r="38">
+      <c r="A38" s="47" t="inlineStr">
+        <is>
+          <t>F3. Notable single partner moves at top firms</t>
+        </is>
+      </c>
+    </row>
+    <row r="39">
+      <c r="A39" s="52" t="inlineStr">
+        <is>
+          <t>Date</t>
+        </is>
+      </c>
+      <c r="B39" s="52" t="inlineStr">
+        <is>
+          <t>Hiring firm</t>
+        </is>
+      </c>
+      <c r="C39" s="52" t="inlineStr">
+        <is>
+          <t>Source firm</t>
+        </is>
+      </c>
+      <c r="D39" s="52" t="inlineStr">
+        <is>
+          <t>Partner</t>
+        </is>
+      </c>
+      <c r="E39" s="52" t="inlineStr">
+        <is>
+          <t>Practice</t>
+        </is>
+      </c>
+    </row>
+    <row r="40">
+      <c r="A40" s="49" t="inlineStr">
+        <is>
+          <t>Jun-2020</t>
+        </is>
+      </c>
+      <c r="B40" s="49" t="inlineStr">
+        <is>
+          <t>Hannes Snellman</t>
+        </is>
+      </c>
+      <c r="C40" s="49" t="inlineStr">
+        <is>
+          <t>Roschier</t>
+        </is>
+      </c>
+      <c r="D40" s="49" t="inlineStr">
+        <is>
+          <t>Ola Åhman</t>
+        </is>
+      </c>
+      <c r="E40" s="49" t="inlineStr">
+        <is>
+          <t>ECM / public M&amp;A</t>
+        </is>
+      </c>
+    </row>
+    <row r="41">
+      <c r="A41" s="49" t="inlineStr">
+        <is>
+          <t>Apr-2021</t>
+        </is>
+      </c>
+      <c r="B41" s="49" t="inlineStr">
+        <is>
+          <t>Bird &amp; Bird</t>
+        </is>
+      </c>
+      <c r="C41" s="49" t="inlineStr">
+        <is>
+          <t>MAQS</t>
+        </is>
+      </c>
+      <c r="D41" s="49" t="inlineStr">
+        <is>
+          <t>Olof Wetterling</t>
+        </is>
+      </c>
+      <c r="E41" s="49" t="inlineStr">
+        <is>
+          <t>Finance</t>
+        </is>
+      </c>
+    </row>
+    <row r="42">
+      <c r="A42" s="49" t="inlineStr">
+        <is>
+          <t>Mar-2023</t>
+        </is>
+      </c>
+      <c r="B42" s="49" t="inlineStr">
+        <is>
+          <t>Skierfe</t>
+        </is>
+      </c>
+      <c r="C42" s="49" t="inlineStr">
+        <is>
+          <t>Cederquist</t>
+        </is>
+      </c>
+      <c r="D42" s="49" t="inlineStr">
+        <is>
+          <t>Christian Johard</t>
+        </is>
+      </c>
+      <c r="E42" s="49" t="inlineStr">
+        <is>
+          <t>Real estate</t>
+        </is>
+      </c>
+    </row>
+    <row r="43">
+      <c r="A43" s="49" t="inlineStr">
+        <is>
+          <t>May-2023</t>
+        </is>
+      </c>
+      <c r="B43" s="49" t="inlineStr">
+        <is>
+          <t>Lindahl</t>
+        </is>
+      </c>
+      <c r="C43" s="49" t="inlineStr">
+        <is>
+          <t>Bird &amp; Bird</t>
+        </is>
+      </c>
+      <c r="D43" s="49" t="inlineStr">
+        <is>
+          <t>Jan Byström</t>
+        </is>
+      </c>
+      <c r="E43" s="49" t="inlineStr">
+        <is>
+          <t>M&amp;A</t>
+        </is>
+      </c>
+    </row>
+    <row r="44">
+      <c r="A44" s="49" t="inlineStr">
+        <is>
+          <t>Aug-2024</t>
+        </is>
+      </c>
+      <c r="B44" s="49" t="inlineStr">
+        <is>
+          <t>Schjødt</t>
+        </is>
+      </c>
+      <c r="C44" s="49" t="inlineStr">
+        <is>
+          <t>Mannheimer Swartling</t>
+        </is>
+      </c>
+      <c r="D44" s="49" t="inlineStr">
+        <is>
+          <t>Tom Wehtje</t>
+        </is>
+      </c>
+      <c r="E44" s="49" t="inlineStr">
+        <is>
+          <t>M&amp;A (later to BAHR)</t>
+        </is>
+      </c>
+    </row>
+    <row r="45">
+      <c r="A45" s="49" t="inlineStr">
+        <is>
+          <t>Sep-2024</t>
+        </is>
+      </c>
+      <c r="B45" s="49" t="inlineStr">
+        <is>
+          <t>Linklaters</t>
+        </is>
+      </c>
+      <c r="C45" s="49" t="inlineStr">
+        <is>
+          <t>White &amp; Case</t>
+        </is>
+      </c>
+      <c r="D45" s="49" t="inlineStr">
+        <is>
+          <t>Magnus Wennerhorn</t>
+        </is>
+      </c>
+      <c r="E45" s="49" t="inlineStr">
+        <is>
+          <t>Banking / finance</t>
+        </is>
+      </c>
+    </row>
+    <row r="46">
+      <c r="A46" s="49" t="inlineStr">
+        <is>
+          <t>Dec-2024</t>
+        </is>
+      </c>
+      <c r="B46" s="49" t="inlineStr">
+        <is>
+          <t>DLA Piper</t>
+        </is>
+      </c>
+      <c r="C46" s="49" t="inlineStr">
+        <is>
+          <t>Snellman</t>
+        </is>
+      </c>
+      <c r="D46" s="49" t="inlineStr">
+        <is>
+          <t>Joel Montin</t>
+        </is>
+      </c>
+      <c r="E46" s="49" t="inlineStr">
+        <is>
+          <t>Financial regulation</t>
+        </is>
+      </c>
+    </row>
+    <row r="47">
+      <c r="A47" s="49" t="inlineStr">
+        <is>
+          <t>Dec-2024</t>
+        </is>
+      </c>
+      <c r="B47" s="49" t="inlineStr">
+        <is>
+          <t>Hammarskiöld</t>
+        </is>
+      </c>
+      <c r="C47" s="49" t="inlineStr">
+        <is>
+          <t>Snellman</t>
+        </is>
+      </c>
+      <c r="D47" s="49" t="inlineStr">
+        <is>
+          <t>Ola Åhman</t>
+        </is>
+      </c>
+      <c r="E47" s="49" t="inlineStr">
+        <is>
+          <t>Corporate / M&amp;A</t>
+        </is>
+      </c>
+    </row>
+    <row r="48">
+      <c r="A48" s="49" t="inlineStr">
+        <is>
+          <t>Mar-2025</t>
+        </is>
+      </c>
+      <c r="B48" s="49" t="inlineStr">
+        <is>
+          <t>DLA Piper</t>
+        </is>
+      </c>
+      <c r="C48" s="49" t="inlineStr">
+        <is>
+          <t>Hammarskiöld</t>
+        </is>
+      </c>
+      <c r="D48" s="49" t="inlineStr">
+        <is>
+          <t>Carl-Johan Pousette</t>
+        </is>
+      </c>
+      <c r="E48" s="49" t="inlineStr">
+        <is>
+          <t>Capital markets</t>
+        </is>
+      </c>
+    </row>
+    <row r="49">
+      <c r="A49" s="49" t="inlineStr">
+        <is>
+          <t>Mar-2025</t>
+        </is>
+      </c>
+      <c r="B49" s="49" t="inlineStr">
+        <is>
+          <t>Bird &amp; Bird</t>
+        </is>
+      </c>
+      <c r="C49" s="49" t="inlineStr">
+        <is>
+          <t>Lindahl</t>
+        </is>
+      </c>
+      <c r="D49" s="49" t="inlineStr">
+        <is>
+          <t>Henrik Nobel</t>
+        </is>
+      </c>
+      <c r="E49" s="49" t="inlineStr">
+        <is>
+          <t>M&amp;A</t>
+        </is>
+      </c>
+    </row>
+    <row r="50">
+      <c r="A50" s="49" t="inlineStr">
+        <is>
+          <t>Mar-2025</t>
+        </is>
+      </c>
+      <c r="B50" s="49" t="inlineStr">
+        <is>
+          <t>Bird &amp; Bird</t>
+        </is>
+      </c>
+      <c r="C50" s="49" t="inlineStr">
+        <is>
+          <t>Westerberg &amp; Partners</t>
+        </is>
+      </c>
+      <c r="D50" s="49" t="inlineStr">
+        <is>
+          <t>Wendela Hårdemark</t>
+        </is>
+      </c>
+      <c r="E50" s="49" t="inlineStr">
+        <is>
+          <t>IP / patent litigation</t>
+        </is>
+      </c>
+    </row>
+    <row r="51">
+      <c r="A51" s="49" t="inlineStr">
+        <is>
+          <t>May-2025</t>
+        </is>
+      </c>
+      <c r="B51" s="49" t="inlineStr">
+        <is>
+          <t>Gernandt &amp; Danielsson</t>
+        </is>
+      </c>
+      <c r="C51" s="49" t="inlineStr">
+        <is>
+          <t>Snellman</t>
+        </is>
+      </c>
+      <c r="D51" s="49" t="inlineStr">
+        <is>
+          <t>Peter Forsberg</t>
+        </is>
+      </c>
+      <c r="E51" s="49" t="inlineStr">
+        <is>
+          <t>Competition</t>
+        </is>
+      </c>
+    </row>
+    <row r="52">
+      <c r="A52" s="49" t="inlineStr">
+        <is>
+          <t>Jun-2025 / Feb-2026</t>
+        </is>
+      </c>
+      <c r="B52" s="49" t="inlineStr">
+        <is>
+          <t>Schjødt then BAHR</t>
+        </is>
+      </c>
+      <c r="C52" s="49" t="inlineStr">
+        <is>
+          <t>Roschier then Schjødt</t>
+        </is>
+      </c>
+      <c r="D52" s="49" t="inlineStr">
+        <is>
+          <t>Peder Boström</t>
+        </is>
+      </c>
+      <c r="E52" s="49" t="inlineStr">
+        <is>
+          <t>Employment</t>
+        </is>
+      </c>
+    </row>
+    <row r="53">
+      <c r="A53" s="49" t="inlineStr">
+        <is>
+          <t>Oct-2025</t>
+        </is>
+      </c>
+      <c r="B53" s="49" t="inlineStr">
+        <is>
+          <t>BAHR</t>
+        </is>
+      </c>
+      <c r="C53" s="49" t="inlineStr">
+        <is>
+          <t>Snellman</t>
+        </is>
+      </c>
+      <c r="D53" s="49" t="inlineStr">
+        <is>
+          <t>Johanna Wärnberg</t>
+        </is>
+      </c>
+      <c r="E53" s="49" t="inlineStr">
+        <is>
+          <t>M&amp;A</t>
+        </is>
+      </c>
+    </row>
+    <row r="54">
+      <c r="A54" s="49" t="inlineStr">
+        <is>
+          <t>Nov-2025</t>
+        </is>
+      </c>
+      <c r="B54" s="49" t="inlineStr">
+        <is>
+          <t>MAQS</t>
+        </is>
+      </c>
+      <c r="C54" s="49" t="inlineStr">
+        <is>
+          <t>Baker McKenzie</t>
+        </is>
+      </c>
+      <c r="D54" s="49" t="inlineStr">
+        <is>
+          <t>Markus Mueller</t>
+        </is>
+      </c>
+      <c r="E54" s="49" t="inlineStr">
+        <is>
+          <t>Banking / finance</t>
+        </is>
+      </c>
+    </row>
+    <row r="55">
+      <c r="A55" s="49" t="inlineStr">
+        <is>
+          <t>Jan-2026</t>
+        </is>
+      </c>
+      <c r="B55" s="49" t="inlineStr">
+        <is>
+          <t>Lindahl</t>
+        </is>
+      </c>
+      <c r="C55" s="49" t="inlineStr">
+        <is>
+          <t>Vinge</t>
+        </is>
+      </c>
+      <c r="D55" s="49" t="inlineStr">
+        <is>
+          <t>Henrik Schön</t>
+        </is>
+      </c>
+      <c r="E55" s="49" t="inlineStr">
+        <is>
+          <t>Financial services</t>
+        </is>
+      </c>
+    </row>
+    <row r="56">
+      <c r="A56" s="49" t="inlineStr">
+        <is>
+          <t>2026</t>
+        </is>
+      </c>
+      <c r="B56" s="49" t="inlineStr">
+        <is>
+          <t>MAQS</t>
+        </is>
+      </c>
+      <c r="C56" s="49" t="inlineStr">
+        <is>
+          <t>Delphi</t>
+        </is>
+      </c>
+      <c r="D56" s="49" t="inlineStr">
+        <is>
+          <t>Karin Roberts</t>
+        </is>
+      </c>
+      <c r="E56" s="49" t="inlineStr">
+        <is>
+          <t>Defence / security</t>
+        </is>
+      </c>
+    </row>
+    <row r="57">
+      <c r="A57" s="49" t="inlineStr">
+        <is>
+          <t>Apr-2026</t>
+        </is>
+      </c>
+      <c r="B57" s="49" t="inlineStr">
+        <is>
+          <t>Schjødt</t>
+        </is>
+      </c>
+      <c r="C57" s="49" t="inlineStr">
+        <is>
+          <t>(ex-Linklaters)</t>
+        </is>
+      </c>
+      <c r="D57" s="49" t="inlineStr">
+        <is>
+          <t>Patrik Björklund</t>
+        </is>
+      </c>
+      <c r="E57" s="49" t="inlineStr">
+        <is>
+          <t>Banking / finance</t>
+        </is>
+      </c>
+    </row>
+    <row r="58">
+      <c r="A58" s="49" t="inlineStr">
+        <is>
+          <t>Jul-2026</t>
+        </is>
+      </c>
+      <c r="B58" s="49" t="inlineStr">
+        <is>
+          <t>DLA Piper</t>
+        </is>
+      </c>
+      <c r="C58" s="49" t="inlineStr">
+        <is>
+          <t>Baker McKenzie</t>
+        </is>
+      </c>
+      <c r="D58" s="49" t="inlineStr">
+        <is>
+          <t>Olof Forssell</t>
+        </is>
+      </c>
+      <c r="E58" s="49" t="inlineStr">
+        <is>
+          <t>Trade / sanctions</t>
+        </is>
+      </c>
+    </row>
+    <row r="59">
+      <c r="A59" s="49" t="inlineStr">
+        <is>
+          <t>2026</t>
+        </is>
+      </c>
+      <c r="B59" s="49" t="inlineStr">
+        <is>
+          <t>Gernandt &amp; Danielsson</t>
+        </is>
+      </c>
+      <c r="C59" s="49" t="inlineStr">
+        <is>
+          <t>Snellman</t>
+        </is>
+      </c>
+      <c r="D59" s="49" t="inlineStr">
+        <is>
+          <t>Pontus Ewerlöf</t>
+        </is>
+      </c>
+      <c r="E59" s="49" t="inlineStr">
+        <is>
+          <t>Disputes</t>
+        </is>
+      </c>
+    </row>
+    <row r="61">
+      <c r="A61" s="47" t="inlineStr">
+        <is>
+          <t>F4. Net partner flow 2020 - Oct 2026 (named partners in F2-F3 plus Legal 500 departures)</t>
+        </is>
+      </c>
+    </row>
+    <row r="62">
+      <c r="A62" s="99" t="inlineStr">
+        <is>
+          <t>Firm</t>
+        </is>
+      </c>
+      <c r="B62" s="99" t="inlineStr">
+        <is>
+          <t>Partner gains</t>
+        </is>
+      </c>
+      <c r="C62" s="99" t="inlineStr">
+        <is>
+          <t>Partner losses</t>
+        </is>
+      </c>
+      <c r="D62" s="99" t="inlineStr">
+        <is>
+          <t>Net</t>
+        </is>
+      </c>
+    </row>
+    <row r="63">
+      <c r="A63" s="49" t="inlineStr">
+        <is>
+          <t>BAHR</t>
+        </is>
+      </c>
+      <c r="B63" s="90" t="n">
+        <v>10</v>
+      </c>
+      <c r="C63" s="90" t="n">
+        <v>0</v>
+      </c>
+      <c r="D63" s="107">
+        <f>B63-C63</f>
+        <v/>
+      </c>
+    </row>
+    <row r="64">
+      <c r="A64" s="49" t="inlineStr">
+        <is>
+          <t>MAQS</t>
+        </is>
+      </c>
+      <c r="B64" s="90" t="n">
+        <v>6</v>
+      </c>
+      <c r="C64" s="90" t="n">
+        <v>1</v>
+      </c>
+      <c r="D64" s="107">
+        <f>B64-C64</f>
+        <v/>
+      </c>
+    </row>
+    <row r="65">
+      <c r="A65" s="49" t="inlineStr">
+        <is>
+          <t>Lindahl</t>
+        </is>
+      </c>
+      <c r="B65" s="90" t="n">
+        <v>4</v>
+      </c>
+      <c r="C65" s="90" t="n">
+        <v>2</v>
+      </c>
+      <c r="D65" s="107">
+        <f>B65-C65</f>
+        <v/>
+      </c>
+    </row>
+    <row r="66">
+      <c r="A66" s="49" t="inlineStr">
+        <is>
+          <t>Gernandt &amp; Danielsson</t>
+        </is>
+      </c>
+      <c r="B66" s="90" t="n">
+        <v>4</v>
+      </c>
+      <c r="C66" s="90" t="n">
+        <v>2</v>
+      </c>
+      <c r="D66" s="107">
+        <f>B66-C66</f>
+        <v/>
+      </c>
+    </row>
+    <row r="67">
+      <c r="A67" s="49" t="inlineStr">
+        <is>
+          <t>Cirio</t>
+        </is>
+      </c>
+      <c r="B67" s="90" t="n">
+        <v>3</v>
+      </c>
+      <c r="C67" s="90" t="n">
+        <v>1</v>
+      </c>
+      <c r="D67" s="107">
+        <f>B67-C67</f>
+        <v/>
+      </c>
+    </row>
+    <row r="68">
+      <c r="A68" s="49" t="inlineStr">
+        <is>
+          <t>Bird &amp; Bird</t>
+        </is>
+      </c>
+      <c r="B68" s="90" t="n">
+        <v>3</v>
+      </c>
+      <c r="C68" s="90" t="n">
+        <v>2</v>
+      </c>
+      <c r="D68" s="107">
+        <f>B68-C68</f>
+        <v/>
+      </c>
+    </row>
+    <row r="69">
+      <c r="A69" s="49" t="inlineStr">
+        <is>
+          <t>DLA Piper</t>
+        </is>
+      </c>
+      <c r="B69" s="90" t="n">
+        <v>3</v>
+      </c>
+      <c r="C69" s="90" t="n">
+        <v>2</v>
+      </c>
+      <c r="D69" s="107">
+        <f>B69-C69</f>
+        <v/>
+      </c>
+    </row>
+    <row r="70">
+      <c r="A70" s="49" t="inlineStr">
+        <is>
+          <t>Hammarskiöld</t>
+        </is>
+      </c>
+      <c r="B70" s="90" t="n">
+        <v>1</v>
+      </c>
+      <c r="C70" s="90" t="n">
+        <v>1</v>
+      </c>
+      <c r="D70" s="107">
+        <f>B70-C70</f>
+        <v/>
+      </c>
+    </row>
+    <row r="71">
+      <c r="A71" s="49" t="inlineStr">
+        <is>
+          <t>Linklaters</t>
+        </is>
+      </c>
+      <c r="B71" s="90" t="n">
+        <v>1</v>
+      </c>
+      <c r="C71" s="90" t="n">
+        <v>2</v>
+      </c>
+      <c r="D71" s="107">
+        <f>B71-C71</f>
+        <v/>
+      </c>
+    </row>
+    <row r="72">
+      <c r="A72" s="49" t="inlineStr">
+        <is>
+          <t>Mannheimer Swartling</t>
+        </is>
+      </c>
+      <c r="B72" s="90" t="n">
+        <v>0</v>
+      </c>
+      <c r="C72" s="90" t="n">
+        <v>2</v>
+      </c>
+      <c r="D72" s="107">
+        <f>B72-C72</f>
+        <v/>
+      </c>
+    </row>
+    <row r="73">
+      <c r="A73" s="49" t="inlineStr">
+        <is>
+          <t>Baker McKenzie</t>
+        </is>
+      </c>
+      <c r="B73" s="90" t="n">
+        <v>0</v>
+      </c>
+      <c r="C73" s="90" t="n">
+        <v>2</v>
+      </c>
+      <c r="D73" s="107">
+        <f>B73-C73</f>
+        <v/>
+      </c>
+    </row>
+    <row r="74">
+      <c r="A74" s="49" t="inlineStr">
+        <is>
+          <t>Roschier</t>
+        </is>
+      </c>
+      <c r="B74" s="90" t="n">
+        <v>0</v>
+      </c>
+      <c r="C74" s="90" t="n">
+        <v>3</v>
+      </c>
+      <c r="D74" s="107">
+        <f>B74-C74</f>
+        <v/>
+      </c>
+    </row>
+    <row r="75">
+      <c r="A75" s="49" t="inlineStr">
+        <is>
+          <t>Cederquist</t>
+        </is>
+      </c>
+      <c r="B75" s="90" t="n">
+        <v>0</v>
+      </c>
+      <c r="C75" s="90" t="n">
+        <v>3</v>
+      </c>
+      <c r="D75" s="107">
+        <f>B75-C75</f>
+        <v/>
+      </c>
+    </row>
+    <row r="76">
+      <c r="A76" s="49" t="inlineStr">
+        <is>
+          <t>Snellman</t>
+        </is>
+      </c>
+      <c r="B76" s="90" t="n">
+        <v>1</v>
+      </c>
+      <c r="C76" s="90" t="n">
+        <v>5</v>
+      </c>
+      <c r="D76" s="107">
+        <f>B76-C76</f>
+        <v/>
+      </c>
+    </row>
+    <row r="77">
+      <c r="A77" s="49" t="inlineStr">
+        <is>
+          <t>Delphi</t>
+        </is>
+      </c>
+      <c r="B77" s="90" t="n">
+        <v>0</v>
+      </c>
+      <c r="C77" s="90" t="n">
+        <v>4</v>
+      </c>
+      <c r="D77" s="107">
+        <f>B77-C77</f>
+        <v/>
+      </c>
+    </row>
+    <row r="78">
+      <c r="A78" s="49" t="inlineStr">
+        <is>
+          <t>AG Advokat</t>
+        </is>
+      </c>
+      <c r="B78" s="90" t="n">
+        <v>0</v>
+      </c>
+      <c r="C78" s="90" t="n">
+        <v>4</v>
+      </c>
+      <c r="D78" s="107">
+        <f>B78-C78</f>
+        <v/>
+      </c>
+    </row>
+    <row r="79">
+      <c r="A79" s="49" t="inlineStr">
+        <is>
+          <t>Schjødt</t>
+        </is>
+      </c>
+      <c r="B79" s="90" t="n">
+        <v>2</v>
+      </c>
+      <c r="C79" s="90" t="n">
+        <v>9</v>
+      </c>
+      <c r="D79" s="107">
+        <f>B79-C79</f>
+        <v/>
+      </c>
+    </row>
+    <row r="80">
+      <c r="A80" s="49" t="inlineStr">
+        <is>
+          <t>Setterwalls</t>
+        </is>
+      </c>
+      <c r="B80" s="90" t="n">
+        <v>0</v>
+      </c>
+      <c r="C80" s="90" t="n">
+        <v>13</v>
+      </c>
+      <c r="D80" s="107">
+        <f>B80-C80</f>
+        <v/>
+      </c>
+    </row>
+    <row r="82">
+      <c r="A82" s="45" t="inlineStr">
+        <is>
+          <t>Schjødt gains: Wehtje, Boström, Björklund (counted in losses again when they left). Setterwalls losses include 12 Malmö partners to Ascente/AGRD. Snellman: Montin partner status unconfirmed.</t>
+        </is>
+      </c>
+    </row>
+    <row r="84">
+      <c r="A84" s="47" t="inlineStr">
+        <is>
+          <t>F5. Key takeaways</t>
+        </is>
+      </c>
+    </row>
+    <row r="85">
+      <c r="A85" t="inlineStr">
+        <is>
+          <t>- Consolidation accelerated from 2025: AGRD (Axcel) has assembled 11 firms in ~13 months (incl. Setterwalls Malmö, Wigge, Moll Wendén) and says more acquisitions are planned. AGRD firms must leave the Bar (no external ownership of advokat firms).</t>
+        </is>
+      </c>
+    </row>
+    <row r="86">
+      <c r="A86" t="inlineStr">
+        <is>
+          <t>- Nordic firms enter Sweden via combinations and lifts: Schjødt (Hamilton, 2020), CMS (Wistrand, 2024), BAHR (8 Schjødt partners, 2026).</t>
+        </is>
+      </c>
+    </row>
+    <row r="87">
+      <c r="A87" t="inlineStr">
+        <is>
+          <t>- Team lifts concentrate in real estate (G&amp;D from Linklaters; Cirio from AG Advokat) and M&amp;A/finance (MAQS from Delphi; BAHR from Schjødt).</t>
+        </is>
+      </c>
+    </row>
+    <row r="88">
+      <c r="A88" t="inlineStr">
+        <is>
+          <t>- Net losers of partners: Setterwalls (Malmö exit), Schjødt, Snellman, Delphi and AG Advokat. The Big 3 (MSA, Vinge, Roschier) show no team losses.</t>
+        </is>
+      </c>
+    </row>
+    <row r="89">
+      <c r="A89" t="inlineStr">
+        <is>
+          <t>- Splits are rising: Hannes Snellman (2024), MAQS (2026/27) and Glimstedt's Stockholm/Göteborg offices (2021).</t>
+        </is>
+      </c>
+    </row>
+    <row r="91">
+      <c r="A91" s="45" t="inlineStr">
+        <is>
+          <t>Not verified / gaps: Hannes Snellman Sweden rename to "Snellman" (no formal notice found); no qualifying team moves found out of MSA, Vinge or Roschier; 2020-23 coverage thinner. All URLs prefixed https://www.</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+  <mergeCells count="1">
+    <mergeCell ref="A2:J2"/>
+  </mergeCells>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
@@ -1408,21 +3676,21 @@
   <dimension ref="A1:O40"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
-    <col width="4" customWidth="1" min="1" max="1"/>
-    <col width="26" customWidth="1" min="2" max="2"/>
-    <col width="13" customWidth="1" min="3" max="3"/>
-    <col width="11" customWidth="1" min="4" max="4"/>
-    <col width="30" customWidth="1" min="5" max="5"/>
-    <col width="9" customWidth="1" min="6" max="6"/>
-    <col width="30" customWidth="1" min="7" max="7"/>
-    <col width="9" customWidth="1" min="8" max="8"/>
-    <col width="11" customWidth="1" min="9" max="9"/>
-    <col width="24" customWidth="1" min="10" max="10"/>
-    <col width="10" customWidth="1" min="11" max="11"/>
-    <col width="10" customWidth="1" min="12" max="12"/>
-    <col width="10" customWidth="1" min="13" max="13"/>
-    <col width="11" customWidth="1" min="14" max="14"/>
-    <col width="40" customWidth="1" min="15" max="15"/>
+    <col width="4" customWidth="1" style="108" min="1" max="1"/>
+    <col width="26" customWidth="1" style="108" min="2" max="2"/>
+    <col width="13" customWidth="1" style="108" min="3" max="3"/>
+    <col width="11" customWidth="1" style="108" min="4" max="4"/>
+    <col width="30" customWidth="1" style="108" min="5" max="5"/>
+    <col width="9" customWidth="1" style="108" min="6" max="6"/>
+    <col width="30" customWidth="1" style="108" min="7" max="7"/>
+    <col width="9" customWidth="1" style="108" min="8" max="8"/>
+    <col width="11" customWidth="1" style="108" min="9" max="9"/>
+    <col width="24" customWidth="1" style="108" min="10" max="10"/>
+    <col width="10" customWidth="1" style="108" min="11" max="11"/>
+    <col width="10" customWidth="1" style="108" min="12" max="12"/>
+    <col width="10" customWidth="1" style="108" min="13" max="13"/>
+    <col width="11" customWidth="1" style="108" min="14" max="14"/>
+    <col width="40" customWidth="1" style="108" min="15" max="15"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -1432,7 +3700,7 @@
         </is>
       </c>
     </row>
-    <row r="2" ht="55" customHeight="1">
+    <row r="2" ht="55" customHeight="1" s="108">
       <c r="A2" s="2" t="inlineStr">
         <is>
           <t>Revenue = latest available year per firm (SEK m). Affärsvärlden figures are fee income; company accounts (AB) are net sales of the main legal entity and are not strictly comparable. Partners and lawyers mostly firm-supplied to Chambers (2026). Employees = headcount, used as a proxy for FTEs (no FTE data is published); AB headcounts usually exclude partners who bill via own companies. Ratios are calculated only where both inputs exist. Grey = not found.</t>
@@ -1517,20 +3785,20 @@
       </c>
     </row>
     <row r="5">
-      <c r="A5" s="81" t="n">
+      <c r="A5" s="109" t="n">
         <v>1</v>
       </c>
-      <c r="B5" s="81" t="inlineStr">
+      <c r="B5" s="109" t="inlineStr">
         <is>
           <t>Vinge</t>
         </is>
       </c>
-      <c r="C5" s="81" t="inlineStr">
+      <c r="C5" s="109" t="inlineStr">
         <is>
           <t>2025</t>
         </is>
       </c>
-      <c r="D5" s="82" t="n">
+      <c r="D5" s="110" t="n">
         <v>2036</v>
       </c>
       <c r="E5" s="49" t="inlineStr">
@@ -1538,7 +3806,7 @@
           <t>Group, annual reports (DJ via Realtid)</t>
         </is>
       </c>
-      <c r="F5" s="81" t="n">
+      <c r="F5" s="109" t="n">
         <v>71</v>
       </c>
       <c r="G5" s="49" t="inlineStr">
@@ -1546,10 +3814,10 @@
           <t>Firm website count, Oct-26 (lawyers incl. ~46 on leave)</t>
         </is>
       </c>
-      <c r="H5" s="81" t="n">
+      <c r="H5" s="109" t="n">
         <v>389</v>
       </c>
-      <c r="I5" s="81" t="n">
+      <c r="I5" s="109" t="n">
         <v>550</v>
       </c>
       <c r="J5" s="49" t="inlineStr">
@@ -1580,20 +3848,20 @@
       </c>
     </row>
     <row r="6">
-      <c r="A6" s="81" t="n">
+      <c r="A6" s="109" t="n">
         <v>2</v>
       </c>
-      <c r="B6" s="81" t="inlineStr">
+      <c r="B6" s="109" t="inlineStr">
         <is>
           <t>Mannheimer Swartling</t>
         </is>
       </c>
-      <c r="C6" s="81" t="inlineStr">
+      <c r="C6" s="109" t="inlineStr">
         <is>
           <t>2025</t>
         </is>
       </c>
-      <c r="D6" s="82" t="n">
+      <c r="D6" s="110" t="n">
         <v>2002</v>
       </c>
       <c r="E6" s="49" t="inlineStr">
@@ -1601,7 +3869,7 @@
           <t>Group, annual report (DJ via Realtid)</t>
         </is>
       </c>
-      <c r="F6" s="81" t="n">
+      <c r="F6" s="109" t="n">
         <v>92</v>
       </c>
       <c r="G6" s="49" t="inlineStr">
@@ -1609,10 +3877,10 @@
           <t>DJ (dividend split), 2025</t>
         </is>
       </c>
-      <c r="H6" s="81" t="n">
+      <c r="H6" s="109" t="n">
         <v>430</v>
       </c>
-      <c r="I6" s="81" t="n">
+      <c r="I6" s="109" t="n">
         <v>650</v>
       </c>
       <c r="J6" s="49" t="inlineStr">
@@ -1643,20 +3911,20 @@
       </c>
     </row>
     <row r="7">
-      <c r="A7" s="81" t="n">
+      <c r="A7" s="109" t="n">
         <v>3</v>
       </c>
-      <c r="B7" s="81" t="inlineStr">
+      <c r="B7" s="109" t="inlineStr">
         <is>
           <t>Roschier (Sweden)</t>
         </is>
       </c>
-      <c r="C7" s="81" t="inlineStr">
+      <c r="C7" s="109" t="inlineStr">
         <is>
           <t>FY Jun24-May25</t>
         </is>
       </c>
-      <c r="D7" s="82" t="n">
+      <c r="D7" s="110" t="n">
         <v>1254</v>
       </c>
       <c r="E7" s="49" t="inlineStr">
@@ -1664,7 +3932,7 @@
           <t>Affärsvärlden Oct-25</t>
         </is>
       </c>
-      <c r="F7" s="81" t="n">
+      <c r="F7" s="109" t="n">
         <v>26</v>
       </c>
       <c r="G7" s="49" t="inlineStr">
@@ -1672,10 +3940,10 @@
           <t>Firm website count, Oct-26 (Stockholm)</t>
         </is>
       </c>
-      <c r="H7" s="81" t="n">
+      <c r="H7" s="109" t="n">
         <v>181</v>
       </c>
-      <c r="I7" s="81" t="n">
+      <c r="I7" s="109" t="n">
         <v>226</v>
       </c>
       <c r="J7" s="49" t="inlineStr">
@@ -1706,20 +3974,20 @@
       </c>
     </row>
     <row r="8">
-      <c r="A8" s="81" t="n">
+      <c r="A8" s="109" t="n">
         <v>4</v>
       </c>
-      <c r="B8" s="81" t="inlineStr">
+      <c r="B8" s="109" t="inlineStr">
         <is>
           <t>White &amp; Case (Stockholm)</t>
         </is>
       </c>
-      <c r="C8" s="81" t="inlineStr">
+      <c r="C8" s="109" t="inlineStr">
         <is>
           <t>2025</t>
         </is>
       </c>
-      <c r="D8" s="82" t="n">
+      <c r="D8" s="110" t="n">
         <v>1108</v>
       </c>
       <c r="E8" s="49" t="inlineStr">
@@ -1727,7 +3995,7 @@
           <t>Company accounts, net sales (AB)</t>
         </is>
       </c>
-      <c r="F8" s="81" t="n">
+      <c r="F8" s="109" t="n">
         <v>16</v>
       </c>
       <c r="G8" s="49" t="inlineStr">
@@ -1735,10 +4003,10 @@
           <t>Implied (est.): DJ "&gt;SEK 69m per partner"</t>
         </is>
       </c>
-      <c r="H8" s="81" t="n">
+      <c r="H8" s="109" t="n">
         <v>70</v>
       </c>
-      <c r="I8" s="81" t="n">
+      <c r="I8" s="109" t="n">
         <v>120</v>
       </c>
       <c r="J8" s="49" t="inlineStr">
@@ -1769,20 +4037,20 @@
       </c>
     </row>
     <row r="9">
-      <c r="A9" s="81" t="n">
+      <c r="A9" s="109" t="n">
         <v>5</v>
       </c>
-      <c r="B9" s="81" t="inlineStr">
+      <c r="B9" s="109" t="inlineStr">
         <is>
           <t>Setterwalls</t>
         </is>
       </c>
-      <c r="C9" s="81" t="inlineStr">
+      <c r="C9" s="109" t="inlineStr">
         <is>
           <t>2025</t>
         </is>
       </c>
-      <c r="D9" s="82" t="n">
+      <c r="D9" s="110" t="n">
         <v>1000</v>
       </c>
       <c r="E9" s="49" t="inlineStr">
@@ -1790,7 +4058,7 @@
           <t>Affärsvärlden ("&gt;1bn"); parent AB 1,056</t>
         </is>
       </c>
-      <c r="F9" s="81" t="n">
+      <c r="F9" s="109" t="n">
         <v>38</v>
       </c>
       <c r="G9" s="49" t="inlineStr">
@@ -1798,10 +4066,10 @@
           <t>Firm website count, Oct-26 (Sthlm + Gbg; Malmö left Sep-26)</t>
         </is>
       </c>
-      <c r="H9" s="81" t="n">
+      <c r="H9" s="109" t="n">
         <v>177</v>
       </c>
-      <c r="I9" s="81" t="n">
+      <c r="I9" s="109" t="n">
         <v>306</v>
       </c>
       <c r="J9" s="49" t="inlineStr">
@@ -1832,20 +4100,20 @@
       </c>
     </row>
     <row r="10">
-      <c r="A10" s="81" t="n">
+      <c r="A10" s="109" t="n">
         <v>6</v>
       </c>
-      <c r="B10" s="81" t="inlineStr">
+      <c r="B10" s="109" t="inlineStr">
         <is>
           <t>Lindahl</t>
         </is>
       </c>
-      <c r="C10" s="81" t="inlineStr">
+      <c r="C10" s="109" t="inlineStr">
         <is>
           <t>2024</t>
         </is>
       </c>
-      <c r="D10" s="82" t="n">
+      <c r="D10" s="110" t="n">
         <v>737</v>
       </c>
       <c r="E10" s="49" t="inlineStr">
@@ -1853,7 +4121,7 @@
           <t>Affärsvärlden Apr-25</t>
         </is>
       </c>
-      <c r="F10" s="81" t="n">
+      <c r="F10" s="109" t="n">
         <v>68</v>
       </c>
       <c r="G10" s="49" t="inlineStr">
@@ -1861,10 +4129,10 @@
           <t>Legal 500 (firm-supplied, 2026)</t>
         </is>
       </c>
-      <c r="H10" s="81" t="n">
+      <c r="H10" s="109" t="n">
         <v>220</v>
       </c>
-      <c r="I10" s="81" t="n">
+      <c r="I10" s="109" t="n">
         <v>300</v>
       </c>
       <c r="J10" s="49" t="inlineStr">
@@ -1895,20 +4163,20 @@
       </c>
     </row>
     <row r="11">
-      <c r="A11" s="81" t="n">
+      <c r="A11" s="109" t="n">
         <v>7</v>
       </c>
-      <c r="B11" s="81" t="inlineStr">
+      <c r="B11" s="109" t="inlineStr">
         <is>
           <t>Gernandt &amp; Danielsson</t>
         </is>
       </c>
-      <c r="C11" s="81" t="inlineStr">
+      <c r="C11" s="109" t="inlineStr">
         <is>
           <t>FY24/25</t>
         </is>
       </c>
-      <c r="D11" s="82" t="n">
+      <c r="D11" s="110" t="n">
         <v>676</v>
       </c>
       <c r="E11" s="49" t="inlineStr">
@@ -1916,7 +4184,7 @@
           <t>Affärsvärlden Oct-25</t>
         </is>
       </c>
-      <c r="F11" s="81" t="n">
+      <c r="F11" s="109" t="n">
         <v>20</v>
       </c>
       <c r="G11" s="49" t="inlineStr">
@@ -1924,10 +4192,10 @@
           <t>Firm website count, Oct-26</t>
         </is>
       </c>
-      <c r="H11" s="81" t="n">
+      <c r="H11" s="109" t="n">
         <v>91</v>
       </c>
-      <c r="I11" s="81" t="n">
+      <c r="I11" s="109" t="n">
         <v>150</v>
       </c>
       <c r="J11" s="49" t="inlineStr">
@@ -1958,20 +4226,20 @@
       </c>
     </row>
     <row r="12">
-      <c r="A12" s="81" t="n">
+      <c r="A12" s="109" t="n">
         <v>8</v>
       </c>
-      <c r="B12" s="81" t="inlineStr">
+      <c r="B12" s="109" t="inlineStr">
         <is>
           <t>DLA Piper (Sweden)</t>
         </is>
       </c>
-      <c r="C12" s="81" t="inlineStr">
+      <c r="C12" s="109" t="inlineStr">
         <is>
           <t>FY24/25</t>
         </is>
       </c>
-      <c r="D12" s="82" t="n">
+      <c r="D12" s="110" t="n">
         <v>602</v>
       </c>
       <c r="E12" s="49" t="inlineStr">
@@ -1979,7 +4247,7 @@
           <t>Affärsvärlden Oct-25</t>
         </is>
       </c>
-      <c r="F12" s="81" t="n">
+      <c r="F12" s="109" t="n">
         <v>37</v>
       </c>
       <c r="G12" s="49" t="inlineStr">
@@ -1987,10 +4255,10 @@
           <t>Firm website count, Oct-26 (profile pages)</t>
         </is>
       </c>
-      <c r="H12" s="81" t="n">
+      <c r="H12" s="109" t="n">
         <v>148</v>
       </c>
-      <c r="I12" s="83" t="n"/>
+      <c r="I12" s="111" t="n"/>
       <c r="J12" s="49" t="inlineStr"/>
       <c r="K12" s="56">
         <f>D12/F12</f>
@@ -2012,20 +4280,20 @@
       </c>
     </row>
     <row r="13">
-      <c r="A13" s="81" t="n">
+      <c r="A13" s="109" t="n">
         <v>9</v>
       </c>
-      <c r="B13" s="81" t="inlineStr">
+      <c r="B13" s="109" t="inlineStr">
         <is>
           <t>CMS Wistrand</t>
         </is>
       </c>
-      <c r="C13" s="81" t="inlineStr">
+      <c r="C13" s="109" t="inlineStr">
         <is>
           <t>2024</t>
         </is>
       </c>
-      <c r="D13" s="82" t="n">
+      <c r="D13" s="110" t="n">
         <v>558</v>
       </c>
       <c r="E13" s="49" t="inlineStr">
@@ -2033,7 +4301,7 @@
           <t>Affärsvärlden Apr-25</t>
         </is>
       </c>
-      <c r="F13" s="81" t="n">
+      <c r="F13" s="109" t="n">
         <v>51</v>
       </c>
       <c r="G13" s="49" t="inlineStr">
@@ -2041,10 +4309,10 @@
           <t>Firm statement (cms.law)</t>
         </is>
       </c>
-      <c r="H13" s="81" t="n">
+      <c r="H13" s="109" t="n">
         <v>150</v>
       </c>
-      <c r="I13" s="83" t="n"/>
+      <c r="I13" s="111" t="n"/>
       <c r="J13" s="49" t="inlineStr"/>
       <c r="K13" s="56">
         <f>D13/F13</f>
@@ -2062,20 +4330,20 @@
       <c r="O13" s="49" t="inlineStr"/>
     </row>
     <row r="14">
-      <c r="A14" s="81" t="n">
+      <c r="A14" s="109" t="n">
         <v>10</v>
       </c>
-      <c r="B14" s="81" t="inlineStr">
+      <c r="B14" s="109" t="inlineStr">
         <is>
           <t>Schjødt (Sweden)</t>
         </is>
       </c>
-      <c r="C14" s="81" t="inlineStr">
+      <c r="C14" s="109" t="inlineStr">
         <is>
           <t>2025</t>
         </is>
       </c>
-      <c r="D14" s="82" t="n">
+      <c r="D14" s="110" t="n">
         <v>534</v>
       </c>
       <c r="E14" s="49" t="inlineStr">
@@ -2083,7 +4351,7 @@
           <t>Est.: "&gt;SEK 0.5bn", +25% on 427</t>
         </is>
       </c>
-      <c r="F14" s="81" t="n">
+      <c r="F14" s="109" t="n">
         <v>20</v>
       </c>
       <c r="G14" s="49" t="inlineStr">
@@ -2091,10 +4359,10 @@
           <t>Firm website count, Oct-26 (may include leavers to BAHR)</t>
         </is>
       </c>
-      <c r="H14" s="81" t="n">
+      <c r="H14" s="109" t="n">
         <v>65</v>
       </c>
-      <c r="I14" s="83" t="n"/>
+      <c r="I14" s="111" t="n"/>
       <c r="J14" s="49" t="inlineStr"/>
       <c r="K14" s="56">
         <f>D14/F14</f>
@@ -2116,20 +4384,20 @@
       </c>
     </row>
     <row r="15">
-      <c r="A15" s="81" t="n">
+      <c r="A15" s="109" t="n">
         <v>11</v>
       </c>
-      <c r="B15" s="81" t="inlineStr">
+      <c r="B15" s="109" t="inlineStr">
         <is>
           <t>Delphi</t>
         </is>
       </c>
-      <c r="C15" s="81" t="inlineStr">
+      <c r="C15" s="109" t="inlineStr">
         <is>
           <t>2024</t>
         </is>
       </c>
-      <c r="D15" s="82" t="n">
+      <c r="D15" s="110" t="n">
         <v>516</v>
       </c>
       <c r="E15" s="49" t="inlineStr">
@@ -2137,7 +4405,7 @@
           <t>Affärsvärlden Apr-25</t>
         </is>
       </c>
-      <c r="F15" s="81" t="n">
+      <c r="F15" s="109" t="n">
         <v>49</v>
       </c>
       <c r="G15" s="49" t="inlineStr">
@@ -2145,10 +4413,10 @@
           <t>Chambers 2026</t>
         </is>
       </c>
-      <c r="H15" s="81" t="n">
+      <c r="H15" s="109" t="n">
         <v>150</v>
       </c>
-      <c r="I15" s="81" t="n">
+      <c r="I15" s="109" t="n">
         <v>220</v>
       </c>
       <c r="J15" s="49" t="inlineStr">
@@ -2179,20 +4447,20 @@
       </c>
     </row>
     <row r="16">
-      <c r="A16" s="81" t="n">
+      <c r="A16" s="109" t="n">
         <v>12</v>
       </c>
-      <c r="B16" s="81" t="inlineStr">
+      <c r="B16" s="109" t="inlineStr">
         <is>
           <t>Cirio</t>
         </is>
       </c>
-      <c r="C16" s="81" t="inlineStr">
+      <c r="C16" s="109" t="inlineStr">
         <is>
           <t>2025</t>
         </is>
       </c>
-      <c r="D16" s="82" t="n">
+      <c r="D16" s="110" t="n">
         <v>431</v>
       </c>
       <c r="E16" s="49" t="inlineStr">
@@ -2200,7 +4468,7 @@
           <t>Company accounts, net sales (AB)</t>
         </is>
       </c>
-      <c r="F16" s="81" t="n">
+      <c r="F16" s="109" t="n">
         <v>27</v>
       </c>
       <c r="G16" s="49" t="inlineStr">
@@ -2208,10 +4476,10 @@
           <t>Legal 500 (firm-supplied, 2026)</t>
         </is>
       </c>
-      <c r="H16" s="81" t="n">
+      <c r="H16" s="109" t="n">
         <v>76</v>
       </c>
-      <c r="I16" s="81" t="n">
+      <c r="I16" s="109" t="n">
         <v>127</v>
       </c>
       <c r="J16" s="49" t="inlineStr">
@@ -2242,20 +4510,20 @@
       </c>
     </row>
     <row r="17">
-      <c r="A17" s="81" t="n">
+      <c r="A17" s="109" t="n">
         <v>13</v>
       </c>
-      <c r="B17" s="81" t="inlineStr">
+      <c r="B17" s="109" t="inlineStr">
         <is>
           <t>MAQS</t>
         </is>
       </c>
-      <c r="C17" s="81" t="inlineStr">
+      <c r="C17" s="109" t="inlineStr">
         <is>
           <t>2024</t>
         </is>
       </c>
-      <c r="D17" s="82" t="n">
+      <c r="D17" s="110" t="n">
         <v>417</v>
       </c>
       <c r="E17" s="49" t="inlineStr">
@@ -2263,7 +4531,7 @@
           <t>Affärsvärlden Apr-25</t>
         </is>
       </c>
-      <c r="F17" s="81" t="n">
+      <c r="F17" s="109" t="n">
         <v>48</v>
       </c>
       <c r="G17" s="49" t="inlineStr">
@@ -2271,10 +4539,10 @@
           <t>Firm website count, Oct-26</t>
         </is>
       </c>
-      <c r="H17" s="81" t="n">
+      <c r="H17" s="109" t="n">
         <v>144</v>
       </c>
-      <c r="I17" s="81" t="n">
+      <c r="I17" s="109" t="n">
         <v>180</v>
       </c>
       <c r="J17" s="49" t="inlineStr">
@@ -2305,20 +4573,20 @@
       </c>
     </row>
     <row r="18">
-      <c r="A18" s="81" t="n">
+      <c r="A18" s="109" t="n">
         <v>14</v>
       </c>
-      <c r="B18" s="81" t="inlineStr">
+      <c r="B18" s="109" t="inlineStr">
         <is>
           <t>Baker McKenzie (Stockholm)</t>
         </is>
       </c>
-      <c r="C18" s="81" t="inlineStr">
+      <c r="C18" s="109" t="inlineStr">
         <is>
           <t>FY23/24</t>
         </is>
       </c>
-      <c r="D18" s="82" t="n">
+      <c r="D18" s="110" t="n">
         <v>334</v>
       </c>
       <c r="E18" s="49" t="inlineStr">
@@ -2326,7 +4594,7 @@
           <t>Affärsvärlden Apr-25</t>
         </is>
       </c>
-      <c r="F18" s="81" t="n">
+      <c r="F18" s="109" t="n">
         <v>12</v>
       </c>
       <c r="G18" s="49" t="inlineStr">
@@ -2334,10 +4602,10 @@
           <t>Firm website count, Oct-26 (+2 principals)</t>
         </is>
       </c>
-      <c r="H18" s="81" t="n">
+      <c r="H18" s="109" t="n">
         <v>73</v>
       </c>
-      <c r="I18" s="83" t="n"/>
+      <c r="I18" s="111" t="n"/>
       <c r="J18" s="49" t="inlineStr"/>
       <c r="K18" s="56">
         <f>D18/F18</f>
@@ -2359,20 +4627,20 @@
       </c>
     </row>
     <row r="19">
-      <c r="A19" s="81" t="n">
+      <c r="A19" s="109" t="n">
         <v>15</v>
       </c>
-      <c r="B19" s="81" t="inlineStr">
+      <c r="B19" s="109" t="inlineStr">
         <is>
           <t>Snellman (Sweden)</t>
         </is>
       </c>
-      <c r="C19" s="81" t="inlineStr">
+      <c r="C19" s="109" t="inlineStr">
         <is>
           <t>2025</t>
         </is>
       </c>
-      <c r="D19" s="82" t="n">
+      <c r="D19" s="110" t="n">
         <v>279</v>
       </c>
       <c r="E19" s="49" t="inlineStr">
@@ -2380,10 +4648,10 @@
           <t>Company accounts, net sales (AB)</t>
         </is>
       </c>
-      <c r="F19" s="83" t="n"/>
+      <c r="F19" s="111" t="n"/>
       <c r="G19" s="49" t="inlineStr"/>
-      <c r="H19" s="83" t="n"/>
-      <c r="I19" s="81" t="n">
+      <c r="H19" s="111" t="n"/>
+      <c r="I19" s="109" t="n">
         <v>107</v>
       </c>
       <c r="J19" s="49" t="inlineStr">
@@ -2405,20 +4673,20 @@
       </c>
     </row>
     <row r="20">
-      <c r="A20" s="81" t="n">
+      <c r="A20" s="109" t="n">
         <v>16</v>
       </c>
-      <c r="B20" s="81" t="inlineStr">
+      <c r="B20" s="109" t="inlineStr">
         <is>
           <t>Foyen</t>
         </is>
       </c>
-      <c r="C20" s="81" t="inlineStr">
+      <c r="C20" s="109" t="inlineStr">
         <is>
           <t>2024</t>
         </is>
       </c>
-      <c r="D20" s="82" t="n">
+      <c r="D20" s="110" t="n">
         <v>277</v>
       </c>
       <c r="E20" s="49" t="inlineStr">
@@ -2426,7 +4694,7 @@
           <t>Affärsvärlden Apr-25</t>
         </is>
       </c>
-      <c r="F20" s="81" t="n">
+      <c r="F20" s="109" t="n">
         <v>23</v>
       </c>
       <c r="G20" s="49" t="inlineStr">
@@ -2434,10 +4702,10 @@
           <t>Firm website count, Oct-26</t>
         </is>
       </c>
-      <c r="H20" s="81" t="n">
+      <c r="H20" s="109" t="n">
         <v>73</v>
       </c>
-      <c r="I20" s="81" t="n">
+      <c r="I20" s="109" t="n">
         <v>106</v>
       </c>
       <c r="J20" s="49" t="inlineStr">
@@ -2464,20 +4732,20 @@
       <c r="O20" s="49" t="inlineStr"/>
     </row>
     <row r="21">
-      <c r="A21" s="81" t="n">
+      <c r="A21" s="109" t="n">
         <v>17</v>
       </c>
-      <c r="B21" s="81" t="inlineStr">
+      <c r="B21" s="109" t="inlineStr">
         <is>
           <t>Glimstedt</t>
         </is>
       </c>
-      <c r="C21" s="81" t="inlineStr">
+      <c r="C21" s="109" t="inlineStr">
         <is>
           <t>2024</t>
         </is>
       </c>
-      <c r="D21" s="82" t="n">
+      <c r="D21" s="110" t="n">
         <v>196</v>
       </c>
       <c r="E21" s="49" t="inlineStr">
@@ -2485,7 +4753,7 @@
           <t>Affärsvärlden Apr-25</t>
         </is>
       </c>
-      <c r="F21" s="81" t="n">
+      <c r="F21" s="109" t="n">
         <v>41</v>
       </c>
       <c r="G21" s="49" t="inlineStr">
@@ -2493,10 +4761,10 @@
           <t>Firm website count, Oct-26 (Sweden)</t>
         </is>
       </c>
-      <c r="H21" s="81" t="n">
+      <c r="H21" s="109" t="n">
         <v>78</v>
       </c>
-      <c r="I21" s="83" t="n"/>
+      <c r="I21" s="111" t="n"/>
       <c r="J21" s="49" t="inlineStr"/>
       <c r="K21" s="56">
         <f>D21/F21</f>
@@ -2518,20 +4786,20 @@
       </c>
     </row>
     <row r="22">
-      <c r="A22" s="81" t="n">
+      <c r="A22" s="109" t="n">
         <v>18</v>
       </c>
-      <c r="B22" s="81" t="inlineStr">
+      <c r="B22" s="109" t="inlineStr">
         <is>
           <t>Eversheds Sutherland</t>
         </is>
       </c>
-      <c r="C22" s="81" t="inlineStr">
+      <c r="C22" s="109" t="inlineStr">
         <is>
           <t>2025</t>
         </is>
       </c>
-      <c r="D22" s="82" t="n">
+      <c r="D22" s="110" t="n">
         <v>166</v>
       </c>
       <c r="E22" s="49" t="inlineStr">
@@ -2539,10 +4807,10 @@
           <t>Company accounts, net sales (AB)</t>
         </is>
       </c>
-      <c r="F22" s="83" t="n"/>
+      <c r="F22" s="111" t="n"/>
       <c r="G22" s="49" t="inlineStr"/>
-      <c r="H22" s="83" t="n"/>
-      <c r="I22" s="81" t="n">
+      <c r="H22" s="111" t="n"/>
+      <c r="I22" s="109" t="n">
         <v>59</v>
       </c>
       <c r="J22" s="49" t="inlineStr">
@@ -2564,20 +4832,20 @@
       </c>
     </row>
     <row r="23">
-      <c r="A23" s="81" t="n">
+      <c r="A23" s="109" t="n">
         <v>19</v>
       </c>
-      <c r="B23" s="81" t="inlineStr">
+      <c r="B23" s="109" t="inlineStr">
         <is>
           <t>Fylgia</t>
         </is>
       </c>
-      <c r="C23" s="81" t="inlineStr">
+      <c r="C23" s="109" t="inlineStr">
         <is>
           <t>2024</t>
         </is>
       </c>
-      <c r="D23" s="82" t="n">
+      <c r="D23" s="110" t="n">
         <v>131</v>
       </c>
       <c r="E23" s="49" t="inlineStr">
@@ -2585,7 +4853,7 @@
           <t>Affärsvärlden Apr-25</t>
         </is>
       </c>
-      <c r="F23" s="81" t="n">
+      <c r="F23" s="109" t="n">
         <v>21</v>
       </c>
       <c r="G23" s="49" t="inlineStr">
@@ -2593,10 +4861,10 @@
           <t>Firm website count, Oct-26</t>
         </is>
       </c>
-      <c r="H23" s="81" t="n">
+      <c r="H23" s="109" t="n">
         <v>35</v>
       </c>
-      <c r="I23" s="83" t="n"/>
+      <c r="I23" s="111" t="n"/>
       <c r="J23" s="49" t="inlineStr"/>
       <c r="K23" s="56">
         <f>D23/F23</f>
@@ -2618,20 +4886,20 @@
       </c>
     </row>
     <row r="24">
-      <c r="A24" s="81" t="n">
+      <c r="A24" s="109" t="n">
         <v>20</v>
       </c>
-      <c r="B24" s="81" t="inlineStr">
+      <c r="B24" s="109" t="inlineStr">
         <is>
           <t>Westerberg &amp; Partners</t>
         </is>
       </c>
-      <c r="C24" s="81" t="inlineStr">
+      <c r="C24" s="109" t="inlineStr">
         <is>
           <t>2025</t>
         </is>
       </c>
-      <c r="D24" s="82" t="n">
+      <c r="D24" s="110" t="n">
         <v>107</v>
       </c>
       <c r="E24" s="49" t="inlineStr">
@@ -2639,7 +4907,7 @@
           <t>Company accounts, net sales (AB)</t>
         </is>
       </c>
-      <c r="F24" s="81" t="n">
+      <c r="F24" s="109" t="n">
         <v>12</v>
       </c>
       <c r="G24" s="49" t="inlineStr">
@@ -2647,10 +4915,10 @@
           <t>Firm website count, Oct-26</t>
         </is>
       </c>
-      <c r="H24" s="81" t="n">
+      <c r="H24" s="109" t="n">
         <v>24</v>
       </c>
-      <c r="I24" s="81" t="n">
+      <c r="I24" s="109" t="n">
         <v>35</v>
       </c>
       <c r="J24" s="49" t="inlineStr">
@@ -2677,20 +4945,20 @@
       <c r="O24" s="49" t="inlineStr"/>
     </row>
     <row r="25">
-      <c r="A25" s="81" t="n">
+      <c r="A25" s="109" t="n">
         <v>21</v>
       </c>
-      <c r="B25" s="81" t="inlineStr">
+      <c r="B25" s="109" t="inlineStr">
         <is>
           <t>Moll Wendén</t>
         </is>
       </c>
-      <c r="C25" s="81" t="inlineStr">
+      <c r="C25" s="109" t="inlineStr">
         <is>
           <t>2025</t>
         </is>
       </c>
-      <c r="D25" s="82" t="n">
+      <c r="D25" s="110" t="n">
         <v>101</v>
       </c>
       <c r="E25" s="49" t="inlineStr">
@@ -2698,7 +4966,7 @@
           <t>Company accounts, net sales (AB)</t>
         </is>
       </c>
-      <c r="F25" s="81" t="n">
+      <c r="F25" s="109" t="n">
         <v>8</v>
       </c>
       <c r="G25" s="49" t="inlineStr">
@@ -2706,10 +4974,10 @@
           <t>Firm website count, Oct-26</t>
         </is>
       </c>
-      <c r="H25" s="81" t="n">
+      <c r="H25" s="109" t="n">
         <v>37</v>
       </c>
-      <c r="I25" s="81" t="n">
+      <c r="I25" s="109" t="n">
         <v>44</v>
       </c>
       <c r="J25" s="49" t="inlineStr">
@@ -2736,20 +5004,20 @@
       <c r="O25" s="49" t="inlineStr"/>
     </row>
     <row r="26">
-      <c r="A26" s="81" t="n">
+      <c r="A26" s="109" t="n">
         <v>22</v>
       </c>
-      <c r="B26" s="81" t="inlineStr">
+      <c r="B26" s="109" t="inlineStr">
         <is>
           <t>Born</t>
         </is>
       </c>
-      <c r="C26" s="81" t="inlineStr">
+      <c r="C26" s="109" t="inlineStr">
         <is>
           <t>2024</t>
         </is>
       </c>
-      <c r="D26" s="82" t="n">
+      <c r="D26" s="110" t="n">
         <v>86</v>
       </c>
       <c r="E26" s="49" t="inlineStr">
@@ -2757,7 +5025,7 @@
           <t>Affärsvärlden Apr-25</t>
         </is>
       </c>
-      <c r="F26" s="81" t="n">
+      <c r="F26" s="109" t="n">
         <v>9</v>
       </c>
       <c r="G26" s="49" t="inlineStr">
@@ -2765,10 +5033,10 @@
           <t>Firm website count, Oct-26</t>
         </is>
       </c>
-      <c r="H26" s="81" t="n">
+      <c r="H26" s="109" t="n">
         <v>26</v>
       </c>
-      <c r="I26" s="83" t="n"/>
+      <c r="I26" s="111" t="n"/>
       <c r="J26" s="49" t="inlineStr"/>
       <c r="K26" s="56">
         <f>D26/F26</f>
@@ -2790,20 +5058,20 @@
       </c>
     </row>
     <row r="27">
-      <c r="A27" s="81" t="n">
+      <c r="A27" s="109" t="n">
         <v>23</v>
       </c>
-      <c r="B27" s="81" t="inlineStr">
+      <c r="B27" s="109" t="inlineStr">
         <is>
           <t>Harvest</t>
         </is>
       </c>
-      <c r="C27" s="81" t="inlineStr">
+      <c r="C27" s="109" t="inlineStr">
         <is>
           <t>2025</t>
         </is>
       </c>
-      <c r="D27" s="82" t="n">
+      <c r="D27" s="110" t="n">
         <v>82</v>
       </c>
       <c r="E27" s="49" t="inlineStr">
@@ -2811,7 +5079,7 @@
           <t>Company accounts, net sales (AB)</t>
         </is>
       </c>
-      <c r="F27" s="81" t="n">
+      <c r="F27" s="109" t="n">
         <v>5</v>
       </c>
       <c r="G27" s="49" t="inlineStr">
@@ -2819,10 +5087,10 @@
           <t>Firm website count, Oct-26</t>
         </is>
       </c>
-      <c r="H27" s="81" t="n">
+      <c r="H27" s="109" t="n">
         <v>27</v>
       </c>
-      <c r="I27" s="81" t="n">
+      <c r="I27" s="109" t="n">
         <v>27</v>
       </c>
       <c r="J27" s="49" t="inlineStr">
@@ -2849,20 +5117,20 @@
       <c r="O27" s="49" t="inlineStr"/>
     </row>
     <row r="28">
-      <c r="A28" s="81" t="n">
+      <c r="A28" s="109" t="n">
         <v>24</v>
       </c>
-      <c r="B28" s="81" t="inlineStr">
+      <c r="B28" s="109" t="inlineStr">
         <is>
           <t>Synch</t>
         </is>
       </c>
-      <c r="C28" s="81" t="inlineStr">
+      <c r="C28" s="109" t="inlineStr">
         <is>
           <t>2025</t>
         </is>
       </c>
-      <c r="D28" s="82" t="n">
+      <c r="D28" s="110" t="n">
         <v>81</v>
       </c>
       <c r="E28" s="49" t="inlineStr">
@@ -2870,7 +5138,7 @@
           <t>Company accounts, net sales (AB)</t>
         </is>
       </c>
-      <c r="F28" s="81" t="n">
+      <c r="F28" s="109" t="n">
         <v>9</v>
       </c>
       <c r="G28" s="49" t="inlineStr">
@@ -2878,10 +5146,10 @@
           <t>Firm website count, Oct-26</t>
         </is>
       </c>
-      <c r="H28" s="81" t="n">
+      <c r="H28" s="109" t="n">
         <v>38</v>
       </c>
-      <c r="I28" s="81" t="n">
+      <c r="I28" s="109" t="n">
         <v>38</v>
       </c>
       <c r="J28" s="49" t="inlineStr">
@@ -2912,20 +5180,20 @@
       </c>
     </row>
     <row r="29">
-      <c r="A29" s="81" t="n">
+      <c r="A29" s="109" t="n">
         <v>25</v>
       </c>
-      <c r="B29" s="81" t="inlineStr">
+      <c r="B29" s="109" t="inlineStr">
         <is>
           <t>Kastell</t>
         </is>
       </c>
-      <c r="C29" s="81" t="inlineStr">
+      <c r="C29" s="109" t="inlineStr">
         <is>
           <t>2025</t>
         </is>
       </c>
-      <c r="D29" s="82" t="n">
+      <c r="D29" s="110" t="n">
         <v>80</v>
       </c>
       <c r="E29" s="49" t="inlineStr">
@@ -2933,7 +5201,7 @@
           <t>Company accounts, net sales (AB)</t>
         </is>
       </c>
-      <c r="F29" s="81" t="n">
+      <c r="F29" s="109" t="n">
         <v>9</v>
       </c>
       <c r="G29" s="49" t="inlineStr">
@@ -2941,10 +5209,10 @@
           <t>Firm website count, Oct-26</t>
         </is>
       </c>
-      <c r="H29" s="81" t="n">
+      <c r="H29" s="109" t="n">
         <v>18</v>
       </c>
-      <c r="I29" s="81" t="n">
+      <c r="I29" s="109" t="n">
         <v>21</v>
       </c>
       <c r="J29" s="49" t="inlineStr">
@@ -3069,12 +5337,12 @@
   <dimension ref="A1:F23"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
-    <col width="24" customWidth="1" min="1" max="1"/>
-    <col width="22" customWidth="1" min="2" max="2"/>
-    <col width="16" customWidth="1" min="3" max="3"/>
-    <col width="14" customWidth="1" min="4" max="4"/>
-    <col width="80" customWidth="1" min="5" max="5"/>
-    <col width="60" customWidth="1" min="6" max="6"/>
+    <col width="24" customWidth="1" style="108" min="1" max="1"/>
+    <col width="22" customWidth="1" style="108" min="2" max="2"/>
+    <col width="16" customWidth="1" style="108" min="3" max="3"/>
+    <col width="14" customWidth="1" style="108" min="4" max="4"/>
+    <col width="80" customWidth="1" style="108" min="5" max="5"/>
+    <col width="60" customWidth="1" style="108" min="6" max="6"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -3398,7 +5666,7 @@
       </c>
       <c r="E14" s="49" t="inlineStr">
         <is>
-          <t>Linklaters Stockholm real estate team: partners Magnus Lidman and Anna Eriksson + 5 associates (dated Jun-24 by Global Legal Post/Legal 500; Afv says early 2025).</t>
+          <t>Linklaters Stockholm real estate team: partners Magnus Lidman and Anna Eriksson + 5 associates (effective 1 Jun 2024, G&amp;D press release).</t>
         </is>
       </c>
       <c r="F14" s="49" t="inlineStr">
@@ -3628,17 +5896,17 @@
   <dimension ref="A1:K59"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
-    <col width="26" customWidth="1" min="1" max="1"/>
-    <col width="30" customWidth="1" min="2" max="2"/>
-    <col width="10" customWidth="1" min="3" max="3"/>
-    <col width="10" customWidth="1" min="4" max="4"/>
-    <col width="10" customWidth="1" min="5" max="5"/>
-    <col width="9" customWidth="1" min="6" max="6"/>
-    <col width="36" customWidth="1" min="7" max="7"/>
-    <col width="28" customWidth="1" min="8" max="8"/>
-    <col width="9" customWidth="1" min="9" max="9"/>
-    <col width="9" customWidth="1" min="10" max="10"/>
-    <col width="28" customWidth="1" min="11" max="11"/>
+    <col width="26" customWidth="1" style="108" min="1" max="1"/>
+    <col width="30" customWidth="1" style="108" min="2" max="2"/>
+    <col width="10" customWidth="1" style="108" min="3" max="3"/>
+    <col width="10" customWidth="1" style="108" min="4" max="4"/>
+    <col width="10" customWidth="1" style="108" min="5" max="5"/>
+    <col width="9" customWidth="1" style="108" min="6" max="6"/>
+    <col width="36" customWidth="1" style="108" min="7" max="7"/>
+    <col width="28" customWidth="1" style="108" min="8" max="8"/>
+    <col width="9" customWidth="1" style="108" min="9" max="9"/>
+    <col width="9" customWidth="1" style="108" min="10" max="10"/>
+    <col width="28" customWidth="1" style="108" min="11" max="11"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -3648,7 +5916,7 @@
         </is>
       </c>
     </row>
-    <row r="2" ht="60" customHeight="1">
+    <row r="2" ht="60" customHeight="1" s="108">
       <c r="A2" s="2" t="inlineStr">
         <is>
           <t>Universe: firm-level rankings in Chambers Europe 2026 (Sweden) and Legal 500 EMEA (Sweden), incl. Legal 500 "firms to watch". Excludes international firms and the nine largest Swedish full-service firms. Counts: 45 ranked independents (incl. PE-owned AGRD firms) + 2 firms to watch only = 47; +5 borderline mid-size firms = 52. Partner/lawyer counts: firm website counts (Oct-26) where available, else firm-supplied to Legal 500 / Chambers (2026); blank where not found.</t>
@@ -5631,60 +7899,60 @@
   <dimension ref="A1:BB66"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
-    <col width="24" customWidth="1" min="1" max="1"/>
-    <col width="8" customWidth="1" min="2" max="2"/>
-    <col width="8" customWidth="1" min="3" max="3"/>
-    <col width="8" customWidth="1" min="4" max="4"/>
-    <col width="6.5" customWidth="1" min="5" max="5"/>
-    <col width="6.5" customWidth="1" min="6" max="6"/>
-    <col width="6.5" customWidth="1" min="7" max="7"/>
-    <col width="6.5" customWidth="1" min="8" max="8"/>
-    <col width="6.5" customWidth="1" min="9" max="9"/>
-    <col width="6.5" customWidth="1" min="10" max="10"/>
-    <col width="6.5" customWidth="1" min="11" max="11"/>
-    <col width="6.5" customWidth="1" min="12" max="12"/>
-    <col width="6.5" customWidth="1" min="13" max="13"/>
-    <col width="6.5" customWidth="1" min="14" max="14"/>
-    <col width="6.5" customWidth="1" min="15" max="15"/>
-    <col width="6.5" customWidth="1" min="16" max="16"/>
-    <col width="6.5" customWidth="1" min="17" max="17"/>
-    <col width="6.5" customWidth="1" min="18" max="18"/>
-    <col width="6.5" customWidth="1" min="19" max="19"/>
-    <col width="6.5" customWidth="1" min="20" max="20"/>
-    <col width="6.5" customWidth="1" min="21" max="21"/>
-    <col width="6.5" customWidth="1" min="22" max="22"/>
-    <col width="6.5" customWidth="1" min="23" max="23"/>
-    <col width="6.5" customWidth="1" min="24" max="24"/>
-    <col width="6.5" customWidth="1" min="25" max="25"/>
-    <col width="6.5" customWidth="1" min="26" max="26"/>
-    <col width="6.5" customWidth="1" min="27" max="27"/>
-    <col width="6.5" customWidth="1" min="28" max="28"/>
-    <col width="6.5" customWidth="1" min="29" max="29"/>
-    <col width="6.5" customWidth="1" min="30" max="30"/>
-    <col width="6.5" customWidth="1" min="31" max="31"/>
-    <col width="6.5" customWidth="1" min="32" max="32"/>
-    <col width="6.5" customWidth="1" min="33" max="33"/>
-    <col width="6.5" customWidth="1" min="34" max="34"/>
-    <col width="6.5" customWidth="1" min="35" max="35"/>
-    <col width="6.5" customWidth="1" min="36" max="36"/>
-    <col width="6.5" customWidth="1" min="37" max="37"/>
-    <col width="6.5" customWidth="1" min="38" max="38"/>
-    <col width="6.5" customWidth="1" min="39" max="39"/>
-    <col width="6.5" customWidth="1" min="40" max="40"/>
-    <col width="6.5" customWidth="1" min="41" max="41"/>
-    <col width="6.5" customWidth="1" min="42" max="42"/>
-    <col width="6.5" customWidth="1" min="43" max="43"/>
-    <col width="6.5" customWidth="1" min="44" max="44"/>
-    <col width="6.5" customWidth="1" min="45" max="45"/>
-    <col width="6.5" customWidth="1" min="46" max="46"/>
-    <col width="6.5" customWidth="1" min="47" max="47"/>
-    <col width="6.5" customWidth="1" min="48" max="48"/>
-    <col width="6.5" customWidth="1" min="49" max="49"/>
-    <col width="6.5" customWidth="1" min="50" max="50"/>
-    <col width="6.5" customWidth="1" min="51" max="51"/>
-    <col width="6.5" customWidth="1" min="52" max="52"/>
-    <col width="6.5" customWidth="1" min="53" max="53"/>
-    <col width="6.5" customWidth="1" min="54" max="54"/>
+    <col width="24" customWidth="1" style="108" min="1" max="1"/>
+    <col width="8" customWidth="1" style="108" min="2" max="2"/>
+    <col width="8" customWidth="1" style="108" min="3" max="3"/>
+    <col width="8" customWidth="1" style="108" min="4" max="4"/>
+    <col width="6.5" customWidth="1" style="108" min="5" max="5"/>
+    <col width="6.5" customWidth="1" style="108" min="6" max="6"/>
+    <col width="6.5" customWidth="1" style="108" min="7" max="7"/>
+    <col width="6.5" customWidth="1" style="108" min="8" max="8"/>
+    <col width="6.5" customWidth="1" style="108" min="9" max="9"/>
+    <col width="6.5" customWidth="1" style="108" min="10" max="10"/>
+    <col width="6.5" customWidth="1" style="108" min="11" max="11"/>
+    <col width="6.5" customWidth="1" style="108" min="12" max="12"/>
+    <col width="6.5" customWidth="1" style="108" min="13" max="13"/>
+    <col width="6.5" customWidth="1" style="108" min="14" max="14"/>
+    <col width="6.5" customWidth="1" style="108" min="15" max="15"/>
+    <col width="6.5" customWidth="1" style="108" min="16" max="16"/>
+    <col width="6.5" customWidth="1" style="108" min="17" max="17"/>
+    <col width="6.5" customWidth="1" style="108" min="18" max="18"/>
+    <col width="6.5" customWidth="1" style="108" min="19" max="19"/>
+    <col width="6.5" customWidth="1" style="108" min="20" max="20"/>
+    <col width="6.5" customWidth="1" style="108" min="21" max="21"/>
+    <col width="6.5" customWidth="1" style="108" min="22" max="22"/>
+    <col width="6.5" customWidth="1" style="108" min="23" max="23"/>
+    <col width="6.5" customWidth="1" style="108" min="24" max="24"/>
+    <col width="6.5" customWidth="1" style="108" min="25" max="25"/>
+    <col width="6.5" customWidth="1" style="108" min="26" max="26"/>
+    <col width="6.5" customWidth="1" style="108" min="27" max="27"/>
+    <col width="6.5" customWidth="1" style="108" min="28" max="28"/>
+    <col width="6.5" customWidth="1" style="108" min="29" max="29"/>
+    <col width="6.5" customWidth="1" style="108" min="30" max="30"/>
+    <col width="6.5" customWidth="1" style="108" min="31" max="31"/>
+    <col width="6.5" customWidth="1" style="108" min="32" max="32"/>
+    <col width="6.5" customWidth="1" style="108" min="33" max="33"/>
+    <col width="6.5" customWidth="1" style="108" min="34" max="34"/>
+    <col width="6.5" customWidth="1" style="108" min="35" max="35"/>
+    <col width="6.5" customWidth="1" style="108" min="36" max="36"/>
+    <col width="6.5" customWidth="1" style="108" min="37" max="37"/>
+    <col width="6.5" customWidth="1" style="108" min="38" max="38"/>
+    <col width="6.5" customWidth="1" style="108" min="39" max="39"/>
+    <col width="6.5" customWidth="1" style="108" min="40" max="40"/>
+    <col width="6.5" customWidth="1" style="108" min="41" max="41"/>
+    <col width="6.5" customWidth="1" style="108" min="42" max="42"/>
+    <col width="6.5" customWidth="1" style="108" min="43" max="43"/>
+    <col width="6.5" customWidth="1" style="108" min="44" max="44"/>
+    <col width="6.5" customWidth="1" style="108" min="45" max="45"/>
+    <col width="6.5" customWidth="1" style="108" min="46" max="46"/>
+    <col width="6.5" customWidth="1" style="108" min="47" max="47"/>
+    <col width="6.5" customWidth="1" style="108" min="48" max="48"/>
+    <col width="6.5" customWidth="1" style="108" min="49" max="49"/>
+    <col width="6.5" customWidth="1" style="108" min="50" max="50"/>
+    <col width="6.5" customWidth="1" style="108" min="51" max="51"/>
+    <col width="6.5" customWidth="1" style="108" min="52" max="52"/>
+    <col width="6.5" customWidth="1" style="108" min="53" max="53"/>
+    <col width="6.5" customWidth="1" style="108" min="54" max="54"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -5694,14 +7962,14 @@
         </is>
       </c>
     </row>
-    <row r="2" ht="45" customHeight="1">
+    <row r="2" ht="45" customHeight="1" s="108">
       <c r="A2" s="2" t="inlineStr">
         <is>
           <t>Chambers Europe 2026 (firm bands, B1 = top) and Legal 500 EMEA, current edition (firm tiers, T1 = top; FTW = firm to watch). Extracted from chambers.com and legal500.com on 2026-10-08. Blank = not ranked. Score = sum of points (band/tier 1 = 5 ... 5 = 1, FTW = 0.5). Rows sorted by score; firms with score &lt; 4 omitted, except boxed firms. Magnusson, Delphi and Lindahl are grouped together so they can share one box.</t>
         </is>
       </c>
     </row>
-    <row r="4" ht="48" customHeight="1">
+    <row r="4" ht="48" customHeight="1" s="108">
       <c r="A4" s="3" t="inlineStr">
         <is>
           <t>Firm</t>
@@ -12544,11 +14812,11 @@
   <dimension ref="A1:E661"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
-    <col width="26" customWidth="1" min="1" max="1"/>
-    <col width="11" customWidth="1" min="2" max="2"/>
-    <col width="14" customWidth="1" min="3" max="3"/>
-    <col width="24" customWidth="1" min="4" max="4"/>
-    <col width="40" customWidth="1" min="5" max="5"/>
+    <col width="26" customWidth="1" style="108" min="1" max="1"/>
+    <col width="11" customWidth="1" style="108" min="2" max="2"/>
+    <col width="14" customWidth="1" style="108" min="3" max="3"/>
+    <col width="24" customWidth="1" style="108" min="4" max="4"/>
+    <col width="40" customWidth="1" style="108" min="5" max="5"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -30413,24 +32681,24 @@
   <dimension ref="A1:R43"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
-    <col width="5" customWidth="1" min="1" max="1"/>
-    <col width="26" customWidth="1" min="2" max="2"/>
-    <col width="11" customWidth="1" min="3" max="3"/>
-    <col width="10" customWidth="1" min="4" max="4"/>
-    <col width="9" customWidth="1" min="5" max="5"/>
-    <col width="10" customWidth="1" min="6" max="6"/>
-    <col width="26" customWidth="1" min="7" max="7"/>
-    <col width="9" customWidth="1" min="8" max="8"/>
-    <col width="10" customWidth="1" min="9" max="9"/>
-    <col width="10" customWidth="1" min="10" max="10"/>
-    <col width="30" customWidth="1" min="11" max="11"/>
-    <col width="10" customWidth="1" min="12" max="12"/>
-    <col width="10" customWidth="1" min="13" max="13"/>
-    <col width="10" customWidth="1" min="14" max="14"/>
-    <col width="12" customWidth="1" min="15" max="15"/>
-    <col width="12" customWidth="1" min="16" max="16"/>
-    <col width="10" customWidth="1" min="17" max="17"/>
-    <col width="40" customWidth="1" min="18" max="18"/>
+    <col width="5" customWidth="1" style="108" min="1" max="1"/>
+    <col width="26" customWidth="1" style="108" min="2" max="2"/>
+    <col width="11" customWidth="1" style="108" min="3" max="3"/>
+    <col width="10" customWidth="1" style="108" min="4" max="4"/>
+    <col width="9" customWidth="1" style="108" min="5" max="5"/>
+    <col width="10" customWidth="1" style="108" min="6" max="6"/>
+    <col width="26" customWidth="1" style="108" min="7" max="7"/>
+    <col width="9" customWidth="1" style="108" min="8" max="8"/>
+    <col width="10" customWidth="1" style="108" min="9" max="9"/>
+    <col width="10" customWidth="1" style="108" min="10" max="10"/>
+    <col width="30" customWidth="1" style="108" min="11" max="11"/>
+    <col width="10" customWidth="1" style="108" min="12" max="12"/>
+    <col width="10" customWidth="1" style="108" min="13" max="13"/>
+    <col width="10" customWidth="1" style="108" min="14" max="14"/>
+    <col width="12" customWidth="1" style="108" min="15" max="15"/>
+    <col width="12" customWidth="1" style="108" min="16" max="16"/>
+    <col width="10" customWidth="1" style="108" min="17" max="17"/>
+    <col width="40" customWidth="1" style="108" min="18" max="18"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -30440,14 +32708,14 @@
         </is>
       </c>
     </row>
-    <row r="2" ht="45" customHeight="1">
+    <row r="2" ht="45" customHeight="1" s="108">
       <c r="A2" s="2" t="inlineStr">
         <is>
           <t>Ranking: Affärsvärlden fee income FY2024 (revised table, 3 Oct 2025; split-year firms on FY24/25). Ratios use the latest available revenue (FY2025 where published, else FY2024; basis shown) against current headcount (mostly Oct-2026), so they are indicative. Leverage (requested) = partners / total employees; partners / lawyers shown alongside. Grey = not available.</t>
         </is>
       </c>
     </row>
-    <row r="4" ht="48" customHeight="1">
+    <row r="4" ht="48" customHeight="1" s="108">
       <c r="A4" s="52" t="inlineStr">
         <is>
           <t>#</t>
@@ -32577,24 +34845,24 @@
   <dimension ref="A1:R55"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
-    <col width="26" customWidth="1" min="1" max="1"/>
-    <col width="20" customWidth="1" min="2" max="2"/>
-    <col width="28" customWidth="1" min="3" max="3"/>
-    <col width="10" customWidth="1" min="4" max="4"/>
-    <col width="10" customWidth="1" min="5" max="5"/>
-    <col width="12" customWidth="1" min="6" max="6"/>
-    <col width="12" customWidth="1" min="7" max="7"/>
-    <col width="10" customWidth="1" min="8" max="8"/>
-    <col width="10" customWidth="1" min="9" max="9"/>
-    <col width="10" customWidth="1" min="10" max="10"/>
-    <col width="10" customWidth="1" min="11" max="11"/>
-    <col width="10" customWidth="1" min="12" max="12"/>
-    <col width="10" customWidth="1" min="13" max="13"/>
-    <col width="10" customWidth="1" min="14" max="14"/>
-    <col width="10" customWidth="1" min="15" max="15"/>
-    <col width="13" customWidth="1" min="16" max="16"/>
-    <col width="40" customWidth="1" min="17" max="17"/>
-    <col width="40" customWidth="1" min="18" max="18"/>
+    <col width="26" customWidth="1" style="108" min="1" max="1"/>
+    <col width="20" customWidth="1" style="108" min="2" max="2"/>
+    <col width="28" customWidth="1" style="108" min="3" max="3"/>
+    <col width="10" customWidth="1" style="108" min="4" max="4"/>
+    <col width="10" customWidth="1" style="108" min="5" max="5"/>
+    <col width="12" customWidth="1" style="108" min="6" max="6"/>
+    <col width="12" customWidth="1" style="108" min="7" max="7"/>
+    <col width="10" customWidth="1" style="108" min="8" max="8"/>
+    <col width="10" customWidth="1" style="108" min="9" max="9"/>
+    <col width="10" customWidth="1" style="108" min="10" max="10"/>
+    <col width="10" customWidth="1" style="108" min="11" max="11"/>
+    <col width="10" customWidth="1" style="108" min="12" max="12"/>
+    <col width="10" customWidth="1" style="108" min="13" max="13"/>
+    <col width="10" customWidth="1" style="108" min="14" max="14"/>
+    <col width="10" customWidth="1" style="108" min="15" max="15"/>
+    <col width="13" customWidth="1" style="108" min="16" max="16"/>
+    <col width="40" customWidth="1" style="108" min="17" max="17"/>
+    <col width="40" customWidth="1" style="108" min="18" max="18"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -32604,7 +34872,7 @@
         </is>
       </c>
     </row>
-    <row r="2" ht="45" customHeight="1">
+    <row r="2" ht="45" customHeight="1" s="108">
       <c r="A2" s="2" t="inlineStr">
         <is>
           <t>Rates are only comparable when dated: Swedish firms typically revise rates annually on 1 January. Public-sector price annexes are usually confidential (Kammarrätten i Stockholm, 2017, Vinge / E-hälsomyndigheten), so firm-level rate cards are scarce. Source type matters: list price (rate card) &gt; court/Chapter 11 filings (actual billed) &gt; public tender (discounted).</t>
@@ -32618,7 +34886,7 @@
         </is>
       </c>
     </row>
-    <row r="5" ht="42" customHeight="1">
+    <row r="5" ht="42" customHeight="1" s="108">
       <c r="A5" s="52" t="inlineStr">
         <is>
           <t>Firm</t>
@@ -32746,7 +35014,7 @@
       <c r="Q6" s="85" t="n"/>
       <c r="R6" s="85" t="n"/>
     </row>
-    <row r="7" ht="60" customHeight="1">
+    <row r="7" ht="60" customHeight="1" s="108">
       <c r="A7" s="49" t="inlineStr">
         <is>
           <t>Mannheimer Swartling</t>
@@ -32814,7 +35082,7 @@
         </is>
       </c>
     </row>
-    <row r="8" ht="60" customHeight="1">
+    <row r="8" ht="60" customHeight="1" s="108">
       <c r="A8" s="49" t="inlineStr">
         <is>
           <t>Cederquist</t>
@@ -34340,22 +36608,22 @@
   <dimension ref="A1:P35"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
-    <col width="24" customWidth="1" min="1" max="1"/>
-    <col width="22" customWidth="1" min="2" max="2"/>
-    <col width="12" customWidth="1" min="3" max="3"/>
-    <col width="10" customWidth="1" min="4" max="4"/>
-    <col width="11" customWidth="1" min="5" max="5"/>
-    <col width="11" customWidth="1" min="6" max="6"/>
-    <col width="11" customWidth="1" min="7" max="7"/>
-    <col width="9" customWidth="1" min="8" max="8"/>
-    <col width="22" customWidth="1" min="9" max="9"/>
-    <col width="11" customWidth="1" min="10" max="10"/>
-    <col width="11" customWidth="1" min="11" max="11"/>
-    <col width="13" customWidth="1" min="12" max="12"/>
-    <col width="10" customWidth="1" min="13" max="13"/>
-    <col width="11" customWidth="1" min="14" max="14"/>
-    <col width="10" customWidth="1" min="15" max="15"/>
-    <col width="50" customWidth="1" min="16" max="16"/>
+    <col width="24" customWidth="1" style="108" min="1" max="1"/>
+    <col width="22" customWidth="1" style="108" min="2" max="2"/>
+    <col width="12" customWidth="1" style="108" min="3" max="3"/>
+    <col width="10" customWidth="1" style="108" min="4" max="4"/>
+    <col width="11" customWidth="1" style="108" min="5" max="5"/>
+    <col width="11" customWidth="1" style="108" min="6" max="6"/>
+    <col width="11" customWidth="1" style="108" min="7" max="7"/>
+    <col width="9" customWidth="1" style="108" min="8" max="8"/>
+    <col width="22" customWidth="1" style="108" min="9" max="9"/>
+    <col width="11" customWidth="1" style="108" min="10" max="10"/>
+    <col width="11" customWidth="1" style="108" min="11" max="11"/>
+    <col width="13" customWidth="1" style="108" min="12" max="12"/>
+    <col width="10" customWidth="1" style="108" min="13" max="13"/>
+    <col width="11" customWidth="1" style="108" min="14" max="14"/>
+    <col width="10" customWidth="1" style="108" min="15" max="15"/>
+    <col width="50" customWidth="1" style="108" min="16" max="16"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -34365,14 +36633,14 @@
         </is>
       </c>
     </row>
-    <row r="2" ht="75" customHeight="1">
+    <row r="2" ht="75" customHeight="1" s="108">
       <c r="A2" s="2" t="inlineStr">
         <is>
           <t>Source: annual reports filed with Bolagsverket, read via allabolag.se (Oct-2026); amounts SEK m. Swedish law firms pay partners mainly through the profit of the firm company (dividends to partners or their holding companies) plus any salary. "Profit pool per partner" = profit before tax (+ disclosed board/CEO salaries, typically partners) / partners: a proxy for AVERAGE equity-partner compensation before personal tax. It understates pay where partners are also on the payroll (salaries are not split out) and overstates local partner pay where profits flow to an international or cross-border partnership (amber rows). Limited partnerships (KB: Gernandt &amp; Danielsson, DLA Piper, Baker McKenzie, CMS Wistrand, Magnusson) do not file public accounts.</t>
         </is>
       </c>
     </row>
-    <row r="4" ht="45" customHeight="1">
+    <row r="4" ht="45" customHeight="1" s="108">
       <c r="A4" s="52" t="inlineStr">
         <is>
           <t>Firm</t>

</xml_diff>

<commit_message>
Add Nordic market comparison (SE/NO/DK/FI), FX conversions and A. Nordic market tab
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01Tu61bPEQej1E6sErbEFanY
</commit_message>
<xml_diff>
--- a/research/swedish_legal_market.xlsx
+++ b/research/swedish_legal_market.xlsx
@@ -8,20 +8,21 @@
   </bookViews>
   <sheets>
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="A. Market size" sheetId="1" state="visible" r:id="rId1"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="A. Growth drivers" sheetId="2" state="visible" r:id="rId2"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="A. Niche firms" sheetId="3" state="visible" r:id="rId3"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="B. Practice rankings" sheetId="4" state="visible" r:id="rId4"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="B. Rankings raw" sheetId="5" state="visible" r:id="rId5"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="B. Top lawyers" sheetId="6" state="visible" r:id="rId6"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="B. Partner pipeline" sheetId="7" state="visible" r:id="rId7"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="C. Benchmarking" sheetId="8" state="visible" r:id="rId8"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="D. Rate cards" sheetId="9" state="visible" r:id="rId9"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="E. Partner compensation" sheetId="10" state="visible" r:id="rId10"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="F. M&amp;A &amp; team lifts" sheetId="11" state="visible" r:id="rId11"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="A. Nordic market" sheetId="2" state="visible" r:id="rId2"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="A. Growth drivers" sheetId="3" state="visible" r:id="rId3"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="A. Niche firms" sheetId="4" state="visible" r:id="rId4"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="B. Practice rankings" sheetId="5" state="visible" r:id="rId5"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="B. Rankings raw" sheetId="6" state="visible" r:id="rId6"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="B. Top lawyers" sheetId="7" state="visible" r:id="rId7"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="B. Partner pipeline" sheetId="8" state="visible" r:id="rId8"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="C. Benchmarking" sheetId="9" state="visible" r:id="rId9"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="D. Rate cards" sheetId="10" state="visible" r:id="rId10"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="E. Partner compensation" sheetId="11" state="visible" r:id="rId11"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="F. M&amp;A &amp; team lifts" sheetId="12" state="visible" r:id="rId12"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="4" hidden="1">'B. Rankings raw'!$A$1:$E$661</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="6" hidden="1">'B. Partner pipeline'!$A$4:$K$176</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="5" hidden="1">'B. Rankings raw'!$A$1:$E$661</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="7" hidden="1">'B. Partner pipeline'!$A$4:$K$176</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -29,12 +30,13 @@
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <numFmts count="3">
+  <numFmts count="4">
     <numFmt numFmtId="164" formatCode="0.0"/>
     <numFmt numFmtId="165" formatCode="+0%;-0%"/>
     <numFmt numFmtId="166" formatCode="#,##0.0"/>
+    <numFmt numFmtId="167" formatCode="0.0000"/>
   </numFmts>
-  <fonts count="10">
+  <fonts count="11">
     <font>
       <name val="Calibri"/>
       <family val="2"/>
@@ -74,6 +76,11 @@
       <b val="1"/>
       <color rgb="001F3864"/>
       <sz val="12"/>
+    </font>
+    <font>
+      <b val="1"/>
+      <color rgb="001F3864"/>
+      <sz val="11"/>
     </font>
   </fonts>
   <fills count="12">
@@ -380,7 +387,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="124">
+  <cellXfs count="128">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
@@ -702,6 +709,12 @@
     </xf>
     <xf numFmtId="0" fontId="0" fillId="9" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="10" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="167" fontId="0" fillId="0" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="3" fontId="5" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="1" fontId="0" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="top" wrapText="1"/>
     </xf>
   </cellXfs>
   <cellStyles count="1">
@@ -1472,6 +1485,1192 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
+  <dimension ref="A1:Q44"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="26" customWidth="1" style="112" min="1" max="1"/>
+    <col width="20" customWidth="1" style="112" min="2" max="2"/>
+    <col width="28" customWidth="1" style="112" min="3" max="3"/>
+    <col width="10" customWidth="1" style="112" min="4" max="4"/>
+    <col width="10" customWidth="1" style="112" min="5" max="5"/>
+    <col width="12" customWidth="1" style="112" min="6" max="6"/>
+    <col width="12" customWidth="1" style="112" min="7" max="7"/>
+    <col width="10" customWidth="1" style="112" min="8" max="8"/>
+    <col width="10" customWidth="1" style="112" min="9" max="9"/>
+    <col width="10" customWidth="1" style="112" min="10" max="10"/>
+    <col width="10" customWidth="1" style="112" min="11" max="11"/>
+    <col width="10" customWidth="1" style="112" min="12" max="12"/>
+    <col width="10" customWidth="1" style="112" min="13" max="13"/>
+    <col width="10" customWidth="1" style="112" min="14" max="14"/>
+    <col width="10" customWidth="1" style="112" min="15" max="15"/>
+    <col width="40" customWidth="1" style="112" min="16" max="16"/>
+    <col width="40" customWidth="1" style="112" min="17" max="17"/>
+  </cols>
+  <sheetData>
+    <row r="1">
+      <c r="A1" s="1" t="inlineStr">
+        <is>
+          <t>Section D. Rate card comparison: Swedish business law firms (SEK per hour, excl. VAT)</t>
+        </is>
+      </c>
+    </row>
+    <row r="2" ht="45" customHeight="1" s="112">
+      <c r="A2" s="2" t="inlineStr">
+        <is>
+          <t>Rates are only comparable when dated: Swedish firms typically revise rates annually on 1 January. Public-sector price annexes are usually confidential (Kammarrätten i Stockholm, 2017, Vinge / E-hälsomyndigheten), so firm-level rate cards are scarce. Source type matters: list price (rate card) vs realised (actual billed) rates. Nordic business-law data only, 2023 onwards.</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" s="47" t="inlineStr">
+        <is>
+          <t>D1. Rate cards by level (list prices)</t>
+        </is>
+      </c>
+    </row>
+    <row r="5" ht="42" customHeight="1" s="112">
+      <c r="A5" s="52" t="inlineStr">
+        <is>
+          <t>Firm</t>
+        </is>
+      </c>
+      <c r="B5" s="52" t="inlineStr">
+        <is>
+          <t>Rate date</t>
+        </is>
+      </c>
+      <c r="C5" s="52" t="inlineStr">
+        <is>
+          <t>Source</t>
+        </is>
+      </c>
+      <c r="D5" s="52" t="inlineStr">
+        <is>
+          <t>Partner</t>
+        </is>
+      </c>
+      <c r="E5" s="84" t="n"/>
+      <c r="F5" s="52" t="inlineStr">
+        <is>
+          <t>Counsel / Senior associate</t>
+        </is>
+      </c>
+      <c r="G5" s="84" t="n"/>
+      <c r="H5" s="52" t="inlineStr">
+        <is>
+          <t>Associate</t>
+        </is>
+      </c>
+      <c r="I5" s="84" t="n"/>
+      <c r="J5" s="52" t="inlineStr">
+        <is>
+          <t>Junior associate</t>
+        </is>
+      </c>
+      <c r="K5" s="84" t="n"/>
+      <c r="L5" s="52" t="inlineStr">
+        <is>
+          <t>Paralegal</t>
+        </is>
+      </c>
+      <c r="M5" s="52" t="inlineStr">
+        <is>
+          <t>Partner mid</t>
+        </is>
+      </c>
+      <c r="N5" s="52" t="inlineStr">
+        <is>
+          <t>Junior mid</t>
+        </is>
+      </c>
+      <c r="O5" s="52" t="inlineStr">
+        <is>
+          <t>Partner / junior (x)</t>
+        </is>
+      </c>
+      <c r="P5" s="52" t="inlineStr">
+        <is>
+          <t>Level definitions in source</t>
+        </is>
+      </c>
+      <c r="Q5" s="52" t="inlineStr">
+        <is>
+          <t>Notes</t>
+        </is>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" s="85" t="n"/>
+      <c r="B6" s="85" t="n"/>
+      <c r="C6" s="85" t="n"/>
+      <c r="D6" s="86" t="inlineStr">
+        <is>
+          <t>Low</t>
+        </is>
+      </c>
+      <c r="E6" s="86" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
+      <c r="F6" s="86" t="inlineStr">
+        <is>
+          <t>Low</t>
+        </is>
+      </c>
+      <c r="G6" s="86" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
+      <c r="H6" s="86" t="inlineStr">
+        <is>
+          <t>Low</t>
+        </is>
+      </c>
+      <c r="I6" s="86" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
+      <c r="J6" s="86" t="inlineStr">
+        <is>
+          <t>Low</t>
+        </is>
+      </c>
+      <c r="K6" s="86" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
+      <c r="L6" s="85" t="n"/>
+      <c r="M6" s="85" t="n"/>
+      <c r="N6" s="85" t="n"/>
+      <c r="O6" s="85" t="n"/>
+      <c r="P6" s="85" t="n"/>
+      <c r="Q6" s="85" t="n"/>
+    </row>
+    <row r="7" ht="60" customHeight="1" s="112">
+      <c r="A7" s="49" t="inlineStr">
+        <is>
+          <t>Mannheimer Swartling</t>
+        </is>
+      </c>
+      <c r="B7" s="49" t="inlineStr">
+        <is>
+          <t>Not stated (provided by colleague, Oct-26)</t>
+        </is>
+      </c>
+      <c r="C7" s="49" t="inlineStr">
+        <is>
+          <t>Firm rate card (client-provided snip)</t>
+        </is>
+      </c>
+      <c r="D7" s="87" t="n">
+        <v>6000</v>
+      </c>
+      <c r="E7" s="87" t="n">
+        <v>10000</v>
+      </c>
+      <c r="F7" s="87" t="n">
+        <v>4550</v>
+      </c>
+      <c r="G7" s="87" t="n">
+        <v>8000</v>
+      </c>
+      <c r="H7" s="87" t="n">
+        <v>3650</v>
+      </c>
+      <c r="I7" s="87" t="n">
+        <v>4150</v>
+      </c>
+      <c r="J7" s="87" t="n">
+        <v>2750</v>
+      </c>
+      <c r="K7" s="87" t="n">
+        <v>3350</v>
+      </c>
+      <c r="L7" s="87" t="n"/>
+      <c r="M7" s="87">
+        <f>AVERAGE(D7:E7)</f>
+        <v/>
+      </c>
+      <c r="N7" s="87">
+        <f>AVERAGE(J7:K7)</f>
+        <v/>
+      </c>
+      <c r="O7" s="88">
+        <f>M7/N7</f>
+        <v/>
+      </c>
+      <c r="P7" s="49" t="inlineStr">
+        <is>
+          <t>Junior Assoc 0-24 months; Associates 25-59 months; Senior Assoc / PDL / Specialist Counsel 60+ months; Partners / Senior Advisor</t>
+        </is>
+      </c>
+      <c r="Q7" s="49" t="inlineStr">
+        <is>
+          <t>Counsel band (4,550-8,000) overlaps partner band. Date to be confirmed.</t>
+        </is>
+      </c>
+    </row>
+    <row r="8" ht="60" customHeight="1" s="112">
+      <c r="A8" s="49" t="inlineStr">
+        <is>
+          <t>Cederquist</t>
+        </is>
+      </c>
+      <c r="B8" s="49" t="inlineStr">
+        <is>
+          <t>2025 (revised annually 1 Jan)</t>
+        </is>
+      </c>
+      <c r="C8" s="49" t="inlineStr">
+        <is>
+          <t>Firm cost estimate / fee structure (client-provided snip)</t>
+        </is>
+      </c>
+      <c r="D8" s="87" t="n">
+        <v>6500</v>
+      </c>
+      <c r="E8" s="87" t="n">
+        <v>8000</v>
+      </c>
+      <c r="F8" s="87" t="n">
+        <v>4500</v>
+      </c>
+      <c r="G8" s="87" t="n">
+        <v>5800</v>
+      </c>
+      <c r="H8" s="87" t="n">
+        <v>3600</v>
+      </c>
+      <c r="I8" s="87" t="n">
+        <v>4100</v>
+      </c>
+      <c r="J8" s="87" t="n">
+        <v>2300</v>
+      </c>
+      <c r="K8" s="87" t="n">
+        <v>3100</v>
+      </c>
+      <c r="L8" s="87" t="n">
+        <v>1500</v>
+      </c>
+      <c r="M8" s="87">
+        <f>AVERAGE(D8:E8)</f>
+        <v/>
+      </c>
+      <c r="N8" s="87">
+        <f>AVERAGE(J8:K8)</f>
+        <v/>
+      </c>
+      <c r="O8" s="88">
+        <f>M8/N8</f>
+        <v/>
+      </c>
+      <c r="P8" s="49" t="inlineStr">
+        <is>
+          <t>Partners; Senior Associates; Associates; Junior Associates; Paralegals</t>
+        </is>
+      </c>
+      <c r="Q8" s="49" t="inlineStr">
+        <is>
+          <t>Time-incurred basis; open to alternative fee arrangements per project.</t>
+        </is>
+      </c>
+    </row>
+    <row r="9" ht="60" customHeight="1" s="112">
+      <c r="A9" s="49" t="inlineStr">
+        <is>
+          <t>MAQS</t>
+        </is>
+      </c>
+      <c r="B9" s="49" t="inlineStr">
+        <is>
+          <t>Sell-side model (Oct-2026)</t>
+        </is>
+      </c>
+      <c r="C9" s="49" t="inlineStr">
+        <is>
+          <t>Sell-side model (vendor financial model)</t>
+        </is>
+      </c>
+      <c r="D9" s="87" t="n">
+        <v>5014.83020687709</v>
+      </c>
+      <c r="E9" s="87" t="n">
+        <v>5014.83020687709</v>
+      </c>
+      <c r="F9" s="87" t="n"/>
+      <c r="G9" s="87" t="n"/>
+      <c r="H9" s="87" t="n">
+        <v>2753.06754681269</v>
+      </c>
+      <c r="I9" s="87" t="n">
+        <v>2753.06754681269</v>
+      </c>
+      <c r="J9" s="87" t="n"/>
+      <c r="K9" s="87" t="n"/>
+      <c r="L9" s="87" t="n"/>
+      <c r="M9" s="87">
+        <f>AVERAGE(D9:E9)</f>
+        <v/>
+      </c>
+      <c r="N9" s="87" t="n"/>
+      <c r="O9" s="88" t="n"/>
+      <c r="P9" s="49" t="inlineStr">
+        <is>
+          <t>Partner; Associate (single rates)</t>
+        </is>
+      </c>
+      <c r="Q9" s="49" t="inlineStr">
+        <is>
+          <t>Single model rates, not a published rate card range; confirm whether list or realised (effective) rates.</t>
+        </is>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" s="46" t="inlineStr">
+        <is>
+          <t>Difference: Mannheimer Swartling vs Cederquist (mid-points)</t>
+        </is>
+      </c>
+      <c r="D10" s="89">
+        <f>AVERAGE(D7:E7)/AVERAGE(D8:E8)-1</f>
+        <v/>
+      </c>
+      <c r="F10" s="89">
+        <f>AVERAGE(F7:G7)/AVERAGE(F8:G8)-1</f>
+        <v/>
+      </c>
+      <c r="H10" s="89">
+        <f>AVERAGE(H7:I7)/AVERAGE(H8:I8)-1</f>
+        <v/>
+      </c>
+      <c r="J10" s="89">
+        <f>AVERAGE(J7:K7)/AVERAGE(J8:K8)-1</f>
+        <v/>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" s="46" t="inlineStr">
+        <is>
+          <t>MAQS (sell-side model) vs Cederquist mid-point</t>
+        </is>
+      </c>
+      <c r="D11" s="89">
+        <f>D9/AVERAGE(D8:E8)-1</f>
+        <v/>
+      </c>
+      <c r="H11" s="89">
+        <f>H9/AVERAGE(H8:I8)-1</f>
+        <v/>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" s="46" t="inlineStr">
+        <is>
+          <t>MAQS (sell-side model) vs Mannheimer Swartling mid-point</t>
+        </is>
+      </c>
+      <c r="D12" s="89">
+        <f>D9/AVERAGE(D7:E7)-1</f>
+        <v/>
+      </c>
+      <c r="H12" s="89">
+        <f>H9/AVERAGE(H7:I7)-1</f>
+        <v/>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" s="47" t="inlineStr">
+        <is>
+          <t>D2. Indicative firm-wide hourly ranges (third-party directory, low reliability)</t>
+        </is>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" s="52" t="inlineStr">
+        <is>
+          <t>Firm</t>
+        </is>
+      </c>
+      <c r="B15" s="52" t="inlineStr">
+        <is>
+          <t>Accessed</t>
+        </is>
+      </c>
+      <c r="C15" s="52" t="inlineStr">
+        <is>
+          <t>Source</t>
+        </is>
+      </c>
+      <c r="D15" s="52" t="inlineStr">
+        <is>
+          <t>Low (~associate)</t>
+        </is>
+      </c>
+      <c r="E15" s="52" t="inlineStr">
+        <is>
+          <t>High (~partner)</t>
+        </is>
+      </c>
+      <c r="F15" s="52" t="inlineStr">
+        <is>
+          <t>Mid</t>
+        </is>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" s="49" t="inlineStr">
+        <is>
+          <t>Mannheimer Swartling</t>
+        </is>
+      </c>
+      <c r="B16" s="49" t="inlineStr">
+        <is>
+          <t>Oct-2026 (undated on site)</t>
+        </is>
+      </c>
+      <c r="C16" s="49" t="inlineStr">
+        <is>
+          <t>skatterätt.se firm pages (tax practice; no level split, no source)</t>
+        </is>
+      </c>
+      <c r="D16" s="87" t="n">
+        <v>4500</v>
+      </c>
+      <c r="E16" s="87" t="n">
+        <v>8000</v>
+      </c>
+      <c r="F16" s="87">
+        <f>AVERAGE(D16:E16)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" s="49" t="inlineStr">
+        <is>
+          <t>Roschier</t>
+        </is>
+      </c>
+      <c r="B17" s="49" t="inlineStr">
+        <is>
+          <t>Oct-2026 (undated on site)</t>
+        </is>
+      </c>
+      <c r="C17" s="49" t="inlineStr">
+        <is>
+          <t>skatterätt.se firm pages (tax practice; no level split, no source)</t>
+        </is>
+      </c>
+      <c r="D17" s="87" t="n">
+        <v>4200</v>
+      </c>
+      <c r="E17" s="87" t="n">
+        <v>7000</v>
+      </c>
+      <c r="F17" s="87">
+        <f>AVERAGE(D17:E17)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="18">
+      <c r="A18" s="49" t="inlineStr">
+        <is>
+          <t>Vinge</t>
+        </is>
+      </c>
+      <c r="B18" s="49" t="inlineStr">
+        <is>
+          <t>Oct-2026 (undated on site)</t>
+        </is>
+      </c>
+      <c r="C18" s="49" t="inlineStr">
+        <is>
+          <t>skatterätt.se firm pages (tax practice; no level split, no source)</t>
+        </is>
+      </c>
+      <c r="D18" s="87" t="n">
+        <v>4000</v>
+      </c>
+      <c r="E18" s="87" t="n">
+        <v>7000</v>
+      </c>
+      <c r="F18" s="87">
+        <f>AVERAGE(D18:E18)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="19">
+      <c r="A19" s="49" t="inlineStr">
+        <is>
+          <t>DLA Piper</t>
+        </is>
+      </c>
+      <c r="B19" s="49" t="inlineStr">
+        <is>
+          <t>Oct-2026 (undated on site)</t>
+        </is>
+      </c>
+      <c r="C19" s="49" t="inlineStr">
+        <is>
+          <t>skatterätt.se firm pages (tax practice; no level split, no source)</t>
+        </is>
+      </c>
+      <c r="D19" s="87" t="n">
+        <v>4000</v>
+      </c>
+      <c r="E19" s="87" t="n">
+        <v>7000</v>
+      </c>
+      <c r="F19" s="87">
+        <f>AVERAGE(D19:E19)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="20">
+      <c r="A20" s="49" t="inlineStr">
+        <is>
+          <t>Schjødt</t>
+        </is>
+      </c>
+      <c r="B20" s="49" t="inlineStr">
+        <is>
+          <t>Oct-2026 (undated on site)</t>
+        </is>
+      </c>
+      <c r="C20" s="49" t="inlineStr">
+        <is>
+          <t>skatterätt.se firm pages (tax practice; no level split, no source)</t>
+        </is>
+      </c>
+      <c r="D20" s="87" t="n">
+        <v>3800</v>
+      </c>
+      <c r="E20" s="87" t="n">
+        <v>6500</v>
+      </c>
+      <c r="F20" s="87">
+        <f>AVERAGE(D20:E20)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="21">
+      <c r="A21" s="49" t="inlineStr">
+        <is>
+          <t>Cederquist</t>
+        </is>
+      </c>
+      <c r="B21" s="49" t="inlineStr">
+        <is>
+          <t>Oct-2026 (undated on site)</t>
+        </is>
+      </c>
+      <c r="C21" s="49" t="inlineStr">
+        <is>
+          <t>skatterätt.se firm pages (tax practice; no level split, no source)</t>
+        </is>
+      </c>
+      <c r="D21" s="87" t="n">
+        <v>3800</v>
+      </c>
+      <c r="E21" s="87" t="n">
+        <v>6500</v>
+      </c>
+      <c r="F21" s="87">
+        <f>AVERAGE(D21:E21)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="22">
+      <c r="A22" s="49" t="inlineStr">
+        <is>
+          <t>Setterwalls</t>
+        </is>
+      </c>
+      <c r="B22" s="49" t="inlineStr">
+        <is>
+          <t>Oct-2026 (undated on site)</t>
+        </is>
+      </c>
+      <c r="C22" s="49" t="inlineStr">
+        <is>
+          <t>skatterätt.se firm pages (tax practice; no level split, no source)</t>
+        </is>
+      </c>
+      <c r="D22" s="87" t="n">
+        <v>3500</v>
+      </c>
+      <c r="E22" s="87" t="n">
+        <v>6000</v>
+      </c>
+      <c r="F22" s="87">
+        <f>AVERAGE(D22:E22)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="23">
+      <c r="A23" s="49" t="inlineStr">
+        <is>
+          <t>Bird &amp; Bird</t>
+        </is>
+      </c>
+      <c r="B23" s="49" t="inlineStr">
+        <is>
+          <t>Oct-2026 (undated on site)</t>
+        </is>
+      </c>
+      <c r="C23" s="49" t="inlineStr">
+        <is>
+          <t>skatterätt.se firm pages (tax practice; no level split, no source)</t>
+        </is>
+      </c>
+      <c r="D23" s="87" t="n">
+        <v>3500</v>
+      </c>
+      <c r="E23" s="87" t="n">
+        <v>6000</v>
+      </c>
+      <c r="F23" s="87">
+        <f>AVERAGE(D23:E23)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="24">
+      <c r="A24" s="49" t="inlineStr">
+        <is>
+          <t>Delphi</t>
+        </is>
+      </c>
+      <c r="B24" s="49" t="inlineStr">
+        <is>
+          <t>Oct-2026 (undated on site)</t>
+        </is>
+      </c>
+      <c r="C24" s="49" t="inlineStr">
+        <is>
+          <t>skatterätt.se firm pages (tax practice; no level split, no source)</t>
+        </is>
+      </c>
+      <c r="D24" s="87" t="n">
+        <v>3200</v>
+      </c>
+      <c r="E24" s="87" t="n">
+        <v>5500</v>
+      </c>
+      <c r="F24" s="87">
+        <f>AVERAGE(D24:E24)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="25">
+      <c r="A25" s="49" t="inlineStr">
+        <is>
+          <t>Lindahl</t>
+        </is>
+      </c>
+      <c r="B25" s="49" t="inlineStr">
+        <is>
+          <t>Oct-2026 (undated on site)</t>
+        </is>
+      </c>
+      <c r="C25" s="49" t="inlineStr">
+        <is>
+          <t>skatterätt.se firm pages (tax practice; no level split, no source)</t>
+        </is>
+      </c>
+      <c r="D25" s="87" t="n">
+        <v>3000</v>
+      </c>
+      <c r="E25" s="87" t="n">
+        <v>5500</v>
+      </c>
+      <c r="F25" s="87">
+        <f>AVERAGE(D25:E25)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="26">
+      <c r="A26" s="45" t="inlineStr">
+        <is>
+          <t>Example: https://www.xn--skattertt-12a.se/byra/vinge-skatt/ (Vinge: "Timarvode 4 000 till 7 000 kr"). Ranges may be estimates; use only for relative positioning.</t>
+        </is>
+      </c>
+    </row>
+    <row r="28">
+      <c r="A28" s="47" t="inlineStr">
+        <is>
+          <t>D3. Dated Nordic rate data points, 2023 onwards (realised rates and market commentary)</t>
+        </is>
+      </c>
+    </row>
+    <row r="29">
+      <c r="A29" s="52" t="inlineStr">
+        <is>
+          <t>Firm</t>
+        </is>
+      </c>
+      <c r="B29" s="52" t="inlineStr">
+        <is>
+          <t>Rate date</t>
+        </is>
+      </c>
+      <c r="C29" s="52" t="inlineStr">
+        <is>
+          <t>Level (as stated)</t>
+        </is>
+      </c>
+      <c r="D29" s="52" t="inlineStr">
+        <is>
+          <t>Mapped level</t>
+        </is>
+      </c>
+      <c r="E29" s="52" t="inlineStr">
+        <is>
+          <t>Rate low</t>
+        </is>
+      </c>
+      <c r="F29" s="52" t="inlineStr">
+        <is>
+          <t>Rate high</t>
+        </is>
+      </c>
+      <c r="G29" s="52" t="inlineStr">
+        <is>
+          <t>Context</t>
+        </is>
+      </c>
+      <c r="H29" s="52" t="inlineStr">
+        <is>
+          <t>Source type</t>
+        </is>
+      </c>
+      <c r="I29" s="52" t="inlineStr">
+        <is>
+          <t>Relevance</t>
+        </is>
+      </c>
+      <c r="J29" s="52" t="inlineStr">
+        <is>
+          <t>Source</t>
+        </is>
+      </c>
+    </row>
+    <row r="30">
+      <c r="A30" s="49" t="inlineStr">
+        <is>
+          <t>Mannheimer Swartling</t>
+        </is>
+      </c>
+      <c r="B30" s="49" t="inlineStr">
+        <is>
+          <t>Nov-2024 to Mar-2025</t>
+        </is>
+      </c>
+      <c r="C30" s="49" t="inlineStr">
+        <is>
+          <t>Average across team (~6,000 h, SEK 32m)</t>
+        </is>
+      </c>
+      <c r="D30" s="49" t="inlineStr">
+        <is>
+          <t>Blended (realised)</t>
+        </is>
+      </c>
+      <c r="E30" s="87" t="n">
+        <v>4000</v>
+      </c>
+      <c r="F30" s="87" t="n">
+        <v>4000</v>
+      </c>
+      <c r="G30" s="49" t="inlineStr">
+        <is>
+          <t>Northvolt restructuring (Swedish counsel in US Chapter 11); lowest average of all advisers</t>
+        </is>
+      </c>
+      <c r="H30" s="49" t="inlineStr">
+        <is>
+          <t>Court-approved fee filing (press)</t>
+        </is>
+      </c>
+      <c r="I30" s="49" t="inlineStr">
+        <is>
+          <t>Only published realised blended rate for a top Nordic firm: ~4,000 vs list partner 6,000-10,000</t>
+        </is>
+      </c>
+      <c r="J30" s="49" t="inlineStr">
+        <is>
+          <t>https://www.affarsvarlden.se/artikel/sa-dyrt-blev-northvolts-raddningsforsok-i-usa-debiteras-47-000-timmar</t>
+        </is>
+      </c>
+    </row>
+    <row r="31">
+      <c r="A31" s="49" t="inlineStr">
+        <is>
+          <t>Top-tier firms (Vinge, MSA, Roschier)</t>
+        </is>
+      </c>
+      <c r="B31" s="49" t="inlineStr">
+        <is>
+          <t>2026</t>
+        </is>
+      </c>
+      <c r="C31" s="49" t="inlineStr">
+        <is>
+          <t>Partner</t>
+        </is>
+      </c>
+      <c r="D31" s="49" t="inlineStr">
+        <is>
+          <t>Partner</t>
+        </is>
+      </c>
+      <c r="E31" s="87" t="n">
+        <v>7000</v>
+      </c>
+      <c r="F31" s="87" t="n">
+        <v>9000</v>
+      </c>
+      <c r="G31" s="49" t="inlineStr">
+        <is>
+          <t>Olle Flygt (ex-Vinge/MSA partner): partner bills 7-9k with 3-5 associates beneath</t>
+        </is>
+      </c>
+      <c r="H31" s="49" t="inlineStr">
+        <is>
+          <t>Market commentary</t>
+        </is>
+      </c>
+      <c r="I31" s="49" t="inlineStr">
+        <is>
+          <t>Current top-tier partner rate level</t>
+        </is>
+      </c>
+      <c r="J31" s="49" t="inlineStr">
+        <is>
+          <t>https://www.realtid.se/perfectweekend/affarsjuridikens-karna-det-har-blivit-for-mycket-fokus-pa-pengar/</t>
+        </is>
+      </c>
+    </row>
+    <row r="32">
+      <c r="A32" s="49" t="inlineStr">
+        <is>
+          <t>Top-tier firms (Vinge, MSA, Roschier)</t>
+        </is>
+      </c>
+      <c r="B32" s="49" t="inlineStr">
+        <is>
+          <t>2026</t>
+        </is>
+      </c>
+      <c r="C32" s="49" t="inlineStr">
+        <is>
+          <t>Biträdande jurist (associate)</t>
+        </is>
+      </c>
+      <c r="D32" s="49" t="inlineStr">
+        <is>
+          <t>Associate</t>
+        </is>
+      </c>
+      <c r="E32" s="87" t="n">
+        <v>3000</v>
+      </c>
+      <c r="F32" s="87" t="n">
+        <v>3000</v>
+      </c>
+      <c r="G32" s="49" t="inlineStr">
+        <is>
+          <t>As above: associates bill ~3,000 and cost at most a third of that</t>
+        </is>
+      </c>
+      <c r="H32" s="49" t="inlineStr">
+        <is>
+          <t>Market commentary</t>
+        </is>
+      </c>
+      <c r="I32" s="49" t="inlineStr">
+        <is>
+          <t>Associate rate and margin (leverage)</t>
+        </is>
+      </c>
+      <c r="J32" s="49" t="inlineStr">
+        <is>
+          <t>https://www.realtid.se/perfectweekend/affarsjuridikens-karna-det-har-blivit-for-mycket-fokus-pa-pengar/</t>
+        </is>
+      </c>
+    </row>
+    <row r="33">
+      <c r="A33" s="49" t="inlineStr">
+        <is>
+          <t>Mannheimer Swartling</t>
+        </is>
+      </c>
+      <c r="B33" s="49" t="inlineStr">
+        <is>
+          <t>Final years before 2025 (not specified)</t>
+        </is>
+      </c>
+      <c r="C33" s="49" t="inlineStr">
+        <is>
+          <t>Partner (Olle Flygt)</t>
+        </is>
+      </c>
+      <c r="D33" s="49" t="inlineStr">
+        <is>
+          <t>Partner</t>
+        </is>
+      </c>
+      <c r="E33" s="87" t="n">
+        <v>7000</v>
+      </c>
+      <c r="F33" s="87" t="n">
+        <v>8000</v>
+      </c>
+      <c r="G33" s="49" t="inlineStr">
+        <is>
+          <t>Own billing rate</t>
+        </is>
+      </c>
+      <c r="H33" s="49" t="inlineStr">
+        <is>
+          <t>Market commentary</t>
+        </is>
+      </c>
+      <c r="I33" s="49" t="inlineStr">
+        <is>
+          <t>Individual partner rate at MSA</t>
+        </is>
+      </c>
+      <c r="J33" s="49" t="inlineStr">
+        <is>
+          <t>https://www.realtid.se/juridik/affarsjuridiken-vaxer-men-sprickorna-syns/</t>
+        </is>
+      </c>
+    </row>
+    <row r="34">
+      <c r="A34" s="49" t="inlineStr">
+        <is>
+          <t>Law firm (unnamed)</t>
+        </is>
+      </c>
+      <c r="B34" s="49" t="inlineStr">
+        <is>
+          <t>Apr-2026</t>
+        </is>
+      </c>
+      <c r="C34" s="49" t="inlineStr">
+        <is>
+          <t>Hourly rate held reasonable</t>
+        </is>
+      </c>
+      <c r="D34" s="49" t="inlineStr">
+        <is>
+          <t>Blended</t>
+        </is>
+      </c>
+      <c r="E34" s="87" t="n">
+        <v>4000</v>
+      </c>
+      <c r="F34" s="87" t="n">
+        <v>4000</v>
+      </c>
+      <c r="G34" s="49" t="inlineStr">
+        <is>
+          <t>Luleå tingsrätt cost ruling</t>
+        </is>
+      </c>
+      <c r="H34" s="49" t="inlineStr">
+        <is>
+          <t>Court ruling (press)</t>
+        </is>
+      </c>
+      <c r="I34" s="49" t="inlineStr">
+        <is>
+          <t>Courts accept ~4,000/h as reasonable for business-law counsel</t>
+        </is>
+      </c>
+      <c r="J34" s="49" t="inlineStr">
+        <is>
+          <t>https://www.realtid.se/juridik/ratten-om-timarvoden-4-000-kronor-i-timmen-ar-ok/</t>
+        </is>
+      </c>
+    </row>
+    <row r="35">
+      <c r="A35" s="45" t="inlineStr">
+        <is>
+          <t>Removed: pre-2023 invoices and court claims (2007-2017), US firms, public-sector and legal-aid data (not relevant to a Nordic business-law investment).</t>
+        </is>
+      </c>
+    </row>
+    <row r="37">
+      <c r="A37" s="47" t="inlineStr">
+        <is>
+          <t>D4. Benchmarks (Nordic business law)</t>
+        </is>
+      </c>
+    </row>
+    <row r="38">
+      <c r="A38" s="52" t="inlineStr">
+        <is>
+          <t>Benchmark</t>
+        </is>
+      </c>
+      <c r="B38" s="52" t="inlineStr">
+        <is>
+          <t>Period</t>
+        </is>
+      </c>
+      <c r="C38" s="52" t="inlineStr">
+        <is>
+          <t>Rate</t>
+        </is>
+      </c>
+      <c r="D38" s="52" t="inlineStr">
+        <is>
+          <t>Currency</t>
+        </is>
+      </c>
+      <c r="E38" s="52" t="inlineStr">
+        <is>
+          <t>Notes</t>
+        </is>
+      </c>
+      <c r="F38" s="52" t="inlineStr">
+        <is>
+          <t>Source</t>
+        </is>
+      </c>
+    </row>
+    <row r="39">
+      <c r="A39" s="49" t="inlineStr">
+        <is>
+          <t>Affärsvärlden fee income per lawyer (panel)</t>
+        </is>
+      </c>
+      <c r="B39" s="49" t="inlineStr">
+        <is>
+          <t>2024</t>
+        </is>
+      </c>
+      <c r="C39" s="87" t="n">
+        <v>4130000</v>
+      </c>
+      <c r="D39" s="49" t="inlineStr">
+        <is>
+          <t>SEK p.a.</t>
+        </is>
+      </c>
+      <c r="E39" s="49" t="inlineStr">
+        <is>
+          <t>Implies ~SEK 2,580/h at 1,600 billable hours or ~2,950/h at 1,400 (illustrative)</t>
+        </is>
+      </c>
+      <c r="F39" s="49" t="inlineStr">
+        <is>
+          <t>https://www.realtid.se/affarer/154-miljarder-sa-klarade-affarsjuristerna-tullchocken/</t>
+        </is>
+      </c>
+    </row>
+    <row r="40">
+      <c r="A40" s="49" t="inlineStr">
+        <is>
+          <t>Affärsvärlden fee income per lawyer (panel)</t>
+        </is>
+      </c>
+      <c r="B40" s="49" t="inlineStr">
+        <is>
+          <t>2023</t>
+        </is>
+      </c>
+      <c r="C40" s="87" t="n">
+        <v>4220000</v>
+      </c>
+      <c r="D40" s="49" t="inlineStr">
+        <is>
+          <t>SEK p.a.</t>
+        </is>
+      </c>
+      <c r="E40" s="49" t="inlineStr"/>
+      <c r="F40" s="49" t="inlineStr">
+        <is>
+          <t>https://www.affarsvarlden.se/artikel/affarsjuristerna-om-trenden-pe-bolagen-kommer-vara-motorn</t>
+        </is>
+      </c>
+    </row>
+    <row r="41">
+      <c r="A41" s="49" t="inlineStr">
+        <is>
+          <t>Norway: commercial litigation rates</t>
+        </is>
+      </c>
+      <c r="B41" s="49" t="inlineStr">
+        <is>
+          <t>2026</t>
+        </is>
+      </c>
+      <c r="C41" s="87" t="n">
+        <v>3000</v>
+      </c>
+      <c r="D41" s="49" t="inlineStr">
+        <is>
+          <t>NOK/h (earlier level)</t>
+        </is>
+      </c>
+      <c r="E41" s="49" t="inlineStr">
+        <is>
+          <t>Norwegian Government Attorney: rates of ~NOK 3,000/h have "doubled in a short time"</t>
+        </is>
+      </c>
+      <c r="F41" s="49" t="inlineStr">
+        <is>
+          <t>https://www.realtid.se/juridik/regeringsadvokaten-slar-larm-advokatkostnaderna-skenar/</t>
+        </is>
+      </c>
+    </row>
+    <row r="43">
+      <c r="A43" s="45" t="inlineStr">
+        <is>
+          <t>Gaps: no published rate cards found for Vinge, White &amp; Case, Setterwalls, Lindahl, Gernandt &amp; Danielsson, CMS Wistrand, Cirio, Baker McKenzie, Snellman, Foyen, Glimstedt, Eversheds, Fylgia, Hammarskiöld, Magnusson, Kahn Pedersen, Wigge, Kastell, Westerberg or TM &amp; Partners.</t>
+        </is>
+      </c>
+    </row>
+    <row r="44">
+      <c r="A44" s="45" t="inlineStr">
+        <is>
+          <t>Routes to fill: client invoices (e.g. via Axo, requested); expert calls with Nordic GCs; confirm whether MAQS sell-side rates are list or realised.</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+  <mergeCells count="14">
+    <mergeCell ref="A5:A6"/>
+    <mergeCell ref="O5:O6"/>
+    <mergeCell ref="N5:N6"/>
+    <mergeCell ref="P5:P6"/>
+    <mergeCell ref="Q5:Q6"/>
+    <mergeCell ref="J5:K5"/>
+    <mergeCell ref="L5:L6"/>
+    <mergeCell ref="F5:G5"/>
+    <mergeCell ref="D5:E5"/>
+    <mergeCell ref="A2:Q2"/>
+    <mergeCell ref="H5:I5"/>
+    <mergeCell ref="M5:M6"/>
+    <mergeCell ref="B5:B6"/>
+    <mergeCell ref="C5:C6"/>
+  </mergeCells>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet11.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
   <dimension ref="A1:P51"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
@@ -3317,7 +4516,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet11.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet12.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
     <outlinePr summaryBelow="1" summaryRight="1"/>
@@ -5566,6 +6765,945 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
+  <dimension ref="A1:H46"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="34" customWidth="1" style="112" min="1" max="1"/>
+    <col width="30" customWidth="1" style="112" min="2" max="2"/>
+    <col width="28" customWidth="1" style="112" min="3" max="3"/>
+    <col width="28" customWidth="1" style="112" min="4" max="4"/>
+    <col width="24" customWidth="1" style="112" min="5" max="5"/>
+    <col width="30" customWidth="1" style="112" min="6" max="6"/>
+    <col width="50" customWidth="1" style="112" min="7" max="7"/>
+    <col width="34" customWidth="1" style="112" min="8" max="8"/>
+  </cols>
+  <sheetData>
+    <row r="1">
+      <c r="A1" s="1" t="inlineStr">
+        <is>
+          <t>A5. Nordic legal and business-law market comparison (SE, NO, DK, FI)</t>
+        </is>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" s="124" t="inlineStr">
+        <is>
+          <t>FX: Riksbank fixing, 12 Oct 2026 (latest published; SEK per unit)</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" s="99" t="inlineStr">
+        <is>
+          <t>Currency</t>
+        </is>
+      </c>
+      <c r="B4" s="99" t="inlineStr">
+        <is>
+          <t>SEK per unit</t>
+        </is>
+      </c>
+      <c r="C4" s="99" t="inlineStr">
+        <is>
+          <t>Source</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" s="6" t="inlineStr">
+        <is>
+          <t>USD</t>
+        </is>
+      </c>
+      <c r="B5" s="125" t="n">
+        <v>10.01386</v>
+      </c>
+      <c r="C5" s="6" t="inlineStr">
+        <is>
+          <t>https://api.riksbank.se/swea/v1/Observations/Latest/SEKUSDPMI (cross-checked vs ECB)</t>
+        </is>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" s="6" t="inlineStr">
+        <is>
+          <t>EUR</t>
+        </is>
+      </c>
+      <c r="B6" s="125" t="n">
+        <v>11.1965</v>
+      </c>
+      <c r="C6" s="6" t="inlineStr">
+        <is>
+          <t>https://api.riksbank.se/swea/v1/Observations/Latest/SEKEURPMI (cross-checked vs ECB)</t>
+        </is>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" s="6" t="inlineStr">
+        <is>
+          <t>NOK</t>
+        </is>
+      </c>
+      <c r="B7" s="125" t="n">
+        <v>1.04684</v>
+      </c>
+      <c r="C7" s="6" t="inlineStr">
+        <is>
+          <t>https://api.riksbank.se/swea/v1/Observations/Latest/SEKNOKPMI (cross-checked vs ECB)</t>
+        </is>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" s="6" t="inlineStr">
+        <is>
+          <t>DKK</t>
+        </is>
+      </c>
+      <c r="B8" s="125" t="n">
+        <v>1.4979</v>
+      </c>
+      <c r="C8" s="6" t="inlineStr">
+        <is>
+          <t>https://api.riksbank.se/swea/v1/Observations/Latest/SEKDKKPMI (cross-checked vs ECB)</t>
+        </is>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" s="124" t="inlineStr">
+        <is>
+          <t>Market size, 2024 (local currency m and SEK m at today's FX)</t>
+        </is>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" s="99" t="inlineStr">
+        <is>
+          <t>Measure</t>
+        </is>
+      </c>
+      <c r="B11" s="99" t="inlineStr">
+        <is>
+          <t>Country</t>
+        </is>
+      </c>
+      <c r="C11" s="99" t="inlineStr">
+        <is>
+          <t>Currency</t>
+        </is>
+      </c>
+      <c r="D11" s="99" t="inlineStr">
+        <is>
+          <t>Local (m)</t>
+        </is>
+      </c>
+      <c r="E11" s="99" t="inlineStr">
+        <is>
+          <t>SEK m</t>
+        </is>
+      </c>
+      <c r="F11" s="99" t="inlineStr">
+        <is>
+          <t>Year</t>
+        </is>
+      </c>
+      <c r="G11" s="99" t="inlineStr">
+        <is>
+          <t>Source / note</t>
+        </is>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" s="49" t="inlineStr">
+        <is>
+          <t>Legal activities (NACE 69.1), official</t>
+        </is>
+      </c>
+      <c r="B12" s="90" t="inlineStr">
+        <is>
+          <t>Sweden</t>
+        </is>
+      </c>
+      <c r="C12" s="90" t="inlineStr">
+        <is>
+          <t>SEK</t>
+        </is>
+      </c>
+      <c r="D12" s="100" t="n">
+        <v>38921</v>
+      </c>
+      <c r="E12" s="100">
+        <f>D12*1</f>
+        <v/>
+      </c>
+      <c r="F12" s="90" t="inlineStr">
+        <is>
+          <t>2024</t>
+        </is>
+      </c>
+      <c r="G12" s="49" t="inlineStr">
+        <is>
+          <t>SCB Företagens ekonomi</t>
+        </is>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" s="49" t="inlineStr">
+        <is>
+          <t>Legal activities (NACE 69.1), official</t>
+        </is>
+      </c>
+      <c r="B13" s="90" t="inlineStr">
+        <is>
+          <t>Norway</t>
+        </is>
+      </c>
+      <c r="C13" s="90" t="inlineStr">
+        <is>
+          <t>NOK</t>
+        </is>
+      </c>
+      <c r="D13" s="100" t="n">
+        <v>27518</v>
+      </c>
+      <c r="E13" s="100">
+        <f>D13*$B$7</f>
+        <v/>
+      </c>
+      <c r="F13" s="90" t="inlineStr">
+        <is>
+          <t>2024</t>
+        </is>
+      </c>
+      <c r="G13" s="49" t="inlineStr">
+        <is>
+          <t>SSB table 08206 / 12817</t>
+        </is>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" s="49" t="inlineStr">
+        <is>
+          <t>Legal activities (NACE 69.10), official</t>
+        </is>
+      </c>
+      <c r="B14" s="90" t="inlineStr">
+        <is>
+          <t>Denmark</t>
+        </is>
+      </c>
+      <c r="C14" s="90" t="inlineStr">
+        <is>
+          <t>DKK</t>
+        </is>
+      </c>
+      <c r="D14" s="100" t="n">
+        <v>19480</v>
+      </c>
+      <c r="E14" s="100">
+        <f>D14*$B$8</f>
+        <v/>
+      </c>
+      <c r="F14" s="90" t="inlineStr">
+        <is>
+          <t>2024</t>
+        </is>
+      </c>
+      <c r="G14" s="49" t="inlineStr">
+        <is>
+          <t>Danmarks Statistik GF11</t>
+        </is>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" s="49" t="inlineStr">
+        <is>
+          <t>Legal activities (TOL 691), official</t>
+        </is>
+      </c>
+      <c r="B15" s="90" t="inlineStr">
+        <is>
+          <t>Finland</t>
+        </is>
+      </c>
+      <c r="C15" s="90" t="inlineStr">
+        <is>
+          <t>EUR</t>
+        </is>
+      </c>
+      <c r="D15" s="100" t="n">
+        <v>1177</v>
+      </c>
+      <c r="E15" s="100">
+        <f>D15*$B$6</f>
+        <v/>
+      </c>
+      <c r="F15" s="90" t="inlineStr">
+        <is>
+          <t>2024</t>
+        </is>
+      </c>
+      <c r="G15" s="49" t="inlineStr">
+        <is>
+          <t>Statistics Finland 13w3 (2025: EUR 1,276m; incl. patent offices ~EUR 109m)</t>
+        </is>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" s="49" t="inlineStr">
+        <is>
+          <t>Business law: official / best estimate</t>
+        </is>
+      </c>
+      <c r="B16" s="90" t="inlineStr">
+        <is>
+          <t>Sweden</t>
+        </is>
+      </c>
+      <c r="C16" s="90" t="inlineStr">
+        <is>
+          <t>SEK</t>
+        </is>
+      </c>
+      <c r="D16" s="100" t="n">
+        <v>16000</v>
+      </c>
+      <c r="E16" s="100">
+        <f>D16*1</f>
+        <v/>
+      </c>
+      <c r="F16" s="90" t="inlineStr">
+        <is>
+          <t>2025</t>
+        </is>
+      </c>
+      <c r="G16" s="49" t="inlineStr">
+        <is>
+          <t>Afv panel of 56 largest firms (floor); industry estimate &gt;SEK 25bn</t>
+        </is>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" s="49" t="inlineStr">
+        <is>
+          <t>Business law: official / best estimate</t>
+        </is>
+      </c>
+      <c r="B17" s="90" t="inlineStr">
+        <is>
+          <t>Norway</t>
+        </is>
+      </c>
+      <c r="C17" s="90" t="inlineStr">
+        <is>
+          <t>NOK</t>
+        </is>
+      </c>
+      <c r="D17" s="100" t="n">
+        <v>15604</v>
+      </c>
+      <c r="E17" s="100">
+        <f>D17*$B$7</f>
+        <v/>
+      </c>
+      <c r="F17" s="90" t="inlineStr">
+        <is>
+          <t>2024</t>
+        </is>
+      </c>
+      <c r="G17" s="49" t="inlineStr">
+        <is>
+          <t>SSB service split "forretningsrett" (57% of 69.1)</t>
+        </is>
+      </c>
+    </row>
+    <row r="18">
+      <c r="A18" s="49" t="inlineStr">
+        <is>
+          <t>Business law: official / best estimate</t>
+        </is>
+      </c>
+      <c r="B18" s="90" t="inlineStr">
+        <is>
+          <t>Denmark</t>
+        </is>
+      </c>
+      <c r="C18" s="90" t="inlineStr">
+        <is>
+          <t>DKK</t>
+        </is>
+      </c>
+      <c r="D18" s="100" t="n">
+        <v>13050</v>
+      </c>
+      <c r="E18" s="100">
+        <f>D18*$B$8</f>
+        <v/>
+      </c>
+      <c r="F18" s="90" t="inlineStr">
+        <is>
+          <t>2024e</t>
+        </is>
+      </c>
+      <c r="G18" s="49" t="inlineStr">
+        <is>
+          <t>Estimate: business clients ~67% of sector turnover (2018, Økonomistyrelsen expert group) x 2024 turnover</t>
+        </is>
+      </c>
+    </row>
+    <row r="19">
+      <c r="A19" s="49" t="inlineStr">
+        <is>
+          <t>Business law: official / best estimate</t>
+        </is>
+      </c>
+      <c r="B19" s="90" t="inlineStr">
+        <is>
+          <t>Finland</t>
+        </is>
+      </c>
+      <c r="C19" s="90" t="inlineStr">
+        <is>
+          <t>EUR</t>
+        </is>
+      </c>
+      <c r="D19" s="100" t="n">
+        <v>600</v>
+      </c>
+      <c r="E19" s="100">
+        <f>D19*$B$6</f>
+        <v/>
+      </c>
+      <c r="F19" s="90" t="inlineStr">
+        <is>
+          <t>2025e</t>
+        </is>
+      </c>
+      <c r="G19" s="49" t="inlineStr">
+        <is>
+          <t>Estimate EUR 0.55-0.65bn: top-20 firms ~EUR 581m + tail</t>
+        </is>
+      </c>
+    </row>
+    <row r="20">
+      <c r="A20" s="46" t="inlineStr">
+        <is>
+          <t>Nordic total, legal activities</t>
+        </is>
+      </c>
+      <c r="E20" s="126">
+        <f>SUM(E12:E15)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="21">
+      <c r="A21" s="46" t="inlineStr">
+        <is>
+          <t>Nordic total, business law (estimate)</t>
+        </is>
+      </c>
+      <c r="E21" s="126">
+        <f>SUM(E16:E19)</f>
+        <v/>
+      </c>
+      <c r="G21" s="2" t="inlineStr">
+        <is>
+          <t>Sweden at panel floor (SEK 16bn); using SEK 20-25bn for Sweden gives ~SEK 64-69bn</t>
+        </is>
+      </c>
+    </row>
+    <row r="23">
+      <c r="A23" s="124" t="inlineStr">
+        <is>
+          <t>Structure and growth (Eurostat SBS M69.1, 2024, EUR; consistent basis)</t>
+        </is>
+      </c>
+    </row>
+    <row r="24">
+      <c r="A24" s="99" t="inlineStr">
+        <is>
+          <t>Country</t>
+        </is>
+      </c>
+      <c r="B24" s="99" t="inlineStr">
+        <is>
+          <t>Turnover EUR m</t>
+        </is>
+      </c>
+      <c r="C24" s="99" t="inlineStr">
+        <is>
+          <t>Turnover SEK m</t>
+        </is>
+      </c>
+      <c r="D24" s="99" t="inlineStr">
+        <is>
+          <t>Enterprises</t>
+        </is>
+      </c>
+      <c r="E24" s="99" t="inlineStr">
+        <is>
+          <t>Employees</t>
+        </is>
+      </c>
+      <c r="F24" s="99" t="inlineStr">
+        <is>
+          <t>Turnover / employee EUR k</t>
+        </is>
+      </c>
+      <c r="G24" s="99" t="inlineStr">
+        <is>
+          <t>Local CAGR</t>
+        </is>
+      </c>
+      <c r="H24" s="99" t="inlineStr">
+        <is>
+          <t>Lawyers (Bar)</t>
+        </is>
+      </c>
+    </row>
+    <row r="25">
+      <c r="A25" s="49" t="inlineStr">
+        <is>
+          <t>Sweden</t>
+        </is>
+      </c>
+      <c r="B25" s="100" t="n">
+        <v>3404.44</v>
+      </c>
+      <c r="C25" s="100">
+        <f>B25*$B$6</f>
+        <v/>
+      </c>
+      <c r="D25" s="100" t="n">
+        <v>6965</v>
+      </c>
+      <c r="E25" s="100" t="n">
+        <v>17521</v>
+      </c>
+      <c r="F25" s="127">
+        <f>B25/E25*1000</f>
+        <v/>
+      </c>
+      <c r="G25" s="49" t="inlineStr">
+        <is>
+          <t>~8% p.a. 2022-24 (SCB new series); 5.8% 2010-21</t>
+        </is>
+      </c>
+      <c r="H25" s="49" t="inlineStr">
+        <is>
+          <t>6,712 members (5,963 practising), end-2025</t>
+        </is>
+      </c>
+    </row>
+    <row r="26">
+      <c r="A26" s="49" t="inlineStr">
+        <is>
+          <t>Norway</t>
+        </is>
+      </c>
+      <c r="B26" s="100" t="n">
+        <v>2366.31</v>
+      </c>
+      <c r="C26" s="100">
+        <f>B26*$B$6</f>
+        <v/>
+      </c>
+      <c r="D26" s="100" t="n">
+        <v>2214</v>
+      </c>
+      <c r="E26" s="100" t="n">
+        <v>9264</v>
+      </c>
+      <c r="F26" s="127">
+        <f>B26/E26*1000</f>
+        <v/>
+      </c>
+      <c r="G26" s="49" t="inlineStr">
+        <is>
+          <t>9.3% p.a. 2019-24 (SSB)</t>
+        </is>
+      </c>
+      <c r="H26" s="49" t="inlineStr">
+        <is>
+          <t>10,756 Advokatforeningen members incl. trainees (2025)</t>
+        </is>
+      </c>
+    </row>
+    <row r="27">
+      <c r="A27" s="49" t="inlineStr">
+        <is>
+          <t>Denmark</t>
+        </is>
+      </c>
+      <c r="B27" s="100" t="n">
+        <v>2610.51</v>
+      </c>
+      <c r="C27" s="100">
+        <f>B27*$B$6</f>
+        <v/>
+      </c>
+      <c r="D27" s="100" t="n">
+        <v>1912</v>
+      </c>
+      <c r="E27" s="100" t="n">
+        <v>13158</v>
+      </c>
+      <c r="F27" s="127">
+        <f>B27/E27*1000</f>
+        <v/>
+      </c>
+      <c r="G27" s="49" t="inlineStr">
+        <is>
+          <t>4.5% p.a. 2019-24 (DST)</t>
+        </is>
+      </c>
+      <c r="H27" s="49" t="inlineStr">
+        <is>
+          <t>~7,760 lawyers incl. in-house (end-2025)</t>
+        </is>
+      </c>
+    </row>
+    <row r="28">
+      <c r="A28" s="49" t="inlineStr">
+        <is>
+          <t>Finland</t>
+        </is>
+      </c>
+      <c r="B28" s="100" t="n">
+        <v>1177.38</v>
+      </c>
+      <c r="C28" s="100">
+        <f>B28*$B$6</f>
+        <v/>
+      </c>
+      <c r="D28" s="100" t="n">
+        <v>2726</v>
+      </c>
+      <c r="E28" s="100" t="n">
+        <v>6509</v>
+      </c>
+      <c r="F28" s="127">
+        <f>B28/E28*1000</f>
+        <v/>
+      </c>
+      <c r="G28" s="49" t="inlineStr">
+        <is>
+          <t>4.9% p.a. 2019-25 (StatFin)</t>
+        </is>
+      </c>
+      <c r="H28" s="49" t="inlineStr">
+        <is>
+          <t>2,443 asianajajat + 1,778 licensed counsel (end-2025)</t>
+        </is>
+      </c>
+    </row>
+    <row r="29">
+      <c r="A29" s="46" t="inlineStr">
+        <is>
+          <t>Total</t>
+        </is>
+      </c>
+      <c r="B29" s="58">
+        <f>SUM(B25:B28)</f>
+        <v/>
+      </c>
+      <c r="C29" s="58">
+        <f>SUM(C25:C28)</f>
+        <v/>
+      </c>
+      <c r="D29" s="58">
+        <f>SUM(D25:D28)</f>
+        <v/>
+      </c>
+      <c r="E29" s="58">
+        <f>SUM(E25:E28)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="31">
+      <c r="A31" s="124" t="inlineStr">
+        <is>
+          <t>Leading firms and concentration</t>
+        </is>
+      </c>
+    </row>
+    <row r="32">
+      <c r="A32" s="99" t="inlineStr">
+        <is>
+          <t>Country</t>
+        </is>
+      </c>
+      <c r="B32" s="99" t="inlineStr">
+        <is>
+          <t>Largest firm (revenue)</t>
+        </is>
+      </c>
+      <c r="C32" s="99" t="inlineStr">
+        <is>
+          <t>Top-5 revenue</t>
+        </is>
+      </c>
+      <c r="D32" s="99" t="inlineStr">
+        <is>
+          <t>Concentration</t>
+        </is>
+      </c>
+      <c r="E32" s="99" t="inlineStr">
+        <is>
+          <t>Revenue per employee, large firms</t>
+        </is>
+      </c>
+      <c r="F32" s="99" t="inlineStr">
+        <is>
+          <t>Partner / hourly rate evidence</t>
+        </is>
+      </c>
+      <c r="G32" s="99" t="inlineStr">
+        <is>
+          <t>Ownership rules for external capital</t>
+        </is>
+      </c>
+    </row>
+    <row r="33">
+      <c r="A33" s="49" t="inlineStr">
+        <is>
+          <t>Sweden</t>
+        </is>
+      </c>
+      <c r="B33" s="49" t="inlineStr">
+        <is>
+          <t>Vinge SEK 2,036m (2025)</t>
+        </is>
+      </c>
+      <c r="C33" s="49" t="inlineStr">
+        <is>
+          <t>Top-5 ~46% of Afv panel (FY2024)</t>
+        </is>
+      </c>
+      <c r="D33" s="49" t="inlineStr">
+        <is>
+          <t>Top-10 ~66% of panel</t>
+        </is>
+      </c>
+      <c r="E33" s="49" t="inlineStr">
+        <is>
+          <t>SEK 3.1-3.9m (MSA, Vinge, 2025)</t>
+        </is>
+      </c>
+      <c r="F33" s="49" t="inlineStr">
+        <is>
+          <t>Partner list SEK 6,000-10,000/h (2025-26)</t>
+        </is>
+      </c>
+      <c r="G33" s="49" t="inlineStr">
+        <is>
+          <t>Bar firms lawyer-owned only; route = leave the Bar (AGRD: 9+ firms since 2025); Bar reviewing rules 2026</t>
+        </is>
+      </c>
+    </row>
+    <row r="34">
+      <c r="A34" s="49" t="inlineStr">
+        <is>
+          <t>Norway</t>
+        </is>
+      </c>
+      <c r="B34" s="49" t="inlineStr">
+        <is>
+          <t>Schjødt NOK 2,498m (2025, consolidated incl. SE/DK/UK)</t>
+        </is>
+      </c>
+      <c r="C34" s="49" t="inlineStr">
+        <is>
+          <t>NOK 9.4bn (2025): Schjødt, Wikborg Rein, Thommessen, BAHR, Wiersholm</t>
+        </is>
+      </c>
+      <c r="D34" s="49" t="inlineStr">
+        <is>
+          <t>Top-5 ~31% of SSB 69.1 (2024); top-100 NOK 22.2bn</t>
+        </is>
+      </c>
+      <c r="E34" s="49" t="inlineStr">
+        <is>
+          <t>NOK 4.7-5.5m (Thommessen, Wiersholm, BAHR, 2025)</t>
+        </is>
+      </c>
+      <c r="F34" s="49" t="inlineStr">
+        <is>
+          <t>Blended ~NOK 5,500/h (Wiersholm, court ruling)</t>
+        </is>
+      </c>
+      <c r="G34" s="49" t="inlineStr">
+        <is>
+          <t>Lawyers Act 2025: owners must work in the firm, lawyer board majority; passive / PE ownership not permitted for advokat firms</t>
+        </is>
+      </c>
+    </row>
+    <row r="35">
+      <c r="A35" s="49" t="inlineStr">
+        <is>
+          <t>Denmark</t>
+        </is>
+      </c>
+      <c r="B35" s="49" t="inlineStr">
+        <is>
+          <t>Gorrissen Federspiel DKK 1,311m (2025)</t>
+        </is>
+      </c>
+      <c r="C35" s="49" t="inlineStr">
+        <is>
+          <t>Gorrissen, Plesner, Bech-Bruun, Accura, DLA Piper ~DKK 5.5bn (2025)</t>
+        </is>
+      </c>
+      <c r="D35" s="49" t="inlineStr">
+        <is>
+          <t>Top-10 ~44% of sector (2022, KFST); est. 47-49% (2025)</t>
+        </is>
+      </c>
+      <c r="E35" s="49" t="inlineStr">
+        <is>
+          <t>DKK 2.4-2.55m per FTE (2025)</t>
+        </is>
+      </c>
+      <c r="F35" s="49" t="inlineStr">
+        <is>
+          <t>Partner DKK 2,057-5,400/h (2023, mid-market); Kammeradvokat DKK 2,710</t>
+        </is>
+      </c>
+      <c r="G35" s="49" t="inlineStr">
+        <is>
+          <t>Law-firm shares only for practising lawyers / staff (BEK 1427/2007); advocates' court monopoly</t>
+        </is>
+      </c>
+    </row>
+    <row r="36">
+      <c r="A36" s="49" t="inlineStr">
+        <is>
+          <t>Finland</t>
+        </is>
+      </c>
+      <c r="B36" s="49" t="inlineStr">
+        <is>
+          <t>Roschier EUR 99m (FY05/2026)</t>
+        </is>
+      </c>
+      <c r="C36" s="49" t="inlineStr">
+        <is>
+          <t>EUR ~349m: Roschier, Krogerus, Hannes Snellman, Borenius, Castrén &amp; Snellman</t>
+        </is>
+      </c>
+      <c r="D36" s="49" t="inlineStr">
+        <is>
+          <t>Top-5 ~27% of TOL 691 (2025); top-5 ~55% of top-30</t>
+        </is>
+      </c>
+      <c r="E36" s="49" t="inlineStr">
+        <is>
+          <t>EUR 205-384k per staff (top-10)</t>
+        </is>
+      </c>
+      <c r="F36" s="49" t="inlineStr">
+        <is>
+          <t>No current survey (2012 median EUR 200/h)</t>
+        </is>
+      </c>
+      <c r="G36" s="49" t="inlineStr">
+        <is>
+          <t>Bar firms lawyer-owned; licensed-counsel route gives full rights of audience; Fondia (listed, non-Bar)</t>
+        </is>
+      </c>
+    </row>
+    <row r="38">
+      <c r="A38" s="124" t="inlineStr">
+        <is>
+          <t>Consolidation and international activity, 2020-2026</t>
+        </is>
+      </c>
+    </row>
+    <row r="39">
+      <c r="A39" s="99" t="inlineStr">
+        <is>
+          <t>Country</t>
+        </is>
+      </c>
+      <c r="B39" s="99" t="inlineStr">
+        <is>
+          <t>Activity</t>
+        </is>
+      </c>
+    </row>
+    <row r="40">
+      <c r="A40" s="49" t="inlineStr">
+        <is>
+          <t>Sweden</t>
+        </is>
+      </c>
+      <c r="B40" s="49" t="inlineStr">
+        <is>
+          <t>AGRD (Axcel) roll-up of 9+ firms since Aug-2025 incl. Setterwalls Malmö; CMS-Wistrand (2024); BAHR Stockholm (2026); Schjødt-Hamilton (2020); Magnusson-Gro, Walthon Ramberg (2026); Hannes Snellman split (2024); MAQS split (2027)</t>
+        </is>
+      </c>
+    </row>
+    <row r="41">
+      <c r="A41" s="49" t="inlineStr">
+        <is>
+          <t>Norway</t>
+        </is>
+      </c>
+      <c r="B41" s="49" t="inlineStr">
+        <is>
+          <t>Schjødt-Hamilton SE (2020), Copenhagen (2022), Norrbom Vinding DK (Mar-2026); BAHR opens Stockholm and Copenhagen (2025-26) after hiring ~18 Schjødt partners; Ræder Bing (2023), Lippestad / Bache-Wiig and Tofte Hald (2024); Cedra buys Big-4 regional law offices (Dec-2025)</t>
+        </is>
+      </c>
+    </row>
+    <row r="42">
+      <c r="A42" s="49" t="inlineStr">
+        <is>
+          <t>Denmark</t>
+        </is>
+      </c>
+      <c r="B42" s="49" t="inlineStr">
+        <is>
+          <t>HortenDahl merger (Jan-2026); DLA Piper takes 49 from Lundgrens (Mar-2025); Schjødt-Norrbom Vinding (Mar-2026); Kromann Reumert converts to P/S (Nov-2025); proposal to open Kammeradvokat mandate (~DKK 0.7bn) to competition</t>
+        </is>
+      </c>
+    </row>
+    <row r="43">
+      <c r="A43" s="49" t="inlineStr">
+        <is>
+          <t>Finland</t>
+        </is>
+      </c>
+      <c r="B43" s="49" t="inlineStr">
+        <is>
+          <t>Hannes Snellman split (2024); DLA Piper-Project Law (2023); Merilampi-I&amp;O Partners (2025, single source); no PE investment found; Fondia (listed) shrinking</t>
+        </is>
+      </c>
+    </row>
+    <row r="45">
+      <c r="A45" s="45" t="inlineStr">
+        <is>
+          <t>Sources: SCB; SSB tables 08206 / 12817; Danmarks Statistik GF11 / REGN1; Statistics Finland 13w3; Eurostat sbs_ovw_act (M691); Advokatbladet / Kapital JUS (NO league tables); Proff.dk filed accounts and Økonomisk Ugebrev (DK); Asiakastieto / DM Faster (FI); Økonomistyrelsen expert group Dec-2024 (DK); national Bar associations.</t>
+        </is>
+      </c>
+    </row>
+    <row r="46">
+      <c r="A46" s="45" t="inlineStr">
+        <is>
+          <t>Caveats: official statistics measure all legal activities, not business law only (Norway is the only country publishing a business-law split). Firm revenues use different fiscal years and entity scopes (e.g. Schjødt consolidated). Business-law figures for Sweden, Denmark and Finland are estimates. FX: Riksbank 12 Oct 2026.</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
   <dimension ref="A1:F23"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
@@ -6119,7 +8257,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
     <outlinePr summaryBelow="1" summaryRight="1"/>
@@ -8721,7 +10859,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
     <outlinePr summaryBelow="1" summaryRight="1"/>
@@ -15634,7 +17772,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
     <outlinePr summaryBelow="1" summaryRight="1"/>
@@ -33503,7 +35641,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet7.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
     <outlinePr summaryBelow="1" summaryRight="1"/>
@@ -38011,7 +40149,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet7.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet8.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
     <outlinePr summaryBelow="1" summaryRight="1"/>
@@ -46537,7 +48675,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet8.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet9.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
     <outlinePr summaryBelow="1" summaryRight="1"/>
@@ -48721,1190 +50859,4 @@
   </mergeCells>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
-</file>
-
-<file path=xl/worksheets/sheet9.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <sheetPr>
-    <outlinePr summaryBelow="1" summaryRight="1"/>
-    <pageSetUpPr/>
-  </sheetPr>
-  <dimension ref="A1:Q44"/>
-  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
-  <cols>
-    <col width="26" customWidth="1" style="112" min="1" max="1"/>
-    <col width="20" customWidth="1" style="112" min="2" max="2"/>
-    <col width="28" customWidth="1" style="112" min="3" max="3"/>
-    <col width="10" customWidth="1" style="112" min="4" max="4"/>
-    <col width="10" customWidth="1" style="112" min="5" max="5"/>
-    <col width="12" customWidth="1" style="112" min="6" max="6"/>
-    <col width="12" customWidth="1" style="112" min="7" max="7"/>
-    <col width="10" customWidth="1" style="112" min="8" max="8"/>
-    <col width="10" customWidth="1" style="112" min="9" max="9"/>
-    <col width="10" customWidth="1" style="112" min="10" max="10"/>
-    <col width="10" customWidth="1" style="112" min="11" max="11"/>
-    <col width="10" customWidth="1" style="112" min="12" max="12"/>
-    <col width="10" customWidth="1" style="112" min="13" max="13"/>
-    <col width="10" customWidth="1" style="112" min="14" max="14"/>
-    <col width="10" customWidth="1" style="112" min="15" max="15"/>
-    <col width="40" customWidth="1" style="112" min="16" max="16"/>
-    <col width="40" customWidth="1" style="112" min="17" max="17"/>
-  </cols>
-  <sheetData>
-    <row r="1">
-      <c r="A1" s="1" t="inlineStr">
-        <is>
-          <t>Section D. Rate card comparison: Swedish business law firms (SEK per hour, excl. VAT)</t>
-        </is>
-      </c>
-    </row>
-    <row r="2" ht="45" customHeight="1" s="112">
-      <c r="A2" s="2" t="inlineStr">
-        <is>
-          <t>Rates are only comparable when dated: Swedish firms typically revise rates annually on 1 January. Public-sector price annexes are usually confidential (Kammarrätten i Stockholm, 2017, Vinge / E-hälsomyndigheten), so firm-level rate cards are scarce. Source type matters: list price (rate card) vs realised (actual billed) rates. Nordic business-law data only, 2023 onwards.</t>
-        </is>
-      </c>
-    </row>
-    <row r="4">
-      <c r="A4" s="47" t="inlineStr">
-        <is>
-          <t>D1. Rate cards by level (list prices)</t>
-        </is>
-      </c>
-    </row>
-    <row r="5" ht="42" customHeight="1" s="112">
-      <c r="A5" s="52" t="inlineStr">
-        <is>
-          <t>Firm</t>
-        </is>
-      </c>
-      <c r="B5" s="52" t="inlineStr">
-        <is>
-          <t>Rate date</t>
-        </is>
-      </c>
-      <c r="C5" s="52" t="inlineStr">
-        <is>
-          <t>Source</t>
-        </is>
-      </c>
-      <c r="D5" s="52" t="inlineStr">
-        <is>
-          <t>Partner</t>
-        </is>
-      </c>
-      <c r="E5" s="84" t="n"/>
-      <c r="F5" s="52" t="inlineStr">
-        <is>
-          <t>Counsel / Senior associate</t>
-        </is>
-      </c>
-      <c r="G5" s="84" t="n"/>
-      <c r="H5" s="52" t="inlineStr">
-        <is>
-          <t>Associate</t>
-        </is>
-      </c>
-      <c r="I5" s="84" t="n"/>
-      <c r="J5" s="52" t="inlineStr">
-        <is>
-          <t>Junior associate</t>
-        </is>
-      </c>
-      <c r="K5" s="84" t="n"/>
-      <c r="L5" s="52" t="inlineStr">
-        <is>
-          <t>Paralegal</t>
-        </is>
-      </c>
-      <c r="M5" s="52" t="inlineStr">
-        <is>
-          <t>Partner mid</t>
-        </is>
-      </c>
-      <c r="N5" s="52" t="inlineStr">
-        <is>
-          <t>Junior mid</t>
-        </is>
-      </c>
-      <c r="O5" s="52" t="inlineStr">
-        <is>
-          <t>Partner / junior (x)</t>
-        </is>
-      </c>
-      <c r="P5" s="52" t="inlineStr">
-        <is>
-          <t>Level definitions in source</t>
-        </is>
-      </c>
-      <c r="Q5" s="52" t="inlineStr">
-        <is>
-          <t>Notes</t>
-        </is>
-      </c>
-    </row>
-    <row r="6">
-      <c r="A6" s="85" t="n"/>
-      <c r="B6" s="85" t="n"/>
-      <c r="C6" s="85" t="n"/>
-      <c r="D6" s="86" t="inlineStr">
-        <is>
-          <t>Low</t>
-        </is>
-      </c>
-      <c r="E6" s="86" t="inlineStr">
-        <is>
-          <t>High</t>
-        </is>
-      </c>
-      <c r="F6" s="86" t="inlineStr">
-        <is>
-          <t>Low</t>
-        </is>
-      </c>
-      <c r="G6" s="86" t="inlineStr">
-        <is>
-          <t>High</t>
-        </is>
-      </c>
-      <c r="H6" s="86" t="inlineStr">
-        <is>
-          <t>Low</t>
-        </is>
-      </c>
-      <c r="I6" s="86" t="inlineStr">
-        <is>
-          <t>High</t>
-        </is>
-      </c>
-      <c r="J6" s="86" t="inlineStr">
-        <is>
-          <t>Low</t>
-        </is>
-      </c>
-      <c r="K6" s="86" t="inlineStr">
-        <is>
-          <t>High</t>
-        </is>
-      </c>
-      <c r="L6" s="85" t="n"/>
-      <c r="M6" s="85" t="n"/>
-      <c r="N6" s="85" t="n"/>
-      <c r="O6" s="85" t="n"/>
-      <c r="P6" s="85" t="n"/>
-      <c r="Q6" s="85" t="n"/>
-    </row>
-    <row r="7" ht="60" customHeight="1" s="112">
-      <c r="A7" s="49" t="inlineStr">
-        <is>
-          <t>Mannheimer Swartling</t>
-        </is>
-      </c>
-      <c r="B7" s="49" t="inlineStr">
-        <is>
-          <t>Not stated (provided by colleague, Oct-26)</t>
-        </is>
-      </c>
-      <c r="C7" s="49" t="inlineStr">
-        <is>
-          <t>Firm rate card (client-provided snip)</t>
-        </is>
-      </c>
-      <c r="D7" s="87" t="n">
-        <v>6000</v>
-      </c>
-      <c r="E7" s="87" t="n">
-        <v>10000</v>
-      </c>
-      <c r="F7" s="87" t="n">
-        <v>4550</v>
-      </c>
-      <c r="G7" s="87" t="n">
-        <v>8000</v>
-      </c>
-      <c r="H7" s="87" t="n">
-        <v>3650</v>
-      </c>
-      <c r="I7" s="87" t="n">
-        <v>4150</v>
-      </c>
-      <c r="J7" s="87" t="n">
-        <v>2750</v>
-      </c>
-      <c r="K7" s="87" t="n">
-        <v>3350</v>
-      </c>
-      <c r="L7" s="87" t="n"/>
-      <c r="M7" s="87">
-        <f>AVERAGE(D7:E7)</f>
-        <v/>
-      </c>
-      <c r="N7" s="87">
-        <f>AVERAGE(J7:K7)</f>
-        <v/>
-      </c>
-      <c r="O7" s="88">
-        <f>M7/N7</f>
-        <v/>
-      </c>
-      <c r="P7" s="49" t="inlineStr">
-        <is>
-          <t>Junior Assoc 0-24 months; Associates 25-59 months; Senior Assoc / PDL / Specialist Counsel 60+ months; Partners / Senior Advisor</t>
-        </is>
-      </c>
-      <c r="Q7" s="49" t="inlineStr">
-        <is>
-          <t>Counsel band (4,550-8,000) overlaps partner band. Date to be confirmed.</t>
-        </is>
-      </c>
-    </row>
-    <row r="8" ht="60" customHeight="1" s="112">
-      <c r="A8" s="49" t="inlineStr">
-        <is>
-          <t>Cederquist</t>
-        </is>
-      </c>
-      <c r="B8" s="49" t="inlineStr">
-        <is>
-          <t>2025 (revised annually 1 Jan)</t>
-        </is>
-      </c>
-      <c r="C8" s="49" t="inlineStr">
-        <is>
-          <t>Firm cost estimate / fee structure (client-provided snip)</t>
-        </is>
-      </c>
-      <c r="D8" s="87" t="n">
-        <v>6500</v>
-      </c>
-      <c r="E8" s="87" t="n">
-        <v>8000</v>
-      </c>
-      <c r="F8" s="87" t="n">
-        <v>4500</v>
-      </c>
-      <c r="G8" s="87" t="n">
-        <v>5800</v>
-      </c>
-      <c r="H8" s="87" t="n">
-        <v>3600</v>
-      </c>
-      <c r="I8" s="87" t="n">
-        <v>4100</v>
-      </c>
-      <c r="J8" s="87" t="n">
-        <v>2300</v>
-      </c>
-      <c r="K8" s="87" t="n">
-        <v>3100</v>
-      </c>
-      <c r="L8" s="87" t="n">
-        <v>1500</v>
-      </c>
-      <c r="M8" s="87">
-        <f>AVERAGE(D8:E8)</f>
-        <v/>
-      </c>
-      <c r="N8" s="87">
-        <f>AVERAGE(J8:K8)</f>
-        <v/>
-      </c>
-      <c r="O8" s="88">
-        <f>M8/N8</f>
-        <v/>
-      </c>
-      <c r="P8" s="49" t="inlineStr">
-        <is>
-          <t>Partners; Senior Associates; Associates; Junior Associates; Paralegals</t>
-        </is>
-      </c>
-      <c r="Q8" s="49" t="inlineStr">
-        <is>
-          <t>Time-incurred basis; open to alternative fee arrangements per project.</t>
-        </is>
-      </c>
-    </row>
-    <row r="9" ht="60" customHeight="1" s="112">
-      <c r="A9" s="49" t="inlineStr">
-        <is>
-          <t>MAQS</t>
-        </is>
-      </c>
-      <c r="B9" s="49" t="inlineStr">
-        <is>
-          <t>Sell-side model (Oct-2026)</t>
-        </is>
-      </c>
-      <c r="C9" s="49" t="inlineStr">
-        <is>
-          <t>Sell-side model (vendor financial model)</t>
-        </is>
-      </c>
-      <c r="D9" s="87" t="n">
-        <v>5014.83020687709</v>
-      </c>
-      <c r="E9" s="87" t="n">
-        <v>5014.83020687709</v>
-      </c>
-      <c r="F9" s="87" t="n"/>
-      <c r="G9" s="87" t="n"/>
-      <c r="H9" s="87" t="n">
-        <v>2753.06754681269</v>
-      </c>
-      <c r="I9" s="87" t="n">
-        <v>2753.06754681269</v>
-      </c>
-      <c r="J9" s="87" t="n"/>
-      <c r="K9" s="87" t="n"/>
-      <c r="L9" s="87" t="n"/>
-      <c r="M9" s="87">
-        <f>AVERAGE(D9:E9)</f>
-        <v/>
-      </c>
-      <c r="N9" s="87" t="n"/>
-      <c r="O9" s="88" t="n"/>
-      <c r="P9" s="49" t="inlineStr">
-        <is>
-          <t>Partner; Associate (single rates)</t>
-        </is>
-      </c>
-      <c r="Q9" s="49" t="inlineStr">
-        <is>
-          <t>Single model rates, not a published rate card range; confirm whether list or realised (effective) rates.</t>
-        </is>
-      </c>
-    </row>
-    <row r="10">
-      <c r="A10" s="46" t="inlineStr">
-        <is>
-          <t>Difference: Mannheimer Swartling vs Cederquist (mid-points)</t>
-        </is>
-      </c>
-      <c r="D10" s="89">
-        <f>AVERAGE(D7:E7)/AVERAGE(D8:E8)-1</f>
-        <v/>
-      </c>
-      <c r="F10" s="89">
-        <f>AVERAGE(F7:G7)/AVERAGE(F8:G8)-1</f>
-        <v/>
-      </c>
-      <c r="H10" s="89">
-        <f>AVERAGE(H7:I7)/AVERAGE(H8:I8)-1</f>
-        <v/>
-      </c>
-      <c r="J10" s="89">
-        <f>AVERAGE(J7:K7)/AVERAGE(J8:K8)-1</f>
-        <v/>
-      </c>
-    </row>
-    <row r="11">
-      <c r="A11" s="46" t="inlineStr">
-        <is>
-          <t>MAQS (sell-side model) vs Cederquist mid-point</t>
-        </is>
-      </c>
-      <c r="D11" s="89">
-        <f>D9/AVERAGE(D8:E8)-1</f>
-        <v/>
-      </c>
-      <c r="H11" s="89">
-        <f>H9/AVERAGE(H8:I8)-1</f>
-        <v/>
-      </c>
-    </row>
-    <row r="12">
-      <c r="A12" s="46" t="inlineStr">
-        <is>
-          <t>MAQS (sell-side model) vs Mannheimer Swartling mid-point</t>
-        </is>
-      </c>
-      <c r="D12" s="89">
-        <f>D9/AVERAGE(D7:E7)-1</f>
-        <v/>
-      </c>
-      <c r="H12" s="89">
-        <f>H9/AVERAGE(H7:I7)-1</f>
-        <v/>
-      </c>
-    </row>
-    <row r="14">
-      <c r="A14" s="47" t="inlineStr">
-        <is>
-          <t>D2. Indicative firm-wide hourly ranges (third-party directory, low reliability)</t>
-        </is>
-      </c>
-    </row>
-    <row r="15">
-      <c r="A15" s="52" t="inlineStr">
-        <is>
-          <t>Firm</t>
-        </is>
-      </c>
-      <c r="B15" s="52" t="inlineStr">
-        <is>
-          <t>Accessed</t>
-        </is>
-      </c>
-      <c r="C15" s="52" t="inlineStr">
-        <is>
-          <t>Source</t>
-        </is>
-      </c>
-      <c r="D15" s="52" t="inlineStr">
-        <is>
-          <t>Low (~associate)</t>
-        </is>
-      </c>
-      <c r="E15" s="52" t="inlineStr">
-        <is>
-          <t>High (~partner)</t>
-        </is>
-      </c>
-      <c r="F15" s="52" t="inlineStr">
-        <is>
-          <t>Mid</t>
-        </is>
-      </c>
-    </row>
-    <row r="16">
-      <c r="A16" s="49" t="inlineStr">
-        <is>
-          <t>Mannheimer Swartling</t>
-        </is>
-      </c>
-      <c r="B16" s="49" t="inlineStr">
-        <is>
-          <t>Oct-2026 (undated on site)</t>
-        </is>
-      </c>
-      <c r="C16" s="49" t="inlineStr">
-        <is>
-          <t>skatterätt.se firm pages (tax practice; no level split, no source)</t>
-        </is>
-      </c>
-      <c r="D16" s="87" t="n">
-        <v>4500</v>
-      </c>
-      <c r="E16" s="87" t="n">
-        <v>8000</v>
-      </c>
-      <c r="F16" s="87">
-        <f>AVERAGE(D16:E16)</f>
-        <v/>
-      </c>
-    </row>
-    <row r="17">
-      <c r="A17" s="49" t="inlineStr">
-        <is>
-          <t>Roschier</t>
-        </is>
-      </c>
-      <c r="B17" s="49" t="inlineStr">
-        <is>
-          <t>Oct-2026 (undated on site)</t>
-        </is>
-      </c>
-      <c r="C17" s="49" t="inlineStr">
-        <is>
-          <t>skatterätt.se firm pages (tax practice; no level split, no source)</t>
-        </is>
-      </c>
-      <c r="D17" s="87" t="n">
-        <v>4200</v>
-      </c>
-      <c r="E17" s="87" t="n">
-        <v>7000</v>
-      </c>
-      <c r="F17" s="87">
-        <f>AVERAGE(D17:E17)</f>
-        <v/>
-      </c>
-    </row>
-    <row r="18">
-      <c r="A18" s="49" t="inlineStr">
-        <is>
-          <t>Vinge</t>
-        </is>
-      </c>
-      <c r="B18" s="49" t="inlineStr">
-        <is>
-          <t>Oct-2026 (undated on site)</t>
-        </is>
-      </c>
-      <c r="C18" s="49" t="inlineStr">
-        <is>
-          <t>skatterätt.se firm pages (tax practice; no level split, no source)</t>
-        </is>
-      </c>
-      <c r="D18" s="87" t="n">
-        <v>4000</v>
-      </c>
-      <c r="E18" s="87" t="n">
-        <v>7000</v>
-      </c>
-      <c r="F18" s="87">
-        <f>AVERAGE(D18:E18)</f>
-        <v/>
-      </c>
-    </row>
-    <row r="19">
-      <c r="A19" s="49" t="inlineStr">
-        <is>
-          <t>DLA Piper</t>
-        </is>
-      </c>
-      <c r="B19" s="49" t="inlineStr">
-        <is>
-          <t>Oct-2026 (undated on site)</t>
-        </is>
-      </c>
-      <c r="C19" s="49" t="inlineStr">
-        <is>
-          <t>skatterätt.se firm pages (tax practice; no level split, no source)</t>
-        </is>
-      </c>
-      <c r="D19" s="87" t="n">
-        <v>4000</v>
-      </c>
-      <c r="E19" s="87" t="n">
-        <v>7000</v>
-      </c>
-      <c r="F19" s="87">
-        <f>AVERAGE(D19:E19)</f>
-        <v/>
-      </c>
-    </row>
-    <row r="20">
-      <c r="A20" s="49" t="inlineStr">
-        <is>
-          <t>Schjødt</t>
-        </is>
-      </c>
-      <c r="B20" s="49" t="inlineStr">
-        <is>
-          <t>Oct-2026 (undated on site)</t>
-        </is>
-      </c>
-      <c r="C20" s="49" t="inlineStr">
-        <is>
-          <t>skatterätt.se firm pages (tax practice; no level split, no source)</t>
-        </is>
-      </c>
-      <c r="D20" s="87" t="n">
-        <v>3800</v>
-      </c>
-      <c r="E20" s="87" t="n">
-        <v>6500</v>
-      </c>
-      <c r="F20" s="87">
-        <f>AVERAGE(D20:E20)</f>
-        <v/>
-      </c>
-    </row>
-    <row r="21">
-      <c r="A21" s="49" t="inlineStr">
-        <is>
-          <t>Cederquist</t>
-        </is>
-      </c>
-      <c r="B21" s="49" t="inlineStr">
-        <is>
-          <t>Oct-2026 (undated on site)</t>
-        </is>
-      </c>
-      <c r="C21" s="49" t="inlineStr">
-        <is>
-          <t>skatterätt.se firm pages (tax practice; no level split, no source)</t>
-        </is>
-      </c>
-      <c r="D21" s="87" t="n">
-        <v>3800</v>
-      </c>
-      <c r="E21" s="87" t="n">
-        <v>6500</v>
-      </c>
-      <c r="F21" s="87">
-        <f>AVERAGE(D21:E21)</f>
-        <v/>
-      </c>
-    </row>
-    <row r="22">
-      <c r="A22" s="49" t="inlineStr">
-        <is>
-          <t>Setterwalls</t>
-        </is>
-      </c>
-      <c r="B22" s="49" t="inlineStr">
-        <is>
-          <t>Oct-2026 (undated on site)</t>
-        </is>
-      </c>
-      <c r="C22" s="49" t="inlineStr">
-        <is>
-          <t>skatterätt.se firm pages (tax practice; no level split, no source)</t>
-        </is>
-      </c>
-      <c r="D22" s="87" t="n">
-        <v>3500</v>
-      </c>
-      <c r="E22" s="87" t="n">
-        <v>6000</v>
-      </c>
-      <c r="F22" s="87">
-        <f>AVERAGE(D22:E22)</f>
-        <v/>
-      </c>
-    </row>
-    <row r="23">
-      <c r="A23" s="49" t="inlineStr">
-        <is>
-          <t>Bird &amp; Bird</t>
-        </is>
-      </c>
-      <c r="B23" s="49" t="inlineStr">
-        <is>
-          <t>Oct-2026 (undated on site)</t>
-        </is>
-      </c>
-      <c r="C23" s="49" t="inlineStr">
-        <is>
-          <t>skatterätt.se firm pages (tax practice; no level split, no source)</t>
-        </is>
-      </c>
-      <c r="D23" s="87" t="n">
-        <v>3500</v>
-      </c>
-      <c r="E23" s="87" t="n">
-        <v>6000</v>
-      </c>
-      <c r="F23" s="87">
-        <f>AVERAGE(D23:E23)</f>
-        <v/>
-      </c>
-    </row>
-    <row r="24">
-      <c r="A24" s="49" t="inlineStr">
-        <is>
-          <t>Delphi</t>
-        </is>
-      </c>
-      <c r="B24" s="49" t="inlineStr">
-        <is>
-          <t>Oct-2026 (undated on site)</t>
-        </is>
-      </c>
-      <c r="C24" s="49" t="inlineStr">
-        <is>
-          <t>skatterätt.se firm pages (tax practice; no level split, no source)</t>
-        </is>
-      </c>
-      <c r="D24" s="87" t="n">
-        <v>3200</v>
-      </c>
-      <c r="E24" s="87" t="n">
-        <v>5500</v>
-      </c>
-      <c r="F24" s="87">
-        <f>AVERAGE(D24:E24)</f>
-        <v/>
-      </c>
-    </row>
-    <row r="25">
-      <c r="A25" s="49" t="inlineStr">
-        <is>
-          <t>Lindahl</t>
-        </is>
-      </c>
-      <c r="B25" s="49" t="inlineStr">
-        <is>
-          <t>Oct-2026 (undated on site)</t>
-        </is>
-      </c>
-      <c r="C25" s="49" t="inlineStr">
-        <is>
-          <t>skatterätt.se firm pages (tax practice; no level split, no source)</t>
-        </is>
-      </c>
-      <c r="D25" s="87" t="n">
-        <v>3000</v>
-      </c>
-      <c r="E25" s="87" t="n">
-        <v>5500</v>
-      </c>
-      <c r="F25" s="87">
-        <f>AVERAGE(D25:E25)</f>
-        <v/>
-      </c>
-    </row>
-    <row r="26">
-      <c r="A26" s="45" t="inlineStr">
-        <is>
-          <t>Example: https://www.xn--skattertt-12a.se/byra/vinge-skatt/ (Vinge: "Timarvode 4 000 till 7 000 kr"). Ranges may be estimates; use only for relative positioning.</t>
-        </is>
-      </c>
-    </row>
-    <row r="28">
-      <c r="A28" s="47" t="inlineStr">
-        <is>
-          <t>D3. Dated Nordic rate data points, 2023 onwards (realised rates and market commentary)</t>
-        </is>
-      </c>
-    </row>
-    <row r="29">
-      <c r="A29" s="52" t="inlineStr">
-        <is>
-          <t>Firm</t>
-        </is>
-      </c>
-      <c r="B29" s="52" t="inlineStr">
-        <is>
-          <t>Rate date</t>
-        </is>
-      </c>
-      <c r="C29" s="52" t="inlineStr">
-        <is>
-          <t>Level (as stated)</t>
-        </is>
-      </c>
-      <c r="D29" s="52" t="inlineStr">
-        <is>
-          <t>Mapped level</t>
-        </is>
-      </c>
-      <c r="E29" s="52" t="inlineStr">
-        <is>
-          <t>Rate low</t>
-        </is>
-      </c>
-      <c r="F29" s="52" t="inlineStr">
-        <is>
-          <t>Rate high</t>
-        </is>
-      </c>
-      <c r="G29" s="52" t="inlineStr">
-        <is>
-          <t>Context</t>
-        </is>
-      </c>
-      <c r="H29" s="52" t="inlineStr">
-        <is>
-          <t>Source type</t>
-        </is>
-      </c>
-      <c r="I29" s="52" t="inlineStr">
-        <is>
-          <t>Relevance</t>
-        </is>
-      </c>
-      <c r="J29" s="52" t="inlineStr">
-        <is>
-          <t>Source</t>
-        </is>
-      </c>
-    </row>
-    <row r="30">
-      <c r="A30" s="49" t="inlineStr">
-        <is>
-          <t>Mannheimer Swartling</t>
-        </is>
-      </c>
-      <c r="B30" s="49" t="inlineStr">
-        <is>
-          <t>Nov-2024 to Mar-2025</t>
-        </is>
-      </c>
-      <c r="C30" s="49" t="inlineStr">
-        <is>
-          <t>Average across team (~6,000 h, SEK 32m)</t>
-        </is>
-      </c>
-      <c r="D30" s="49" t="inlineStr">
-        <is>
-          <t>Blended (realised)</t>
-        </is>
-      </c>
-      <c r="E30" s="87" t="n">
-        <v>4000</v>
-      </c>
-      <c r="F30" s="87" t="n">
-        <v>4000</v>
-      </c>
-      <c r="G30" s="49" t="inlineStr">
-        <is>
-          <t>Northvolt restructuring (Swedish counsel in US Chapter 11); lowest average of all advisers</t>
-        </is>
-      </c>
-      <c r="H30" s="49" t="inlineStr">
-        <is>
-          <t>Court-approved fee filing (press)</t>
-        </is>
-      </c>
-      <c r="I30" s="49" t="inlineStr">
-        <is>
-          <t>Only published realised blended rate for a top Nordic firm: ~4,000 vs list partner 6,000-10,000</t>
-        </is>
-      </c>
-      <c r="J30" s="49" t="inlineStr">
-        <is>
-          <t>https://www.affarsvarlden.se/artikel/sa-dyrt-blev-northvolts-raddningsforsok-i-usa-debiteras-47-000-timmar</t>
-        </is>
-      </c>
-    </row>
-    <row r="31">
-      <c r="A31" s="49" t="inlineStr">
-        <is>
-          <t>Top-tier firms (Vinge, MSA, Roschier)</t>
-        </is>
-      </c>
-      <c r="B31" s="49" t="inlineStr">
-        <is>
-          <t>2026</t>
-        </is>
-      </c>
-      <c r="C31" s="49" t="inlineStr">
-        <is>
-          <t>Partner</t>
-        </is>
-      </c>
-      <c r="D31" s="49" t="inlineStr">
-        <is>
-          <t>Partner</t>
-        </is>
-      </c>
-      <c r="E31" s="87" t="n">
-        <v>7000</v>
-      </c>
-      <c r="F31" s="87" t="n">
-        <v>9000</v>
-      </c>
-      <c r="G31" s="49" t="inlineStr">
-        <is>
-          <t>Olle Flygt (ex-Vinge/MSA partner): partner bills 7-9k with 3-5 associates beneath</t>
-        </is>
-      </c>
-      <c r="H31" s="49" t="inlineStr">
-        <is>
-          <t>Market commentary</t>
-        </is>
-      </c>
-      <c r="I31" s="49" t="inlineStr">
-        <is>
-          <t>Current top-tier partner rate level</t>
-        </is>
-      </c>
-      <c r="J31" s="49" t="inlineStr">
-        <is>
-          <t>https://www.realtid.se/perfectweekend/affarsjuridikens-karna-det-har-blivit-for-mycket-fokus-pa-pengar/</t>
-        </is>
-      </c>
-    </row>
-    <row r="32">
-      <c r="A32" s="49" t="inlineStr">
-        <is>
-          <t>Top-tier firms (Vinge, MSA, Roschier)</t>
-        </is>
-      </c>
-      <c r="B32" s="49" t="inlineStr">
-        <is>
-          <t>2026</t>
-        </is>
-      </c>
-      <c r="C32" s="49" t="inlineStr">
-        <is>
-          <t>Biträdande jurist (associate)</t>
-        </is>
-      </c>
-      <c r="D32" s="49" t="inlineStr">
-        <is>
-          <t>Associate</t>
-        </is>
-      </c>
-      <c r="E32" s="87" t="n">
-        <v>3000</v>
-      </c>
-      <c r="F32" s="87" t="n">
-        <v>3000</v>
-      </c>
-      <c r="G32" s="49" t="inlineStr">
-        <is>
-          <t>As above: associates bill ~3,000 and cost at most a third of that</t>
-        </is>
-      </c>
-      <c r="H32" s="49" t="inlineStr">
-        <is>
-          <t>Market commentary</t>
-        </is>
-      </c>
-      <c r="I32" s="49" t="inlineStr">
-        <is>
-          <t>Associate rate and margin (leverage)</t>
-        </is>
-      </c>
-      <c r="J32" s="49" t="inlineStr">
-        <is>
-          <t>https://www.realtid.se/perfectweekend/affarsjuridikens-karna-det-har-blivit-for-mycket-fokus-pa-pengar/</t>
-        </is>
-      </c>
-    </row>
-    <row r="33">
-      <c r="A33" s="49" t="inlineStr">
-        <is>
-          <t>Mannheimer Swartling</t>
-        </is>
-      </c>
-      <c r="B33" s="49" t="inlineStr">
-        <is>
-          <t>Final years before 2025 (not specified)</t>
-        </is>
-      </c>
-      <c r="C33" s="49" t="inlineStr">
-        <is>
-          <t>Partner (Olle Flygt)</t>
-        </is>
-      </c>
-      <c r="D33" s="49" t="inlineStr">
-        <is>
-          <t>Partner</t>
-        </is>
-      </c>
-      <c r="E33" s="87" t="n">
-        <v>7000</v>
-      </c>
-      <c r="F33" s="87" t="n">
-        <v>8000</v>
-      </c>
-      <c r="G33" s="49" t="inlineStr">
-        <is>
-          <t>Own billing rate</t>
-        </is>
-      </c>
-      <c r="H33" s="49" t="inlineStr">
-        <is>
-          <t>Market commentary</t>
-        </is>
-      </c>
-      <c r="I33" s="49" t="inlineStr">
-        <is>
-          <t>Individual partner rate at MSA</t>
-        </is>
-      </c>
-      <c r="J33" s="49" t="inlineStr">
-        <is>
-          <t>https://www.realtid.se/juridik/affarsjuridiken-vaxer-men-sprickorna-syns/</t>
-        </is>
-      </c>
-    </row>
-    <row r="34">
-      <c r="A34" s="49" t="inlineStr">
-        <is>
-          <t>Law firm (unnamed)</t>
-        </is>
-      </c>
-      <c r="B34" s="49" t="inlineStr">
-        <is>
-          <t>Apr-2026</t>
-        </is>
-      </c>
-      <c r="C34" s="49" t="inlineStr">
-        <is>
-          <t>Hourly rate held reasonable</t>
-        </is>
-      </c>
-      <c r="D34" s="49" t="inlineStr">
-        <is>
-          <t>Blended</t>
-        </is>
-      </c>
-      <c r="E34" s="87" t="n">
-        <v>4000</v>
-      </c>
-      <c r="F34" s="87" t="n">
-        <v>4000</v>
-      </c>
-      <c r="G34" s="49" t="inlineStr">
-        <is>
-          <t>Luleå tingsrätt cost ruling</t>
-        </is>
-      </c>
-      <c r="H34" s="49" t="inlineStr">
-        <is>
-          <t>Court ruling (press)</t>
-        </is>
-      </c>
-      <c r="I34" s="49" t="inlineStr">
-        <is>
-          <t>Courts accept ~4,000/h as reasonable for business-law counsel</t>
-        </is>
-      </c>
-      <c r="J34" s="49" t="inlineStr">
-        <is>
-          <t>https://www.realtid.se/juridik/ratten-om-timarvoden-4-000-kronor-i-timmen-ar-ok/</t>
-        </is>
-      </c>
-    </row>
-    <row r="35">
-      <c r="A35" s="45" t="inlineStr">
-        <is>
-          <t>Removed: pre-2023 invoices and court claims (2007-2017), US firms, public-sector and legal-aid data (not relevant to a Nordic business-law investment).</t>
-        </is>
-      </c>
-    </row>
-    <row r="37">
-      <c r="A37" s="47" t="inlineStr">
-        <is>
-          <t>D4. Benchmarks (Nordic business law)</t>
-        </is>
-      </c>
-    </row>
-    <row r="38">
-      <c r="A38" s="52" t="inlineStr">
-        <is>
-          <t>Benchmark</t>
-        </is>
-      </c>
-      <c r="B38" s="52" t="inlineStr">
-        <is>
-          <t>Period</t>
-        </is>
-      </c>
-      <c r="C38" s="52" t="inlineStr">
-        <is>
-          <t>Rate</t>
-        </is>
-      </c>
-      <c r="D38" s="52" t="inlineStr">
-        <is>
-          <t>Currency</t>
-        </is>
-      </c>
-      <c r="E38" s="52" t="inlineStr">
-        <is>
-          <t>Notes</t>
-        </is>
-      </c>
-      <c r="F38" s="52" t="inlineStr">
-        <is>
-          <t>Source</t>
-        </is>
-      </c>
-    </row>
-    <row r="39">
-      <c r="A39" s="49" t="inlineStr">
-        <is>
-          <t>Affärsvärlden fee income per lawyer (panel)</t>
-        </is>
-      </c>
-      <c r="B39" s="49" t="inlineStr">
-        <is>
-          <t>2024</t>
-        </is>
-      </c>
-      <c r="C39" s="87" t="n">
-        <v>4130000</v>
-      </c>
-      <c r="D39" s="49" t="inlineStr">
-        <is>
-          <t>SEK p.a.</t>
-        </is>
-      </c>
-      <c r="E39" s="49" t="inlineStr">
-        <is>
-          <t>Implies ~SEK 2,580/h at 1,600 billable hours or ~2,950/h at 1,400 (illustrative)</t>
-        </is>
-      </c>
-      <c r="F39" s="49" t="inlineStr">
-        <is>
-          <t>https://www.realtid.se/affarer/154-miljarder-sa-klarade-affarsjuristerna-tullchocken/</t>
-        </is>
-      </c>
-    </row>
-    <row r="40">
-      <c r="A40" s="49" t="inlineStr">
-        <is>
-          <t>Affärsvärlden fee income per lawyer (panel)</t>
-        </is>
-      </c>
-      <c r="B40" s="49" t="inlineStr">
-        <is>
-          <t>2023</t>
-        </is>
-      </c>
-      <c r="C40" s="87" t="n">
-        <v>4220000</v>
-      </c>
-      <c r="D40" s="49" t="inlineStr">
-        <is>
-          <t>SEK p.a.</t>
-        </is>
-      </c>
-      <c r="E40" s="49" t="inlineStr"/>
-      <c r="F40" s="49" t="inlineStr">
-        <is>
-          <t>https://www.affarsvarlden.se/artikel/affarsjuristerna-om-trenden-pe-bolagen-kommer-vara-motorn</t>
-        </is>
-      </c>
-    </row>
-    <row r="41">
-      <c r="A41" s="49" t="inlineStr">
-        <is>
-          <t>Norway: commercial litigation rates</t>
-        </is>
-      </c>
-      <c r="B41" s="49" t="inlineStr">
-        <is>
-          <t>2026</t>
-        </is>
-      </c>
-      <c r="C41" s="87" t="n">
-        <v>3000</v>
-      </c>
-      <c r="D41" s="49" t="inlineStr">
-        <is>
-          <t>NOK/h (earlier level)</t>
-        </is>
-      </c>
-      <c r="E41" s="49" t="inlineStr">
-        <is>
-          <t>Norwegian Government Attorney: rates of ~NOK 3,000/h have "doubled in a short time"</t>
-        </is>
-      </c>
-      <c r="F41" s="49" t="inlineStr">
-        <is>
-          <t>https://www.realtid.se/juridik/regeringsadvokaten-slar-larm-advokatkostnaderna-skenar/</t>
-        </is>
-      </c>
-    </row>
-    <row r="43">
-      <c r="A43" s="45" t="inlineStr">
-        <is>
-          <t>Gaps: no published rate cards found for Vinge, White &amp; Case, Setterwalls, Lindahl, Gernandt &amp; Danielsson, CMS Wistrand, Cirio, Baker McKenzie, Snellman, Foyen, Glimstedt, Eversheds, Fylgia, Hammarskiöld, Magnusson, Kahn Pedersen, Wigge, Kastell, Westerberg or TM &amp; Partners.</t>
-        </is>
-      </c>
-    </row>
-    <row r="44">
-      <c r="A44" s="45" t="inlineStr">
-        <is>
-          <t>Routes to fill: client invoices (e.g. via Axo, requested); expert calls with Nordic GCs; confirm whether MAQS sell-side rates are list or realised.</t>
-        </is>
-      </c>
-    </row>
-  </sheetData>
-  <mergeCells count="14">
-    <mergeCell ref="A5:A6"/>
-    <mergeCell ref="O5:O6"/>
-    <mergeCell ref="N5:N6"/>
-    <mergeCell ref="P5:P6"/>
-    <mergeCell ref="Q5:Q6"/>
-    <mergeCell ref="J5:K5"/>
-    <mergeCell ref="L5:L6"/>
-    <mergeCell ref="F5:G5"/>
-    <mergeCell ref="D5:E5"/>
-    <mergeCell ref="A2:Q2"/>
-    <mergeCell ref="H5:I5"/>
-    <mergeCell ref="C5:C6"/>
-    <mergeCell ref="B5:B6"/>
-    <mergeCell ref="M5:M6"/>
-  </mergeCells>
-  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
-</worksheet>
 </file>
</xml_diff>

<commit_message>
Add utilisation benchmarks (C2 block and briefing section 5b); fix sheet order
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01Tu61bPEQej1E6sErbEFanY
</commit_message>
<xml_diff>
--- a/research/swedish_legal_market.xlsx
+++ b/research/swedish_legal_market.xlsx
@@ -36,7 +36,7 @@
     <numFmt numFmtId="166" formatCode="#,##0.0"/>
     <numFmt numFmtId="167" formatCode="0.0000"/>
   </numFmts>
-  <fonts count="11">
+  <fonts count="12">
     <font>
       <name val="Calibri"/>
       <family val="2"/>
@@ -81,6 +81,10 @@
       <b val="1"/>
       <color rgb="001F3864"/>
       <sz val="11"/>
+    </font>
+    <font>
+      <b val="1"/>
+      <sz val="12"/>
     </font>
   </fonts>
   <fills count="12">
@@ -141,7 +145,7 @@
       </patternFill>
     </fill>
   </fills>
-  <borders count="19">
+  <borders count="20">
     <border>
       <left/>
       <right/>
@@ -383,11 +387,22 @@
       </bottom>
       <diagonal/>
     </border>
+    <border>
+      <left/>
+      <right/>
+      <top style="thin">
+        <color rgb="00BFBFBF"/>
+      </top>
+      <bottom style="thin">
+        <color rgb="00BFBFBF"/>
+      </bottom>
+      <diagonal/>
+    </border>
   </borders>
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="128">
+  <cellXfs count="130">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
@@ -716,6 +731,8 @@
     <xf numFmtId="1" fontId="0" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="top" wrapText="1"/>
     </xf>
+    <xf numFmtId="0" fontId="11" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="19" pivotButton="0" quotePrefix="0" xfId="0"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0" hidden="0"/>
@@ -48681,7 +48698,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:R45"/>
+  <dimension ref="A1:R63"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="5" customWidth="1" style="112" min="1" max="1"/>
@@ -50853,9 +50870,473 @@
         </is>
       </c>
     </row>
+    <row r="47">
+      <c r="A47" s="128" t="inlineStr">
+        <is>
+          <t>C2. Utilisation benchmarks: billable-hour targets and Nordic norms</t>
+        </is>
+      </c>
+    </row>
+    <row r="48">
+      <c r="A48" s="99" t="inlineStr"/>
+      <c r="B48" s="99" t="inlineStr">
+        <is>
+          <t>Firm / basis</t>
+        </is>
+      </c>
+      <c r="C48" s="99" t="inlineStr">
+        <is>
+          <t>Metric</t>
+        </is>
+      </c>
+      <c r="D48" s="99" t="inlineStr"/>
+      <c r="E48" s="99" t="inlineStr"/>
+      <c r="F48" s="99" t="inlineStr">
+        <is>
+          <t>Value</t>
+        </is>
+      </c>
+      <c r="G48" s="99" t="inlineStr">
+        <is>
+          <t>Period</t>
+        </is>
+      </c>
+      <c r="H48" s="99" t="inlineStr">
+        <is>
+          <t>Reliability / source</t>
+        </is>
+      </c>
+    </row>
+    <row r="49">
+      <c r="B49" s="49" t="inlineStr">
+        <is>
+          <t>Vinge</t>
+        </is>
+      </c>
+      <c r="C49" s="49" t="inlineStr">
+        <is>
+          <t>Associate billable-hour target</t>
+        </is>
+      </c>
+      <c r="D49" s="129" t="n"/>
+      <c r="E49" s="84" t="n"/>
+      <c r="F49" s="49" t="inlineStr">
+        <is>
+          <t>1,500 h (incl. 100 h qualifying internal)</t>
+        </is>
+      </c>
+      <c r="G49" s="49" t="inlineStr">
+        <is>
+          <t>c.2012-14</t>
+        </is>
+      </c>
+      <c r="H49" s="49" t="inlineStr">
+        <is>
+          <t>Indicative: anonymous crowd-sourced table (juristlon.wordpress.com, 2014)</t>
+        </is>
+      </c>
+    </row>
+    <row r="50">
+      <c r="B50" s="49" t="inlineStr">
+        <is>
+          <t>Mannheimer Swartling</t>
+        </is>
+      </c>
+      <c r="C50" s="49" t="inlineStr">
+        <is>
+          <t>Associate billable-hour target</t>
+        </is>
+      </c>
+      <c r="D50" s="129" t="n"/>
+      <c r="E50" s="84" t="n"/>
+      <c r="F50" s="49" t="inlineStr">
+        <is>
+          <t>1,500 h (none in year 1)</t>
+        </is>
+      </c>
+      <c r="G50" s="49" t="inlineStr">
+        <is>
+          <t>c.2012-14</t>
+        </is>
+      </c>
+      <c r="H50" s="49" t="inlineStr">
+        <is>
+          <t>Indicative: as above</t>
+        </is>
+      </c>
+    </row>
+    <row r="51">
+      <c r="B51" s="49" t="inlineStr">
+        <is>
+          <t>Cederquist</t>
+        </is>
+      </c>
+      <c r="C51" s="49" t="inlineStr">
+        <is>
+          <t>Bonus ladder</t>
+        </is>
+      </c>
+      <c r="D51" s="129" t="n"/>
+      <c r="E51" s="84" t="n"/>
+      <c r="F51" s="49" t="inlineStr">
+        <is>
+          <t>0.75 month at 1,500 h up to 4.25 months at 1,800 h</t>
+        </is>
+      </c>
+      <c r="G51" s="49" t="inlineStr">
+        <is>
+          <t>c.2012-14</t>
+        </is>
+      </c>
+      <c r="H51" s="49" t="inlineStr">
+        <is>
+          <t>Indicative: as above</t>
+        </is>
+      </c>
+    </row>
+    <row r="52">
+      <c r="B52" s="49" t="inlineStr">
+        <is>
+          <t>White &amp; Case (Stockholm)</t>
+        </is>
+      </c>
+      <c r="C52" s="49" t="inlineStr">
+        <is>
+          <t>Associate billable-hour target</t>
+        </is>
+      </c>
+      <c r="D52" s="129" t="n"/>
+      <c r="E52" s="84" t="n"/>
+      <c r="F52" s="49" t="inlineStr">
+        <is>
+          <t>1,700 h</t>
+        </is>
+      </c>
+      <c r="G52" s="49" t="inlineStr">
+        <is>
+          <t>c.2012-14</t>
+        </is>
+      </c>
+      <c r="H52" s="49" t="inlineStr">
+        <is>
+          <t>Indicative: as above</t>
+        </is>
+      </c>
+    </row>
+    <row r="53">
+      <c r="B53" s="49" t="inlineStr">
+        <is>
+          <t>Lindahl</t>
+        </is>
+      </c>
+      <c r="C53" s="49" t="inlineStr">
+        <is>
+          <t>Associate billable-hour target</t>
+        </is>
+      </c>
+      <c r="D53" s="129" t="n"/>
+      <c r="E53" s="84" t="n"/>
+      <c r="F53" s="49" t="inlineStr">
+        <is>
+          <t>1,350 h (up to 200 h internal); bonus from 1,450 h</t>
+        </is>
+      </c>
+      <c r="G53" s="49" t="inlineStr">
+        <is>
+          <t>c.2012-14</t>
+        </is>
+      </c>
+      <c r="H53" s="49" t="inlineStr">
+        <is>
+          <t>Indicative: as above</t>
+        </is>
+      </c>
+    </row>
+    <row r="54">
+      <c r="B54" s="49" t="inlineStr">
+        <is>
+          <t>Fylgia</t>
+        </is>
+      </c>
+      <c r="C54" s="49" t="inlineStr">
+        <is>
+          <t>Target / bonus</t>
+        </is>
+      </c>
+      <c r="D54" s="129" t="n"/>
+      <c r="E54" s="84" t="n"/>
+      <c r="F54" s="49" t="inlineStr">
+        <is>
+          <t>1,400 h; bonus at 1,400 / 1,500 h</t>
+        </is>
+      </c>
+      <c r="G54" s="49" t="inlineStr">
+        <is>
+          <t>c.2012-14</t>
+        </is>
+      </c>
+      <c r="H54" s="49" t="inlineStr">
+        <is>
+          <t>Indicative: as above</t>
+        </is>
+      </c>
+    </row>
+    <row r="55">
+      <c r="B55" s="49" t="inlineStr">
+        <is>
+          <t>Delphi</t>
+        </is>
+      </c>
+      <c r="C55" s="49" t="inlineStr">
+        <is>
+          <t>Bonus threshold</t>
+        </is>
+      </c>
+      <c r="D55" s="129" t="n"/>
+      <c r="E55" s="84" t="n"/>
+      <c r="F55" s="49" t="inlineStr">
+        <is>
+          <t>1,500 h</t>
+        </is>
+      </c>
+      <c r="G55" s="49" t="inlineStr">
+        <is>
+          <t>c.2012-14</t>
+        </is>
+      </c>
+      <c r="H55" s="49" t="inlineStr">
+        <is>
+          <t>Indicative: as above</t>
+        </is>
+      </c>
+    </row>
+    <row r="56">
+      <c r="B56" s="49" t="inlineStr">
+        <is>
+          <t>Baker McKenzie (Stockholm)</t>
+        </is>
+      </c>
+      <c r="C56" s="49" t="inlineStr">
+        <is>
+          <t>Bonus threshold</t>
+        </is>
+      </c>
+      <c r="D56" s="129" t="n"/>
+      <c r="E56" s="84" t="n"/>
+      <c r="F56" s="49" t="inlineStr">
+        <is>
+          <t>from 1,400 billed h</t>
+        </is>
+      </c>
+      <c r="G56" s="49" t="inlineStr">
+        <is>
+          <t>c.2012-14</t>
+        </is>
+      </c>
+      <c r="H56" s="49" t="inlineStr">
+        <is>
+          <t>Indicative: as above</t>
+        </is>
+      </c>
+    </row>
+    <row r="57">
+      <c r="B57" s="49" t="inlineStr">
+        <is>
+          <t>Bird &amp; Bird (Stockholm)</t>
+        </is>
+      </c>
+      <c r="C57" s="49" t="inlineStr">
+        <is>
+          <t>Ramp-up target</t>
+        </is>
+      </c>
+      <c r="D57" s="129" t="n"/>
+      <c r="E57" s="84" t="n"/>
+      <c r="F57" s="49" t="inlineStr">
+        <is>
+          <t>1,000 / 1,200 / 1,450 h (years 1 / 2 / 3+)</t>
+        </is>
+      </c>
+      <c r="G57" s="49" t="inlineStr">
+        <is>
+          <t>2007</t>
+        </is>
+      </c>
+      <c r="H57" s="49" t="inlineStr">
+        <is>
+          <t>Indicative: as above</t>
+        </is>
+      </c>
+    </row>
+    <row r="58">
+      <c r="B58" s="49" t="inlineStr">
+        <is>
+          <t>Swedish business-law firms</t>
+        </is>
+      </c>
+      <c r="C58" s="49" t="inlineStr">
+        <is>
+          <t>Billable-hour requirement</t>
+        </is>
+      </c>
+      <c r="D58" s="129" t="n"/>
+      <c r="E58" s="84" t="n"/>
+      <c r="F58" s="49" t="inlineStr">
+        <is>
+          <t>1,400-1,600 h p.a.</t>
+        </is>
+      </c>
+      <c r="G58" s="49" t="inlineStr">
+        <is>
+          <t>2018</t>
+        </is>
+      </c>
+      <c r="H58" s="49" t="inlineStr">
+        <is>
+          <t>Advokaten no. 7 2018 (snippet)</t>
+        </is>
+      </c>
+    </row>
+    <row r="59">
+      <c r="B59" s="49" t="inlineStr">
+        <is>
+          <t>Swedish law firms</t>
+        </is>
+      </c>
+      <c r="C59" s="49" t="inlineStr">
+        <is>
+          <t>Share of worked time billed</t>
+        </is>
+      </c>
+      <c r="D59" s="129" t="n"/>
+      <c r="E59" s="84" t="n"/>
+      <c r="F59" s="49" t="inlineStr">
+        <is>
+          <t>40-90%, median just over 70%</t>
+        </is>
+      </c>
+      <c r="G59" s="49" t="inlineStr">
+        <is>
+          <t>2012</t>
+        </is>
+      </c>
+      <c r="H59" s="49" t="inlineStr">
+        <is>
+          <t>Advokaten 2012 (snippet)</t>
+        </is>
+      </c>
+    </row>
+    <row r="60">
+      <c r="B60" s="49" t="inlineStr">
+        <is>
+          <t>Norwegian law firms</t>
+        </is>
+      </c>
+      <c r="C60" s="49" t="inlineStr">
+        <is>
+          <t>Billing rate (faktureringsgrad)</t>
+        </is>
+      </c>
+      <c r="D60" s="129" t="n"/>
+      <c r="E60" s="84" t="n"/>
+      <c r="F60" s="49" t="inlineStr">
+        <is>
+          <t>just over 72% (~1,220 h on 1,695 h)</t>
+        </is>
+      </c>
+      <c r="G60" s="49" t="inlineStr">
+        <is>
+          <t>2016</t>
+        </is>
+      </c>
+      <c r="H60" s="49" t="inlineStr">
+        <is>
+          <t>Advokatforeningen industry survey (memo Sep-2017)</t>
+        </is>
+      </c>
+    </row>
+    <row r="61">
+      <c r="B61" s="49" t="inlineStr">
+        <is>
+          <t>Norwegian associates</t>
+        </is>
+      </c>
+      <c r="C61" s="49" t="inlineStr">
+        <is>
+          <t>Actual vs contracted hours</t>
+        </is>
+      </c>
+      <c r="D61" s="129" t="n"/>
+      <c r="E61" s="84" t="n"/>
+      <c r="F61" s="49" t="inlineStr">
+        <is>
+          <t>46 h/week actual (48 h at 50+ lawyer firms) vs 39 h contracted; 27% under-record hours</t>
+        </is>
+      </c>
+      <c r="G61" s="49" t="inlineStr">
+        <is>
+          <t>Nov-2025</t>
+        </is>
+      </c>
+      <c r="H61" s="49" t="inlineStr">
+        <is>
+          <t>Juristforbundet survey (n=279)</t>
+        </is>
+      </c>
+    </row>
+    <row r="62">
+      <c r="B62" s="49" t="inlineStr">
+        <is>
+          <t>Danish associates / lawyers</t>
+        </is>
+      </c>
+      <c r="C62" s="49" t="inlineStr">
+        <is>
+          <t>Fixed billable-hour requirement</t>
+        </is>
+      </c>
+      <c r="D62" s="129" t="n"/>
+      <c r="E62" s="84" t="n"/>
+      <c r="F62" s="49" t="inlineStr">
+        <is>
+          <t>54% / 55% have one; 47 / 46 h worked per week</t>
+        </is>
+      </c>
+      <c r="G62" s="49" t="inlineStr">
+        <is>
+          <t>2018</t>
+        </is>
+      </c>
+      <c r="H62" s="49" t="inlineStr">
+        <is>
+          <t>Djøf Advokat survey</t>
+        </is>
+      </c>
+    </row>
+    <row r="63">
+      <c r="A63" s="45" t="inlineStr">
+        <is>
+          <t>Reading: Nordic norm ~1,200-1,300 billable hours (70-75% of a ~1,650-1,700 h year); large business-law firms target ~1,400-1,600 h for associates. No current published targets found for named Nordic firms or for Finland. See the charging rates briefing for international benchmarks (PwC UK, Thomson Reuters).</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
-  <mergeCells count="1">
+  <mergeCells count="15">
+    <mergeCell ref="C54:E54"/>
+    <mergeCell ref="C58:E58"/>
+    <mergeCell ref="C60:E60"/>
+    <mergeCell ref="C50:E50"/>
+    <mergeCell ref="C57:E57"/>
+    <mergeCell ref="C52:E52"/>
+    <mergeCell ref="C55:E55"/>
     <mergeCell ref="A2:R2"/>
+    <mergeCell ref="C53:E53"/>
+    <mergeCell ref="C61:E61"/>
+    <mergeCell ref="C49:E49"/>
+    <mergeCell ref="C56:E56"/>
+    <mergeCell ref="C59:E59"/>
+    <mergeCell ref="C51:E51"/>
+    <mergeCell ref="C62:E62"/>
   </mergeCells>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Remove legal-aid and public-sector references; focus on business-law firms only
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01Tu61bPEQej1E6sErbEFanY
</commit_message>
<xml_diff>
--- a/research/swedish_legal_market.xlsx
+++ b/research/swedish_legal_market.xlsx
@@ -2518,7 +2518,7 @@
     <row r="35">
       <c r="A35" s="45" t="inlineStr">
         <is>
-          <t>Removed: pre-2023 invoices and court claims (2007-2017), US firms, public-sector and legal-aid data (not relevant to a Nordic business-law investment).</t>
+          <t>Scope: Nordic business-law firms only, 2023 onwards.</t>
         </is>
       </c>
     </row>
@@ -2674,9 +2674,9 @@
     <mergeCell ref="D5:E5"/>
     <mergeCell ref="A2:Q2"/>
     <mergeCell ref="H5:I5"/>
+    <mergeCell ref="C5:C6"/>
+    <mergeCell ref="B5:B6"/>
     <mergeCell ref="M5:M6"/>
-    <mergeCell ref="B5:B6"/>
-    <mergeCell ref="C5:C6"/>
   </mergeCells>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
@@ -4507,7 +4507,7 @@
     <row r="49">
       <c r="A49" s="45" t="inlineStr">
         <is>
-          <t>No Swedish press ranking of business lawyers by taxed income was found for 2020-2026 (recent "best-paid lawyer" lists cover public defenders' state fees, not business law). DI, Expressen and Aftonbladet could not be checked directly.</t>
+          <t>No Swedish press ranking of business lawyers by taxed income was found for 2020-2026. DI, Expressen and Aftonbladet could not be checked directly.</t>
         </is>
       </c>
     </row>
@@ -7583,7 +7583,7 @@
       </c>
       <c r="F35" s="49" t="inlineStr">
         <is>
-          <t>Partner DKK 2,057-5,400/h (2023, mid-market); Kammeradvokat DKK 2,710</t>
+          <t>Partner DKK 2,057-5,400/h (2023, mid-market firms)</t>
         </is>
       </c>
       <c r="G35" s="49" t="inlineStr">
@@ -7680,7 +7680,7 @@
       </c>
       <c r="B42" s="49" t="inlineStr">
         <is>
-          <t>HortenDahl merger (Jan-2026); DLA Piper takes 49 from Lundgrens (Mar-2025); Schjødt-Norrbom Vinding (Mar-2026); Kromann Reumert converts to P/S (Nov-2025); proposal to open Kammeradvokat mandate (~DKK 0.7bn) to competition</t>
+          <t>HortenDahl merger (Jan-2026); DLA Piper takes 49 from Lundgrens (Mar-2025); Schjødt-Norrbom Vinding (Mar-2026); Kromann Reumert converts to P/S (Nov-2025)</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
C. Benchmarking: add FY2025 revenue, like-for-like YoY growth and source/coverage columns
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01Tu61bPEQej1E6sErbEFanY
</commit_message>
<xml_diff>
--- a/research/swedish_legal_market.xlsx
+++ b/research/swedish_legal_market.xlsx
@@ -402,7 +402,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="130">
+  <cellXfs count="133">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
@@ -733,6 +733,15 @@
     </xf>
     <xf numFmtId="0" fontId="11" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="19" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="165" fontId="0" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="3" fontId="0" fillId="5" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="165" fontId="5" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="top" wrapText="1"/>
+    </xf>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0" hidden="0"/>
@@ -2674,9 +2683,9 @@
     <mergeCell ref="D5:E5"/>
     <mergeCell ref="A2:Q2"/>
     <mergeCell ref="H5:I5"/>
+    <mergeCell ref="M5:M6"/>
+    <mergeCell ref="B5:B6"/>
     <mergeCell ref="C5:C6"/>
-    <mergeCell ref="B5:B6"/>
-    <mergeCell ref="M5:M6"/>
   </mergeCells>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
@@ -48698,27 +48707,30 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:R63"/>
+  <dimension ref="A1:U63"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="5" customWidth="1" style="112" min="1" max="1"/>
     <col width="26" customWidth="1" style="112" min="2" max="2"/>
     <col width="11" customWidth="1" style="112" min="3" max="3"/>
     <col width="10" customWidth="1" style="112" min="4" max="4"/>
-    <col width="9" customWidth="1" style="112" min="5" max="5"/>
-    <col width="10" customWidth="1" style="112" min="6" max="6"/>
-    <col width="26" customWidth="1" style="112" min="7" max="7"/>
+    <col width="10" customWidth="1" style="112" min="5" max="5"/>
+    <col width="28" customWidth="1" style="112" min="6" max="6"/>
+    <col width="10" customWidth="1" style="112" min="7" max="7"/>
     <col width="9" customWidth="1" style="112" min="8" max="8"/>
     <col width="10" customWidth="1" style="112" min="9" max="9"/>
-    <col width="10" customWidth="1" style="112" min="10" max="10"/>
-    <col width="30" customWidth="1" style="112" min="11" max="11"/>
+    <col width="26" customWidth="1" style="112" min="10" max="10"/>
+    <col width="9" customWidth="1" style="112" min="11" max="11"/>
     <col width="10" customWidth="1" style="112" min="12" max="12"/>
     <col width="10" customWidth="1" style="112" min="13" max="13"/>
-    <col width="10" customWidth="1" style="112" min="14" max="14"/>
-    <col width="12" customWidth="1" style="112" min="15" max="15"/>
-    <col width="12" customWidth="1" style="112" min="16" max="16"/>
+    <col width="30" customWidth="1" style="112" min="14" max="14"/>
+    <col width="10" customWidth="1" style="112" min="15" max="15"/>
+    <col width="10" customWidth="1" style="112" min="16" max="16"/>
     <col width="10" customWidth="1" style="112" min="17" max="17"/>
-    <col width="40" customWidth="1" style="112" min="18" max="18"/>
+    <col width="12" customWidth="1" style="112" min="18" max="18"/>
+    <col width="12" customWidth="1" style="112" min="19" max="19"/>
+    <col width="10" customWidth="1" style="112" min="20" max="20"/>
+    <col width="40" customWidth="1" style="112" min="21" max="21"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -48731,7 +48743,7 @@
     <row r="2" ht="45" customHeight="1" s="112">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>Ranking: Affärsvärlden fee income FY2024 (revised table, 3 Oct 2025; split-year firms on FY24/25). Ratios use the latest available revenue (FY2025 where published, else FY2024; basis shown) against current headcount (mostly Oct-2026), so they are indicative. Leverage (requested) = partners / total employees; partners / lawyers shown alongside. Grey = not available.</t>
+          <t>Ranking: Affärsvärlden fee income FY2024; FY2025 revenue from filed company accounts / press where available (revised table, 3 Oct 2025; split-year firms on FY24/25). Ratios use the latest available revenue (FY2025 where published, else FY2024; basis shown) against current headcount (mostly Oct-2026), so they are indicative. Leverage (requested) = partners / total employees; partners / lawyers shown alongside. Grey = not available.</t>
         </is>
       </c>
     </row>
@@ -48753,75 +48765,90 @@
       </c>
       <c r="D4" s="52" t="inlineStr">
         <is>
+          <t>Revenue FY2025</t>
+        </is>
+      </c>
+      <c r="E4" s="52" t="inlineStr">
+        <is>
+          <t>YoY FY25 vs FY24 (like-for-like)</t>
+        </is>
+      </c>
+      <c r="F4" s="52" t="inlineStr">
+        <is>
+          <t>FY2025 source / coverage</t>
+        </is>
+      </c>
+      <c r="G4" s="52" t="inlineStr">
+        <is>
           <t>Afv FY2023</t>
         </is>
       </c>
-      <c r="E4" s="52" t="inlineStr">
+      <c r="H4" s="52" t="inlineStr">
         <is>
           <t>Growth FY24</t>
         </is>
       </c>
-      <c r="F4" s="52" t="inlineStr">
+      <c r="I4" s="52" t="inlineStr">
         <is>
           <t>Latest revenue</t>
         </is>
       </c>
-      <c r="G4" s="52" t="inlineStr">
+      <c r="J4" s="52" t="inlineStr">
         <is>
           <t>Latest revenue basis</t>
         </is>
       </c>
-      <c r="H4" s="52" t="inlineStr">
+      <c r="K4" s="52" t="inlineStr">
         <is>
           <t>Partners</t>
         </is>
       </c>
-      <c r="I4" s="52" t="inlineStr">
+      <c r="L4" s="52" t="inlineStr">
         <is>
           <t>Lawyers (incl. partners)</t>
         </is>
       </c>
-      <c r="J4" s="52" t="inlineStr">
+      <c r="M4" s="52" t="inlineStr">
         <is>
           <t>Total employees</t>
         </is>
       </c>
-      <c r="K4" s="52" t="inlineStr">
+      <c r="N4" s="52" t="inlineStr">
         <is>
           <t>Headcount source</t>
         </is>
       </c>
-      <c r="L4" s="52" t="inlineStr">
+      <c r="O4" s="52" t="inlineStr">
         <is>
           <t>Rev / partner</t>
         </is>
       </c>
-      <c r="M4" s="52" t="inlineStr">
+      <c r="P4" s="52" t="inlineStr">
         <is>
           <t>Rev / employee</t>
         </is>
       </c>
-      <c r="N4" s="52" t="inlineStr">
+      <c r="Q4" s="52" t="inlineStr">
         <is>
           <t>Rev / lawyer</t>
         </is>
       </c>
-      <c r="O4" s="52" t="inlineStr">
+      <c r="R4" s="52" t="inlineStr">
         <is>
           <t>Leverage: partners / employees</t>
         </is>
       </c>
-      <c r="P4" s="52" t="inlineStr">
+      <c r="S4" s="52" t="inlineStr">
         <is>
           <t>Leverage: partners / lawyers</t>
         </is>
       </c>
-      <c r="Q4" s="52" t="inlineStr">
+      <c r="T4" s="52" t="inlineStr">
         <is>
           <t>Employees per partner</t>
         </is>
       </c>
-      <c r="R4" s="52" t="inlineStr">
+      <c r="U4" s="52" t="inlineStr">
         <is>
           <t>Notes</t>
         </is>
@@ -48840,59 +48867,71 @@
         <v>2085</v>
       </c>
       <c r="D5" s="100" t="n">
+        <v>2036</v>
+      </c>
+      <c r="E5" s="130">
+        <f>D5/2083-1</f>
+        <v/>
+      </c>
+      <c r="F5" s="49" t="inlineStr">
+        <is>
+          <t>Group annual reports (DJ via Realtid): full firm</t>
+        </is>
+      </c>
+      <c r="G5" s="100" t="n">
         <v>1751</v>
       </c>
-      <c r="E5" s="101">
-        <f>C5/D5-1</f>
+      <c r="H5" s="101">
+        <f>C5/G5-1</f>
         <v/>
       </c>
-      <c r="F5" s="100" t="n">
+      <c r="I5" s="100" t="n">
         <v>2036</v>
       </c>
-      <c r="G5" s="49" t="inlineStr">
+      <c r="J5" s="49" t="inlineStr">
         <is>
           <t>FY2025 group (annual reports, DJ)</t>
         </is>
       </c>
-      <c r="H5" s="90" t="n">
+      <c r="K5" s="90" t="n">
         <v>71</v>
       </c>
-      <c r="I5" s="90" t="n">
+      <c r="L5" s="90" t="n">
         <v>389</v>
       </c>
-      <c r="J5" s="90" t="n">
+      <c r="M5" s="90" t="n">
         <v>529</v>
       </c>
-      <c r="K5" s="49" t="inlineStr">
+      <c r="N5" s="49" t="inlineStr">
         <is>
           <t>Firm website count Oct-26; employees: 3 ABs 2025 accounts</t>
         </is>
       </c>
-      <c r="L5" s="92">
-        <f>F5/H5</f>
+      <c r="O5" s="92">
+        <f>I5/K5</f>
         <v/>
       </c>
-      <c r="M5" s="93">
-        <f>F5/J5</f>
+      <c r="P5" s="93">
+        <f>I5/M5</f>
         <v/>
       </c>
-      <c r="N5" s="93">
-        <f>F5/I5</f>
+      <c r="Q5" s="93">
+        <f>I5/L5</f>
         <v/>
       </c>
-      <c r="O5" s="101">
-        <f>H5/J5</f>
+      <c r="R5" s="101">
+        <f>K5/M5</f>
         <v/>
       </c>
-      <c r="P5" s="101">
-        <f>H5/I5</f>
+      <c r="S5" s="101">
+        <f>K5/L5</f>
         <v/>
       </c>
-      <c r="Q5" s="92">
-        <f>J5/H5</f>
+      <c r="T5" s="92">
+        <f>M5/K5</f>
         <v/>
       </c>
-      <c r="R5" s="49" t="inlineStr">
+      <c r="U5" s="49" t="inlineStr">
         <is>
           <t>Lawyers incl. ~46 on leave</t>
         </is>
@@ -48911,59 +48950,71 @@
         <v>1911</v>
       </c>
       <c r="D6" s="100" t="n">
+        <v>2002</v>
+      </c>
+      <c r="E6" s="130">
+        <f>D6/1916-1</f>
+        <v/>
+      </c>
+      <c r="F6" s="49" t="inlineStr">
+        <is>
+          <t>Annual report (AB): full firm</t>
+        </is>
+      </c>
+      <c r="G6" s="100" t="n">
         <v>1807</v>
       </c>
-      <c r="E6" s="101">
-        <f>C6/D6-1</f>
+      <c r="H6" s="101">
+        <f>C6/G6-1</f>
         <v/>
       </c>
-      <c r="F6" s="100" t="n">
+      <c r="I6" s="100" t="n">
         <v>2002</v>
       </c>
-      <c r="G6" s="49" t="inlineStr">
+      <c r="J6" s="49" t="inlineStr">
         <is>
           <t>FY2025 (annual report)</t>
         </is>
       </c>
-      <c r="H6" s="90" t="n">
+      <c r="K6" s="90" t="n">
         <v>92</v>
       </c>
-      <c r="I6" s="90" t="n">
+      <c r="L6" s="90" t="n">
         <v>430</v>
       </c>
-      <c r="J6" s="90" t="n">
+      <c r="M6" s="90" t="n">
         <v>649</v>
       </c>
-      <c r="K6" s="49" t="inlineStr">
+      <c r="N6" s="49" t="inlineStr">
         <is>
           <t>DJ/Chambers 2026; employees 2025 accounts</t>
         </is>
       </c>
-      <c r="L6" s="92">
-        <f>F6/H6</f>
+      <c r="O6" s="92">
+        <f>I6/K6</f>
         <v/>
       </c>
-      <c r="M6" s="93">
-        <f>F6/J6</f>
+      <c r="P6" s="93">
+        <f>I6/M6</f>
         <v/>
       </c>
-      <c r="N6" s="93">
-        <f>F6/I6</f>
+      <c r="Q6" s="93">
+        <f>I6/L6</f>
         <v/>
       </c>
-      <c r="O6" s="101">
-        <f>H6/J6</f>
+      <c r="R6" s="101">
+        <f>K6/M6</f>
         <v/>
       </c>
-      <c r="P6" s="101">
-        <f>H6/I6</f>
+      <c r="S6" s="101">
+        <f>K6/L6</f>
         <v/>
       </c>
-      <c r="Q6" s="92">
-        <f>J6/H6</f>
+      <c r="T6" s="92">
+        <f>M6/K6</f>
         <v/>
       </c>
-      <c r="R6" s="49" t="inlineStr"/>
+      <c r="U6" s="49" t="inlineStr"/>
     </row>
     <row r="7">
       <c r="A7" s="90" t="n">
@@ -48978,59 +49029,71 @@
         <v>1254</v>
       </c>
       <c r="D7" s="100" t="n">
+        <v>1304</v>
+      </c>
+      <c r="E7" s="130">
+        <f>D7/1254-1</f>
+        <v/>
+      </c>
+      <c r="F7" s="49" t="inlineStr">
+        <is>
+          <t>AB accounts FY Jun25-May26 vs FY24/25: full firm</t>
+        </is>
+      </c>
+      <c r="G7" s="100" t="n">
         <v>1026</v>
       </c>
-      <c r="E7" s="101">
-        <f>C7/D7-1</f>
+      <c r="H7" s="101">
+        <f>C7/G7-1</f>
         <v/>
       </c>
-      <c r="F7" s="100" t="n">
+      <c r="I7" s="100" t="n">
         <v>1304</v>
       </c>
-      <c r="G7" s="49" t="inlineStr">
+      <c r="J7" s="49" t="inlineStr">
         <is>
           <t>FY Jun25-May26 net sales (AB)</t>
         </is>
       </c>
-      <c r="H7" s="90" t="n">
+      <c r="K7" s="90" t="n">
         <v>26</v>
       </c>
-      <c r="I7" s="90" t="n">
+      <c r="L7" s="90" t="n">
         <v>181</v>
       </c>
-      <c r="J7" s="90" t="n">
+      <c r="M7" s="90" t="n">
         <v>220</v>
       </c>
-      <c r="K7" s="49" t="inlineStr">
+      <c r="N7" s="49" t="inlineStr">
         <is>
           <t>Firm website count Oct-26 (Stockholm); employees AB accounts</t>
         </is>
       </c>
-      <c r="L7" s="92">
-        <f>F7/H7</f>
+      <c r="O7" s="92">
+        <f>I7/K7</f>
         <v/>
       </c>
-      <c r="M7" s="93">
-        <f>F7/J7</f>
+      <c r="P7" s="93">
+        <f>I7/M7</f>
         <v/>
       </c>
-      <c r="N7" s="93">
-        <f>F7/I7</f>
+      <c r="Q7" s="93">
+        <f>I7/L7</f>
         <v/>
       </c>
-      <c r="O7" s="101">
-        <f>H7/J7</f>
+      <c r="R7" s="101">
+        <f>K7/M7</f>
         <v/>
       </c>
-      <c r="P7" s="101">
-        <f>H7/I7</f>
+      <c r="S7" s="101">
+        <f>K7/L7</f>
         <v/>
       </c>
-      <c r="Q7" s="92">
-        <f>J7/H7</f>
+      <c r="T7" s="92">
+        <f>M7/K7</f>
         <v/>
       </c>
-      <c r="R7" s="49" t="inlineStr">
+      <c r="U7" s="49" t="inlineStr">
         <is>
           <t>Split year; Afv FY24 = FY Jun24-May25</t>
         </is>
@@ -49049,59 +49112,71 @@
         <v>918</v>
       </c>
       <c r="D8" s="100" t="n">
+        <v>1056</v>
+      </c>
+      <c r="E8" s="130">
+        <f>D8/996-1</f>
+        <v/>
+      </c>
+      <c r="F8" s="49" t="inlineStr">
+        <is>
+          <t>Parent AB accounts (pass-through, incl. Malmö); Afv "&gt;1bn"</t>
+        </is>
+      </c>
+      <c r="G8" s="100" t="n">
         <v>899</v>
       </c>
-      <c r="E8" s="101">
-        <f>C8/D8-1</f>
+      <c r="H8" s="101">
+        <f>C8/G8-1</f>
         <v/>
       </c>
-      <c r="F8" s="100" t="n">
+      <c r="I8" s="100" t="n">
         <v>1000</v>
       </c>
-      <c r="G8" s="49" t="inlineStr">
+      <c r="J8" s="49" t="inlineStr">
         <is>
           <t>FY2025 (Afv "&gt;1bn")</t>
         </is>
       </c>
-      <c r="H8" s="90" t="n">
+      <c r="K8" s="90" t="n">
         <v>38</v>
       </c>
-      <c r="I8" s="90" t="n">
+      <c r="L8" s="90" t="n">
         <v>177</v>
       </c>
-      <c r="J8" s="90" t="n">
+      <c r="M8" s="90" t="n">
         <v>306</v>
       </c>
-      <c r="K8" s="49" t="inlineStr">
+      <c r="N8" s="49" t="inlineStr">
         <is>
           <t>Firm website count Oct-26; employees 3 entities 2025</t>
         </is>
       </c>
-      <c r="L8" s="92">
-        <f>F8/H8</f>
+      <c r="O8" s="92">
+        <f>I8/K8</f>
         <v/>
       </c>
-      <c r="M8" s="93">
-        <f>F8/J8</f>
+      <c r="P8" s="93">
+        <f>I8/M8</f>
         <v/>
       </c>
-      <c r="N8" s="93">
-        <f>F8/I8</f>
+      <c r="Q8" s="93">
+        <f>I8/L8</f>
         <v/>
       </c>
-      <c r="O8" s="101">
-        <f>H8/J8</f>
+      <c r="R8" s="101">
+        <f>K8/M8</f>
         <v/>
       </c>
-      <c r="P8" s="101">
-        <f>H8/I8</f>
+      <c r="S8" s="101">
+        <f>K8/L8</f>
         <v/>
       </c>
-      <c r="Q8" s="92">
-        <f>J8/H8</f>
+      <c r="T8" s="92">
+        <f>M8/K8</f>
         <v/>
       </c>
-      <c r="R8" s="49" t="inlineStr">
+      <c r="U8" s="49" t="inlineStr">
         <is>
           <t>Revenue/employees incl. Malmö (left Sep-26); partners/lawyers exclude it</t>
         </is>
@@ -49120,59 +49195,71 @@
         <v>737</v>
       </c>
       <c r="D9" s="100" t="n">
+        <v>438</v>
+      </c>
+      <c r="E9" s="130">
+        <f>D9/406-1</f>
+        <v/>
+      </c>
+      <c r="F9" s="69" t="inlineStr">
+        <is>
+          <t>PARTIAL: Malmö, Stockholm, Göteborg ABs only</t>
+        </is>
+      </c>
+      <c r="G9" s="100" t="n">
         <v>707</v>
       </c>
-      <c r="E9" s="101">
-        <f>C9/D9-1</f>
+      <c r="H9" s="101">
+        <f>C9/G9-1</f>
         <v/>
       </c>
-      <c r="F9" s="100" t="n">
+      <c r="I9" s="100" t="n">
         <v>737</v>
       </c>
-      <c r="G9" s="49" t="inlineStr">
+      <c r="J9" s="49" t="inlineStr">
         <is>
           <t>FY2024 (Afv)</t>
         </is>
       </c>
-      <c r="H9" s="90" t="n">
+      <c r="K9" s="90" t="n">
         <v>68</v>
       </c>
-      <c r="I9" s="90" t="n">
+      <c r="L9" s="90" t="n">
         <v>220</v>
       </c>
-      <c r="J9" s="90" t="n">
+      <c r="M9" s="90" t="n">
         <v>300</v>
       </c>
-      <c r="K9" s="49" t="inlineStr">
+      <c r="N9" s="49" t="inlineStr">
         <is>
           <t>Legal 500 / Chambers (firm-supplied)</t>
         </is>
       </c>
-      <c r="L9" s="92">
-        <f>F9/H9</f>
+      <c r="O9" s="92">
+        <f>I9/K9</f>
         <v/>
       </c>
-      <c r="M9" s="93">
-        <f>F9/J9</f>
+      <c r="P9" s="93">
+        <f>I9/M9</f>
         <v/>
       </c>
-      <c r="N9" s="93">
-        <f>F9/I9</f>
+      <c r="Q9" s="93">
+        <f>I9/L9</f>
         <v/>
       </c>
-      <c r="O9" s="101">
-        <f>H9/J9</f>
+      <c r="R9" s="101">
+        <f>K9/M9</f>
         <v/>
       </c>
-      <c r="P9" s="101">
-        <f>H9/I9</f>
+      <c r="S9" s="101">
+        <f>K9/L9</f>
         <v/>
       </c>
-      <c r="Q9" s="92">
-        <f>J9/H9</f>
+      <c r="T9" s="92">
+        <f>M9/K9</f>
         <v/>
       </c>
-      <c r="R9" s="49" t="inlineStr"/>
+      <c r="U9" s="49" t="inlineStr"/>
     </row>
     <row r="10">
       <c r="A10" s="90" t="n">
@@ -49186,60 +49273,67 @@
       <c r="C10" s="100" t="n">
         <v>676</v>
       </c>
-      <c r="D10" s="100" t="n">
+      <c r="D10" s="131" t="n"/>
+      <c r="E10" s="98" t="n"/>
+      <c r="F10" s="49" t="inlineStr">
+        <is>
+          <t>Not filed (KB)</t>
+        </is>
+      </c>
+      <c r="G10" s="100" t="n">
         <v>601</v>
       </c>
-      <c r="E10" s="101">
-        <f>C10/D10-1</f>
+      <c r="H10" s="101">
+        <f>C10/G10-1</f>
         <v/>
       </c>
-      <c r="F10" s="100" t="n">
+      <c r="I10" s="100" t="n">
         <v>676</v>
       </c>
-      <c r="G10" s="49" t="inlineStr">
+      <c r="J10" s="49" t="inlineStr">
         <is>
           <t>FY24/25 (Afv)</t>
         </is>
       </c>
-      <c r="H10" s="90" t="n">
+      <c r="K10" s="90" t="n">
         <v>20</v>
       </c>
-      <c r="I10" s="90" t="n">
+      <c r="L10" s="90" t="n">
         <v>91</v>
       </c>
-      <c r="J10" s="90" t="n">
+      <c r="M10" s="90" t="n">
         <v>150</v>
       </c>
-      <c r="K10" s="49" t="inlineStr">
+      <c r="N10" s="49" t="inlineStr">
         <is>
           <t>Firm website count Oct-26; employees firm website</t>
         </is>
       </c>
-      <c r="L10" s="92">
-        <f>F10/H10</f>
+      <c r="O10" s="92">
+        <f>I10/K10</f>
         <v/>
       </c>
-      <c r="M10" s="93">
-        <f>F10/J10</f>
+      <c r="P10" s="93">
+        <f>I10/M10</f>
         <v/>
       </c>
-      <c r="N10" s="93">
-        <f>F10/I10</f>
+      <c r="Q10" s="93">
+        <f>I10/L10</f>
         <v/>
       </c>
-      <c r="O10" s="101">
-        <f>H10/J10</f>
+      <c r="R10" s="101">
+        <f>K10/M10</f>
         <v/>
       </c>
-      <c r="P10" s="101">
-        <f>H10/I10</f>
+      <c r="S10" s="101">
+        <f>K10/L10</f>
         <v/>
       </c>
-      <c r="Q10" s="92">
-        <f>J10/H10</f>
+      <c r="T10" s="92">
+        <f>M10/K10</f>
         <v/>
       </c>
-      <c r="R10" s="49" t="inlineStr">
+      <c r="U10" s="49" t="inlineStr">
         <is>
           <t>KB - no public accounts</t>
         </is>
@@ -49257,49 +49351,56 @@
       <c r="C11" s="100" t="n">
         <v>602</v>
       </c>
-      <c r="D11" s="100" t="n">
+      <c r="D11" s="131" t="n"/>
+      <c r="E11" s="98" t="n"/>
+      <c r="F11" s="49" t="inlineStr">
+        <is>
+          <t>Not filed (KB)</t>
+        </is>
+      </c>
+      <c r="G11" s="100" t="n">
         <v>660</v>
       </c>
-      <c r="E11" s="101">
-        <f>C11/D11-1</f>
+      <c r="H11" s="101">
+        <f>C11/G11-1</f>
         <v/>
       </c>
-      <c r="F11" s="100" t="n">
+      <c r="I11" s="100" t="n">
         <v>602</v>
       </c>
-      <c r="G11" s="49" t="inlineStr">
+      <c r="J11" s="49" t="inlineStr">
         <is>
           <t>FY24/25 (Afv)</t>
         </is>
       </c>
-      <c r="H11" s="90" t="n">
+      <c r="K11" s="90" t="n">
         <v>37</v>
       </c>
-      <c r="I11" s="90" t="n">
+      <c r="L11" s="90" t="n">
         <v>148</v>
       </c>
-      <c r="J11" s="98" t="n"/>
-      <c r="K11" s="49" t="inlineStr">
+      <c r="M11" s="98" t="n"/>
+      <c r="N11" s="49" t="inlineStr">
         <is>
           <t>Firm website count Oct-26</t>
         </is>
       </c>
-      <c r="L11" s="92">
-        <f>F11/H11</f>
+      <c r="O11" s="92">
+        <f>I11/K11</f>
         <v/>
       </c>
-      <c r="M11" s="98" t="n"/>
-      <c r="N11" s="93">
-        <f>F11/I11</f>
+      <c r="P11" s="98" t="n"/>
+      <c r="Q11" s="93">
+        <f>I11/L11</f>
         <v/>
       </c>
-      <c r="O11" s="98" t="n"/>
-      <c r="P11" s="101">
-        <f>H11/I11</f>
+      <c r="R11" s="98" t="n"/>
+      <c r="S11" s="101">
+        <f>K11/L11</f>
         <v/>
       </c>
-      <c r="Q11" s="98" t="n"/>
-      <c r="R11" s="49" t="inlineStr">
+      <c r="T11" s="98" t="n"/>
+      <c r="U11" s="49" t="inlineStr">
         <is>
           <t>Employees: allabolag band 200-499 only</t>
         </is>
@@ -49317,60 +49418,67 @@
       <c r="C12" s="100" t="n">
         <v>558</v>
       </c>
-      <c r="D12" s="100" t="n">
+      <c r="D12" s="131" t="n"/>
+      <c r="E12" s="98" t="n"/>
+      <c r="F12" s="49" t="inlineStr">
+        <is>
+          <t>Not filed (KB)</t>
+        </is>
+      </c>
+      <c r="G12" s="100" t="n">
         <v>529</v>
       </c>
-      <c r="E12" s="101">
-        <f>C12/D12-1</f>
+      <c r="H12" s="101">
+        <f>C12/G12-1</f>
         <v/>
       </c>
-      <c r="F12" s="100" t="n">
+      <c r="I12" s="100" t="n">
         <v>558</v>
       </c>
-      <c r="G12" s="49" t="inlineStr">
+      <c r="J12" s="49" t="inlineStr">
         <is>
           <t>FY2024 (Afv)</t>
         </is>
       </c>
-      <c r="H12" s="90" t="n">
+      <c r="K12" s="90" t="n">
         <v>51</v>
       </c>
-      <c r="I12" s="90" t="n">
+      <c r="L12" s="90" t="n">
         <v>150</v>
       </c>
-      <c r="J12" s="90" t="n">
+      <c r="M12" s="90" t="n">
         <v>220</v>
       </c>
-      <c r="K12" s="49" t="inlineStr">
+      <c r="N12" s="49" t="inlineStr">
         <is>
           <t>Firm statement / Chambers 2026 ("&gt;220")</t>
         </is>
       </c>
-      <c r="L12" s="92">
-        <f>F12/H12</f>
+      <c r="O12" s="92">
+        <f>I12/K12</f>
         <v/>
       </c>
-      <c r="M12" s="93">
-        <f>F12/J12</f>
+      <c r="P12" s="93">
+        <f>I12/M12</f>
         <v/>
       </c>
-      <c r="N12" s="93">
-        <f>F12/I12</f>
+      <c r="Q12" s="93">
+        <f>I12/L12</f>
         <v/>
       </c>
-      <c r="O12" s="101">
-        <f>H12/J12</f>
+      <c r="R12" s="101">
+        <f>K12/M12</f>
         <v/>
       </c>
-      <c r="P12" s="101">
-        <f>H12/I12</f>
+      <c r="S12" s="101">
+        <f>K12/L12</f>
         <v/>
       </c>
-      <c r="Q12" s="92">
-        <f>J12/H12</f>
+      <c r="T12" s="92">
+        <f>M12/K12</f>
         <v/>
       </c>
-      <c r="R12" s="49" t="inlineStr"/>
+      <c r="U12" s="49" t="inlineStr"/>
     </row>
     <row r="13">
       <c r="A13" s="90" t="n">
@@ -49385,59 +49493,71 @@
         <v>516</v>
       </c>
       <c r="D13" s="100" t="n">
+        <v>356</v>
+      </c>
+      <c r="E13" s="130">
+        <f>D13/355-1</f>
+        <v/>
+      </c>
+      <c r="F13" s="69" t="inlineStr">
+        <is>
+          <t>PARTIAL: Stockholm, Göteborg, Malmö ABs</t>
+        </is>
+      </c>
+      <c r="G13" s="100" t="n">
         <v>505</v>
       </c>
-      <c r="E13" s="101">
-        <f>C13/D13-1</f>
+      <c r="H13" s="101">
+        <f>C13/G13-1</f>
         <v/>
       </c>
-      <c r="F13" s="100" t="n">
+      <c r="I13" s="100" t="n">
         <v>516</v>
       </c>
-      <c r="G13" s="49" t="inlineStr">
+      <c r="J13" s="49" t="inlineStr">
         <is>
           <t>FY2024 (Afv)</t>
         </is>
       </c>
-      <c r="H13" s="90" t="n">
+      <c r="K13" s="90" t="n">
         <v>49</v>
       </c>
-      <c r="I13" s="90" t="n">
+      <c r="L13" s="90" t="n">
         <v>150</v>
       </c>
-      <c r="J13" s="90" t="n">
+      <c r="M13" s="90" t="n">
         <v>220</v>
       </c>
-      <c r="K13" s="49" t="inlineStr">
+      <c r="N13" s="49" t="inlineStr">
         <is>
           <t>Chambers 2026 / firm website</t>
         </is>
       </c>
-      <c r="L13" s="92">
-        <f>F13/H13</f>
+      <c r="O13" s="92">
+        <f>I13/K13</f>
         <v/>
       </c>
-      <c r="M13" s="93">
-        <f>F13/J13</f>
+      <c r="P13" s="93">
+        <f>I13/M13</f>
         <v/>
       </c>
-      <c r="N13" s="93">
-        <f>F13/I13</f>
+      <c r="Q13" s="93">
+        <f>I13/L13</f>
         <v/>
       </c>
-      <c r="O13" s="101">
-        <f>H13/J13</f>
+      <c r="R13" s="101">
+        <f>K13/M13</f>
         <v/>
       </c>
-      <c r="P13" s="101">
-        <f>H13/I13</f>
+      <c r="S13" s="101">
+        <f>K13/L13</f>
         <v/>
       </c>
-      <c r="Q13" s="92">
-        <f>J13/H13</f>
+      <c r="T13" s="92">
+        <f>M13/K13</f>
         <v/>
       </c>
-      <c r="R13" s="49" t="inlineStr"/>
+      <c r="U13" s="49" t="inlineStr"/>
     </row>
     <row r="14">
       <c r="A14" s="90" t="n">
@@ -49452,48 +49572,60 @@
         <v>500</v>
       </c>
       <c r="D14" s="100" t="n">
+        <v>555</v>
+      </c>
+      <c r="E14" s="130">
+        <f>D14/500-1</f>
+        <v/>
+      </c>
+      <c r="F14" s="69" t="inlineStr">
+        <is>
+          <t>Press snippet (Afv FY2025), unverified; KB not filed</t>
+        </is>
+      </c>
+      <c r="G14" s="100" t="n">
         <v>472</v>
       </c>
-      <c r="E14" s="101">
-        <f>C14/D14-1</f>
+      <c r="H14" s="101">
+        <f>C14/G14-1</f>
         <v/>
       </c>
-      <c r="F14" s="100" t="n">
+      <c r="I14" s="100" t="n">
         <v>500</v>
       </c>
-      <c r="G14" s="49" t="inlineStr">
+      <c r="J14" s="49" t="inlineStr">
         <is>
           <t>FY2024 (Afv)</t>
         </is>
       </c>
-      <c r="H14" s="90" t="n">
+      <c r="K14" s="90" t="n">
         <v>26</v>
       </c>
-      <c r="I14" s="90" t="n">
+      <c r="L14" s="90" t="n">
         <v>124</v>
       </c>
-      <c r="J14" s="98" t="n"/>
-      <c r="K14" s="49" t="inlineStr">
+      <c r="M14" s="98" t="n"/>
+      <c r="N14" s="49" t="inlineStr">
         <is>
           <t>Legal 500 (firm-supplied)</t>
         </is>
       </c>
-      <c r="L14" s="92">
-        <f>F14/H14</f>
+      <c r="O14" s="92">
+        <f>I14/K14</f>
         <v/>
       </c>
-      <c r="M14" s="98" t="n"/>
-      <c r="N14" s="93">
-        <f>F14/I14</f>
+      <c r="P14" s="98" t="n"/>
+      <c r="Q14" s="93">
+        <f>I14/L14</f>
         <v/>
       </c>
-      <c r="O14" s="98" t="n"/>
-      <c r="P14" s="101">
-        <f>H14/I14</f>
+      <c r="R14" s="98" t="n"/>
+      <c r="S14" s="101">
+        <f>K14/L14</f>
         <v/>
       </c>
-      <c r="Q14" s="98" t="n"/>
-      <c r="R14" s="49" t="inlineStr">
+      <c r="T14" s="98" t="n"/>
+      <c r="U14" s="49" t="inlineStr">
         <is>
           <t>KB - no public accounts; Chambers 120 lawyers</t>
         </is>
@@ -49512,48 +49644,60 @@
         <v>427</v>
       </c>
       <c r="D15" s="100" t="n">
+        <v>534</v>
+      </c>
+      <c r="E15" s="130">
+        <f>D15/427-1</f>
+        <v/>
+      </c>
+      <c r="F15" s="69" t="inlineStr">
+        <is>
+          <t>Press estimate (Afv: "&gt;0.5bn", +25%)</t>
+        </is>
+      </c>
+      <c r="G15" s="100" t="n">
         <v>343</v>
       </c>
-      <c r="E15" s="101">
-        <f>C15/D15-1</f>
+      <c r="H15" s="101">
+        <f>C15/G15-1</f>
         <v/>
       </c>
-      <c r="F15" s="100" t="n">
+      <c r="I15" s="100" t="n">
         <v>534</v>
       </c>
-      <c r="G15" s="49" t="inlineStr">
+      <c r="J15" s="49" t="inlineStr">
         <is>
           <t>FY2025 est. ("&gt;0.5bn", +25%)</t>
         </is>
       </c>
-      <c r="H15" s="90" t="n">
+      <c r="K15" s="90" t="n">
         <v>20</v>
       </c>
-      <c r="I15" s="90" t="n">
+      <c r="L15" s="90" t="n">
         <v>65</v>
       </c>
-      <c r="J15" s="98" t="n"/>
-      <c r="K15" s="49" t="inlineStr">
+      <c r="M15" s="98" t="n"/>
+      <c r="N15" s="49" t="inlineStr">
         <is>
           <t>Firm website count Oct-26 (Stockholm)</t>
         </is>
       </c>
-      <c r="L15" s="92">
-        <f>F15/H15</f>
+      <c r="O15" s="92">
+        <f>I15/K15</f>
         <v/>
       </c>
-      <c r="M15" s="98" t="n"/>
-      <c r="N15" s="93">
-        <f>F15/I15</f>
+      <c r="P15" s="98" t="n"/>
+      <c r="Q15" s="93">
+        <f>I15/L15</f>
         <v/>
       </c>
-      <c r="O15" s="98" t="n"/>
-      <c r="P15" s="101">
-        <f>H15/I15</f>
+      <c r="R15" s="98" t="n"/>
+      <c r="S15" s="101">
+        <f>K15/L15</f>
         <v/>
       </c>
-      <c r="Q15" s="98" t="n"/>
-      <c r="R15" s="49" t="inlineStr">
+      <c r="T15" s="98" t="n"/>
+      <c r="U15" s="49" t="inlineStr">
         <is>
           <t>May include leavers to BAHR; branch band 50-99 employees</t>
         </is>
@@ -49572,59 +49716,71 @@
         <v>417</v>
       </c>
       <c r="D16" s="100" t="n">
+        <v>324</v>
+      </c>
+      <c r="E16" s="130">
+        <f>D16/301-1</f>
+        <v/>
+      </c>
+      <c r="F16" s="49" t="inlineStr">
+        <is>
+          <t>MAQS AB accounts (excl. Malmö KB)</t>
+        </is>
+      </c>
+      <c r="G16" s="100" t="n">
         <v>346</v>
       </c>
-      <c r="E16" s="101">
-        <f>C16/D16-1</f>
+      <c r="H16" s="101">
+        <f>C16/G16-1</f>
         <v/>
       </c>
-      <c r="F16" s="100" t="n">
+      <c r="I16" s="100" t="n">
         <v>417</v>
       </c>
-      <c r="G16" s="49" t="inlineStr">
+      <c r="J16" s="49" t="inlineStr">
         <is>
           <t>FY2024 (Afv)</t>
         </is>
       </c>
-      <c r="H16" s="90" t="n">
+      <c r="K16" s="90" t="n">
         <v>48</v>
       </c>
-      <c r="I16" s="90" t="n">
+      <c r="L16" s="90" t="n">
         <v>144</v>
       </c>
-      <c r="J16" s="90" t="n">
+      <c r="M16" s="90" t="n">
         <v>180</v>
       </c>
-      <c r="K16" s="49" t="inlineStr">
+      <c r="N16" s="49" t="inlineStr">
         <is>
           <t>Firm website count Oct-26; employees Chambers 2026</t>
         </is>
       </c>
-      <c r="L16" s="92">
-        <f>F16/H16</f>
+      <c r="O16" s="92">
+        <f>I16/K16</f>
         <v/>
       </c>
-      <c r="M16" s="93">
-        <f>F16/J16</f>
+      <c r="P16" s="93">
+        <f>I16/M16</f>
         <v/>
       </c>
-      <c r="N16" s="93">
-        <f>F16/I16</f>
+      <c r="Q16" s="93">
+        <f>I16/L16</f>
         <v/>
       </c>
-      <c r="O16" s="101">
-        <f>H16/J16</f>
+      <c r="R16" s="101">
+        <f>K16/M16</f>
         <v/>
       </c>
-      <c r="P16" s="101">
-        <f>H16/I16</f>
+      <c r="S16" s="101">
+        <f>K16/L16</f>
         <v/>
       </c>
-      <c r="Q16" s="92">
-        <f>J16/H16</f>
+      <c r="T16" s="92">
+        <f>M16/K16</f>
         <v/>
       </c>
-      <c r="R16" s="49" t="inlineStr">
+      <c r="U16" s="49" t="inlineStr">
         <is>
           <t>Splitting from 1 Jan 2027: Malmö (MAQS KB) vs Sthlm/Gbg/Sundsvall (MAQS AB)</t>
         </is>
@@ -49643,59 +49799,71 @@
         <v>363</v>
       </c>
       <c r="D17" s="100" t="n">
+        <v>431</v>
+      </c>
+      <c r="E17" s="130">
+        <f>D17/373-1</f>
+        <v/>
+      </c>
+      <c r="F17" s="49" t="inlineStr">
+        <is>
+          <t>AB accounts: full firm</t>
+        </is>
+      </c>
+      <c r="G17" s="100" t="n">
         <v>317</v>
       </c>
-      <c r="E17" s="101">
-        <f>C17/D17-1</f>
+      <c r="H17" s="101">
+        <f>C17/G17-1</f>
         <v/>
       </c>
-      <c r="F17" s="100" t="n">
+      <c r="I17" s="100" t="n">
         <v>431</v>
       </c>
-      <c r="G17" s="49" t="inlineStr">
+      <c r="J17" s="49" t="inlineStr">
         <is>
           <t>FY2025 net sales (AB)</t>
         </is>
       </c>
-      <c r="H17" s="90" t="n">
+      <c r="K17" s="90" t="n">
         <v>27</v>
       </c>
-      <c r="I17" s="90" t="n">
+      <c r="L17" s="90" t="n">
         <v>76</v>
       </c>
-      <c r="J17" s="90" t="n">
+      <c r="M17" s="90" t="n">
         <v>127</v>
       </c>
-      <c r="K17" s="49" t="inlineStr">
+      <c r="N17" s="49" t="inlineStr">
         <is>
           <t>Legal 500; employees 2025 accounts</t>
         </is>
       </c>
-      <c r="L17" s="92">
-        <f>F17/H17</f>
+      <c r="O17" s="92">
+        <f>I17/K17</f>
         <v/>
       </c>
-      <c r="M17" s="93">
-        <f>F17/J17</f>
+      <c r="P17" s="93">
+        <f>I17/M17</f>
         <v/>
       </c>
-      <c r="N17" s="93">
-        <f>F17/I17</f>
+      <c r="Q17" s="93">
+        <f>I17/L17</f>
         <v/>
       </c>
-      <c r="O17" s="101">
-        <f>H17/J17</f>
+      <c r="R17" s="101">
+        <f>K17/M17</f>
         <v/>
       </c>
-      <c r="P17" s="101">
-        <f>H17/I17</f>
+      <c r="S17" s="101">
+        <f>K17/L17</f>
         <v/>
       </c>
-      <c r="Q17" s="92">
-        <f>J17/H17</f>
+      <c r="T17" s="92">
+        <f>M17/K17</f>
         <v/>
       </c>
-      <c r="R17" s="49" t="inlineStr"/>
+      <c r="U17" s="49" t="inlineStr"/>
     </row>
     <row r="18">
       <c r="A18" s="90" t="n">
@@ -49710,51 +49878,63 @@
         <v>295</v>
       </c>
       <c r="D18" s="100" t="n">
+        <v>279</v>
+      </c>
+      <c r="E18" s="130">
+        <f>D18/299-1</f>
+        <v/>
+      </c>
+      <c r="F18" s="49" t="inlineStr">
+        <is>
+          <t>AB accounts: full firm</t>
+        </is>
+      </c>
+      <c r="G18" s="100" t="n">
         <v>300</v>
       </c>
-      <c r="E18" s="101">
-        <f>C18/D18-1</f>
+      <c r="H18" s="101">
+        <f>C18/G18-1</f>
         <v/>
       </c>
-      <c r="F18" s="100" t="n">
+      <c r="I18" s="100" t="n">
         <v>279</v>
       </c>
-      <c r="G18" s="49" t="inlineStr">
+      <c r="J18" s="49" t="inlineStr">
         <is>
           <t>FY2025 net sales (AB)</t>
         </is>
       </c>
-      <c r="H18" s="90" t="n">
+      <c r="K18" s="90" t="n">
         <v>17</v>
       </c>
-      <c r="I18" s="98" t="n"/>
-      <c r="J18" s="90" t="n">
+      <c r="L18" s="98" t="n"/>
+      <c r="M18" s="90" t="n">
         <v>107</v>
       </c>
-      <c r="K18" s="49" t="inlineStr">
+      <c r="N18" s="49" t="inlineStr">
         <is>
           <t>Legal 500 (stale); employees 2025 accounts</t>
         </is>
       </c>
-      <c r="L18" s="92">
-        <f>F18/H18</f>
+      <c r="O18" s="92">
+        <f>I18/K18</f>
         <v/>
       </c>
-      <c r="M18" s="93">
-        <f>F18/J18</f>
+      <c r="P18" s="93">
+        <f>I18/M18</f>
         <v/>
       </c>
-      <c r="N18" s="98" t="n"/>
-      <c r="O18" s="101">
-        <f>H18/J18</f>
+      <c r="Q18" s="98" t="n"/>
+      <c r="R18" s="101">
+        <f>K18/M18</f>
         <v/>
       </c>
-      <c r="P18" s="98" t="n"/>
-      <c r="Q18" s="92">
-        <f>J18/H18</f>
+      <c r="S18" s="98" t="n"/>
+      <c r="T18" s="92">
+        <f>M18/K18</f>
         <v/>
       </c>
-      <c r="R18" s="49" t="inlineStr">
+      <c r="U18" s="49" t="inlineStr">
         <is>
           <t>Partner count unverified</t>
         </is>
@@ -49773,59 +49953,71 @@
         <v>277</v>
       </c>
       <c r="D19" s="100" t="n">
+        <v>172</v>
+      </c>
+      <c r="E19" s="130">
+        <f>D19/164-1</f>
+        <v/>
+      </c>
+      <c r="F19" s="69" t="inlineStr">
+        <is>
+          <t>PARTIAL: main Swedish AB</t>
+        </is>
+      </c>
+      <c r="G19" s="100" t="n">
         <v>263</v>
       </c>
-      <c r="E19" s="101">
-        <f>C19/D19-1</f>
+      <c r="H19" s="101">
+        <f>C19/G19-1</f>
         <v/>
       </c>
-      <c r="F19" s="100" t="n">
+      <c r="I19" s="100" t="n">
         <v>277</v>
       </c>
-      <c r="G19" s="49" t="inlineStr">
+      <c r="J19" s="49" t="inlineStr">
         <is>
           <t>FY2024 (Afv)</t>
         </is>
       </c>
-      <c r="H19" s="90" t="n">
+      <c r="K19" s="90" t="n">
         <v>23</v>
       </c>
-      <c r="I19" s="90" t="n">
+      <c r="L19" s="90" t="n">
         <v>73</v>
       </c>
-      <c r="J19" s="90" t="n">
+      <c r="M19" s="90" t="n">
         <v>106</v>
       </c>
-      <c r="K19" s="49" t="inlineStr">
+      <c r="N19" s="49" t="inlineStr">
         <is>
           <t>Firm website count Oct-26; employees AB accounts</t>
         </is>
       </c>
-      <c r="L19" s="92">
-        <f>F19/H19</f>
+      <c r="O19" s="92">
+        <f>I19/K19</f>
         <v/>
       </c>
-      <c r="M19" s="93">
-        <f>F19/J19</f>
+      <c r="P19" s="93">
+        <f>I19/M19</f>
         <v/>
       </c>
-      <c r="N19" s="93">
-        <f>F19/I19</f>
+      <c r="Q19" s="93">
+        <f>I19/L19</f>
         <v/>
       </c>
-      <c r="O19" s="101">
-        <f>H19/J19</f>
+      <c r="R19" s="101">
+        <f>K19/M19</f>
         <v/>
       </c>
-      <c r="P19" s="101">
-        <f>H19/I19</f>
+      <c r="S19" s="101">
+        <f>K19/L19</f>
         <v/>
       </c>
-      <c r="Q19" s="92">
-        <f>J19/H19</f>
+      <c r="T19" s="92">
+        <f>M19/K19</f>
         <v/>
       </c>
-      <c r="R19" s="49" t="inlineStr"/>
+      <c r="U19" s="49" t="inlineStr"/>
     </row>
     <row r="20">
       <c r="A20" s="90" t="n">
@@ -49839,41 +50031,48 @@
       <c r="C20" s="100" t="n">
         <v>198</v>
       </c>
-      <c r="D20" s="100" t="n">
+      <c r="D20" s="131" t="n"/>
+      <c r="E20" s="98" t="n"/>
+      <c r="F20" s="49" t="inlineStr">
+        <is>
+          <t>Not filed (KB)</t>
+        </is>
+      </c>
+      <c r="G20" s="100" t="n">
         <v>228</v>
       </c>
-      <c r="E20" s="101">
-        <f>C20/D20-1</f>
+      <c r="H20" s="101">
+        <f>C20/G20-1</f>
         <v/>
       </c>
-      <c r="F20" s="100" t="n">
+      <c r="I20" s="100" t="n">
         <v>198</v>
       </c>
-      <c r="G20" s="49" t="inlineStr">
+      <c r="J20" s="49" t="inlineStr">
         <is>
           <t>FY2024 (Afv)</t>
         </is>
       </c>
-      <c r="H20" s="98" t="n"/>
-      <c r="I20" s="90" t="n">
+      <c r="K20" s="98" t="n"/>
+      <c r="L20" s="90" t="n">
         <v>41</v>
       </c>
-      <c r="J20" s="98" t="n"/>
-      <c r="K20" s="49" t="inlineStr">
+      <c r="M20" s="98" t="n"/>
+      <c r="N20" s="49" t="inlineStr">
         <is>
           <t>Legal 500</t>
         </is>
-      </c>
-      <c r="L20" s="98" t="n"/>
-      <c r="M20" s="98" t="n"/>
-      <c r="N20" s="93">
-        <f>F20/I20</f>
-        <v/>
       </c>
       <c r="O20" s="98" t="n"/>
       <c r="P20" s="98" t="n"/>
-      <c r="Q20" s="98" t="n"/>
-      <c r="R20" s="49" t="inlineStr">
+      <c r="Q20" s="93">
+        <f>I20/L20</f>
+        <v/>
+      </c>
+      <c r="R20" s="98" t="n"/>
+      <c r="S20" s="98" t="n"/>
+      <c r="T20" s="98" t="n"/>
+      <c r="U20" s="49" t="inlineStr">
         <is>
           <t>Lost 12-person team to Cirio (Jan-25)</t>
         </is>
@@ -49891,49 +50090,56 @@
       <c r="C21" s="100" t="n">
         <v>196</v>
       </c>
-      <c r="D21" s="100" t="n">
+      <c r="D21" s="131" t="n"/>
+      <c r="E21" s="98" t="n"/>
+      <c r="F21" s="49" t="inlineStr">
+        <is>
+          <t>Not collected (multiple regional ABs)</t>
+        </is>
+      </c>
+      <c r="G21" s="100" t="n">
         <v>174</v>
       </c>
-      <c r="E21" s="101">
-        <f>C21/D21-1</f>
+      <c r="H21" s="101">
+        <f>C21/G21-1</f>
         <v/>
       </c>
-      <c r="F21" s="100" t="n">
+      <c r="I21" s="100" t="n">
         <v>196</v>
       </c>
-      <c r="G21" s="49" t="inlineStr">
+      <c r="J21" s="49" t="inlineStr">
         <is>
           <t>FY2024 (Afv)</t>
         </is>
       </c>
-      <c r="H21" s="90" t="n">
+      <c r="K21" s="90" t="n">
         <v>41</v>
       </c>
-      <c r="I21" s="90" t="n">
+      <c r="L21" s="90" t="n">
         <v>78</v>
       </c>
-      <c r="J21" s="98" t="n"/>
-      <c r="K21" s="49" t="inlineStr">
+      <c r="M21" s="98" t="n"/>
+      <c r="N21" s="49" t="inlineStr">
         <is>
           <t>Firm website count Oct-26 (Sweden)</t>
         </is>
       </c>
-      <c r="L21" s="92">
-        <f>F21/H21</f>
+      <c r="O21" s="92">
+        <f>I21/K21</f>
         <v/>
       </c>
-      <c r="M21" s="98" t="n"/>
-      <c r="N21" s="93">
-        <f>F21/I21</f>
+      <c r="P21" s="98" t="n"/>
+      <c r="Q21" s="93">
+        <f>I21/L21</f>
         <v/>
       </c>
-      <c r="O21" s="98" t="n"/>
-      <c r="P21" s="101">
-        <f>H21/I21</f>
+      <c r="R21" s="98" t="n"/>
+      <c r="S21" s="101">
+        <f>K21/L21</f>
         <v/>
       </c>
-      <c r="Q21" s="98" t="n"/>
-      <c r="R21" s="49" t="inlineStr">
+      <c r="T21" s="98" t="n"/>
+      <c r="U21" s="49" t="inlineStr">
         <is>
           <t>~200 staff incl. Baltics (not used)</t>
         </is>
@@ -49952,48 +50158,60 @@
         <v>188</v>
       </c>
       <c r="D22" s="100" t="n">
+        <v>103</v>
+      </c>
+      <c r="E22" s="130">
+        <f>D22/92-1</f>
+        <v/>
+      </c>
+      <c r="F22" s="69" t="inlineStr">
+        <is>
+          <t>PARTIAL: TM &amp; Partners Law AB</t>
+        </is>
+      </c>
+      <c r="G22" s="100" t="n">
         <v>175</v>
       </c>
-      <c r="E22" s="101">
-        <f>C22/D22-1</f>
+      <c r="H22" s="101">
+        <f>C22/G22-1</f>
         <v/>
       </c>
-      <c r="F22" s="100" t="n">
+      <c r="I22" s="100" t="n">
         <v>188</v>
       </c>
-      <c r="G22" s="49" t="inlineStr">
+      <c r="J22" s="49" t="inlineStr">
         <is>
           <t>FY2024 (Afv)</t>
         </is>
       </c>
-      <c r="H22" s="90" t="n">
+      <c r="K22" s="90" t="n">
         <v>18</v>
       </c>
-      <c r="I22" s="90" t="n">
+      <c r="L22" s="90" t="n">
         <v>63</v>
       </c>
-      <c r="J22" s="98" t="n"/>
-      <c r="K22" s="49" t="inlineStr">
+      <c r="M22" s="98" t="n"/>
+      <c r="N22" s="49" t="inlineStr">
         <is>
           <t>Firm website count Oct-26</t>
         </is>
       </c>
-      <c r="L22" s="92">
-        <f>F22/H22</f>
+      <c r="O22" s="92">
+        <f>I22/K22</f>
         <v/>
       </c>
-      <c r="M22" s="98" t="n"/>
-      <c r="N22" s="93">
-        <f>F22/I22</f>
+      <c r="P22" s="98" t="n"/>
+      <c r="Q22" s="93">
+        <f>I22/L22</f>
         <v/>
       </c>
-      <c r="O22" s="98" t="n"/>
-      <c r="P22" s="101">
-        <f>H22/I22</f>
+      <c r="R22" s="98" t="n"/>
+      <c r="S22" s="101">
+        <f>K22/L22</f>
         <v/>
       </c>
-      <c r="Q22" s="98" t="n"/>
-      <c r="R22" s="49" t="inlineStr">
+      <c r="T22" s="98" t="n"/>
+      <c r="U22" s="49" t="inlineStr">
         <is>
           <t>Part of AGRD since 2025; AB (73 staff) is partial</t>
         </is>
@@ -50011,32 +50229,39 @@
       <c r="C23" s="100" t="n">
         <v>165</v>
       </c>
-      <c r="D23" s="100" t="n">
+      <c r="D23" s="131" t="n"/>
+      <c r="E23" s="98" t="n"/>
+      <c r="F23" s="49" t="inlineStr">
+        <is>
+          <t>Not collected</t>
+        </is>
+      </c>
+      <c r="G23" s="100" t="n">
         <v>164</v>
       </c>
-      <c r="E23" s="101">
-        <f>C23/D23-1</f>
+      <c r="H23" s="101">
+        <f>C23/G23-1</f>
         <v/>
       </c>
-      <c r="F23" s="100" t="n">
+      <c r="I23" s="100" t="n">
         <v>165</v>
       </c>
-      <c r="G23" s="49" t="inlineStr">
+      <c r="J23" s="49" t="inlineStr">
         <is>
           <t>FY2024 (Afv)</t>
         </is>
       </c>
-      <c r="H23" s="98" t="n"/>
-      <c r="I23" s="98" t="n"/>
-      <c r="J23" s="98" t="n"/>
-      <c r="K23" s="49" t="inlineStr"/>
+      <c r="K23" s="98" t="n"/>
       <c r="L23" s="98" t="n"/>
       <c r="M23" s="98" t="n"/>
-      <c r="N23" s="98" t="n"/>
+      <c r="N23" s="49" t="inlineStr"/>
       <c r="O23" s="98" t="n"/>
       <c r="P23" s="98" t="n"/>
       <c r="Q23" s="98" t="n"/>
-      <c r="R23" s="49" t="inlineStr">
+      <c r="R23" s="98" t="n"/>
+      <c r="S23" s="98" t="n"/>
+      <c r="T23" s="98" t="n"/>
+      <c r="U23" s="49" t="inlineStr">
         <is>
           <t>Headcount not researched</t>
         </is>
@@ -50054,41 +50279,48 @@
       <c r="C24" s="100" t="n">
         <v>163</v>
       </c>
-      <c r="D24" s="100" t="n">
+      <c r="D24" s="131" t="n"/>
+      <c r="E24" s="98" t="n"/>
+      <c r="F24" s="49" t="inlineStr">
+        <is>
+          <t>Not collected</t>
+        </is>
+      </c>
+      <c r="G24" s="100" t="n">
         <v>151</v>
       </c>
-      <c r="E24" s="101">
-        <f>C24/D24-1</f>
+      <c r="H24" s="101">
+        <f>C24/G24-1</f>
         <v/>
       </c>
-      <c r="F24" s="100" t="n">
+      <c r="I24" s="100" t="n">
         <v>163</v>
       </c>
-      <c r="G24" s="49" t="inlineStr">
+      <c r="J24" s="49" t="inlineStr">
         <is>
           <t>FY2024 (Afv)</t>
         </is>
       </c>
-      <c r="H24" s="98" t="n"/>
-      <c r="I24" s="90" t="n">
+      <c r="K24" s="98" t="n"/>
+      <c r="L24" s="90" t="n">
         <v>56</v>
       </c>
-      <c r="J24" s="98" t="n"/>
-      <c r="K24" s="49" t="inlineStr">
+      <c r="M24" s="98" t="n"/>
+      <c r="N24" s="49" t="inlineStr">
         <is>
           <t>Legal 500</t>
         </is>
-      </c>
-      <c r="L24" s="98" t="n"/>
-      <c r="M24" s="98" t="n"/>
-      <c r="N24" s="93">
-        <f>F24/I24</f>
-        <v/>
       </c>
       <c r="O24" s="98" t="n"/>
       <c r="P24" s="98" t="n"/>
-      <c r="Q24" s="98" t="n"/>
-      <c r="R24" s="49" t="inlineStr">
+      <c r="Q24" s="93">
+        <f>I24/L24</f>
+        <v/>
+      </c>
+      <c r="R24" s="98" t="n"/>
+      <c r="S24" s="98" t="n"/>
+      <c r="T24" s="98" t="n"/>
+      <c r="U24" s="49" t="inlineStr">
         <is>
           <t>Part of AGRD since 2025</t>
         </is>
@@ -50107,45 +50339,57 @@
         <v>158</v>
       </c>
       <c r="D25" s="100" t="n">
+        <v>178</v>
+      </c>
+      <c r="E25" s="130">
+        <f>D25/160-1</f>
+        <v/>
+      </c>
+      <c r="F25" s="49" t="inlineStr">
+        <is>
+          <t>AB accounts: full firm</t>
+        </is>
+      </c>
+      <c r="G25" s="100" t="n">
         <v>133</v>
       </c>
-      <c r="E25" s="101">
-        <f>C25/D25-1</f>
+      <c r="H25" s="101">
+        <f>C25/G25-1</f>
         <v/>
       </c>
-      <c r="F25" s="100" t="n">
+      <c r="I25" s="100" t="n">
         <v>178</v>
       </c>
-      <c r="G25" s="49" t="inlineStr">
+      <c r="J25" s="49" t="inlineStr">
         <is>
           <t>FY2025 net sales (AB)</t>
         </is>
       </c>
-      <c r="H25" s="98" t="n"/>
-      <c r="I25" s="90" t="n">
+      <c r="K25" s="98" t="n"/>
+      <c r="L25" s="90" t="n">
         <v>47</v>
       </c>
-      <c r="J25" s="90" t="n">
+      <c r="M25" s="90" t="n">
         <v>63</v>
       </c>
-      <c r="K25" s="49" t="inlineStr">
+      <c r="N25" s="49" t="inlineStr">
         <is>
           <t>Chambers 2026; employees 2025 accounts</t>
         </is>
       </c>
-      <c r="L25" s="98" t="n"/>
-      <c r="M25" s="93">
-        <f>F25/J25</f>
+      <c r="O25" s="98" t="n"/>
+      <c r="P25" s="93">
+        <f>I25/M25</f>
         <v/>
       </c>
-      <c r="N25" s="93">
-        <f>F25/I25</f>
+      <c r="Q25" s="93">
+        <f>I25/L25</f>
         <v/>
       </c>
-      <c r="O25" s="98" t="n"/>
-      <c r="P25" s="98" t="n"/>
-      <c r="Q25" s="98" t="n"/>
-      <c r="R25" s="49" t="inlineStr"/>
+      <c r="R25" s="98" t="n"/>
+      <c r="S25" s="98" t="n"/>
+      <c r="T25" s="98" t="n"/>
+      <c r="U25" s="49" t="inlineStr"/>
     </row>
     <row r="26">
       <c r="A26" s="90" t="n">
@@ -50159,49 +50403,56 @@
       <c r="C26" s="100" t="n">
         <v>146</v>
       </c>
-      <c r="D26" s="100" t="n">
+      <c r="D26" s="131" t="n"/>
+      <c r="E26" s="98" t="n"/>
+      <c r="F26" s="49" t="inlineStr">
+        <is>
+          <t>Service AB only (not comparable)</t>
+        </is>
+      </c>
+      <c r="G26" s="100" t="n">
         <v>122</v>
       </c>
-      <c r="E26" s="101">
-        <f>C26/D26-1</f>
+      <c r="H26" s="101">
+        <f>C26/G26-1</f>
         <v/>
       </c>
-      <c r="F26" s="100" t="n">
+      <c r="I26" s="100" t="n">
         <v>146</v>
       </c>
-      <c r="G26" s="49" t="inlineStr">
+      <c r="J26" s="49" t="inlineStr">
         <is>
           <t>FY2024 (Afv)</t>
         </is>
       </c>
-      <c r="H26" s="90" t="n">
+      <c r="K26" s="90" t="n">
         <v>11</v>
       </c>
-      <c r="I26" s="90" t="n">
+      <c r="L26" s="90" t="n">
         <v>40</v>
       </c>
-      <c r="J26" s="98" t="n"/>
-      <c r="K26" s="49" t="inlineStr">
+      <c r="M26" s="98" t="n"/>
+      <c r="N26" s="49" t="inlineStr">
         <is>
           <t>Firm website count Oct-26</t>
         </is>
       </c>
-      <c r="L26" s="92">
-        <f>F26/H26</f>
+      <c r="O26" s="92">
+        <f>I26/K26</f>
         <v/>
       </c>
-      <c r="M26" s="98" t="n"/>
-      <c r="N26" s="93">
-        <f>F26/I26</f>
+      <c r="P26" s="98" t="n"/>
+      <c r="Q26" s="93">
+        <f>I26/L26</f>
         <v/>
       </c>
-      <c r="O26" s="98" t="n"/>
-      <c r="P26" s="101">
-        <f>H26/I26</f>
+      <c r="R26" s="98" t="n"/>
+      <c r="S26" s="101">
+        <f>K26/L26</f>
         <v/>
       </c>
-      <c r="Q26" s="98" t="n"/>
-      <c r="R26" s="49" t="inlineStr">
+      <c r="T26" s="98" t="n"/>
+      <c r="U26" s="49" t="inlineStr">
         <is>
           <t>Service AB (53 staff) is partial; joined AGRD Jan-26</t>
         </is>
@@ -50219,41 +50470,48 @@
       <c r="C27" s="100" t="n">
         <v>141</v>
       </c>
-      <c r="D27" s="100" t="n">
+      <c r="D27" s="131" t="n"/>
+      <c r="E27" s="98" t="n"/>
+      <c r="F27" s="49" t="inlineStr">
+        <is>
+          <t>Not collected</t>
+        </is>
+      </c>
+      <c r="G27" s="100" t="n">
         <v>117</v>
       </c>
-      <c r="E27" s="101">
-        <f>C27/D27-1</f>
+      <c r="H27" s="101">
+        <f>C27/G27-1</f>
         <v/>
       </c>
-      <c r="F27" s="100" t="n">
+      <c r="I27" s="100" t="n">
         <v>141</v>
       </c>
-      <c r="G27" s="49" t="inlineStr">
+      <c r="J27" s="49" t="inlineStr">
         <is>
           <t>FY2024 (Afv)</t>
         </is>
       </c>
-      <c r="H27" s="98" t="n"/>
-      <c r="I27" s="90" t="n">
+      <c r="K27" s="98" t="n"/>
+      <c r="L27" s="90" t="n">
         <v>41</v>
       </c>
-      <c r="J27" s="98" t="n"/>
-      <c r="K27" s="49" t="inlineStr">
+      <c r="M27" s="98" t="n"/>
+      <c r="N27" s="49" t="inlineStr">
         <is>
           <t>Legal 500</t>
         </is>
-      </c>
-      <c r="L27" s="98" t="n"/>
-      <c r="M27" s="98" t="n"/>
-      <c r="N27" s="93">
-        <f>F27/I27</f>
-        <v/>
       </c>
       <c r="O27" s="98" t="n"/>
       <c r="P27" s="98" t="n"/>
-      <c r="Q27" s="98" t="n"/>
-      <c r="R27" s="49" t="inlineStr"/>
+      <c r="Q27" s="93">
+        <f>I27/L27</f>
+        <v/>
+      </c>
+      <c r="R27" s="98" t="n"/>
+      <c r="S27" s="98" t="n"/>
+      <c r="T27" s="98" t="n"/>
+      <c r="U27" s="49" t="inlineStr"/>
     </row>
     <row r="28">
       <c r="A28" s="90" t="n">
@@ -50268,40 +50526,52 @@
         <v>140</v>
       </c>
       <c r="D28" s="100" t="n">
+        <v>166</v>
+      </c>
+      <c r="E28" s="130">
+        <f>D28/160-1</f>
+        <v/>
+      </c>
+      <c r="F28" s="49" t="inlineStr">
+        <is>
+          <t>AB accounts: full firm</t>
+        </is>
+      </c>
+      <c r="G28" s="100" t="n">
         <v>148</v>
       </c>
-      <c r="E28" s="101">
-        <f>C28/D28-1</f>
+      <c r="H28" s="101">
+        <f>C28/G28-1</f>
         <v/>
       </c>
-      <c r="F28" s="100" t="n">
+      <c r="I28" s="100" t="n">
         <v>166</v>
       </c>
-      <c r="G28" s="49" t="inlineStr">
+      <c r="J28" s="49" t="inlineStr">
         <is>
           <t>FY2025 net sales (AB)</t>
         </is>
       </c>
-      <c r="H28" s="98" t="n"/>
-      <c r="I28" s="98" t="n"/>
-      <c r="J28" s="90" t="n">
+      <c r="K28" s="98" t="n"/>
+      <c r="L28" s="98" t="n"/>
+      <c r="M28" s="90" t="n">
         <v>59</v>
       </c>
-      <c r="K28" s="49" t="inlineStr">
+      <c r="N28" s="49" t="inlineStr">
         <is>
           <t>2025 accounts</t>
         </is>
       </c>
-      <c r="L28" s="98" t="n"/>
-      <c r="M28" s="93">
-        <f>F28/J28</f>
+      <c r="O28" s="98" t="n"/>
+      <c r="P28" s="93">
+        <f>I28/M28</f>
         <v/>
       </c>
-      <c r="N28" s="98" t="n"/>
-      <c r="O28" s="98" t="n"/>
-      <c r="P28" s="98" t="n"/>
       <c r="Q28" s="98" t="n"/>
-      <c r="R28" s="49" t="inlineStr"/>
+      <c r="R28" s="98" t="n"/>
+      <c r="S28" s="98" t="n"/>
+      <c r="T28" s="98" t="n"/>
+      <c r="U28" s="49" t="inlineStr"/>
     </row>
     <row r="29">
       <c r="A29" s="90" t="n">
@@ -50315,49 +50585,56 @@
       <c r="C29" s="100" t="n">
         <v>131</v>
       </c>
-      <c r="D29" s="100" t="n">
+      <c r="D29" s="131" t="n"/>
+      <c r="E29" s="98" t="n"/>
+      <c r="F29" s="49" t="inlineStr">
+        <is>
+          <t>Not filed (KB)</t>
+        </is>
+      </c>
+      <c r="G29" s="100" t="n">
         <v>120</v>
       </c>
-      <c r="E29" s="101">
-        <f>C29/D29-1</f>
+      <c r="H29" s="101">
+        <f>C29/G29-1</f>
         <v/>
       </c>
-      <c r="F29" s="100" t="n">
+      <c r="I29" s="100" t="n">
         <v>131</v>
       </c>
-      <c r="G29" s="49" t="inlineStr">
+      <c r="J29" s="49" t="inlineStr">
         <is>
           <t>FY2024 (Afv)</t>
         </is>
       </c>
-      <c r="H29" s="90" t="n">
+      <c r="K29" s="90" t="n">
         <v>21</v>
       </c>
-      <c r="I29" s="90" t="n">
+      <c r="L29" s="90" t="n">
         <v>35</v>
       </c>
-      <c r="J29" s="98" t="n"/>
-      <c r="K29" s="49" t="inlineStr">
+      <c r="M29" s="98" t="n"/>
+      <c r="N29" s="49" t="inlineStr">
         <is>
           <t>Firm website count Oct-26</t>
         </is>
       </c>
-      <c r="L29" s="92">
-        <f>F29/H29</f>
+      <c r="O29" s="92">
+        <f>I29/K29</f>
         <v/>
       </c>
-      <c r="M29" s="98" t="n"/>
-      <c r="N29" s="93">
-        <f>F29/I29</f>
+      <c r="P29" s="98" t="n"/>
+      <c r="Q29" s="93">
+        <f>I29/L29</f>
         <v/>
       </c>
-      <c r="O29" s="98" t="n"/>
-      <c r="P29" s="101">
-        <f>H29/I29</f>
+      <c r="R29" s="98" t="n"/>
+      <c r="S29" s="101">
+        <f>K29/L29</f>
         <v/>
       </c>
-      <c r="Q29" s="98" t="n"/>
-      <c r="R29" s="49" t="inlineStr">
+      <c r="T29" s="98" t="n"/>
+      <c r="U29" s="49" t="inlineStr">
         <is>
           <t>KB band 20-49 employees</t>
         </is>
@@ -50375,32 +50652,39 @@
       <c r="C30" s="100" t="n">
         <v>130</v>
       </c>
-      <c r="D30" s="100" t="n">
+      <c r="D30" s="131" t="n"/>
+      <c r="E30" s="98" t="n"/>
+      <c r="F30" s="49" t="inlineStr">
+        <is>
+          <t>Service AB only (not comparable)</t>
+        </is>
+      </c>
+      <c r="G30" s="100" t="n">
         <v>114</v>
       </c>
-      <c r="E30" s="101">
-        <f>C30/D30-1</f>
+      <c r="H30" s="101">
+        <f>C30/G30-1</f>
         <v/>
       </c>
-      <c r="F30" s="100" t="n">
+      <c r="I30" s="100" t="n">
         <v>130</v>
       </c>
-      <c r="G30" s="49" t="inlineStr">
+      <c r="J30" s="49" t="inlineStr">
         <is>
           <t>FY2024 (Afv)</t>
         </is>
       </c>
-      <c r="H30" s="98" t="n"/>
-      <c r="I30" s="98" t="n"/>
-      <c r="J30" s="98" t="n"/>
-      <c r="K30" s="49" t="inlineStr"/>
+      <c r="K30" s="98" t="n"/>
       <c r="L30" s="98" t="n"/>
       <c r="M30" s="98" t="n"/>
-      <c r="N30" s="98" t="n"/>
+      <c r="N30" s="49" t="inlineStr"/>
       <c r="O30" s="98" t="n"/>
       <c r="P30" s="98" t="n"/>
       <c r="Q30" s="98" t="n"/>
-      <c r="R30" s="49" t="inlineStr">
+      <c r="R30" s="98" t="n"/>
+      <c r="S30" s="98" t="n"/>
+      <c r="T30" s="98" t="n"/>
+      <c r="U30" s="49" t="inlineStr">
         <is>
           <t>AB (49 staff) is partial</t>
         </is>
@@ -50418,41 +50702,48 @@
       <c r="C31" s="100" t="n">
         <v>126</v>
       </c>
-      <c r="D31" s="100" t="n">
+      <c r="D31" s="131" t="n"/>
+      <c r="E31" s="98" t="n"/>
+      <c r="F31" s="49" t="inlineStr">
+        <is>
+          <t>Not collected</t>
+        </is>
+      </c>
+      <c r="G31" s="100" t="n">
         <v>126</v>
       </c>
-      <c r="E31" s="101">
-        <f>C31/D31-1</f>
+      <c r="H31" s="101">
+        <f>C31/G31-1</f>
         <v/>
       </c>
-      <c r="F31" s="100" t="n">
+      <c r="I31" s="100" t="n">
         <v>126</v>
       </c>
-      <c r="G31" s="49" t="inlineStr">
+      <c r="J31" s="49" t="inlineStr">
         <is>
           <t>FY2024 (Afv)</t>
         </is>
       </c>
-      <c r="H31" s="98" t="n"/>
-      <c r="I31" s="98" t="n"/>
-      <c r="J31" s="90" t="n">
+      <c r="K31" s="98" t="n"/>
+      <c r="L31" s="98" t="n"/>
+      <c r="M31" s="90" t="n">
         <v>96</v>
       </c>
-      <c r="K31" s="49" t="inlineStr">
+      <c r="N31" s="49" t="inlineStr">
         <is>
           <t>Legal 500 ("number of staff")</t>
         </is>
       </c>
-      <c r="L31" s="98" t="n"/>
-      <c r="M31" s="93">
-        <f>F31/J31</f>
+      <c r="O31" s="98" t="n"/>
+      <c r="P31" s="93">
+        <f>I31/M31</f>
         <v/>
       </c>
-      <c r="N31" s="98" t="n"/>
-      <c r="O31" s="98" t="n"/>
-      <c r="P31" s="98" t="n"/>
       <c r="Q31" s="98" t="n"/>
-      <c r="R31" s="49" t="inlineStr"/>
+      <c r="R31" s="98" t="n"/>
+      <c r="S31" s="98" t="n"/>
+      <c r="T31" s="98" t="n"/>
+      <c r="U31" s="49" t="inlineStr"/>
     </row>
     <row r="32">
       <c r="A32" s="90" t="n">
@@ -50466,32 +50757,39 @@
       <c r="C32" s="100" t="n">
         <v>122</v>
       </c>
-      <c r="D32" s="100" t="n">
+      <c r="D32" s="131" t="n"/>
+      <c r="E32" s="98" t="n"/>
+      <c r="F32" s="49" t="inlineStr">
+        <is>
+          <t>Not collected</t>
+        </is>
+      </c>
+      <c r="G32" s="100" t="n">
         <v>117</v>
       </c>
-      <c r="E32" s="101">
-        <f>C32/D32-1</f>
+      <c r="H32" s="101">
+        <f>C32/G32-1</f>
         <v/>
       </c>
-      <c r="F32" s="100" t="n">
+      <c r="I32" s="100" t="n">
         <v>122</v>
       </c>
-      <c r="G32" s="49" t="inlineStr">
+      <c r="J32" s="49" t="inlineStr">
         <is>
           <t>FY24/25 (Afv)</t>
         </is>
       </c>
-      <c r="H32" s="98" t="n"/>
-      <c r="I32" s="98" t="n"/>
-      <c r="J32" s="98" t="n"/>
-      <c r="K32" s="49" t="inlineStr"/>
+      <c r="K32" s="98" t="n"/>
       <c r="L32" s="98" t="n"/>
       <c r="M32" s="98" t="n"/>
-      <c r="N32" s="98" t="n"/>
+      <c r="N32" s="49" t="inlineStr"/>
       <c r="O32" s="98" t="n"/>
       <c r="P32" s="98" t="n"/>
       <c r="Q32" s="98" t="n"/>
-      <c r="R32" s="49" t="inlineStr">
+      <c r="R32" s="98" t="n"/>
+      <c r="S32" s="98" t="n"/>
+      <c r="T32" s="98" t="n"/>
+      <c r="U32" s="49" t="inlineStr">
         <is>
           <t>Headcount not researched</t>
         </is>
@@ -50510,59 +50808,71 @@
         <v>112</v>
       </c>
       <c r="D33" s="100" t="n">
+        <v>125</v>
+      </c>
+      <c r="E33" s="130">
+        <f>D33/112-1</f>
+        <v/>
+      </c>
+      <c r="F33" s="49" t="inlineStr">
+        <is>
+          <t>AB accounts: full firm</t>
+        </is>
+      </c>
+      <c r="G33" s="100" t="n">
         <v>124</v>
       </c>
-      <c r="E33" s="101">
-        <f>C33/D33-1</f>
+      <c r="H33" s="101">
+        <f>C33/G33-1</f>
         <v/>
       </c>
-      <c r="F33" s="100" t="n">
+      <c r="I33" s="100" t="n">
         <v>125</v>
       </c>
-      <c r="G33" s="49" t="inlineStr">
+      <c r="J33" s="49" t="inlineStr">
         <is>
           <t>FY2025 net sales (AB)</t>
         </is>
       </c>
-      <c r="H33" s="90" t="n">
+      <c r="K33" s="90" t="n">
         <v>13</v>
       </c>
-      <c r="I33" s="90" t="n">
+      <c r="L33" s="90" t="n">
         <v>47</v>
       </c>
-      <c r="J33" s="90" t="n">
+      <c r="M33" s="90" t="n">
         <v>46</v>
       </c>
-      <c r="K33" s="49" t="inlineStr">
+      <c r="N33" s="49" t="inlineStr">
         <is>
           <t>Firm website count Oct-26; employees 2025 accounts</t>
         </is>
       </c>
-      <c r="L33" s="92">
-        <f>F33/H33</f>
+      <c r="O33" s="92">
+        <f>I33/K33</f>
         <v/>
       </c>
-      <c r="M33" s="93">
-        <f>F33/J33</f>
+      <c r="P33" s="93">
+        <f>I33/M33</f>
         <v/>
       </c>
-      <c r="N33" s="93">
-        <f>F33/I33</f>
+      <c r="Q33" s="93">
+        <f>I33/L33</f>
         <v/>
       </c>
-      <c r="O33" s="101">
-        <f>H33/J33</f>
+      <c r="R33" s="101">
+        <f>K33/M33</f>
         <v/>
       </c>
-      <c r="P33" s="101">
-        <f>H33/I33</f>
+      <c r="S33" s="101">
+        <f>K33/L33</f>
         <v/>
       </c>
-      <c r="Q33" s="92">
-        <f>J33/H33</f>
+      <c r="T33" s="92">
+        <f>M33/K33</f>
         <v/>
       </c>
-      <c r="R33" s="49" t="inlineStr">
+      <c r="U33" s="49" t="inlineStr">
         <is>
           <t>Merged with Gro Advokatbyrå 1 Oct 2026 (~SEK 20m)</t>
         </is>
@@ -50581,59 +50891,71 @@
         <v>108</v>
       </c>
       <c r="D34" s="100" t="n">
+        <v>101</v>
+      </c>
+      <c r="E34" s="130">
+        <f>D34/108-1</f>
+        <v/>
+      </c>
+      <c r="F34" s="49" t="inlineStr">
+        <is>
+          <t>AB accounts: full firm</t>
+        </is>
+      </c>
+      <c r="G34" s="100" t="n">
         <v>89</v>
       </c>
-      <c r="E34" s="101">
-        <f>C34/D34-1</f>
+      <c r="H34" s="101">
+        <f>C34/G34-1</f>
         <v/>
       </c>
-      <c r="F34" s="100" t="n">
+      <c r="I34" s="100" t="n">
         <v>101</v>
       </c>
-      <c r="G34" s="49" t="inlineStr">
+      <c r="J34" s="49" t="inlineStr">
         <is>
           <t>FY2025 net sales (AB)</t>
         </is>
       </c>
-      <c r="H34" s="90" t="n">
+      <c r="K34" s="90" t="n">
         <v>8</v>
       </c>
-      <c r="I34" s="90" t="n">
+      <c r="L34" s="90" t="n">
         <v>37</v>
       </c>
-      <c r="J34" s="90" t="n">
+      <c r="M34" s="90" t="n">
         <v>44</v>
       </c>
-      <c r="K34" s="49" t="inlineStr">
+      <c r="N34" s="49" t="inlineStr">
         <is>
           <t>Firm website count Oct-26; employees 2025 accounts</t>
         </is>
       </c>
-      <c r="L34" s="92">
-        <f>F34/H34</f>
+      <c r="O34" s="92">
+        <f>I34/K34</f>
         <v/>
       </c>
-      <c r="M34" s="93">
-        <f>F34/J34</f>
+      <c r="P34" s="93">
+        <f>I34/M34</f>
         <v/>
       </c>
-      <c r="N34" s="93">
-        <f>F34/I34</f>
+      <c r="Q34" s="93">
+        <f>I34/L34</f>
         <v/>
       </c>
-      <c r="O34" s="101">
-        <f>H34/J34</f>
+      <c r="R34" s="101">
+        <f>K34/M34</f>
         <v/>
       </c>
-      <c r="P34" s="101">
-        <f>H34/I34</f>
+      <c r="S34" s="101">
+        <f>K34/L34</f>
         <v/>
       </c>
-      <c r="Q34" s="92">
-        <f>J34/H34</f>
+      <c r="T34" s="92">
+        <f>M34/K34</f>
         <v/>
       </c>
-      <c r="R34" s="49" t="inlineStr">
+      <c r="U34" s="49" t="inlineStr">
         <is>
           <t>Joined AGRD May-26</t>
         </is>
@@ -50653,60 +50975,67 @@
       <c r="C35" s="100" t="n">
         <v>334</v>
       </c>
-      <c r="D35" s="100" t="n">
+      <c r="D35" s="131" t="n"/>
+      <c r="E35" s="98" t="n"/>
+      <c r="F35" s="49" t="inlineStr">
+        <is>
+          <t>Not filed (KB)</t>
+        </is>
+      </c>
+      <c r="G35" s="100" t="n">
         <v>323</v>
       </c>
-      <c r="E35" s="101">
-        <f>C35/D35-1</f>
+      <c r="H35" s="101">
+        <f>C35/G35-1</f>
         <v/>
       </c>
-      <c r="F35" s="100" t="n">
+      <c r="I35" s="100" t="n">
         <v>334</v>
       </c>
-      <c r="G35" s="49" t="inlineStr">
+      <c r="J35" s="49" t="inlineStr">
         <is>
           <t>FY23/24 (Afv Apr-25; not in revised table)</t>
         </is>
       </c>
-      <c r="H35" s="90" t="n">
+      <c r="K35" s="90" t="n">
         <v>12</v>
       </c>
-      <c r="I35" s="90" t="n">
+      <c r="L35" s="90" t="n">
         <v>73</v>
       </c>
-      <c r="J35" s="90" t="n">
+      <c r="M35" s="90" t="n">
         <v>125</v>
       </c>
-      <c r="K35" s="49" t="inlineStr">
+      <c r="N35" s="49" t="inlineStr">
         <is>
           <t>Firm website count Oct-26; "~125 professionals" (Mar-26)</t>
         </is>
       </c>
-      <c r="L35" s="92">
-        <f>F35/H35</f>
+      <c r="O35" s="92">
+        <f>I35/K35</f>
         <v/>
       </c>
-      <c r="M35" s="93">
-        <f>F35/J35</f>
+      <c r="P35" s="93">
+        <f>I35/M35</f>
         <v/>
       </c>
-      <c r="N35" s="93">
-        <f>F35/I35</f>
+      <c r="Q35" s="93">
+        <f>I35/L35</f>
         <v/>
       </c>
-      <c r="O35" s="101">
-        <f>H35/J35</f>
+      <c r="R35" s="101">
+        <f>K35/M35</f>
         <v/>
       </c>
-      <c r="P35" s="101">
-        <f>H35/I35</f>
+      <c r="S35" s="101">
+        <f>K35/L35</f>
         <v/>
       </c>
-      <c r="Q35" s="92">
-        <f>J35/H35</f>
+      <c r="T35" s="92">
+        <f>M35/K35</f>
         <v/>
       </c>
-      <c r="R35" s="49" t="inlineStr">
+      <c r="U35" s="49" t="inlineStr">
         <is>
           <t>Would rank ~14</t>
         </is>
@@ -50727,40 +51056,52 @@
         <v>195</v>
       </c>
       <c r="D36" s="100" t="n">
+        <v>376</v>
+      </c>
+      <c r="E36" s="130">
+        <f>D36/422-1</f>
+        <v/>
+      </c>
+      <c r="F36" s="69" t="inlineStr">
+        <is>
+          <t>AB accounts FY May24-Apr25 vs prior year; basis unclear</t>
+        </is>
+      </c>
+      <c r="G36" s="100" t="n">
         <v>199</v>
       </c>
-      <c r="E36" s="101">
-        <f>C36/D36-1</f>
+      <c r="H36" s="101">
+        <f>C36/G36-1</f>
         <v/>
       </c>
-      <c r="F36" s="100" t="n">
+      <c r="I36" s="100" t="n">
         <v>195</v>
       </c>
-      <c r="G36" s="49" t="inlineStr">
+      <c r="J36" s="49" t="inlineStr">
         <is>
           <t>FY23/24 (Afv Apr-25; not in revised table)</t>
         </is>
       </c>
-      <c r="H36" s="98" t="n"/>
-      <c r="I36" s="98" t="n"/>
-      <c r="J36" s="90" t="n">
+      <c r="K36" s="98" t="n"/>
+      <c r="L36" s="98" t="n"/>
+      <c r="M36" s="90" t="n">
         <v>75</v>
       </c>
-      <c r="K36" s="49" t="inlineStr">
+      <c r="N36" s="49" t="inlineStr">
         <is>
           <t>AB accounts FY24/25</t>
         </is>
       </c>
-      <c r="L36" s="98" t="n"/>
-      <c r="M36" s="93">
-        <f>F36/J36</f>
+      <c r="O36" s="98" t="n"/>
+      <c r="P36" s="93">
+        <f>I36/M36</f>
         <v/>
       </c>
-      <c r="N36" s="98" t="n"/>
-      <c r="O36" s="98" t="n"/>
-      <c r="P36" s="98" t="n"/>
       <c r="Q36" s="98" t="n"/>
-      <c r="R36" s="49" t="inlineStr">
+      <c r="R36" s="98" t="n"/>
+      <c r="S36" s="98" t="n"/>
+      <c r="T36" s="98" t="n"/>
+      <c r="U36" s="49" t="inlineStr">
         <is>
           <t>AB net sales 376 (basis unclear)</t>
         </is>
@@ -50772,28 +51113,32 @@
           <t>Median (top 30)</t>
         </is>
       </c>
-      <c r="L37" s="102">
-        <f>MEDIAN(L5:L34)</f>
+      <c r="E37" s="132">
+        <f>MEDIAN(E5:E34)</f>
         <v/>
       </c>
-      <c r="M37" s="103">
-        <f>MEDIAN(M5:M34)</f>
-        <v/>
-      </c>
-      <c r="N37" s="103">
-        <f>MEDIAN(N5:N34)</f>
-        <v/>
-      </c>
-      <c r="O37" s="104">
+      <c r="O37" s="102">
         <f>MEDIAN(O5:O34)</f>
         <v/>
       </c>
-      <c r="P37" s="104">
+      <c r="P37" s="103">
         <f>MEDIAN(P5:P34)</f>
         <v/>
       </c>
-      <c r="Q37" s="102">
+      <c r="Q37" s="103">
         <f>MEDIAN(Q5:Q34)</f>
+        <v/>
+      </c>
+      <c r="R37" s="104">
+        <f>MEDIAN(R5:R34)</f>
+        <v/>
+      </c>
+      <c r="S37" s="104">
+        <f>MEDIAN(S5:S34)</f>
+        <v/>
+      </c>
+      <c r="T37" s="102">
+        <f>MEDIAN(T5:T34)</f>
         <v/>
       </c>
     </row>
@@ -50807,12 +51152,12 @@
         <f>SUM(C5:C34)</f>
         <v/>
       </c>
-      <c r="D38" s="58">
-        <f>SUM(D5:D34)</f>
+      <c r="G38" s="58">
+        <f>SUM(G5:G34)</f>
         <v/>
       </c>
-      <c r="E38" s="59">
-        <f>C38/D38-1</f>
+      <c r="H38" s="59">
+        <f>C38/G38-1</f>
         <v/>
       </c>
     </row>
@@ -50852,7 +51197,7 @@
     <row r="43">
       <c r="A43" s="45" t="inlineStr">
         <is>
-          <t>Units: SEK m; ratios in SEK m per head. Revenue per partner/employee/lawyer uses "Latest revenue" (column F).</t>
+          <t>Units: SEK m; ratios in SEK m per head. Revenue per partner/employee/lawyer uses "Latest revenue" (column I). FY2025 YoY is like-for-like on the same basis (company accounts vs prior-year company accounts; group vs group); yellow = partial entity coverage, press figure or unclear basis. The full Afv FY2025 table is paywalled; limited partnerships (KB) do not file.</t>
         </is>
       </c>
     </row>
@@ -51326,11 +51671,11 @@
     <mergeCell ref="C58:E58"/>
     <mergeCell ref="C60:E60"/>
     <mergeCell ref="C50:E50"/>
-    <mergeCell ref="C57:E57"/>
+    <mergeCell ref="A2:U2"/>
     <mergeCell ref="C52:E52"/>
     <mergeCell ref="C55:E55"/>
-    <mergeCell ref="A2:R2"/>
     <mergeCell ref="C53:E53"/>
+    <mergeCell ref="C57:E57"/>
     <mergeCell ref="C61:E61"/>
     <mergeCell ref="C49:E49"/>
     <mergeCell ref="C56:E56"/>

</xml_diff>